<commit_message>
CRM actualizado — 06/05/2026 17:41
</commit_message>
<xml_diff>
--- a/CRM_PowerBI_BrendaLuna_actualizado.xlsx
+++ b/CRM_PowerBI_BrendaLuna_actualizado.xlsx
@@ -1,25 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CRM_Datos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="CRM_Datos" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,29 +27,13 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="10"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF1F3864"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFCE4D6"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -64,18 +48,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -439,3243 +417,3031 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:M75"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
-  <cols>
-    <col width="59.85546875" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="12.28515625" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="22.42578125" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="23" bestFit="1" customWidth="1" min="4" max="4"/>
-    <col width="65.28515625" bestFit="1" customWidth="1" min="5" max="5"/>
-    <col width="25.7109375" bestFit="1" customWidth="1" min="6" max="6"/>
-    <col width="18.140625" bestFit="1" customWidth="1" min="7" max="8"/>
-    <col width="12.85546875" bestFit="1" customWidth="1" min="9" max="9"/>
-    <col width="14" bestFit="1" customWidth="1" min="10" max="10"/>
-    <col width="10.85546875" bestFit="1" customWidth="1" min="11" max="11"/>
-    <col width="11.42578125" bestFit="1" customWidth="1" min="12" max="12"/>
-    <col width="18.85546875" bestFit="1" customWidth="1" min="13" max="13"/>
-  </cols>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Correo_electronico</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Etapa</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Ingreso_esperado_COP</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Nombre_contacto</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Oportunidad</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Vendedor</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Fecha_creacion</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Fecha_cierre</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Semana_ISO</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Anio_creacion</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Mes_cierre</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Anio_cierre</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Es_Lead_Calificado</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>macaballero@comfenalcovalle.com.co</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>Contactado</t>
         </is>
       </c>
-      <c r="C2" s="2" t="n">
+      <c r="C2" t="n">
         <v>10000000</v>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Maria Alejandra Caballero Martínez</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>WAB Gestión Equipo Comercial</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Richard Castaño</t>
         </is>
       </c>
-      <c r="G2" s="3" t="n">
+      <c r="G2" s="1" t="n">
         <v>46148.44212962963</v>
       </c>
-      <c r="H2" s="4" t="n">
+      <c r="H2" s="1" t="n">
         <v>46163</v>
       </c>
-      <c r="I2" s="2" t="n">
+      <c r="I2" t="n">
         <v>19</v>
       </c>
-      <c r="J2" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K2" s="2" t="n">
+      <c r="J2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K2" t="n">
         <v>5</v>
       </c>
-      <c r="L2" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="L2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M2" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>mflorez@comfenalcovalle.com.co</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Negociación</t>
         </is>
       </c>
-      <c r="C3" s="2" t="n">
-        <v>9000000</v>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="C3" t="n">
+        <v>11000000</v>
+      </c>
+      <c r="D3" t="inlineStr">
         <is>
           <t>Monica Florez</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Seguros de la gente Comfenalco EPS</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="n">
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G3" s="1" t="n">
         <v>46106.60332175926</v>
       </c>
-      <c r="H3" s="3" t="n">
+      <c r="H3" s="1" t="n">
         <v>46167</v>
       </c>
-      <c r="I3" s="2" t="n">
+      <c r="I3" t="n">
         <v>13</v>
       </c>
-      <c r="J3" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K3" s="2" t="n">
+      <c r="J3" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K3" t="n">
         <v>5</v>
       </c>
-      <c r="L3" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M3" s="2" t="inlineStr">
+      <c r="L3" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M3" t="inlineStr">
         <is>
           <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>medifar624@gmail.com</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>Ganado</t>
         </is>
       </c>
-      <c r="C4" s="2" t="n">
+      <c r="C4" t="n">
         <v>11491202</v>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>Daniel Gallo</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>Oportunidad de MEDISFARMA SAS</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="n">
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G4" s="1" t="n">
         <v>46091.44133101852</v>
       </c>
-      <c r="H4" s="4" t="n">
+      <c r="H4" s="1" t="n">
         <v>46146</v>
       </c>
-      <c r="I4" s="2" t="n">
+      <c r="I4" t="n">
         <v>11</v>
       </c>
-      <c r="J4" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K4" s="2" t="n">
+      <c r="J4" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K4" t="n">
         <v>5</v>
       </c>
-      <c r="L4" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="L4" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M4" t="inlineStr">
         <is>
           <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>auditoria@clinicalosandes.com</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>Ganado</t>
         </is>
       </c>
-      <c r="C5" s="2" t="n">
+      <c r="C5" t="n">
         <v>16914000</v>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>Juan Carlos Garcia</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>BPO Clinica Los Andes Asignacion de Citas y SC</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="n">
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G5" s="1" t="n">
         <v>46056.62674768519</v>
       </c>
-      <c r="H5" s="4" t="n">
+      <c r="H5" s="1" t="n">
         <v>46146</v>
       </c>
-      <c r="I5" s="2" t="n">
+      <c r="I5" t="n">
         <v>6</v>
       </c>
-      <c r="J5" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K5" s="2" t="n">
+      <c r="J5" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K5" t="n">
         <v>5</v>
       </c>
-      <c r="L5" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M5" s="2" t="inlineStr">
+      <c r="L5" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M5" t="inlineStr">
         <is>
           <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>ingrid.torres@archies.co</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>Ganado</t>
         </is>
       </c>
-      <c r="C6" s="2" t="n">
+      <c r="C6" t="n">
         <v>30000000</v>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>INGRID TORRES</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>SERVICIO BPO - DOMICILIOS</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>Richard Castaño</t>
         </is>
       </c>
-      <c r="G6" s="3" t="n">
+      <c r="G6" s="1" t="n">
         <v>46037.44476851852</v>
       </c>
-      <c r="H6" s="4" t="n">
+      <c r="H6" s="1" t="n">
         <v>46079</v>
       </c>
-      <c r="I6" s="2" t="n">
+      <c r="I6" t="n">
         <v>3</v>
       </c>
-      <c r="J6" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K6" s="2" t="n">
+      <c r="J6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K6" t="n">
         <v>2</v>
       </c>
-      <c r="L6" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="L6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M6" t="inlineStr">
         <is>
           <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n"/>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>Ganado</t>
         </is>
       </c>
-      <c r="C7" s="2" t="n">
+      <c r="C7" t="n">
         <v>2674000</v>
       </c>
-      <c r="D7" s="2" t="n"/>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>Desarrollo Bot</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>Richard Castaño</t>
         </is>
       </c>
-      <c r="G7" s="3" t="n">
+      <c r="G7" s="1" t="n">
         <v>45965.4525</v>
       </c>
-      <c r="H7" s="4" t="n">
+      <c r="H7" s="1" t="n">
         <v>46108</v>
       </c>
-      <c r="I7" s="2" t="n">
+      <c r="I7" t="n">
         <v>45</v>
       </c>
-      <c r="J7" s="2" t="n">
+      <c r="J7" t="n">
         <v>2025</v>
       </c>
-      <c r="K7" s="2" t="n">
+      <c r="K7" t="n">
         <v>3</v>
       </c>
-      <c r="L7" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="L7" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M7" t="inlineStr">
         <is>
           <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n"/>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>Ganado</t>
         </is>
       </c>
-      <c r="C8" s="2" t="n">
+      <c r="C8" t="n">
         <v>10300000</v>
       </c>
-      <c r="D8" s="2" t="n"/>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>Agentes Contact Center</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>Richard Castaño</t>
         </is>
       </c>
-      <c r="G8" s="3" t="n">
+      <c r="G8" s="1" t="n">
         <v>45940.49733796297</v>
       </c>
-      <c r="H8" s="4" t="n">
+      <c r="H8" s="1" t="n">
         <v>46027</v>
       </c>
-      <c r="I8" s="2" t="n">
+      <c r="I8" t="n">
         <v>41</v>
       </c>
-      <c r="J8" s="2" t="n">
+      <c r="J8" t="n">
         <v>2025</v>
       </c>
-      <c r="K8" s="2" t="n">
+      <c r="K8" t="n">
         <v>1</v>
       </c>
-      <c r="L8" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="L8" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M8" t="inlineStr">
         <is>
           <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>stefania.bolivar@clinicadeoccidente.com</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>Seguimiento</t>
         </is>
       </c>
-      <c r="C9" s="2" t="n">
+      <c r="C9" t="n">
         <v>40000000</v>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>STEFANIA BOLIVAR</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>Oportunidad Clinica de Occidente</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>Richard Castaño</t>
         </is>
       </c>
-      <c r="G9" s="3" t="n">
+      <c r="G9" s="1" t="n">
         <v>45916.67493055556</v>
       </c>
-      <c r="H9" s="4" t="n">
+      <c r="H9" s="1" t="n">
         <v>45930</v>
       </c>
-      <c r="I9" s="2" t="n">
+      <c r="I9" t="n">
         <v>38</v>
       </c>
-      <c r="J9" s="2" t="n">
+      <c r="J9" t="n">
         <v>2025</v>
       </c>
-      <c r="K9" s="2" t="n">
+      <c r="K9" t="n">
         <v>9</v>
       </c>
-      <c r="L9" s="2" t="n">
+      <c r="L9" t="n">
         <v>2025</v>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>cserna@surtifamiliar.com.co</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>Ganado</t>
         </is>
       </c>
-      <c r="C10" s="2" t="n">
+      <c r="C10" t="n">
         <v>5800000</v>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>Claudia Patricia Serna</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>Nuevo CRM 360, Agente IA y Audio IA</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>Richard Castaño</t>
         </is>
       </c>
-      <c r="G10" s="3" t="n">
+      <c r="G10" s="1" t="n">
         <v>45915.47034722222</v>
       </c>
-      <c r="H10" s="4" t="n">
+      <c r="H10" s="1" t="n">
         <v>46141</v>
       </c>
-      <c r="I10" s="2" t="n">
+      <c r="I10" t="n">
         <v>38</v>
       </c>
-      <c r="J10" s="2" t="n">
+      <c r="J10" t="n">
         <v>2025</v>
       </c>
-      <c r="K10" s="2" t="n">
+      <c r="K10" t="n">
         <v>4</v>
       </c>
-      <c r="L10" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="L10" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M10" t="inlineStr">
         <is>
           <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n"/>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>Nuevo</t>
         </is>
       </c>
-      <c r="C11" s="2" t="n">
+      <c r="C11" t="n">
         <v>0</v>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>MADERKIT</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>Oportunidad de MADERKIT</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G11" s="3" t="n">
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G11" s="1" t="n">
         <v>46147.66540509259</v>
       </c>
-      <c r="H11" s="3" t="n"/>
-      <c r="I11" s="2" t="n">
+      <c r="I11" t="n">
         <v>19</v>
       </c>
-      <c r="J11" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K11" s="2" t="n"/>
-      <c r="L11" s="2" t="n"/>
-      <c r="M11" s="2" t="inlineStr">
+      <c r="J11" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M11" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>omer120395@gmail.com</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>Nuevo</t>
         </is>
       </c>
-      <c r="C12" s="2" t="n">
+      <c r="C12" t="n">
         <v>0</v>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>Omer Peñaloza</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>Oportunidad de Omer Peñaloza</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="n">
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G12" s="1" t="n">
         <v>46147.66090277778</v>
       </c>
-      <c r="H12" s="2" t="n"/>
-      <c r="I12" s="2" t="n">
+      <c r="I12" t="n">
         <v>19</v>
       </c>
-      <c r="J12" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K12" s="2" t="n"/>
-      <c r="L12" s="2" t="n"/>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="J12" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M12" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" t="inlineStr">
         <is>
           <t>directora.it@supermercadobelalcazar.com.co</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>Contactado</t>
         </is>
       </c>
-      <c r="C13" s="2" t="n">
+      <c r="C13" t="n">
         <v>6000000</v>
       </c>
-      <c r="D13" s="2" t="n"/>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>Oportunidad de ABASTECEMOS DE OCCIDENTE</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="n">
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G13" s="1" t="n">
         <v>46147.64170138889</v>
       </c>
-      <c r="H13" s="4" t="n">
+      <c r="H13" s="1" t="n">
         <v>46157</v>
       </c>
-      <c r="I13" s="2" t="n">
+      <c r="I13" t="n">
         <v>19</v>
       </c>
-      <c r="J13" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K13" s="2" t="n">
+      <c r="J13" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K13" t="n">
         <v>5</v>
       </c>
-      <c r="L13" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M13" s="2" t="inlineStr">
+      <c r="L13" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M13" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" t="inlineStr">
         <is>
           <t>oscar.molina@terrenoshouston.com</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>Propuesta</t>
         </is>
       </c>
-      <c r="C14" s="2" t="n">
+      <c r="C14" t="n">
         <v>37623040</v>
       </c>
-      <c r="D14" s="2" t="n"/>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>Oportunidad de COLONY RIDGE</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="n">
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G14" s="1" t="n">
         <v>46147.60297453704</v>
       </c>
-      <c r="H14" s="4" t="n">
+      <c r="H14" s="1" t="n">
         <v>46150</v>
       </c>
-      <c r="I14" s="2" t="n">
+      <c r="I14" t="n">
         <v>19</v>
       </c>
-      <c r="J14" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K14" s="2" t="n">
+      <c r="J14" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K14" t="n">
         <v>5</v>
       </c>
-      <c r="L14" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M14" s="2" t="inlineStr">
+      <c r="L14" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M14" t="inlineStr">
         <is>
           <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="A15" t="inlineStr">
         <is>
           <t>jsantacr@ccc.org.co</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>Contactado</t>
         </is>
       </c>
-      <c r="C15" s="2" t="n">
+      <c r="C15" t="n">
         <v>55000000</v>
       </c>
-      <c r="D15" s="2" t="n"/>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>Oportunidad de CAMARA DE COMERCIO CALI</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G15" s="3" t="n">
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G15" s="1" t="n">
         <v>46141.62370370371</v>
       </c>
-      <c r="H15" s="4" t="n">
+      <c r="H15" s="1" t="n">
         <v>46289</v>
       </c>
-      <c r="I15" s="2" t="n">
+      <c r="I15" t="n">
         <v>18</v>
       </c>
-      <c r="J15" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K15" s="2" t="n">
+      <c r="J15" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K15" t="n">
         <v>9</v>
       </c>
-      <c r="L15" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M15" s="2" t="inlineStr">
+      <c r="L15" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M15" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="A16" t="inlineStr">
         <is>
           <t>exportaciones@laprovincia.com</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>Nuevo</t>
         </is>
       </c>
-      <c r="C16" s="2" t="n">
+      <c r="C16" t="n">
         <v>6000000</v>
       </c>
-      <c r="D16" s="2" t="n"/>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>Oportunidad de PRODUCTOS LA PROVINCIA SAS</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G16" s="3" t="n">
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G16" s="1" t="n">
         <v>46141.62021990741</v>
       </c>
-      <c r="H16" s="2" t="n"/>
-      <c r="I16" s="2" t="n">
+      <c r="I16" t="n">
         <v>18</v>
       </c>
-      <c r="J16" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K16" s="2" t="n"/>
-      <c r="L16" s="2" t="n"/>
-      <c r="M16" s="2" t="inlineStr">
+      <c r="J16" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M16" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A17" t="inlineStr">
         <is>
           <t>coordinador.mercadeo@regency.com.co</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="n">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
         <v>0</v>
       </c>
-      <c r="D17" s="2" t="n"/>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>Oportunidad de REGENCY TECH SAS</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G17" s="3" t="n">
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G17" s="1" t="n">
         <v>46141.59664351852</v>
       </c>
-      <c r="H17" s="2" t="n"/>
-      <c r="I17" s="2" t="n">
+      <c r="I17" t="n">
         <v>18</v>
       </c>
-      <c r="J17" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K17" s="2" t="n"/>
-      <c r="L17" s="2" t="n"/>
-      <c r="M17" s="2" t="inlineStr">
+      <c r="J17" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M17" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="n"/>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>Contactado</t>
         </is>
       </c>
-      <c r="C18" s="2" t="n">
+      <c r="C18" t="n">
         <v>1200000000</v>
       </c>
-      <c r="D18" s="2" t="n"/>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>Oportunidad de EMCALI E.I.C.E ESP</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G18" s="3" t="n">
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G18" s="1" t="n">
         <v>46141.59045138889</v>
       </c>
-      <c r="H18" s="3" t="n">
+      <c r="H18" s="1" t="n">
         <v>46352</v>
       </c>
-      <c r="I18" s="2" t="n">
+      <c r="I18" t="n">
         <v>18</v>
       </c>
-      <c r="J18" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K18" s="2" t="n">
+      <c r="J18" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K18" t="n">
         <v>11</v>
       </c>
-      <c r="L18" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M18" s="2" t="inlineStr">
+      <c r="L18" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M18" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="A19" t="inlineStr">
         <is>
           <t>angie_feligrana@eficacia.com.co</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>Negociación</t>
         </is>
       </c>
-      <c r="C19" s="2" t="n">
+      <c r="C19" t="n">
         <v>6000000</v>
       </c>
-      <c r="D19" s="2" t="n"/>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>Oportunidad de Eficacia sas / Angie Feligrana</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G19" s="3" t="n">
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G19" s="1" t="n">
         <v>46126.63210648148</v>
       </c>
-      <c r="H19" s="4" t="n">
+      <c r="H19" s="1" t="n">
         <v>46150</v>
       </c>
-      <c r="I19" s="2" t="n">
+      <c r="I19" t="n">
         <v>16</v>
       </c>
-      <c r="J19" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K19" s="2" t="n">
+      <c r="J19" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K19" t="n">
         <v>5</v>
       </c>
-      <c r="L19" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M19" s="2" t="inlineStr">
+      <c r="L19" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M19" t="inlineStr">
         <is>
           <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="A20" t="inlineStr">
         <is>
           <t>Estrategiadigital@zuluagaysoto.com</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="n">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
         <v>0</v>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>Maryuri Arguello</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>Oportunidad de Maryuri Arguello</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G20" s="3" t="n">
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G20" s="1" t="n">
         <v>46125.71925925926</v>
       </c>
-      <c r="H20" s="2" t="n"/>
-      <c r="I20" s="2" t="n">
+      <c r="I20" t="n">
         <v>16</v>
       </c>
-      <c r="J20" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K20" s="2" t="n"/>
-      <c r="L20" s="2" t="n"/>
-      <c r="M20" s="2" t="inlineStr">
+      <c r="J20" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M20" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="A21" t="inlineStr">
         <is>
           <t>gabrielrodriguez@arrozsupremo.com</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>Ganado</t>
         </is>
       </c>
-      <c r="C21" s="2" t="n">
+      <c r="C21" t="n">
         <v>8000000</v>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>GABRIEL RODRIGUEZ</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>Agente de Ventas</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>Richard Castaño</t>
         </is>
       </c>
-      <c r="G21" s="3" t="n">
+      <c r="G21" s="1" t="n">
         <v>46119.62108796297</v>
       </c>
-      <c r="H21" s="4" t="n">
+      <c r="H21" s="1" t="n">
         <v>46141</v>
       </c>
-      <c r="I21" s="2" t="n">
+      <c r="I21" t="n">
         <v>15</v>
       </c>
-      <c r="J21" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K21" s="2" t="n">
+      <c r="J21" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K21" t="n">
         <v>4</v>
       </c>
-      <c r="L21" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M21" s="2" t="inlineStr">
+      <c r="L21" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M21" t="inlineStr">
         <is>
           <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="A22" t="inlineStr">
         <is>
           <t>Belkis.jimenez@agrauto.com.co</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="n">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
         <v>0</v>
       </c>
-      <c r="D22" s="2" t="n"/>
-      <c r="E22" s="2" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>Oportunidad de AGRICOLA AUTOMOTRIZ SAS</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G22" s="3" t="n">
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G22" s="1" t="n">
         <v>46119.38914351852</v>
       </c>
-      <c r="H22" s="3" t="n"/>
-      <c r="I22" s="2" t="n">
+      <c r="I22" t="n">
         <v>15</v>
       </c>
-      <c r="J22" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K22" s="2" t="n"/>
-      <c r="L22" s="2" t="n"/>
-      <c r="M22" s="2" t="inlineStr">
+      <c r="J22" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M22" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+      <c r="A23" t="inlineStr">
         <is>
           <t>anyela.aponza@cotel.com.co</t>
         </is>
       </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="n">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
         <v>0</v>
       </c>
-      <c r="D23" s="2" t="n"/>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>Oportunidad de COTEL SAL</t>
         </is>
       </c>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G23" s="3" t="n">
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G23" s="1" t="n">
         <v>46112.61271990741</v>
       </c>
-      <c r="H23" s="2" t="n"/>
-      <c r="I23" s="2" t="n">
+      <c r="I23" t="n">
         <v>14</v>
       </c>
-      <c r="J23" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K23" s="2" t="n"/>
-      <c r="L23" s="2" t="n"/>
-      <c r="M23" s="2" t="inlineStr">
+      <c r="J23" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M23" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
+      <c r="A24" t="inlineStr">
         <is>
           <t>liliana.patino@quironsalud.com</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="n">
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
         <v>0</v>
       </c>
-      <c r="D24" s="2" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>CLINICA IMBANACO</t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>Oportunidad de Liliana Patiño Flórez</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G24" s="3" t="n">
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G24" s="1" t="n">
         <v>46112.60853009259</v>
       </c>
-      <c r="H24" s="2" t="n"/>
-      <c r="I24" s="2" t="n">
+      <c r="I24" t="n">
         <v>14</v>
       </c>
-      <c r="J24" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K24" s="2" t="n"/>
-      <c r="L24" s="2" t="n"/>
-      <c r="M24" s="2" t="inlineStr">
+      <c r="J24" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M24" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
+      <c r="A25" t="inlineStr">
         <is>
           <t>casanchez@jgb.com.co</t>
         </is>
       </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="n">
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
         <v>0</v>
       </c>
-      <c r="D25" s="2" t="n"/>
-      <c r="E25" s="2" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>Oportunidad de JGB S.A.</t>
         </is>
       </c>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G25" s="3" t="n">
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G25" s="1" t="n">
         <v>46112.6052662037</v>
       </c>
-      <c r="H25" s="3" t="n"/>
-      <c r="I25" s="2" t="n">
+      <c r="I25" t="n">
         <v>14</v>
       </c>
-      <c r="J25" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K25" s="2" t="n"/>
-      <c r="L25" s="2" t="n"/>
-      <c r="M25" s="2" t="inlineStr">
+      <c r="J25" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M25" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="A26" t="inlineStr">
         <is>
           <t>damaris.gomez@disfarma.com.co</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>Propuesta</t>
         </is>
       </c>
-      <c r="C26" s="2" t="n">
+      <c r="C26" t="n">
         <v>0</v>
       </c>
-      <c r="D26" s="2" t="n"/>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="E26" t="inlineStr">
         <is>
           <t>Oportunidad de DISFARMA</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G26" s="3" t="n">
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G26" s="1" t="n">
         <v>46112.60325231482</v>
       </c>
-      <c r="H26" s="2" t="n"/>
-      <c r="I26" s="2" t="n">
+      <c r="I26" t="n">
         <v>14</v>
       </c>
-      <c r="J26" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K26" s="2" t="n"/>
-      <c r="L26" s="2" t="n"/>
-      <c r="M26" s="2" t="inlineStr">
+      <c r="J26" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M26" t="inlineStr">
         <is>
           <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
+      <c r="A27" t="inlineStr">
         <is>
           <t>alergologosdeoccidente@gmail.com</t>
         </is>
       </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="n">
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
         <v>0</v>
       </c>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>Johana Gonzalez</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
+      <c r="E27" t="inlineStr">
         <is>
           <t>Oportunidad de Johana Gonzalez</t>
         </is>
       </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G27" s="3" t="n">
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G27" s="1" t="n">
         <v>46107.51248842593</v>
       </c>
-      <c r="H27" s="2" t="n"/>
-      <c r="I27" s="2" t="n">
+      <c r="I27" t="n">
         <v>13</v>
       </c>
-      <c r="J27" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K27" s="2" t="n"/>
-      <c r="L27" s="2" t="n"/>
-      <c r="M27" s="2" t="inlineStr">
+      <c r="J27" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M27" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr">
+      <c r="A28" t="inlineStr">
         <is>
           <t>DavidEsteban.Porras@alfalaval.com</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B28" t="inlineStr">
         <is>
           <t>Ganado</t>
         </is>
       </c>
-      <c r="C28" s="2" t="n">
+      <c r="C28" t="n">
         <v>15000000</v>
       </c>
-      <c r="D28" s="2" t="n"/>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="E28" t="inlineStr">
         <is>
           <t>Oportunidad de OPORTUNIDAD ENCUESTAS ALFALAVAL</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="F28" t="inlineStr">
         <is>
           <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
-      <c r="G28" s="3" t="n">
+      <c r="G28" s="1" t="n">
         <v>46101.72893518519</v>
       </c>
-      <c r="H28" s="4" t="n">
+      <c r="H28" s="1" t="n">
         <v>46141</v>
       </c>
-      <c r="I28" s="2" t="n">
+      <c r="I28" t="n">
         <v>12</v>
       </c>
-      <c r="J28" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K28" s="2" t="n">
+      <c r="J28" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K28" t="n">
         <v>4</v>
       </c>
-      <c r="L28" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M28" s="2" t="inlineStr">
+      <c r="L28" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M28" t="inlineStr">
         <is>
           <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr">
+      <c r="A29" t="inlineStr">
         <is>
           <t>Dr.arcarmona@gmail.com</t>
         </is>
       </c>
-      <c r="B29" s="2" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>Contactado</t>
         </is>
       </c>
-      <c r="C29" s="2" t="n">
+      <c r="C29" t="n">
         <v>0</v>
       </c>
-      <c r="D29" s="2" t="n"/>
-      <c r="E29" s="2" t="inlineStr">
+      <c r="E29" t="inlineStr">
         <is>
           <t>Oportunidad de GAMANUCLEAR LTDA - Dr Alberto Carmona</t>
         </is>
       </c>
-      <c r="F29" s="2" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G29" s="3" t="n">
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G29" s="1" t="n">
         <v>46098.65114583333</v>
       </c>
-      <c r="H29" s="3" t="n"/>
-      <c r="I29" s="2" t="n">
+      <c r="I29" t="n">
         <v>12</v>
       </c>
-      <c r="J29" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K29" s="2" t="n"/>
-      <c r="L29" s="2" t="n"/>
-      <c r="M29" s="2" t="inlineStr">
+      <c r="J29" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M29" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
+      <c r="A30" t="inlineStr">
         <is>
           <t>cecilia.guevara@cosmitet.net / administracion.crd@cosmitet.net</t>
         </is>
       </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="n">
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
         <v>0</v>
       </c>
-      <c r="D30" s="2" t="inlineStr">
+      <c r="D30" t="inlineStr">
         <is>
           <t>Cecilia Guevara</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr">
+      <c r="E30" t="inlineStr">
         <is>
           <t>Oportunidad de CLINICA REY DAVID Walter Charria</t>
         </is>
       </c>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G30" s="3" t="n">
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G30" s="1" t="n">
         <v>46094.69002314815</v>
       </c>
-      <c r="H30" s="2" t="n"/>
-      <c r="I30" s="2" t="n">
+      <c r="I30" t="n">
         <v>11</v>
       </c>
-      <c r="J30" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K30" s="2" t="n"/>
-      <c r="L30" s="2" t="n"/>
-      <c r="M30" s="2" t="inlineStr">
+      <c r="J30" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M30" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="inlineStr">
+      <c r="A31" t="inlineStr">
         <is>
           <t>vicerrectoriacademica@unicatolica.edu.co</t>
         </is>
       </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="n">
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
         <v>0</v>
       </c>
-      <c r="D31" s="2" t="inlineStr">
+      <c r="D31" t="inlineStr">
         <is>
           <t>Jorge Silva</t>
         </is>
       </c>
-      <c r="E31" s="2" t="inlineStr">
+      <c r="E31" t="inlineStr">
         <is>
           <t>Oportunidad de Jorge Silva</t>
         </is>
       </c>
-      <c r="F31" s="2" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G31" s="3" t="n">
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G31" s="1" t="n">
         <v>46094.66880787037</v>
       </c>
-      <c r="H31" s="2" t="n"/>
-      <c r="I31" s="2" t="n">
+      <c r="I31" t="n">
         <v>11</v>
       </c>
-      <c r="J31" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K31" s="2" t="n"/>
-      <c r="L31" s="2" t="n"/>
-      <c r="M31" s="2" t="inlineStr">
+      <c r="J31" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M31" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr">
+      <c r="A32" t="inlineStr">
         <is>
           <t>pedroperea02@gmail.com</t>
         </is>
       </c>
-      <c r="B32" s="2" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>Ganado</t>
         </is>
       </c>
-      <c r="C32" s="2" t="n">
+      <c r="C32" t="n">
         <v>2160000</v>
       </c>
-      <c r="D32" s="2" t="inlineStr">
+      <c r="D32" t="inlineStr">
         <is>
           <t>Pedro Pablo Perea Mafla</t>
         </is>
       </c>
-      <c r="E32" s="2" t="inlineStr">
+      <c r="E32" t="inlineStr">
         <is>
           <t>Oportunidad de Encuestas</t>
         </is>
       </c>
-      <c r="F32" s="2" t="inlineStr">
+      <c r="F32" t="inlineStr">
         <is>
           <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
-      <c r="G32" s="3" t="n">
+      <c r="G32" s="1" t="n">
         <v>46094.65905092593</v>
       </c>
-      <c r="H32" s="4" t="n">
+      <c r="H32" s="1" t="n">
         <v>46141</v>
       </c>
-      <c r="I32" s="2" t="n">
+      <c r="I32" t="n">
         <v>11</v>
       </c>
-      <c r="J32" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K32" s="2" t="n">
+      <c r="J32" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K32" t="n">
         <v>4</v>
       </c>
-      <c r="L32" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M32" s="2" t="inlineStr">
+      <c r="L32" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M32" t="inlineStr">
         <is>
           <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
+      <c r="A33" t="inlineStr">
         <is>
           <t>cristina.papamija@bmm.com.co</t>
         </is>
       </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="n">
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
         <v>8071000</v>
       </c>
-      <c r="D33" s="2" t="n"/>
-      <c r="E33" s="2" t="inlineStr">
+      <c r="E33" t="inlineStr">
         <is>
           <t>Oportunidad de BANCO MUNDO MUJER</t>
         </is>
       </c>
-      <c r="F33" s="2" t="inlineStr">
+      <c r="F33" t="inlineStr">
         <is>
           <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
-      <c r="G33" s="3" t="n">
+      <c r="G33" s="1" t="n">
         <v>46094.65019675926</v>
       </c>
-      <c r="H33" s="2" t="n"/>
-      <c r="I33" s="2" t="n">
+      <c r="I33" t="n">
         <v>11</v>
       </c>
-      <c r="J33" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K33" s="2" t="n"/>
-      <c r="L33" s="2" t="n"/>
-      <c r="M33" s="2" t="inlineStr">
+      <c r="J33" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M33" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr">
+      <c r="A34" t="inlineStr">
         <is>
           <t>capacitacionvirtual@fundacionwwbcol.org</t>
         </is>
       </c>
-      <c r="B34" s="2" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>Propuesta</t>
         </is>
       </c>
-      <c r="C34" s="2" t="n">
+      <c r="C34" t="n">
         <v>1600000</v>
       </c>
-      <c r="D34" s="2" t="n"/>
-      <c r="E34" s="2" t="inlineStr">
+      <c r="E34" t="inlineStr">
         <is>
           <t>Licenciamiento y ajuste WhatsApp FUNDACIÓN WWB</t>
         </is>
       </c>
-      <c r="F34" s="2" t="inlineStr">
+      <c r="F34" t="inlineStr">
         <is>
           <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
-      <c r="G34" s="3" t="n">
+      <c r="G34" s="1" t="n">
         <v>46094.64826388889</v>
       </c>
-      <c r="H34" s="2" t="n"/>
-      <c r="I34" s="2" t="n">
+      <c r="I34" t="n">
         <v>11</v>
       </c>
-      <c r="J34" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K34" s="2" t="n"/>
-      <c r="L34" s="2" t="n"/>
-      <c r="M34" s="2" t="inlineStr">
+      <c r="J34" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M34" t="inlineStr">
         <is>
           <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="inlineStr">
+      <c r="A35" t="inlineStr">
         <is>
           <t>carol.cuesta@cbolivar.com</t>
         </is>
       </c>
-      <c r="B35" s="2" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>Ganado</t>
         </is>
       </c>
-      <c r="C35" s="2" t="n">
+      <c r="C35" t="n">
         <v>2900000</v>
       </c>
-      <c r="D35" s="2" t="inlineStr">
+      <c r="D35" t="inlineStr">
         <is>
           <t>CAROL CUESTA</t>
         </is>
       </c>
-      <c r="E35" s="2" t="inlineStr">
+      <c r="E35" t="inlineStr">
         <is>
           <t>Gestión de Subsidios CB Bogotá</t>
         </is>
       </c>
-      <c r="F35" s="2" t="inlineStr">
+      <c r="F35" t="inlineStr">
         <is>
           <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
-      <c r="G35" s="3" t="n">
+      <c r="G35" s="1" t="n">
         <v>46094.64454861111</v>
       </c>
-      <c r="H35" s="4" t="n">
+      <c r="H35" s="1" t="n">
         <v>46135</v>
       </c>
-      <c r="I35" s="2" t="n">
+      <c r="I35" t="n">
         <v>11</v>
       </c>
-      <c r="J35" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K35" s="2" t="n">
+      <c r="J35" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K35" t="n">
         <v>4</v>
       </c>
-      <c r="L35" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M35" s="2" t="inlineStr">
+      <c r="L35" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M35" t="inlineStr">
         <is>
           <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="A36" t="inlineStr">
         <is>
           <t>edwin.munoz.v@uniminuto.edu</t>
         </is>
       </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C36" s="2" t="n">
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
         <v>0</v>
       </c>
-      <c r="D36" s="2" t="n"/>
-      <c r="E36" s="2" t="inlineStr">
+      <c r="E36" t="inlineStr">
         <is>
           <t>Oportunidad de UNIMINUTO</t>
         </is>
       </c>
-      <c r="F36" s="2" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G36" s="3" t="n">
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G36" s="1" t="n">
         <v>46092.63626157407</v>
       </c>
-      <c r="H36" s="2" t="n"/>
-      <c r="I36" s="2" t="n">
+      <c r="I36" t="n">
         <v>11</v>
       </c>
-      <c r="J36" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K36" s="2" t="n"/>
-      <c r="L36" s="2" t="n"/>
-      <c r="M36" s="2" t="inlineStr">
+      <c r="J36" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M36" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="inlineStr">
+      <c r="A37" t="inlineStr">
         <is>
           <t>jaime_zuluaga@eficacia.com.co</t>
         </is>
       </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C37" s="2" t="n">
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
         <v>0</v>
       </c>
-      <c r="D37" s="2" t="inlineStr">
+      <c r="D37" t="inlineStr">
         <is>
           <t>Jaime Alberto</t>
         </is>
       </c>
-      <c r="E37" s="2" t="inlineStr">
+      <c r="E37" t="inlineStr">
         <is>
           <t>Oportunidad de Jaime Alberto Zuluaga</t>
         </is>
       </c>
-      <c r="F37" s="2" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G37" s="3" t="n">
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G37" s="1" t="n">
         <v>46092.63153935185</v>
       </c>
-      <c r="H37" s="2" t="n"/>
-      <c r="I37" s="2" t="n">
+      <c r="I37" t="n">
         <v>11</v>
       </c>
-      <c r="J37" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K37" s="2" t="n"/>
-      <c r="L37" s="2" t="n"/>
-      <c r="M37" s="2" t="inlineStr">
+      <c r="J37" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M37" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="inlineStr">
+      <c r="A38" t="inlineStr">
         <is>
           <t>comercial@isyscol.com</t>
         </is>
       </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="n">
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
         <v>0</v>
       </c>
-      <c r="D38" s="2" t="inlineStr">
+      <c r="D38" t="inlineStr">
         <is>
           <t>Andres Nader</t>
         </is>
       </c>
-      <c r="E38" s="2" t="inlineStr">
+      <c r="E38" t="inlineStr">
         <is>
           <t>Oportunidad de Andres Nader</t>
         </is>
       </c>
-      <c r="F38" s="2" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G38" s="3" t="n">
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G38" s="1" t="n">
         <v>46091.59211805555</v>
       </c>
-      <c r="H38" s="2" t="n"/>
-      <c r="I38" s="2" t="n">
+      <c r="I38" t="n">
         <v>11</v>
       </c>
-      <c r="J38" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K38" s="2" t="n"/>
-      <c r="L38" s="2" t="n"/>
-      <c r="M38" s="2" t="inlineStr">
+      <c r="J38" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M38" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="inlineStr">
+      <c r="A39" t="inlineStr">
         <is>
           <t>mercadeo@norteysur.co</t>
         </is>
       </c>
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C39" s="2" t="n">
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
         <v>0</v>
       </c>
-      <c r="D39" s="2" t="inlineStr">
+      <c r="D39" t="inlineStr">
         <is>
           <t>Isabella Mesa</t>
         </is>
       </c>
-      <c r="E39" s="2" t="inlineStr">
+      <c r="E39" t="inlineStr">
         <is>
           <t>Oportunidad de Isabella Mesa</t>
         </is>
       </c>
-      <c r="F39" s="2" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G39" s="3" t="n">
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G39" s="1" t="n">
         <v>46091.40078703704</v>
       </c>
-      <c r="H39" s="2" t="n"/>
-      <c r="I39" s="2" t="n">
+      <c r="I39" t="n">
         <v>11</v>
       </c>
-      <c r="J39" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K39" s="2" t="n"/>
-      <c r="L39" s="2" t="n"/>
-      <c r="M39" s="2" t="inlineStr">
+      <c r="J39" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M39" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="n"/>
-      <c r="B40" s="2" t="inlineStr">
+      <c r="B40" t="inlineStr">
         <is>
           <t>Propuesta</t>
         </is>
       </c>
-      <c r="C40" s="2" t="n">
+      <c r="C40" t="n">
         <v>0</v>
       </c>
-      <c r="D40" s="2" t="n"/>
-      <c r="E40" s="2" t="inlineStr">
+      <c r="E40" t="inlineStr">
         <is>
           <t>Clasificación EMAIL Comfenalco Cartagena</t>
         </is>
       </c>
-      <c r="F40" s="2" t="inlineStr">
+      <c r="F40" t="inlineStr">
         <is>
           <t>Maria Fernanda Gaviria</t>
         </is>
       </c>
-      <c r="G40" s="3" t="n">
+      <c r="G40" s="1" t="n">
         <v>46091.3665625</v>
       </c>
-      <c r="H40" s="2" t="n"/>
-      <c r="I40" s="2" t="n">
+      <c r="I40" t="n">
         <v>11</v>
       </c>
-      <c r="J40" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K40" s="2" t="n"/>
-      <c r="L40" s="2" t="n"/>
-      <c r="M40" s="2" t="inlineStr">
+      <c r="J40" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M40" t="inlineStr">
         <is>
           <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="n"/>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C41" s="2" t="n">
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
         <v>0</v>
       </c>
-      <c r="D41" s="2" t="n"/>
-      <c r="E41" s="2" t="inlineStr">
+      <c r="E41" t="inlineStr">
         <is>
           <t>Oportunidad de ESE HOSPITAL LA MARIA</t>
         </is>
       </c>
-      <c r="F41" s="2" t="inlineStr">
+      <c r="F41" t="inlineStr">
         <is>
           <t>Laura Alejandra Castañeda</t>
         </is>
       </c>
-      <c r="G41" s="3" t="n">
+      <c r="G41" s="1" t="n">
         <v>46083.67605324074</v>
       </c>
-      <c r="H41" s="2" t="n"/>
-      <c r="I41" s="2" t="n">
+      <c r="I41" t="n">
         <v>10</v>
       </c>
-      <c r="J41" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K41" s="2" t="n"/>
-      <c r="L41" s="2" t="n"/>
-      <c r="M41" s="2" t="inlineStr">
+      <c r="J41" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M41" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="n"/>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C42" s="2" t="n">
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
         <v>0</v>
       </c>
-      <c r="D42" s="2" t="n"/>
-      <c r="E42" s="2" t="inlineStr">
+      <c r="E42" t="inlineStr">
         <is>
           <t>Oportunidad de SUPER TRANSPORTE</t>
         </is>
       </c>
-      <c r="F42" s="2" t="inlineStr">
+      <c r="F42" t="inlineStr">
         <is>
           <t>Laura Alejandra Castañeda</t>
         </is>
       </c>
-      <c r="G42" s="3" t="n">
+      <c r="G42" s="1" t="n">
         <v>46083.6706712963</v>
       </c>
-      <c r="H42" s="2" t="n"/>
-      <c r="I42" s="2" t="n">
+      <c r="I42" t="n">
         <v>10</v>
       </c>
-      <c r="J42" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K42" s="2" t="n"/>
-      <c r="L42" s="2" t="n"/>
-      <c r="M42" s="2" t="inlineStr">
+      <c r="J42" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M42" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="n"/>
-      <c r="B43" s="2" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C43" s="2" t="n">
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
         <v>0</v>
       </c>
-      <c r="D43" s="2" t="n"/>
-      <c r="E43" s="2" t="inlineStr">
+      <c r="E43" t="inlineStr">
         <is>
           <t>Oportunidad de ENLACES IP S.A.S</t>
         </is>
       </c>
-      <c r="F43" s="2" t="inlineStr">
+      <c r="F43" t="inlineStr">
         <is>
           <t>Laura Alejandra Castañeda</t>
         </is>
       </c>
-      <c r="G43" s="3" t="n">
+      <c r="G43" s="1" t="n">
         <v>46083.50145833333</v>
       </c>
-      <c r="H43" s="3" t="n"/>
-      <c r="I43" s="2" t="n">
+      <c r="I43" t="n">
         <v>10</v>
       </c>
-      <c r="J43" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K43" s="2" t="n"/>
-      <c r="L43" s="2" t="n"/>
-      <c r="M43" s="2" t="inlineStr">
+      <c r="J43" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M43" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="inlineStr">
+      <c r="A44" t="inlineStr">
         <is>
           <t>accounting@diaza.com</t>
         </is>
       </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C44" s="2" t="n">
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
         <v>0</v>
       </c>
-      <c r="D44" s="2" t="inlineStr">
+      <c r="D44" t="inlineStr">
         <is>
           <t>JOHANA RODRIGUEZ</t>
         </is>
       </c>
-      <c r="E44" s="2" t="inlineStr">
+      <c r="E44" t="inlineStr">
         <is>
           <t>Oportunidad de JOHANA RODRIGUEZ</t>
         </is>
       </c>
-      <c r="F44" s="2" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G44" s="3" t="n">
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G44" s="1" t="n">
         <v>46079.73486111111</v>
       </c>
-      <c r="H44" s="2" t="n"/>
-      <c r="I44" s="2" t="n">
+      <c r="I44" t="n">
         <v>9</v>
       </c>
-      <c r="J44" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K44" s="2" t="n"/>
-      <c r="L44" s="2" t="n"/>
-      <c r="M44" s="2" t="inlineStr">
+      <c r="J44" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M44" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="inlineStr">
+      <c r="A45" t="inlineStr">
         <is>
           <t>mensajeriamyr@gmail.com</t>
         </is>
       </c>
-      <c r="B45" s="2" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C45" s="2" t="n">
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
         <v>0</v>
       </c>
-      <c r="D45" s="2" t="n"/>
-      <c r="E45" s="2" t="inlineStr">
+      <c r="E45" t="inlineStr">
         <is>
           <t>Oportunidad de MENSAJERIA M&amp;R SAS</t>
         </is>
       </c>
-      <c r="F45" s="2" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G45" s="3" t="n">
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G45" s="1" t="n">
         <v>46079.72262731481</v>
       </c>
-      <c r="H45" s="2" t="n"/>
-      <c r="I45" s="2" t="n">
+      <c r="I45" t="n">
         <v>9</v>
       </c>
-      <c r="J45" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K45" s="2" t="n"/>
-      <c r="L45" s="2" t="n"/>
-      <c r="M45" s="2" t="inlineStr">
+      <c r="J45" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M45" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="inlineStr">
+      <c r="A46" t="inlineStr">
         <is>
           <t>sistemaspanaderialeal@gmail.com</t>
         </is>
       </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C46" s="2" t="n">
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
         <v>0</v>
       </c>
-      <c r="D46" s="2" t="inlineStr">
+      <c r="D46" t="inlineStr">
         <is>
           <t>Diego Rios</t>
         </is>
       </c>
-      <c r="E46" s="2" t="inlineStr">
+      <c r="E46" t="inlineStr">
         <is>
           <t>JAMDAC SAS, Diego Rios</t>
         </is>
       </c>
-      <c r="F46" s="2" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G46" s="3" t="n">
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G46" s="1" t="n">
         <v>46071.63706018519</v>
       </c>
-      <c r="H46" s="3" t="n"/>
-      <c r="I46" s="2" t="n">
+      <c r="I46" t="n">
         <v>8</v>
       </c>
-      <c r="J46" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K46" s="2" t="n"/>
-      <c r="L46" s="2" t="n"/>
-      <c r="M46" s="2" t="inlineStr">
+      <c r="J46" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M46" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="inlineStr">
+      <c r="A47" t="inlineStr">
         <is>
           <t>efernandez@unico.com.co</t>
         </is>
       </c>
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C47" s="2" t="n">
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
         <v>0</v>
       </c>
-      <c r="D47" s="2" t="inlineStr">
+      <c r="D47" t="inlineStr">
         <is>
           <t>Erick Fernandez</t>
         </is>
       </c>
-      <c r="E47" s="2" t="inlineStr">
+      <c r="E47" t="inlineStr">
         <is>
           <t>Oportunidad de Erick Fernandez</t>
         </is>
       </c>
-      <c r="F47" s="2" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G47" s="3" t="n">
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G47" s="1" t="n">
         <v>46064.3750462963</v>
       </c>
-      <c r="H47" s="2" t="n"/>
-      <c r="I47" s="2" t="n">
+      <c r="I47" t="n">
         <v>7</v>
       </c>
-      <c r="J47" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K47" s="2" t="n"/>
-      <c r="L47" s="2" t="n"/>
-      <c r="M47" s="2" t="inlineStr">
+      <c r="J47" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M47" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="inlineStr">
+      <c r="A48" t="inlineStr">
         <is>
           <t>kabenitez@icesi.edu.co</t>
         </is>
       </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C48" s="2" t="n">
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
         <v>10000000</v>
       </c>
-      <c r="D48" s="2" t="inlineStr">
+      <c r="D48" t="inlineStr">
         <is>
           <t>KENI BENITEZ</t>
         </is>
       </c>
-      <c r="E48" s="2" t="inlineStr">
+      <c r="E48" t="inlineStr">
         <is>
           <t>Oportunidad de KENI BENITEZ</t>
         </is>
       </c>
-      <c r="F48" s="2" t="inlineStr">
+      <c r="F48" t="inlineStr">
         <is>
           <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
-      <c r="G48" s="3" t="n">
+      <c r="G48" s="1" t="n">
         <v>46059.34918981481</v>
       </c>
-      <c r="H48" s="3" t="n"/>
-      <c r="I48" s="2" t="n">
+      <c r="I48" t="n">
         <v>6</v>
       </c>
-      <c r="J48" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K48" s="2" t="n"/>
-      <c r="L48" s="2" t="n"/>
-      <c r="M48" s="2" t="inlineStr">
+      <c r="J48" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M48" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="inlineStr">
+      <c r="A49" t="inlineStr">
         <is>
           <t>patovar@uao.edu.co</t>
         </is>
       </c>
-      <c r="B49" s="2" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C49" s="2" t="n">
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
         <v>0</v>
       </c>
-      <c r="D49" s="2" t="inlineStr">
+      <c r="D49" t="inlineStr">
         <is>
           <t>Paula Tovar</t>
         </is>
       </c>
-      <c r="E49" s="2" t="inlineStr">
+      <c r="E49" t="inlineStr">
         <is>
           <t>Oportunidad de UNIVERSIDAD AUTONOMA DE OCCIDENTE</t>
         </is>
       </c>
-      <c r="F49" s="2" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G49" s="3" t="n">
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G49" s="1" t="n">
         <v>46058.72516203704</v>
       </c>
-      <c r="H49" s="2" t="n"/>
-      <c r="I49" s="2" t="n">
+      <c r="I49" t="n">
         <v>6</v>
       </c>
-      <c r="J49" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K49" s="2" t="n"/>
-      <c r="L49" s="2" t="n"/>
-      <c r="M49" s="2" t="inlineStr">
+      <c r="J49" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M49" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="inlineStr">
+      <c r="A50" t="inlineStr">
         <is>
           <t>comercial@isyscol.com</t>
         </is>
       </c>
-      <c r="B50" s="2" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C50" s="2" t="n">
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
         <v>0</v>
       </c>
-      <c r="D50" s="2" t="n"/>
-      <c r="E50" s="2" t="inlineStr">
+      <c r="E50" t="inlineStr">
         <is>
           <t>Oportunidad de TECNOLOGIAS ISYSCOL SAS</t>
         </is>
       </c>
-      <c r="F50" s="2" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G50" s="3" t="n">
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G50" s="1" t="n">
         <v>46057.58993055556</v>
       </c>
-      <c r="H50" s="2" t="n"/>
-      <c r="I50" s="2" t="n">
+      <c r="I50" t="n">
         <v>6</v>
       </c>
-      <c r="J50" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K50" s="2" t="n"/>
-      <c r="L50" s="2" t="n"/>
-      <c r="M50" s="2" t="inlineStr">
+      <c r="J50" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M50" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="n"/>
-      <c r="B51" s="2" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C51" s="2" t="n">
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
         <v>15000000</v>
       </c>
-      <c r="D51" s="2" t="n"/>
-      <c r="E51" s="2" t="inlineStr">
+      <c r="E51" t="inlineStr">
         <is>
           <t>Oportunidad de VOICE IA EFICACIA</t>
         </is>
       </c>
-      <c r="F51" s="2" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G51" s="3" t="n">
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G51" s="1" t="n">
         <v>46057.3409837963</v>
       </c>
-      <c r="H51" s="2" t="n"/>
-      <c r="I51" s="2" t="n">
+      <c r="I51" t="n">
         <v>6</v>
       </c>
-      <c r="J51" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K51" s="2" t="n"/>
-      <c r="L51" s="2" t="n"/>
-      <c r="M51" s="2" t="inlineStr">
+      <c r="J51" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M51" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="n"/>
-      <c r="B52" s="2" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C52" s="2" t="n">
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
         <v>4000000</v>
       </c>
-      <c r="D52" s="2" t="n"/>
-      <c r="E52" s="2" t="inlineStr">
+      <c r="E52" t="inlineStr">
         <is>
           <t>Oportunidad de Eficacia WhatsApp</t>
         </is>
       </c>
-      <c r="F52" s="2" t="inlineStr">
+      <c r="F52" t="inlineStr">
         <is>
           <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
-      <c r="G52" s="3" t="n">
+      <c r="G52" s="1" t="n">
         <v>46049.67292824074</v>
       </c>
-      <c r="H52" s="2" t="n"/>
-      <c r="I52" s="2" t="n">
+      <c r="I52" t="n">
         <v>5</v>
       </c>
-      <c r="J52" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K52" s="2" t="n"/>
-      <c r="L52" s="2" t="n"/>
-      <c r="M52" s="2" t="inlineStr">
+      <c r="J52" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M52" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="n"/>
-      <c r="B53" s="2" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C53" s="2" t="n">
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
         <v>20000000</v>
       </c>
-      <c r="D53" s="2" t="n"/>
-      <c r="E53" s="2" t="inlineStr">
+      <c r="E53" t="inlineStr">
         <is>
           <t>Oportunidad de CRUZ ROJA COLOMBIANA SECCIONAL VALLE DEL CAUCA</t>
         </is>
       </c>
-      <c r="F53" s="2" t="inlineStr">
+      <c r="F53" t="inlineStr">
         <is>
           <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
-      <c r="G53" s="3" t="n">
+      <c r="G53" s="1" t="n">
         <v>46006.49650462963</v>
       </c>
-      <c r="H53" s="2" t="n"/>
-      <c r="I53" s="2" t="n">
+      <c r="I53" t="n">
         <v>51</v>
       </c>
-      <c r="J53" s="2" t="n">
+      <c r="J53" t="n">
         <v>2025</v>
       </c>
-      <c r="K53" s="2" t="n"/>
-      <c r="L53" s="2" t="n"/>
-      <c r="M53" s="2" t="inlineStr">
+      <c r="M53" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="inlineStr">
+      <c r="A54" t="inlineStr">
         <is>
           <t>silvia.figueroa@neurithmedia.com</t>
         </is>
       </c>
-      <c r="B54" s="2" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C54" s="2" t="n">
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
         <v>25000000</v>
       </c>
-      <c r="D54" s="2" t="n"/>
-      <c r="E54" s="2" t="inlineStr">
+      <c r="E54" t="inlineStr">
         <is>
           <t>Contact center ventas España</t>
         </is>
       </c>
-      <c r="F54" s="2" t="inlineStr">
+      <c r="F54" t="inlineStr">
         <is>
           <t>Richard Castaño</t>
         </is>
       </c>
-      <c r="G54" s="3" t="n">
+      <c r="G54" s="1" t="n">
         <v>45960.61145833333</v>
       </c>
-      <c r="H54" s="2" t="n"/>
-      <c r="I54" s="2" t="n">
+      <c r="I54" t="n">
         <v>44</v>
       </c>
-      <c r="J54" s="2" t="n">
+      <c r="J54" t="n">
         <v>2025</v>
       </c>
-      <c r="K54" s="2" t="n"/>
-      <c r="L54" s="2" t="n"/>
-      <c r="M54" s="2" t="inlineStr">
+      <c r="M54" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="n"/>
-      <c r="B55" s="2" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C55" s="2" t="n">
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
         <v>37000000</v>
       </c>
-      <c r="D55" s="2" t="inlineStr">
+      <c r="D55" t="inlineStr">
         <is>
           <t>Mabel</t>
         </is>
       </c>
-      <c r="E55" s="2" t="inlineStr">
+      <c r="E55" t="inlineStr">
         <is>
           <t>Masivos Licitacion</t>
         </is>
       </c>
-      <c r="F55" s="2" t="inlineStr">
+      <c r="F55" t="inlineStr">
         <is>
           <t>Richard Castaño</t>
         </is>
       </c>
-      <c r="G55" s="3" t="n">
+      <c r="G55" s="1" t="n">
         <v>45940.49372685186</v>
       </c>
-      <c r="H55" s="2" t="n"/>
-      <c r="I55" s="2" t="n">
+      <c r="I55" t="n">
         <v>41</v>
       </c>
-      <c r="J55" s="2" t="n">
+      <c r="J55" t="n">
         <v>2025</v>
       </c>
-      <c r="K55" s="2" t="n"/>
-      <c r="L55" s="2" t="n"/>
-      <c r="M55" s="2" t="inlineStr">
+      <c r="M55" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="inlineStr">
+      <c r="A56" t="inlineStr">
         <is>
           <t>ana.zuniga@cbolivar.com</t>
         </is>
       </c>
-      <c r="B56" s="2" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C56" s="2" t="n">
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
         <v>4997000</v>
       </c>
-      <c r="D56" s="2" t="inlineStr">
+      <c r="D56" t="inlineStr">
         <is>
           <t>Ana Lucia Zuñiga</t>
         </is>
       </c>
-      <c r="E56" s="2" t="inlineStr">
+      <c r="E56" t="inlineStr">
         <is>
           <t>Constructora Bolivar Agente Redes</t>
         </is>
       </c>
-      <c r="F56" s="2" t="inlineStr">
+      <c r="F56" t="inlineStr">
         <is>
           <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
-      <c r="G56" s="3" t="n">
+      <c r="G56" s="1" t="n">
         <v>45940.49215277778</v>
       </c>
-      <c r="H56" s="2" t="n"/>
-      <c r="I56" s="2" t="n">
+      <c r="I56" t="n">
         <v>41</v>
       </c>
-      <c r="J56" s="2" t="n">
+      <c r="J56" t="n">
         <v>2025</v>
       </c>
-      <c r="K56" s="2" t="n"/>
-      <c r="L56" s="2" t="n"/>
-      <c r="M56" s="2" t="inlineStr">
+      <c r="M56" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="2" t="inlineStr">
+      <c r="A57" t="inlineStr">
         <is>
           <t>julian_mendez@extras.com.co</t>
         </is>
       </c>
-      <c r="B57" s="2" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C57" s="2" t="n">
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
         <v>15000000</v>
       </c>
-      <c r="D57" s="2" t="inlineStr">
+      <c r="D57" t="inlineStr">
         <is>
           <t>Julian Mendez.</t>
         </is>
       </c>
-      <c r="E57" s="2" t="inlineStr">
+      <c r="E57" t="inlineStr">
         <is>
           <t>Oportunidad de EFICACIA S A S</t>
         </is>
       </c>
-      <c r="F57" s="2" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G57" s="3" t="n">
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G57" s="1" t="n">
         <v>45922.66201388889</v>
       </c>
-      <c r="H57" s="2" t="n"/>
-      <c r="I57" s="2" t="n">
+      <c r="I57" t="n">
         <v>39</v>
       </c>
-      <c r="J57" s="2" t="n">
+      <c r="J57" t="n">
         <v>2025</v>
       </c>
-      <c r="K57" s="2" t="n"/>
-      <c r="L57" s="2" t="n"/>
-      <c r="M57" s="2" t="inlineStr">
+      <c r="M57" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="inlineStr">
+      <c r="A58" t="inlineStr">
         <is>
           <t>info@eficacia.com.co</t>
         </is>
       </c>
-      <c r="B58" s="2" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C58" s="2" t="n">
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
         <v>0</v>
       </c>
-      <c r="D58" s="2" t="n"/>
-      <c r="E58" s="2" t="inlineStr">
+      <c r="E58" t="inlineStr">
         <is>
           <t>Nutresa</t>
         </is>
       </c>
-      <c r="F58" s="2" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G58" s="3" t="n">
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G58" s="1" t="n">
         <v>45922.66199074074</v>
       </c>
-      <c r="H58" s="2" t="n"/>
-      <c r="I58" s="2" t="n">
+      <c r="I58" t="n">
         <v>39</v>
       </c>
-      <c r="J58" s="2" t="n">
+      <c r="J58" t="n">
         <v>2025</v>
       </c>
-      <c r="K58" s="2" t="n"/>
-      <c r="L58" s="2" t="n"/>
-      <c r="M58" s="2" t="inlineStr">
+      <c r="M58" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="inlineStr">
+      <c r="A59" t="inlineStr">
         <is>
           <t>hrodriguez@jaramillomora.com</t>
         </is>
       </c>
-      <c r="B59" s="2" t="inlineStr">
+      <c r="B59" t="inlineStr">
         <is>
           <t>Seguimiento</t>
         </is>
       </c>
-      <c r="C59" s="2" t="n">
+      <c r="C59" t="n">
         <v>0</v>
       </c>
-      <c r="D59" s="2" t="inlineStr">
+      <c r="D59" t="inlineStr">
         <is>
           <t>HANNA</t>
         </is>
       </c>
-      <c r="E59" s="2" t="inlineStr">
+      <c r="E59" t="inlineStr">
         <is>
           <t>Oportunidad de JARAMILLO MORA CONSTRUCTORA S A</t>
         </is>
       </c>
-      <c r="F59" s="2" t="inlineStr">
+      <c r="F59" t="inlineStr">
         <is>
           <t>Richard Castaño</t>
         </is>
       </c>
-      <c r="G59" s="3" t="n">
+      <c r="G59" s="1" t="n">
         <v>45916.71618055556</v>
       </c>
-      <c r="H59" s="2" t="n"/>
-      <c r="I59" s="2" t="n">
+      <c r="I59" t="n">
         <v>38</v>
       </c>
-      <c r="J59" s="2" t="n">
+      <c r="J59" t="n">
         <v>2025</v>
       </c>
-      <c r="K59" s="2" t="n"/>
-      <c r="L59" s="2" t="n"/>
-      <c r="M59" s="2" t="inlineStr">
+      <c r="M59" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="n"/>
-      <c r="B60" s="2" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C60" s="2" t="n">
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
         <v>147000000</v>
       </c>
-      <c r="D60" s="2" t="n"/>
-      <c r="E60" s="2" t="inlineStr">
+      <c r="E60" t="inlineStr">
         <is>
           <t>Contact Center Agendamiento citas</t>
         </is>
       </c>
-      <c r="F60" s="2" t="inlineStr">
+      <c r="F60" t="inlineStr">
         <is>
           <t>Richard Castaño</t>
         </is>
       </c>
-      <c r="G60" s="3" t="n">
+      <c r="G60" s="1" t="n">
         <v>45916.67502314815</v>
       </c>
-      <c r="H60" s="2" t="n"/>
-      <c r="I60" s="2" t="n">
+      <c r="I60" t="n">
         <v>38</v>
       </c>
-      <c r="J60" s="2" t="n">
+      <c r="J60" t="n">
         <v>2025</v>
       </c>
-      <c r="K60" s="2" t="n"/>
-      <c r="L60" s="2" t="n"/>
-      <c r="M60" s="2" t="inlineStr">
+      <c r="M60" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="2" t="inlineStr">
+      <c r="A61" t="inlineStr">
         <is>
           <t>jaime_zuluaga@eficacia.com.co</t>
         </is>
       </c>
-      <c r="B61" s="2" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C61" s="2" t="n">
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
         <v>14700000</v>
       </c>
-      <c r="D61" s="2" t="n"/>
-      <c r="E61" s="2" t="inlineStr">
+      <c r="E61" t="inlineStr">
         <is>
           <t>Agentes contact center encuestas</t>
         </is>
       </c>
-      <c r="F61" s="2" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G61" s="3" t="n">
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G61" s="1" t="n">
         <v>45916.65275462963</v>
       </c>
-      <c r="H61" s="3" t="n">
+      <c r="H61" s="1" t="n">
         <v>45930</v>
       </c>
-      <c r="I61" s="2" t="n">
+      <c r="I61" t="n">
         <v>38</v>
       </c>
-      <c r="J61" s="2" t="n">
+      <c r="J61" t="n">
         <v>2025</v>
       </c>
-      <c r="K61" s="2" t="n">
+      <c r="K61" t="n">
         <v>9</v>
       </c>
-      <c r="L61" s="2" t="n">
+      <c r="L61" t="n">
         <v>2025</v>
       </c>
-      <c r="M61" s="2" t="inlineStr">
+      <c r="M61" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="2" t="n"/>
-      <c r="B62" s="2" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C62" s="2" t="n">
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
         <v>4796000</v>
       </c>
-      <c r="D62" s="2" t="inlineStr">
+      <c r="D62" t="inlineStr">
         <is>
           <t>Juan Grisales</t>
         </is>
       </c>
-      <c r="E62" s="2" t="inlineStr">
+      <c r="E62" t="inlineStr">
         <is>
           <t>Agente Call Center Outbound</t>
         </is>
       </c>
-      <c r="F62" s="2" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G62" s="3" t="n">
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G62" s="1" t="n">
         <v>45915.4809375</v>
       </c>
-      <c r="H62" s="2" t="n"/>
-      <c r="I62" s="2" t="n">
+      <c r="I62" t="n">
         <v>38</v>
       </c>
-      <c r="J62" s="2" t="n">
+      <c r="J62" t="n">
         <v>2025</v>
       </c>
-      <c r="K62" s="2" t="n"/>
-      <c r="L62" s="2" t="n"/>
-      <c r="M62" s="2" t="inlineStr">
+      <c r="M62" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="2" t="inlineStr">
+      <c r="A63" t="inlineStr">
         <is>
           <t>gestormercadeo@lamontana.co</t>
         </is>
       </c>
-      <c r="B63" s="2" t="inlineStr">
+      <c r="B63" t="inlineStr">
         <is>
           <t>Seguimiento</t>
         </is>
       </c>
-      <c r="C63" s="2" t="n">
+      <c r="C63" t="n">
         <v>25000000</v>
       </c>
-      <c r="D63" s="2" t="inlineStr">
+      <c r="D63" t="inlineStr">
         <is>
           <t>Alejandra Ossa</t>
         </is>
       </c>
-      <c r="E63" s="2" t="inlineStr">
+      <c r="E63" t="inlineStr">
         <is>
           <t>Voice BOT</t>
         </is>
       </c>
-      <c r="F63" s="2" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G63" s="3" t="n">
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G63" s="1" t="n">
         <v>45915.48023148148</v>
       </c>
-      <c r="H63" s="4" t="n">
+      <c r="H63" s="1" t="n">
         <v>46150</v>
       </c>
-      <c r="I63" s="2" t="n">
+      <c r="I63" t="n">
         <v>38</v>
       </c>
-      <c r="J63" s="2" t="n">
+      <c r="J63" t="n">
         <v>2025</v>
       </c>
-      <c r="K63" s="2" t="n">
+      <c r="K63" t="n">
         <v>5</v>
       </c>
-      <c r="L63" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M63" s="2" t="inlineStr">
+      <c r="L63" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M63" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="2" t="inlineStr">
+      <c r="A64" t="inlineStr">
         <is>
           <t>elkinmarquezconsuegra@gmail.com</t>
         </is>
       </c>
-      <c r="B64" s="2" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C64" s="2" t="n">
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
         <v>2500000</v>
       </c>
-      <c r="D64" s="2" t="n"/>
-      <c r="E64" s="2" t="inlineStr">
+      <c r="E64" t="inlineStr">
         <is>
           <t>Venta Masivos</t>
         </is>
       </c>
-      <c r="F64" s="2" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G64" s="3" t="n">
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G64" s="1" t="n">
         <v>45915.47924768519</v>
       </c>
-      <c r="H64" s="2" t="n"/>
-      <c r="I64" s="2" t="n">
+      <c r="I64" t="n">
         <v>38</v>
       </c>
-      <c r="J64" s="2" t="n">
+      <c r="J64" t="n">
         <v>2025</v>
       </c>
-      <c r="K64" s="2" t="n"/>
-      <c r="L64" s="2" t="n"/>
-      <c r="M64" s="2" t="inlineStr">
+      <c r="M64" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="2" t="inlineStr">
+      <c r="A65" t="inlineStr">
         <is>
           <t>bladimir.munoz@uptc.edu.co</t>
         </is>
       </c>
-      <c r="B65" s="2" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C65" s="2" t="n">
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
         <v>22000000</v>
       </c>
-      <c r="D65" s="2" t="inlineStr">
+      <c r="D65" t="inlineStr">
         <is>
           <t>Bladimir Muñoz Forero</t>
         </is>
       </c>
-      <c r="E65" s="2" t="inlineStr">
+      <c r="E65" t="inlineStr">
         <is>
           <t>Oportunidad Venta BPO</t>
         </is>
       </c>
-      <c r="F65" s="2" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G65" s="3" t="n">
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G65" s="1" t="n">
         <v>45915.47494212963</v>
       </c>
-      <c r="H65" s="2" t="n"/>
-      <c r="I65" s="2" t="n">
+      <c r="I65" t="n">
         <v>38</v>
       </c>
-      <c r="J65" s="2" t="n">
+      <c r="J65" t="n">
         <v>2025</v>
       </c>
-      <c r="K65" s="2" t="n"/>
-      <c r="L65" s="2" t="n"/>
-      <c r="M65" s="2" t="inlineStr">
+      <c r="M65" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="inlineStr">
+      <c r="A66" t="inlineStr">
         <is>
           <t>gerencia@alitasfactory.com</t>
         </is>
       </c>
-      <c r="B66" s="2" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C66" s="2" t="n">
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
         <v>40000000</v>
       </c>
-      <c r="D66" s="2" t="n"/>
-      <c r="E66" s="2" t="inlineStr">
+      <c r="E66" t="inlineStr">
         <is>
           <t>1 agente IA para ventas y asesoramiento</t>
         </is>
       </c>
-      <c r="F66" s="2" t="inlineStr">
+      <c r="F66" t="inlineStr">
         <is>
           <t>Richard Castaño</t>
         </is>
       </c>
-      <c r="G66" s="3" t="n">
+      <c r="G66" s="1" t="n">
         <v>45915.47300925926</v>
       </c>
-      <c r="H66" s="2" t="n"/>
-      <c r="I66" s="2" t="n">
+      <c r="I66" t="n">
         <v>38</v>
       </c>
-      <c r="J66" s="2" t="n">
+      <c r="J66" t="n">
         <v>2025</v>
       </c>
-      <c r="K66" s="2" t="n"/>
-      <c r="L66" s="2" t="n"/>
-      <c r="M66" s="2" t="inlineStr">
+      <c r="M66" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="2" t="inlineStr">
+      <c r="A67" t="inlineStr">
         <is>
           <t>mmonroy@falabella.com.co</t>
         </is>
       </c>
-      <c r="B67" s="2" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C67" s="2" t="n">
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
         <v>60000000</v>
       </c>
-      <c r="D67" s="2" t="n"/>
-      <c r="E67" s="2" t="inlineStr">
+      <c r="E67" t="inlineStr">
         <is>
           <t>Agente IA Try and Buy Inbound y Outbound</t>
         </is>
       </c>
-      <c r="F67" s="2" t="inlineStr">
+      <c r="F67" t="inlineStr">
         <is>
           <t>Richard Castaño</t>
         </is>
       </c>
-      <c r="G67" s="3" t="n">
+      <c r="G67" s="1" t="n">
         <v>45915.46633101852</v>
       </c>
-      <c r="H67" s="2" t="n"/>
-      <c r="I67" s="2" t="n">
+      <c r="I67" t="n">
         <v>38</v>
       </c>
-      <c r="J67" s="2" t="n">
+      <c r="J67" t="n">
         <v>2025</v>
       </c>
-      <c r="K67" s="2" t="n"/>
-      <c r="L67" s="2" t="n"/>
-      <c r="M67" s="2" t="inlineStr">
+      <c r="M67" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="2" t="inlineStr">
+      <c r="A68" t="inlineStr">
         <is>
           <t>gerencia@motosymotoselpaisa.com</t>
         </is>
       </c>
-      <c r="B68" s="2" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C68" s="2" t="n">
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
         <v>40000000</v>
       </c>
-      <c r="D68" s="2" t="n"/>
-      <c r="E68" s="2" t="inlineStr">
+      <c r="E68" t="inlineStr">
         <is>
           <t>Oportunidad de MOTOS Y MOTOS EL PAISA S A S</t>
         </is>
       </c>
-      <c r="F68" s="2" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G68" s="3" t="n">
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G68" s="1" t="n">
         <v>45915.46252314815</v>
       </c>
-      <c r="H68" s="2" t="n"/>
-      <c r="I68" s="2" t="n">
+      <c r="I68" t="n">
         <v>38</v>
       </c>
-      <c r="J68" s="2" t="n">
+      <c r="J68" t="n">
         <v>2025</v>
       </c>
-      <c r="K68" s="2" t="n"/>
-      <c r="L68" s="2" t="n"/>
-      <c r="M68" s="2" t="inlineStr">
+      <c r="M68" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="2" t="inlineStr">
+      <c r="A69" t="inlineStr">
         <is>
           <t>isanchez@unico.com.co</t>
         </is>
       </c>
-      <c r="B69" s="2" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C69" s="2" t="n">
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
         <v>0</v>
       </c>
-      <c r="D69" s="2" t="n"/>
-      <c r="E69" s="2" t="inlineStr">
+      <c r="E69" t="inlineStr">
         <is>
           <t>1 agente IA para relacionamiento con locatarios</t>
         </is>
       </c>
-      <c r="F69" s="2" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G69" s="3" t="n">
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G69" s="1" t="n">
         <v>45915.46157407408</v>
       </c>
-      <c r="H69" s="2" t="n"/>
-      <c r="I69" s="2" t="n">
+      <c r="I69" t="n">
         <v>38</v>
       </c>
-      <c r="J69" s="2" t="n">
+      <c r="J69" t="n">
         <v>2025</v>
       </c>
-      <c r="K69" s="2" t="n"/>
-      <c r="L69" s="2" t="n"/>
-      <c r="M69" s="2" t="inlineStr">
+      <c r="M69" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="2" t="inlineStr">
+      <c r="A70" t="inlineStr">
         <is>
           <t>asantiago@stop.com.co</t>
         </is>
       </c>
-      <c r="B70" s="2" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C70" s="2" t="n">
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
         <v>30000000</v>
       </c>
-      <c r="D70" s="2" t="n"/>
-      <c r="E70" s="2" t="inlineStr">
+      <c r="E70" t="inlineStr">
         <is>
           <t>1 Agente IA en cobranzas</t>
         </is>
       </c>
-      <c r="F70" s="2" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G70" s="3" t="n">
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G70" s="1" t="n">
         <v>45915.46052083333</v>
       </c>
-      <c r="H70" s="2" t="n"/>
-      <c r="I70" s="2" t="n">
+      <c r="I70" t="n">
         <v>38</v>
       </c>
-      <c r="J70" s="2" t="n">
+      <c r="J70" t="n">
         <v>2025</v>
       </c>
-      <c r="K70" s="2" t="n"/>
-      <c r="L70" s="2" t="n"/>
-      <c r="M70" s="2" t="inlineStr">
+      <c r="M70" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>
@@ -3705,7 +3471,7 @@
           <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
-      <c r="G71" s="5" t="n">
+      <c r="G71" s="1" t="n">
         <v>45915.35666666667</v>
       </c>
       <c r="I71" t="n">
@@ -3744,7 +3510,7 @@
           <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
-      <c r="G72" s="5" t="n">
+      <c r="G72" s="1" t="n">
         <v>45915.35537037037</v>
       </c>
       <c r="I72" t="n">
@@ -3783,7 +3549,7 @@
           <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
-      <c r="G73" s="5" t="n">
+      <c r="G73" s="1" t="n">
         <v>45915.35351851852</v>
       </c>
       <c r="I73" t="n">
@@ -3827,7 +3593,7 @@
           <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
-      <c r="G74" s="5" t="n">
+      <c r="G74" s="1" t="n">
         <v>45915.34180555555</v>
       </c>
       <c r="I74" t="n">
@@ -3866,7 +3632,7 @@
           <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
-      <c r="G75" s="5" t="n">
+      <c r="G75" s="1" t="n">
         <v>45915.33471064815</v>
       </c>
       <c r="I75" t="n">
@@ -3882,6 +3648,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
CRM actualizado — 07/05/2026 08:38
</commit_message>
<xml_diff>
--- a/CRM_PowerBI_BrendaLuna_actualizado.xlsx
+++ b/CRM_PowerBI_BrendaLuna_actualizado.xlsx
@@ -849,7 +849,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>40000000</v>
+        <v>30000000</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -1255,7 +1255,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>1200000000</v>
+        <v>1200000</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -2963,7 +2963,7 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>0</v>
+        <v>30000000</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
CRM actualizado — 12/05/2026 17:02
</commit_message>
<xml_diff>
--- a/CRM_PowerBI_BrendaLuna_actualizado.xlsx
+++ b/CRM_PowerBI_BrendaLuna_actualizado.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M75"/>
+  <dimension ref="A1:M81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -944,6 +944,11 @@
       </c>
     </row>
     <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>administración@fullredtotal.com</t>
+        </is>
+      </c>
       <c r="B11" t="inlineStr">
         <is>
           <t>Nuevo</t>
@@ -954,12 +959,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>MADERKIT</t>
+          <t>Eivar Eñasco</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Oportunidad de MADERKIT</t>
+          <t>Oportunidad de Eivar Eñasco</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -968,10 +973,10 @@
         </is>
       </c>
       <c r="G11" s="1" t="n">
-        <v>46147.66540509259</v>
+        <v>46154.67546296296</v>
       </c>
       <c r="I11" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J11" t="n">
         <v>2026</v>
@@ -985,25 +990,25 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>omer120395@gmail.com</t>
+          <t>cserna@surtifamiliar.com.co</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Negociación</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0</v>
+        <v>1950000</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Omer Peñaloza</t>
+          <t>Claudia Patricia Serna</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Oportunidad de Omer Peñaloza</t>
+          <t>Oportunidad de Claudia Patricia Serna</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1012,37 +1017,42 @@
         </is>
       </c>
       <c r="G12" s="1" t="n">
-        <v>46147.66090277778</v>
+        <v>46154.66616898148</v>
       </c>
       <c r="I12" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J12" t="n">
         <v>2026</v>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>directora.it@supermercadobelalcazar.com.co</t>
+          <t>coordmercadeo@pacificcenter.co</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>6000000</v>
+        <v>0</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Claudia Castro</t>
+        </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Oportunidad de ABASTECEMOS DE OCCIDENTE</t>
+          <t>Oportunidad de Claudia Castro</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1051,21 +1061,12 @@
         </is>
       </c>
       <c r="G13" s="1" t="n">
-        <v>46147.64170138889</v>
-      </c>
-      <c r="H13" s="1" t="n">
-        <v>46157</v>
+        <v>46154.66341435185</v>
       </c>
       <c r="I13" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J13" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K13" t="n">
-        <v>5</v>
-      </c>
-      <c r="L13" t="n">
         <v>2026</v>
       </c>
       <c r="M13" t="inlineStr">
@@ -1077,20 +1078,25 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>oscar.molina@terrenoshouston.com</t>
+          <t>isabellarengifo27@gmail.com</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>37623040</v>
+        <v>0</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Isabella Rengifo</t>
+        </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Oportunidad de COLONY RIDGE</t>
+          <t>Oportunidad de Isabella Rengifo</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1099,67 +1105,58 @@
         </is>
       </c>
       <c r="G14" s="1" t="n">
-        <v>46147.60297453704</v>
-      </c>
-      <c r="H14" s="1" t="n">
-        <v>46150</v>
+        <v>46154.65981481481</v>
       </c>
       <c r="I14" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J14" t="n">
         <v>2026</v>
       </c>
-      <c r="K14" t="n">
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>No calificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Contactado</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>50000000</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Paola Gómez - Agente Inmobiliaria Independiente</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Puesto de Trabajo CC Medellin</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Richard Castaño</t>
+        </is>
+      </c>
+      <c r="G15" s="1" t="n">
+        <v>46154.49104166667</v>
+      </c>
+      <c r="H15" s="1" t="n">
+        <v>46170</v>
+      </c>
+      <c r="I15" t="n">
+        <v>20</v>
+      </c>
+      <c r="J15" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K15" t="n">
         <v>5</v>
-      </c>
-      <c r="L14" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>Calificado</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>jsantacr@ccc.org.co</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Contactado</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>55000000</v>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Oportunidad de CAMARA DE COMERCIO CALI</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G15" s="1" t="n">
-        <v>46141.62370370371</v>
-      </c>
-      <c r="H15" s="1" t="n">
-        <v>46289</v>
-      </c>
-      <c r="I15" t="n">
-        <v>18</v>
-      </c>
-      <c r="J15" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K15" t="n">
-        <v>9</v>
       </c>
       <c r="L15" t="n">
         <v>2026</v>
@@ -1173,59 +1170,59 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>exportaciones@laprovincia.com</t>
+          <t>alberto.ramirez@constructorabolivar.com</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
+          <t>Propuesta</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Oportunidad de NPS Relacional</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Jennifer Hoyos Gallego</t>
+        </is>
+      </c>
+      <c r="G16" s="1" t="n">
+        <v>46154.44511574074</v>
+      </c>
+      <c r="I16" t="n">
+        <v>20</v>
+      </c>
+      <c r="J16" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Calificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" t="inlineStr">
+        <is>
           <t>Nuevo</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>6000000</v>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Oportunidad de PRODUCTOS LA PROVINCIA SAS</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G16" s="1" t="n">
-        <v>46141.62021990741</v>
-      </c>
-      <c r="I16" t="n">
-        <v>18</v>
-      </c>
-      <c r="J16" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>No calificado</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>coordinador.mercadeo@regency.com.co</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Perdido</t>
         </is>
       </c>
       <c r="C17" t="n">
         <v>0</v>
       </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>MADERKIT</t>
+        </is>
+      </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Oportunidad de REGENCY TECH SAS</t>
+          <t>Oportunidad de MADERKIT</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1234,10 +1231,10 @@
         </is>
       </c>
       <c r="G17" s="1" t="n">
-        <v>46141.59664351852</v>
+        <v>46147.66540509259</v>
       </c>
       <c r="I17" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J17" t="n">
         <v>2026</v>
@@ -1249,17 +1246,27 @@
       </c>
     </row>
     <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>omer120395@gmail.com</t>
+        </is>
+      </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>1200000</v>
+        <v>0</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Omer Peñaloza</t>
+        </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Oportunidad de EMCALI E.I.C.E ESP</t>
+          <t>Oportunidad de Omer Peñaloza</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1268,21 +1275,12 @@
         </is>
       </c>
       <c r="G18" s="1" t="n">
-        <v>46141.59045138889</v>
-      </c>
-      <c r="H18" s="1" t="n">
-        <v>46352</v>
+        <v>46147.66090277778</v>
       </c>
       <c r="I18" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J18" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K18" t="n">
-        <v>11</v>
-      </c>
-      <c r="L18" t="n">
         <v>2026</v>
       </c>
       <c r="M18" t="inlineStr">
@@ -1294,12 +1292,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>angie_feligrana@eficacia.com.co</t>
+          <t>directora.it@supermercadobelalcazar.com.co</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Negociación</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -1307,7 +1305,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Oportunidad de Eficacia sas / Angie Feligrana</t>
+          <t>Oportunidad de ABASTECEMOS DE OCCIDENTE</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1316,13 +1314,13 @@
         </is>
       </c>
       <c r="G19" s="1" t="n">
-        <v>46126.63210648148</v>
+        <v>46147.64170138889</v>
       </c>
       <c r="H19" s="1" t="n">
-        <v>46150</v>
+        <v>46157</v>
       </c>
       <c r="I19" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="J19" t="n">
         <v>2026</v>
@@ -1335,32 +1333,27 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Estrategiadigital@zuluagaysoto.com</t>
+          <t>oscar.molina@terrenoshouston.com</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>0</v>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Maryuri Arguello</t>
-        </is>
+        <v>37623040</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Oportunidad de Maryuri Arguello</t>
+          <t>Oportunidad de COLONY RIDGE</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1369,90 +1362,94 @@
         </is>
       </c>
       <c r="G20" s="1" t="n">
-        <v>46125.71925925926</v>
+        <v>46147.60297453704</v>
+      </c>
+      <c r="H20" s="1" t="n">
+        <v>46150</v>
       </c>
       <c r="I20" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="J20" t="n">
         <v>2026</v>
       </c>
+      <c r="K20" t="n">
+        <v>5</v>
+      </c>
+      <c r="L20" t="n">
+        <v>2026</v>
+      </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>gabrielrodriguez@arrozsupremo.com</t>
+          <t>jsantacr@ccc.org.co</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Ganado</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>8000000</v>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>GABRIEL RODRIGUEZ</t>
-        </is>
+        <v>55000000</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Agente de Ventas</t>
+          <t>Oportunidad de CAMARA DE COMERCIO CALI</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Richard Castaño</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G21" s="1" t="n">
-        <v>46119.62108796297</v>
+        <v>46141.62370370371</v>
       </c>
       <c r="H21" s="1" t="n">
-        <v>46141</v>
+        <v>46289</v>
       </c>
       <c r="I21" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="J21" t="n">
         <v>2026</v>
       </c>
       <c r="K21" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="L21" t="n">
         <v>2026</v>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Belkis.jimenez@agrauto.com.co</t>
+          <t>exportaciones@laprovincia.com</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>0</v>
+        <v>6000000</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Oportunidad de AGRICOLA AUTOMOTRIZ SAS</t>
+          <t>Oportunidad de PRODUCTOS LA PROVINCIA SAS</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1461,10 +1458,10 @@
         </is>
       </c>
       <c r="G22" s="1" t="n">
-        <v>46119.38914351852</v>
+        <v>46141.62021990741</v>
       </c>
       <c r="I22" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="J22" t="n">
         <v>2026</v>
@@ -1478,7 +1475,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>anyela.aponza@cotel.com.co</t>
+          <t>coordinador.mercadeo@regency.com.co</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1491,7 +1488,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Oportunidad de COTEL SAL</t>
+          <t>Oportunidad de REGENCY TECH SAS</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1500,10 +1497,10 @@
         </is>
       </c>
       <c r="G23" s="1" t="n">
-        <v>46112.61271990741</v>
+        <v>46141.59664351852</v>
       </c>
       <c r="I23" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="J23" t="n">
         <v>2026</v>
@@ -1515,27 +1512,17 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>liliana.patino@quironsalud.com</t>
-        </is>
-      </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>CLINICA IMBANACO</t>
-        </is>
+        <v>1200000</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Oportunidad de Liliana Patiño Flórez</t>
+          <t>Oportunidad de EMCALI E.I.C.E ESP</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1544,12 +1531,21 @@
         </is>
       </c>
       <c r="G24" s="1" t="n">
-        <v>46112.60853009259</v>
+        <v>46141.59045138889</v>
+      </c>
+      <c r="H24" s="1" t="n">
+        <v>46352</v>
       </c>
       <c r="I24" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="J24" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K24" t="n">
+        <v>11</v>
+      </c>
+      <c r="L24" t="n">
         <v>2026</v>
       </c>
       <c r="M24" t="inlineStr">
@@ -1561,20 +1557,20 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>casanchez@jgb.com.co</t>
+          <t>angie_feligrana@eficacia.com.co</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Negociación</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>0</v>
+        <v>6000000</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Oportunidad de JGB S.A.</t>
+          <t>Oportunidad de Eficacia sas / Angie Feligrana</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1583,37 +1579,51 @@
         </is>
       </c>
       <c r="G25" s="1" t="n">
-        <v>46112.6052662037</v>
+        <v>46126.63210648148</v>
+      </c>
+      <c r="H25" s="1" t="n">
+        <v>46150</v>
       </c>
       <c r="I25" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="J25" t="n">
         <v>2026</v>
       </c>
+      <c r="K25" t="n">
+        <v>5</v>
+      </c>
+      <c r="L25" t="n">
+        <v>2026</v>
+      </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>damaris.gomez@disfarma.com.co</t>
+          <t>Estrategiadigital@zuluagaysoto.com</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C26" t="n">
         <v>0</v>
       </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Maryuri Arguello</t>
+        </is>
+      </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Oportunidad de DISFARMA</t>
+          <t>Oportunidad de Maryuri Arguello</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1622,121 +1632,121 @@
         </is>
       </c>
       <c r="G26" s="1" t="n">
-        <v>46112.60325231482</v>
+        <v>46125.71925925926</v>
       </c>
       <c r="I26" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="J26" t="n">
         <v>2026</v>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>alergologosdeoccidente@gmail.com</t>
+          <t>gabrielrodriguez@arrozsupremo.com</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Ganado</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>0</v>
+        <v>8000000</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Johana Gonzalez</t>
+          <t>GABRIEL RODRIGUEZ</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Oportunidad de Johana Gonzalez</t>
+          <t>Agente de Ventas</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Richard Castaño</t>
         </is>
       </c>
       <c r="G27" s="1" t="n">
-        <v>46107.51248842593</v>
+        <v>46119.62108796297</v>
+      </c>
+      <c r="H27" s="1" t="n">
+        <v>46141</v>
       </c>
       <c r="I27" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="J27" t="n">
         <v>2026</v>
       </c>
+      <c r="K27" t="n">
+        <v>4</v>
+      </c>
+      <c r="L27" t="n">
+        <v>2026</v>
+      </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>DavidEsteban.Porras@alfalaval.com</t>
+          <t>Belkis.jimenez@agrauto.com.co</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Ganado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>15000000</v>
+        <v>0</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Oportunidad de OPORTUNIDAD ENCUESTAS ALFALAVAL</t>
+          <t>Oportunidad de AGRICOLA AUTOMOTRIZ SAS</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G28" s="1" t="n">
-        <v>46101.72893518519</v>
-      </c>
-      <c r="H28" s="1" t="n">
-        <v>46141</v>
+        <v>46119.38914351852</v>
       </c>
       <c r="I28" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="J28" t="n">
         <v>2026</v>
       </c>
-      <c r="K28" t="n">
-        <v>4</v>
-      </c>
-      <c r="L28" t="n">
-        <v>2026</v>
-      </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Dr.arcarmona@gmail.com</t>
+          <t>anyela.aponza@cotel.com.co</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -1744,7 +1754,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Oportunidad de GAMANUCLEAR LTDA - Dr Alberto Carmona</t>
+          <t>Oportunidad de COTEL SAL</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1753,10 +1763,10 @@
         </is>
       </c>
       <c r="G29" s="1" t="n">
-        <v>46098.65114583333</v>
+        <v>46112.61271990741</v>
       </c>
       <c r="I29" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="J29" t="n">
         <v>2026</v>
@@ -1770,7 +1780,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>cecilia.guevara@cosmitet.net / administracion.crd@cosmitet.net</t>
+          <t>liliana.patino@quironsalud.com</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1783,12 +1793,12 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Cecilia Guevara</t>
+          <t>CLINICA IMBANACO</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Oportunidad de CLINICA REY DAVID Walter Charria</t>
+          <t>Oportunidad de Liliana Patiño Flórez</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1797,10 +1807,10 @@
         </is>
       </c>
       <c r="G30" s="1" t="n">
-        <v>46094.69002314815</v>
+        <v>46112.60853009259</v>
       </c>
       <c r="I30" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="J30" t="n">
         <v>2026</v>
@@ -1814,7 +1824,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>vicerrectoriacademica@unicatolica.edu.co</t>
+          <t>casanchez@jgb.com.co</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1825,14 +1835,9 @@
       <c r="C31" t="n">
         <v>0</v>
       </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>Jorge Silva</t>
-        </is>
-      </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Oportunidad de Jorge Silva</t>
+          <t>Oportunidad de JGB S.A.</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1841,10 +1846,10 @@
         </is>
       </c>
       <c r="G31" s="1" t="n">
-        <v>46094.66880787037</v>
+        <v>46112.6052662037</v>
       </c>
       <c r="I31" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="J31" t="n">
         <v>2026</v>
@@ -1858,48 +1863,34 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>pedroperea02@gmail.com</t>
+          <t>damaris.gomez@disfarma.com.co</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Ganado</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>2160000</v>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Pedro Pablo Perea Mafla</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Oportunidad de Encuestas</t>
+          <t>Oportunidad de DISFARMA</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G32" s="1" t="n">
-        <v>46094.65905092593</v>
-      </c>
-      <c r="H32" s="1" t="n">
-        <v>46141</v>
+        <v>46112.60325231482</v>
       </c>
       <c r="I32" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="J32" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K32" t="n">
-        <v>4</v>
-      </c>
-      <c r="L32" t="n">
         <v>2026</v>
       </c>
       <c r="M32" t="inlineStr">
@@ -1911,7 +1902,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>cristina.papamija@bmm.com.co</t>
+          <t>alergologosdeoccidente@gmail.com</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1920,23 +1911,28 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>8071000</v>
+        <v>0</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Johana Gonzalez</t>
+        </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Oportunidad de BANCO MUNDO MUJER</t>
+          <t>Oportunidad de Johana Gonzalez</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G33" s="1" t="n">
-        <v>46094.65019675926</v>
+        <v>46107.51248842593</v>
       </c>
       <c r="I33" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="J33" t="n">
         <v>2026</v>
@@ -1950,20 +1946,20 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>capacitacionvirtual@fundacionwwbcol.org</t>
+          <t>DavidEsteban.Porras@alfalaval.com</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Ganado</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>1600000</v>
+        <v>15000000</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Licenciamiento y ajuste WhatsApp FUNDACIÓN WWB</t>
+          <t>Oportunidad de OPORTUNIDAD ENCUESTAS ALFALAVAL</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1972,12 +1968,21 @@
         </is>
       </c>
       <c r="G34" s="1" t="n">
-        <v>46094.64826388889</v>
+        <v>46101.72893518519</v>
+      </c>
+      <c r="H34" s="1" t="n">
+        <v>46141</v>
       </c>
       <c r="I34" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J34" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K34" t="n">
+        <v>4</v>
+      </c>
+      <c r="L34" t="n">
         <v>2026</v>
       </c>
       <c r="M34" t="inlineStr">
@@ -1989,60 +1994,46 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>carol.cuesta@cbolivar.com</t>
+          <t>Dr.arcarmona@gmail.com</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Ganado</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>2900000</v>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>CAROL CUESTA</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Gestión de Subsidios CB Bogotá</t>
+          <t>Oportunidad de GAMANUCLEAR LTDA - Dr Alberto Carmona</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G35" s="1" t="n">
-        <v>46094.64454861111</v>
-      </c>
-      <c r="H35" s="1" t="n">
-        <v>46135</v>
+        <v>46098.65114583333</v>
       </c>
       <c r="I35" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J35" t="n">
         <v>2026</v>
       </c>
-      <c r="K35" t="n">
-        <v>4</v>
-      </c>
-      <c r="L35" t="n">
-        <v>2026</v>
-      </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>edwin.munoz.v@uniminuto.edu</t>
+          <t>cecilia.guevara@cosmitet.net / administracion.crd@cosmitet.net</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2053,9 +2044,14 @@
       <c r="C36" t="n">
         <v>0</v>
       </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Cecilia Guevara</t>
+        </is>
+      </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Oportunidad de UNIMINUTO</t>
+          <t>Oportunidad de CLINICA REY DAVID Walter Charria</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -2064,7 +2060,7 @@
         </is>
       </c>
       <c r="G36" s="1" t="n">
-        <v>46092.63626157407</v>
+        <v>46094.69002314815</v>
       </c>
       <c r="I36" t="n">
         <v>11</v>
@@ -2081,7 +2077,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>jaime_zuluaga@eficacia.com.co</t>
+          <t>vicerrectoriacademica@unicatolica.edu.co</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2094,12 +2090,12 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Jaime Alberto</t>
+          <t>Jorge Silva</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Oportunidad de Jaime Alberto Zuluaga</t>
+          <t>Oportunidad de Jorge Silva</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -2108,7 +2104,7 @@
         </is>
       </c>
       <c r="G37" s="1" t="n">
-        <v>46092.63153935185</v>
+        <v>46094.66880787037</v>
       </c>
       <c r="I37" t="n">
         <v>11</v>
@@ -2125,34 +2121,37 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>comercial@isyscol.com</t>
+          <t>pedroperea02@gmail.com</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Ganado</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>0</v>
+        <v>2160000</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Andres Nader</t>
+          <t>Pedro Pablo Perea Mafla</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Oportunidad de Andres Nader</t>
+          <t>Oportunidad de Encuestas</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G38" s="1" t="n">
-        <v>46091.59211805555</v>
+        <v>46094.65905092593</v>
+      </c>
+      <c r="H38" s="1" t="n">
+        <v>46141</v>
       </c>
       <c r="I38" t="n">
         <v>11</v>
@@ -2160,16 +2159,22 @@
       <c r="J38" t="n">
         <v>2026</v>
       </c>
+      <c r="K38" t="n">
+        <v>4</v>
+      </c>
+      <c r="L38" t="n">
+        <v>2026</v>
+      </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>mercadeo@norteysur.co</t>
+          <t>cristina.papamija@bmm.com.co</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2178,25 +2183,20 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>0</v>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>Isabella Mesa</t>
-        </is>
+        <v>8071000</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Oportunidad de Isabella Mesa</t>
+          <t>Oportunidad de BANCO MUNDO MUJER</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G39" s="1" t="n">
-        <v>46091.40078703704</v>
+        <v>46094.65019675926</v>
       </c>
       <c r="I39" t="n">
         <v>11</v>
@@ -2211,26 +2211,31 @@
       </c>
     </row>
     <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>capacitacionvirtual@fundacionwwbcol.org</t>
+        </is>
+      </c>
       <c r="B40" t="inlineStr">
         <is>
           <t>Propuesta</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>0</v>
+        <v>1600000</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Clasificación EMAIL Comfenalco Cartagena</t>
+          <t>Licenciamiento y ajuste WhatsApp FUNDACIÓN WWB</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Maria Fernanda Gaviria</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G40" s="1" t="n">
-        <v>46091.3665625</v>
+        <v>46094.64826388889</v>
       </c>
       <c r="I40" t="n">
         <v>11</v>
@@ -2245,40 +2250,64 @@
       </c>
     </row>
     <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>carol.cuesta@cbolivar.com</t>
+        </is>
+      </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Ganado</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>0</v>
+        <v>2900000</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>CAROL CUESTA</t>
+        </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Oportunidad de ESE HOSPITAL LA MARIA</t>
+          <t>Gestión de Subsidios CB Bogotá</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Laura Alejandra Castañeda</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G41" s="1" t="n">
-        <v>46083.67605324074</v>
+        <v>46094.64454861111</v>
+      </c>
+      <c r="H41" s="1" t="n">
+        <v>46135</v>
       </c>
       <c r="I41" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J41" t="n">
         <v>2026</v>
       </c>
+      <c r="K41" t="n">
+        <v>4</v>
+      </c>
+      <c r="L41" t="n">
+        <v>2026</v>
+      </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>edwin.munoz.v@uniminuto.edu</t>
+        </is>
+      </c>
       <c r="B42" t="inlineStr">
         <is>
           <t>Perdido</t>
@@ -2289,19 +2318,19 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Oportunidad de SUPER TRANSPORTE</t>
+          <t>Oportunidad de UNIMINUTO</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Laura Alejandra Castañeda</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G42" s="1" t="n">
-        <v>46083.6706712963</v>
+        <v>46092.63626157407</v>
       </c>
       <c r="I42" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J42" t="n">
         <v>2026</v>
@@ -2313,6 +2342,11 @@
       </c>
     </row>
     <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>jaime_zuluaga@eficacia.com.co</t>
+        </is>
+      </c>
       <c r="B43" t="inlineStr">
         <is>
           <t>Perdido</t>
@@ -2321,21 +2355,26 @@
       <c r="C43" t="n">
         <v>0</v>
       </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Jaime Alberto</t>
+        </is>
+      </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Oportunidad de ENLACES IP S.A.S</t>
+          <t>Oportunidad de Jaime Alberto Zuluaga</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Laura Alejandra Castañeda</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G43" s="1" t="n">
-        <v>46083.50145833333</v>
+        <v>46092.63153935185</v>
       </c>
       <c r="I43" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J43" t="n">
         <v>2026</v>
@@ -2349,7 +2388,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>accounting@diaza.com</t>
+          <t>comercial@isyscol.com</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2362,12 +2401,12 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>JOHANA RODRIGUEZ</t>
+          <t>Andres Nader</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Oportunidad de JOHANA RODRIGUEZ</t>
+          <t>Oportunidad de Andres Nader</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -2376,10 +2415,10 @@
         </is>
       </c>
       <c r="G44" s="1" t="n">
-        <v>46079.73486111111</v>
+        <v>46091.59211805555</v>
       </c>
       <c r="I44" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="J44" t="n">
         <v>2026</v>
@@ -2393,7 +2432,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>mensajeriamyr@gmail.com</t>
+          <t>mercadeo@norteysur.co</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2404,9 +2443,14 @@
       <c r="C45" t="n">
         <v>0</v>
       </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Isabella Mesa</t>
+        </is>
+      </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Oportunidad de MENSAJERIA M&amp;R SAS</t>
+          <t>Oportunidad de Isabella Mesa</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -2415,10 +2459,10 @@
         </is>
       </c>
       <c r="G45" s="1" t="n">
-        <v>46079.72262731481</v>
+        <v>46091.40078703704</v>
       </c>
       <c r="I45" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="J45" t="n">
         <v>2026</v>
@@ -2430,55 +2474,40 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>sistemaspanaderialeal@gmail.com</t>
-        </is>
-      </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C46" t="n">
         <v>0</v>
       </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>Diego Rios</t>
-        </is>
-      </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>JAMDAC SAS, Diego Rios</t>
+          <t>Clasificación EMAIL Comfenalco Cartagena</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Maria Fernanda Gaviria</t>
         </is>
       </c>
       <c r="G46" s="1" t="n">
-        <v>46071.63706018519</v>
+        <v>46091.3665625</v>
       </c>
       <c r="I46" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="J46" t="n">
         <v>2026</v>
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>efernandez@unico.com.co</t>
-        </is>
-      </c>
       <c r="B47" t="inlineStr">
         <is>
           <t>Perdido</t>
@@ -2487,26 +2516,21 @@
       <c r="C47" t="n">
         <v>0</v>
       </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>Erick Fernandez</t>
-        </is>
-      </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Oportunidad de Erick Fernandez</t>
+          <t>Oportunidad de ESE HOSPITAL LA MARIA</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Laura Alejandra Castañeda</t>
         </is>
       </c>
       <c r="G47" s="1" t="n">
-        <v>46064.3750462963</v>
+        <v>46083.67605324074</v>
       </c>
       <c r="I47" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="J47" t="n">
         <v>2026</v>
@@ -2518,39 +2542,29 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>kabenitez@icesi.edu.co</t>
-        </is>
-      </c>
       <c r="B48" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>10000000</v>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>KENI BENITEZ</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Oportunidad de KENI BENITEZ</t>
+          <t>Oportunidad de SUPER TRANSPORTE</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Laura Alejandra Castañeda</t>
         </is>
       </c>
       <c r="G48" s="1" t="n">
-        <v>46059.34918981481</v>
+        <v>46083.6706712963</v>
       </c>
       <c r="I48" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="J48" t="n">
         <v>2026</v>
@@ -2562,11 +2576,6 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>patovar@uao.edu.co</t>
-        </is>
-      </c>
       <c r="B49" t="inlineStr">
         <is>
           <t>Perdido</t>
@@ -2575,26 +2584,21 @@
       <c r="C49" t="n">
         <v>0</v>
       </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>Paula Tovar</t>
-        </is>
-      </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Oportunidad de UNIVERSIDAD AUTONOMA DE OCCIDENTE</t>
+          <t>Oportunidad de ENLACES IP S.A.S</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Laura Alejandra Castañeda</t>
         </is>
       </c>
       <c r="G49" s="1" t="n">
-        <v>46058.72516203704</v>
+        <v>46083.50145833333</v>
       </c>
       <c r="I49" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="J49" t="n">
         <v>2026</v>
@@ -2608,7 +2612,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>comercial@isyscol.com</t>
+          <t>accounting@diaza.com</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2619,9 +2623,14 @@
       <c r="C50" t="n">
         <v>0</v>
       </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>JOHANA RODRIGUEZ</t>
+        </is>
+      </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Oportunidad de TECNOLOGIAS ISYSCOL SAS</t>
+          <t>Oportunidad de JOHANA RODRIGUEZ</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -2630,10 +2639,10 @@
         </is>
       </c>
       <c r="G50" s="1" t="n">
-        <v>46057.58993055556</v>
+        <v>46079.73486111111</v>
       </c>
       <c r="I50" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J50" t="n">
         <v>2026</v>
@@ -2645,17 +2654,22 @@
       </c>
     </row>
     <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>mensajeriamyr@gmail.com</t>
+        </is>
+      </c>
       <c r="B51" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>15000000</v>
+        <v>0</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Oportunidad de VOICE IA EFICACIA</t>
+          <t>Oportunidad de MENSAJERIA M&amp;R SAS</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -2664,10 +2678,10 @@
         </is>
       </c>
       <c r="G51" s="1" t="n">
-        <v>46057.3409837963</v>
+        <v>46079.72262731481</v>
       </c>
       <c r="I51" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J51" t="n">
         <v>2026</v>
@@ -2679,29 +2693,39 @@
       </c>
     </row>
     <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>sistemaspanaderialeal@gmail.com</t>
+        </is>
+      </c>
       <c r="B52" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>4000000</v>
+        <v>0</v>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Diego Rios</t>
+        </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Oportunidad de Eficacia WhatsApp</t>
+          <t>JAMDAC SAS, Diego Rios</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G52" s="1" t="n">
-        <v>46049.67292824074</v>
+        <v>46071.63706018519</v>
       </c>
       <c r="I52" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="J52" t="n">
         <v>2026</v>
@@ -2713,32 +2737,42 @@
       </c>
     </row>
     <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>efernandez@unico.com.co</t>
+        </is>
+      </c>
       <c r="B53" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>20000000</v>
+        <v>0</v>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Erick Fernandez</t>
+        </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Oportunidad de CRUZ ROJA COLOMBIANA SECCIONAL VALLE DEL CAUCA</t>
+          <t>Oportunidad de Erick Fernandez</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G53" s="1" t="n">
-        <v>46006.49650462963</v>
+        <v>46064.3750462963</v>
       </c>
       <c r="I53" t="n">
-        <v>51</v>
+        <v>7</v>
       </c>
       <c r="J53" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="M53" t="inlineStr">
         <is>
@@ -2749,7 +2783,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>silvia.figueroa@neurithmedia.com</t>
+          <t>kabenitez@icesi.edu.co</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2758,26 +2792,31 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>25000000</v>
+        <v>10000000</v>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>KENI BENITEZ</t>
+        </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Contact center ventas España</t>
+          <t>Oportunidad de KENI BENITEZ</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Richard Castaño</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G54" s="1" t="n">
-        <v>45960.61145833333</v>
+        <v>46059.34918981481</v>
       </c>
       <c r="I54" t="n">
-        <v>44</v>
+        <v>6</v>
       </c>
       <c r="J54" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="M54" t="inlineStr">
         <is>
@@ -2786,37 +2825,42 @@
       </c>
     </row>
     <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>patovar@uao.edu.co</t>
+        </is>
+      </c>
       <c r="B55" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>37000000</v>
+        <v>0</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Mabel</t>
+          <t>Paula Tovar</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Masivos Licitacion</t>
+          <t>Oportunidad de UNIVERSIDAD AUTONOMA DE OCCIDENTE</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Richard Castaño</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G55" s="1" t="n">
-        <v>45940.49372685186</v>
+        <v>46058.72516203704</v>
       </c>
       <c r="I55" t="n">
-        <v>41</v>
+        <v>6</v>
       </c>
       <c r="J55" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="M55" t="inlineStr">
         <is>
@@ -2827,7 +2871,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>ana.zuniga@cbolivar.com</t>
+          <t>comercial@isyscol.com</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2836,31 +2880,26 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>4997000</v>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>Ana Lucia Zuñiga</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Constructora Bolivar Agente Redes</t>
+          <t>Oportunidad de TECNOLOGIAS ISYSCOL SAS</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G56" s="1" t="n">
-        <v>45940.49215277778</v>
+        <v>46057.58993055556</v>
       </c>
       <c r="I56" t="n">
-        <v>41</v>
+        <v>6</v>
       </c>
       <c r="J56" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="M56" t="inlineStr">
         <is>
@@ -2869,11 +2908,6 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>julian_mendez@extras.com.co</t>
-        </is>
-      </c>
       <c r="B57" t="inlineStr">
         <is>
           <t>Perdido</t>
@@ -2882,14 +2916,9 @@
       <c r="C57" t="n">
         <v>15000000</v>
       </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>Julian Mendez.</t>
-        </is>
-      </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Oportunidad de EFICACIA S A S</t>
+          <t>Oportunidad de VOICE IA EFICACIA</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -2898,13 +2927,13 @@
         </is>
       </c>
       <c r="G57" s="1" t="n">
-        <v>45922.66201388889</v>
+        <v>46057.3409837963</v>
       </c>
       <c r="I57" t="n">
-        <v>39</v>
+        <v>6</v>
       </c>
       <c r="J57" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="M57" t="inlineStr">
         <is>
@@ -2913,37 +2942,32 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>info@eficacia.com.co</t>
-        </is>
-      </c>
       <c r="B58" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>0</v>
+        <v>4000000</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Nutresa</t>
+          <t>Oportunidad de Eficacia WhatsApp</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G58" s="1" t="n">
-        <v>45922.66199074074</v>
+        <v>46049.67292824074</v>
       </c>
       <c r="I58" t="n">
-        <v>39</v>
+        <v>5</v>
       </c>
       <c r="J58" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="M58" t="inlineStr">
         <is>
@@ -2952,39 +2976,29 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>hrodriguez@jaramillomora.com</t>
-        </is>
-      </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Seguimiento</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>30000000</v>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>HANNA</t>
-        </is>
+        <v>20000000</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Oportunidad de JARAMILLO MORA CONSTRUCTORA S A</t>
+          <t>Oportunidad de CRUZ ROJA COLOMBIANA SECCIONAL VALLE DEL CAUCA</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Richard Castaño</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G59" s="1" t="n">
-        <v>45916.71618055556</v>
+        <v>46006.49650462963</v>
       </c>
       <c r="I59" t="n">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="J59" t="n">
         <v>2025</v>
@@ -2996,17 +3010,22 @@
       </c>
     </row>
     <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>silvia.figueroa@neurithmedia.com</t>
+        </is>
+      </c>
       <c r="B60" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>147000000</v>
+        <v>25000000</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Contact Center Agendamiento citas</t>
+          <t>Contact center ventas España</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -3015,10 +3034,10 @@
         </is>
       </c>
       <c r="G60" s="1" t="n">
-        <v>45916.67502314815</v>
+        <v>45960.61145833333</v>
       </c>
       <c r="I60" t="n">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="J60" t="n">
         <v>2025</v>
@@ -3030,47 +3049,38 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>jaime_zuluaga@eficacia.com.co</t>
-        </is>
-      </c>
       <c r="B61" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>14700000</v>
+        <v>37000000</v>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Mabel</t>
+        </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Agentes contact center encuestas</t>
+          <t>Masivos Licitacion</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Richard Castaño</t>
         </is>
       </c>
       <c r="G61" s="1" t="n">
-        <v>45916.65275462963</v>
-      </c>
-      <c r="H61" s="1" t="n">
-        <v>45930</v>
+        <v>45940.49372685186</v>
       </c>
       <c r="I61" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="J61" t="n">
         <v>2025</v>
       </c>
-      <c r="K61" t="n">
-        <v>9</v>
-      </c>
-      <c r="L61" t="n">
-        <v>2025</v>
-      </c>
       <c r="M61" t="inlineStr">
         <is>
           <t>No calificado</t>
@@ -3078,34 +3088,39 @@
       </c>
     </row>
     <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>ana.zuniga@cbolivar.com</t>
+        </is>
+      </c>
       <c r="B62" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>4796000</v>
+        <v>4997000</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Juan Grisales</t>
+          <t>Ana Lucia Zuñiga</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Agente Call Center Outbound</t>
+          <t>Constructora Bolivar Agente Redes</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G62" s="1" t="n">
-        <v>45915.4809375</v>
+        <v>45940.49215277778</v>
       </c>
       <c r="I62" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="J62" t="n">
         <v>2025</v>
@@ -3119,25 +3134,25 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>gestormercadeo@lamontana.co</t>
+          <t>julian_mendez@extras.com.co</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Seguimiento</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>25000000</v>
+        <v>15000000</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Alejandra Ossa</t>
+          <t>Julian Mendez.</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Voice BOT</t>
+          <t>Oportunidad de EFICACIA S A S</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -3146,23 +3161,14 @@
         </is>
       </c>
       <c r="G63" s="1" t="n">
-        <v>45915.48023148148</v>
-      </c>
-      <c r="H63" s="1" t="n">
-        <v>46150</v>
+        <v>45922.66201388889</v>
       </c>
       <c r="I63" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="J63" t="n">
         <v>2025</v>
       </c>
-      <c r="K63" t="n">
-        <v>5</v>
-      </c>
-      <c r="L63" t="n">
-        <v>2026</v>
-      </c>
       <c r="M63" t="inlineStr">
         <is>
           <t>No calificado</t>
@@ -3172,7 +3178,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>elkinmarquezconsuegra@gmail.com</t>
+          <t>info@eficacia.com.co</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3181,11 +3187,11 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>2500000</v>
+        <v>0</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Venta Masivos</t>
+          <t>Nutresa</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -3194,10 +3200,10 @@
         </is>
       </c>
       <c r="G64" s="1" t="n">
-        <v>45915.47924768519</v>
+        <v>45922.66199074074</v>
       </c>
       <c r="I64" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="J64" t="n">
         <v>2025</v>
@@ -3211,34 +3217,34 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>bladimir.munoz@uptc.edu.co</t>
+          <t>hrodriguez@jaramillomora.com</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Seguimiento</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>22000000</v>
+        <v>30000000</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Bladimir Muñoz Forero</t>
+          <t>HANNA</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Oportunidad Venta BPO</t>
+          <t>Oportunidad de JARAMILLO MORA CONSTRUCTORA S A</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Richard Castaño</t>
         </is>
       </c>
       <c r="G65" s="1" t="n">
-        <v>45915.47494212963</v>
+        <v>45916.71618055556</v>
       </c>
       <c r="I65" t="n">
         <v>38</v>
@@ -3253,22 +3259,17 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>gerencia@alitasfactory.com</t>
-        </is>
-      </c>
       <c r="B66" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>40000000</v>
+        <v>147000000</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>1 agente IA para ventas y asesoramiento</t>
+          <t>Contact Center Agendamiento citas</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -3277,7 +3278,7 @@
         </is>
       </c>
       <c r="G66" s="1" t="n">
-        <v>45915.47300925926</v>
+        <v>45916.67502314815</v>
       </c>
       <c r="I66" t="n">
         <v>38</v>
@@ -3294,7 +3295,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>mmonroy@falabella.com.co</t>
+          <t>jaime_zuluaga@eficacia.com.co</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3303,20 +3304,23 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>60000000</v>
+        <v>14700000</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Agente IA Try and Buy Inbound y Outbound</t>
+          <t>Agentes contact center encuestas</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Richard Castaño</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G67" s="1" t="n">
-        <v>45915.46633101852</v>
+        <v>45916.65275462963</v>
+      </c>
+      <c r="H67" s="1" t="n">
+        <v>45930</v>
       </c>
       <c r="I67" t="n">
         <v>38</v>
@@ -3324,6 +3328,12 @@
       <c r="J67" t="n">
         <v>2025</v>
       </c>
+      <c r="K67" t="n">
+        <v>9</v>
+      </c>
+      <c r="L67" t="n">
+        <v>2025</v>
+      </c>
       <c r="M67" t="inlineStr">
         <is>
           <t>No calificado</t>
@@ -3331,22 +3341,22 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>gerencia@motosymotoselpaisa.com</t>
-        </is>
-      </c>
       <c r="B68" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>40000000</v>
+        <v>4796000</v>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Juan Grisales</t>
+        </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Oportunidad de MOTOS Y MOTOS EL PAISA S A S</t>
+          <t>Agente Call Center Outbound</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -3355,7 +3365,7 @@
         </is>
       </c>
       <c r="G68" s="1" t="n">
-        <v>45915.46252314815</v>
+        <v>45915.4809375</v>
       </c>
       <c r="I68" t="n">
         <v>38</v>
@@ -3372,20 +3382,25 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>isanchez@unico.com.co</t>
+          <t>gestormercadeo@lamontana.co</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Seguimiento</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>0</v>
+        <v>25000000</v>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Alejandra Ossa</t>
+        </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>1 agente IA para relacionamiento con locatarios</t>
+          <t>Voice BOT</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -3394,7 +3409,10 @@
         </is>
       </c>
       <c r="G69" s="1" t="n">
-        <v>45915.46157407408</v>
+        <v>45915.48023148148</v>
+      </c>
+      <c r="H69" s="1" t="n">
+        <v>46150</v>
       </c>
       <c r="I69" t="n">
         <v>38</v>
@@ -3402,6 +3420,12 @@
       <c r="J69" t="n">
         <v>2025</v>
       </c>
+      <c r="K69" t="n">
+        <v>5</v>
+      </c>
+      <c r="L69" t="n">
+        <v>2026</v>
+      </c>
       <c r="M69" t="inlineStr">
         <is>
           <t>No calificado</t>
@@ -3411,7 +3435,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>asantiago@stop.com.co</t>
+          <t>elkinmarquezconsuegra@gmail.com</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -3420,11 +3444,11 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>30000000</v>
+        <v>2500000</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>1 Agente IA en cobranzas</t>
+          <t>Venta Masivos</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -3433,7 +3457,7 @@
         </is>
       </c>
       <c r="G70" s="1" t="n">
-        <v>45915.46052083333</v>
+        <v>45915.47924768519</v>
       </c>
       <c r="I70" t="n">
         <v>38</v>
@@ -3450,7 +3474,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>jcastano@mercaldas.com.co</t>
+          <t>bladimir.munoz@uptc.edu.co</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -3459,11 +3483,16 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>30000000</v>
+        <v>22000000</v>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Bladimir Muñoz Forero</t>
+        </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>1 agente IA para ventas y asesoramiento</t>
+          <t>Oportunidad Venta BPO</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -3472,7 +3501,7 @@
         </is>
       </c>
       <c r="G71" s="1" t="n">
-        <v>45915.35666666667</v>
+        <v>45915.47494212963</v>
       </c>
       <c r="I71" t="n">
         <v>38</v>
@@ -3489,7 +3518,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>calidad@cempac.com.co</t>
+          <t>gerencia@alitasfactory.com</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -3498,7 +3527,7 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>42000000</v>
+        <v>40000000</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -3507,11 +3536,11 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Richard Castaño</t>
         </is>
       </c>
       <c r="G72" s="1" t="n">
-        <v>45915.35537037037</v>
+        <v>45915.47300925926</v>
       </c>
       <c r="I72" t="n">
         <v>38</v>
@@ -3528,7 +3557,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>info@eficacia.com.co</t>
+          <t>mmonroy@falabella.com.co</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -3537,20 +3566,20 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>15000000</v>
+        <v>60000000</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Requieren IA para PQRS y exploran otras opciones</t>
+          <t>Agente IA Try and Buy Inbound y Outbound</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Richard Castaño</t>
         </is>
       </c>
       <c r="G73" s="1" t="n">
-        <v>45915.35351851852</v>
+        <v>45915.46633101852</v>
       </c>
       <c r="I73" t="n">
         <v>38</v>
@@ -3567,7 +3596,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>orlandogomez@grupogiraldo.com</t>
+          <t>gerencia@motosymotoselpaisa.com</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -3576,16 +3605,11 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>30000000</v>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>Orlando Gomez</t>
-        </is>
+        <v>40000000</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>1 agente IA para ventas y asesoramiento</t>
+          <t>Oportunidad de MOTOS Y MOTOS EL PAISA S A S</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -3594,7 +3618,7 @@
         </is>
       </c>
       <c r="G74" s="1" t="n">
-        <v>45915.34180555555</v>
+        <v>45915.46252314815</v>
       </c>
       <c r="I74" t="n">
         <v>38</v>
@@ -3611,7 +3635,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>c.roman@chipichape.com.co</t>
+          <t>isanchez@unico.com.co</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -3620,11 +3644,11 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>60000000</v>
+        <v>0</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>3 Agentes IA</t>
+          <t>1 agente IA para relacionamiento con locatarios</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -3633,7 +3657,7 @@
         </is>
       </c>
       <c r="G75" s="1" t="n">
-        <v>45915.33471064815</v>
+        <v>45915.46157407408</v>
       </c>
       <c r="I75" t="n">
         <v>38</v>
@@ -3642,6 +3666,245 @@
         <v>2025</v>
       </c>
       <c r="M75" t="inlineStr">
+        <is>
+          <t>No calificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>asantiago@stop.com.co</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>30000000</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>1 Agente IA en cobranzas</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G76" s="1" t="n">
+        <v>45915.46052083333</v>
+      </c>
+      <c r="I76" t="n">
+        <v>38</v>
+      </c>
+      <c r="J76" t="n">
+        <v>2025</v>
+      </c>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t>No calificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>jcastano@mercaldas.com.co</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>30000000</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>1 agente IA para ventas y asesoramiento</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G77" s="1" t="n">
+        <v>45915.35666666667</v>
+      </c>
+      <c r="I77" t="n">
+        <v>38</v>
+      </c>
+      <c r="J77" t="n">
+        <v>2025</v>
+      </c>
+      <c r="M77" t="inlineStr">
+        <is>
+          <t>No calificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>calidad@cempac.com.co</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>42000000</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>1 agente IA para ventas y asesoramiento</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G78" s="1" t="n">
+        <v>45915.35537037037</v>
+      </c>
+      <c r="I78" t="n">
+        <v>38</v>
+      </c>
+      <c r="J78" t="n">
+        <v>2025</v>
+      </c>
+      <c r="M78" t="inlineStr">
+        <is>
+          <t>No calificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>info@eficacia.com.co</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>15000000</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Requieren IA para PQRS y exploran otras opciones</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Jennifer Hoyos Gallego</t>
+        </is>
+      </c>
+      <c r="G79" s="1" t="n">
+        <v>45915.35351851852</v>
+      </c>
+      <c r="I79" t="n">
+        <v>38</v>
+      </c>
+      <c r="J79" t="n">
+        <v>2025</v>
+      </c>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t>No calificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>orlandogomez@grupogiraldo.com</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>30000000</v>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Orlando Gomez</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>1 agente IA para ventas y asesoramiento</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G80" s="1" t="n">
+        <v>45915.34180555555</v>
+      </c>
+      <c r="I80" t="n">
+        <v>38</v>
+      </c>
+      <c r="J80" t="n">
+        <v>2025</v>
+      </c>
+      <c r="M80" t="inlineStr">
+        <is>
+          <t>No calificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>c.roman@chipichape.com.co</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>60000000</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>3 Agentes IA</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G81" s="1" t="n">
+        <v>45915.33471064815</v>
+      </c>
+      <c r="I81" t="n">
+        <v>38</v>
+      </c>
+      <c r="J81" t="n">
+        <v>2025</v>
+      </c>
+      <c r="M81" t="inlineStr">
         <is>
           <t>No calificado</t>
         </is>

</xml_diff>

<commit_message>
CRM actualizado — 12/05/2026 17:17
</commit_message>
<xml_diff>
--- a/CRM_PowerBI_BrendaLuna_actualizado.xlsx
+++ b/CRM_PowerBI_BrendaLuna_actualizado.xlsx
@@ -657,7 +657,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>16914000</v>
+        <v>17627400</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -1087,7 +1087,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0</v>
+        <v>16000000</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -1122,7 +1122,7 @@
     <row r="15">
       <c r="B15" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -1163,7 +1163,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
@@ -1209,11 +1209,11 @@
     <row r="17">
       <c r="B17" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0</v>
+        <v>3000000</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -1297,7 +1297,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -1333,7 +1333,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
@@ -1441,7 +1441,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -1868,7 +1868,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Seguimiento</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -1895,7 +1895,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
@@ -1999,7 +1999,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -2476,7 +2476,7 @@
     <row r="46">
       <c r="B46" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Seguimiento</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -2503,7 +2503,7 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
CRM actualizado — 13/05/2026 08:51
</commit_message>
<xml_diff>
--- a/CRM_PowerBI_BrendaLuna_actualizado.xlsx
+++ b/CRM_PowerBI_BrendaLuna_actualizado.xlsx
@@ -565,7 +565,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Richard Castaño</t>
         </is>
       </c>
       <c r="G3" s="1" t="n">
@@ -2218,7 +2218,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -2245,7 +2245,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
CRM actualizado — 20/05/2026 10:01
</commit_message>
<xml_diff>
--- a/CRM_PowerBI_BrendaLuna_actualizado.xlsx
+++ b/CRM_PowerBI_BrendaLuna_actualizado.xlsx
@@ -946,7 +946,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>administración@fullredtotal.com</t>
+          <t>asantiago@stop.com.co</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -957,14 +957,9 @@
       <c r="C11" t="n">
         <v>0</v>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Eivar Eñasco</t>
-        </is>
-      </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Oportunidad de Eivar Eñasco</t>
+          <t>Oportunidad de STOP SAS</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -973,10 +968,10 @@
         </is>
       </c>
       <c r="G11" s="1" t="n">
-        <v>46154.67546296296</v>
+        <v>46161.63508101852</v>
       </c>
       <c r="I11" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J11" t="n">
         <v>2026</v>
@@ -990,25 +985,25 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>cserna@surtifamiliar.com.co</t>
+          <t>aestrada@teker.co</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Negociación</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1950000</v>
+        <v>0</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Claudia Patricia Serna</t>
+          <t>TEKER SALUD SAS</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Oportunidad de Claudia Patricia Serna</t>
+          <t>Oportunidad de TEKER SALUD SAS</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1017,26 +1012,21 @@
         </is>
       </c>
       <c r="G12" s="1" t="n">
-        <v>46154.66616898148</v>
+        <v>46161.62922453704</v>
       </c>
       <c r="I12" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J12" t="n">
         <v>2026</v>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>coordmercadeo@pacificcenter.co</t>
-        </is>
-      </c>
       <c r="B13" t="inlineStr">
         <is>
           <t>Nuevo</t>
@@ -1045,14 +1035,9 @@
       <c r="C13" t="n">
         <v>0</v>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Claudia Castro</t>
-        </is>
-      </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Oportunidad de Claudia Castro</t>
+          <t>Oportunidad de TIAN IPS SAS</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1061,10 +1046,10 @@
         </is>
       </c>
       <c r="G13" s="1" t="n">
-        <v>46154.66341435185</v>
+        <v>46161.61643518518</v>
       </c>
       <c r="I13" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J13" t="n">
         <v>2026</v>
@@ -1078,7 +1063,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>isabellarengifo27@gmail.com</t>
+          <t>administración@fullredtotal.com</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1087,16 +1072,16 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>16000000</v>
+        <v>0</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Isabella Rengifo</t>
+          <t>Eivar Eñasco</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Oportunidad de Isabella Rengifo</t>
+          <t>Oportunidad de Eivar Eñasco</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1105,7 +1090,7 @@
         </is>
       </c>
       <c r="G14" s="1" t="n">
-        <v>46154.65981481481</v>
+        <v>46154.67546296296</v>
       </c>
       <c r="I14" t="n">
         <v>20</v>
@@ -1120,34 +1105,36 @@
       </c>
     </row>
     <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>cserna@surtifamiliar.com.co</t>
+        </is>
+      </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Negociación</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>50000000</v>
+        <v>1950000</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Paola Gómez - Agente Inmobiliaria Independiente</t>
+          <t>Claudia Patricia Serna</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Puesto de Trabajo CC Medellin</t>
+          <t>Oportunidad de Claudia Patricia Serna</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Richard Castaño</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G15" s="1" t="n">
-        <v>46154.49104166667</v>
-      </c>
-      <c r="H15" s="1" t="n">
-        <v>46170</v>
+        <v>46154.66616898148</v>
       </c>
       <c r="I15" t="n">
         <v>20</v>
@@ -1155,12 +1142,6 @@
       <c r="J15" t="n">
         <v>2026</v>
       </c>
-      <c r="K15" t="n">
-        <v>5</v>
-      </c>
-      <c r="L15" t="n">
-        <v>2026</v>
-      </c>
       <c r="M15" t="inlineStr">
         <is>
           <t>Calificado</t>
@@ -1170,29 +1151,34 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>alberto.ramirez@constructorabolivar.com</t>
+          <t>coordmercadeo@pacificcenter.co</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>3000000</v>
+        <v>0</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Claudia Castro</t>
+        </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Oportunidad de NPS Relacional</t>
+          <t>Oportunidad de Claudia Castro</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G16" s="1" t="n">
-        <v>46154.44511574074</v>
+        <v>46154.66341435185</v>
       </c>
       <c r="I16" t="n">
         <v>20</v>
@@ -1202,97 +1188,106 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
+          <t>No calificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>isabellarengifo27@gmail.com</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>16000000</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Isabella Rengifo</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Oportunidad de Isabella Rengifo</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G17" s="1" t="n">
+        <v>46154.65981481481</v>
+      </c>
+      <c r="I17" t="n">
+        <v>20</v>
+      </c>
+      <c r="J17" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>No calificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Propuesta</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>50000000</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Paola Gómez - Agente Inmobiliaria Independiente</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Puesto de Trabajo CC Medellin</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Richard Castaño</t>
+        </is>
+      </c>
+      <c r="G18" s="1" t="n">
+        <v>46154.49104166667</v>
+      </c>
+      <c r="H18" s="1" t="n">
+        <v>46170</v>
+      </c>
+      <c r="I18" t="n">
+        <v>20</v>
+      </c>
+      <c r="J18" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K18" t="n">
+        <v>5</v>
+      </c>
+      <c r="L18" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
           <t>Calificado</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Contactado</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
-        <v>3000000</v>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>MADERKIT</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>Oportunidad de MADERKIT</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G17" s="1" t="n">
-        <v>46147.66540509259</v>
-      </c>
-      <c r="I17" t="n">
-        <v>19</v>
-      </c>
-      <c r="J17" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>No calificado</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>omer120395@gmail.com</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
-        <v>0</v>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Omer Peñaloza</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>Oportunidad de Omer Peñaloza</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G18" s="1" t="n">
-        <v>46147.66090277778</v>
-      </c>
-      <c r="I18" t="n">
-        <v>19</v>
-      </c>
-      <c r="J18" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>directora.it@supermercadobelalcazar.com.co</t>
+          <t>alberto.ramirez@constructorabolivar.com</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1301,36 +1296,27 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>6000000</v>
+        <v>3000000</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Oportunidad de ABASTECEMOS DE OCCIDENTE</t>
+          <t>Oportunidad de NPS Relacional</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G19" s="1" t="n">
-        <v>46147.64170138889</v>
-      </c>
-      <c r="H19" s="1" t="n">
-        <v>46157</v>
+        <v>46154.44511574074</v>
       </c>
       <c r="I19" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J19" t="n">
         <v>2026</v>
       </c>
-      <c r="K19" t="n">
-        <v>5</v>
-      </c>
-      <c r="L19" t="n">
-        <v>2026</v>
-      </c>
       <c r="M19" t="inlineStr">
         <is>
           <t>Calificado</t>
@@ -1338,22 +1324,22 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>oscar.molina@terrenoshouston.com</t>
-        </is>
-      </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Negociación</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>37623040</v>
+        <v>3000000</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>MADERKIT</t>
+        </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Oportunidad de COLONY RIDGE</t>
+          <t>Oportunidad de MADERKIT</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1362,10 +1348,7 @@
         </is>
       </c>
       <c r="G20" s="1" t="n">
-        <v>46147.60297453704</v>
-      </c>
-      <c r="H20" s="1" t="n">
-        <v>46150</v>
+        <v>46147.66540509259</v>
       </c>
       <c r="I20" t="n">
         <v>19</v>
@@ -1373,35 +1356,34 @@
       <c r="J20" t="n">
         <v>2026</v>
       </c>
-      <c r="K20" t="n">
-        <v>5</v>
-      </c>
-      <c r="L20" t="n">
-        <v>2026</v>
-      </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>jsantacr@ccc.org.co</t>
+          <t>omer120395@gmail.com</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>55000000</v>
+        <v>0</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Omer Peñaloza</t>
+        </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Oportunidad de CAMARA DE COMERCIO CALI</t>
+          <t>Oportunidad de Omer Peñaloza</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1410,21 +1392,12 @@
         </is>
       </c>
       <c r="G21" s="1" t="n">
-        <v>46141.62370370371</v>
-      </c>
-      <c r="H21" s="1" t="n">
-        <v>46289</v>
+        <v>46147.66090277778</v>
       </c>
       <c r="I21" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J21" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K21" t="n">
-        <v>9</v>
-      </c>
-      <c r="L21" t="n">
         <v>2026</v>
       </c>
       <c r="M21" t="inlineStr">
@@ -1436,12 +1409,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>exportaciones@laprovincia.com</t>
+          <t>directora.it@supermercadobelalcazar.com.co</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -1449,7 +1422,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Oportunidad de PRODUCTOS LA PROVINCIA SAS</t>
+          <t>Oportunidad de ABASTECEMOS DE OCCIDENTE</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1458,12 +1431,21 @@
         </is>
       </c>
       <c r="G22" s="1" t="n">
-        <v>46141.62021990741</v>
+        <v>46147.64170138889</v>
+      </c>
+      <c r="H22" s="1" t="n">
+        <v>46157</v>
       </c>
       <c r="I22" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J22" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K22" t="n">
+        <v>5</v>
+      </c>
+      <c r="L22" t="n">
         <v>2026</v>
       </c>
       <c r="M22" t="inlineStr">
@@ -1475,20 +1457,20 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>coordinador.mercadeo@regency.com.co</t>
+          <t>oscar.molina@terrenoshouston.com</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Negociación</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>0</v>
+        <v>37623040</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Oportunidad de REGENCY TECH SAS</t>
+          <t>Oportunidad de COLONY RIDGE</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1497,32 +1479,46 @@
         </is>
       </c>
       <c r="G23" s="1" t="n">
-        <v>46141.59664351852</v>
+        <v>46147.60297453704</v>
+      </c>
+      <c r="H23" s="1" t="n">
+        <v>46150</v>
       </c>
       <c r="I23" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J23" t="n">
         <v>2026</v>
       </c>
+      <c r="K23" t="n">
+        <v>5</v>
+      </c>
+      <c r="L23" t="n">
+        <v>2026</v>
+      </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>jsantacr@ccc.org.co</t>
+        </is>
+      </c>
       <c r="B24" t="inlineStr">
         <is>
           <t>Contactado</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>1200000</v>
+        <v>55000000</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Oportunidad de EMCALI E.I.C.E ESP</t>
+          <t>Oportunidad de CAMARA DE COMERCIO CALI</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1531,10 +1527,10 @@
         </is>
       </c>
       <c r="G24" s="1" t="n">
-        <v>46141.59045138889</v>
+        <v>46141.62370370371</v>
       </c>
       <c r="H24" s="1" t="n">
-        <v>46352</v>
+        <v>46289</v>
       </c>
       <c r="I24" t="n">
         <v>18</v>
@@ -1543,7 +1539,7 @@
         <v>2026</v>
       </c>
       <c r="K24" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="L24" t="n">
         <v>2026</v>
@@ -1557,12 +1553,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>angie_feligrana@eficacia.com.co</t>
+          <t>exportaciones@laprovincia.com</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Negociación</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -1570,7 +1566,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Oportunidad de Eficacia sas / Angie Feligrana</t>
+          <t>Oportunidad de PRODUCTOS LA PROVINCIA SAS</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1579,33 +1575,24 @@
         </is>
       </c>
       <c r="G25" s="1" t="n">
-        <v>46126.63210648148</v>
-      </c>
-      <c r="H25" s="1" t="n">
-        <v>46150</v>
+        <v>46141.62021990741</v>
       </c>
       <c r="I25" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J25" t="n">
         <v>2026</v>
       </c>
-      <c r="K25" t="n">
-        <v>5</v>
-      </c>
-      <c r="L25" t="n">
-        <v>2026</v>
-      </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Estrategiadigital@zuluagaysoto.com</t>
+          <t>coordinador.mercadeo@regency.com.co</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1616,14 +1603,9 @@
       <c r="C26" t="n">
         <v>0</v>
       </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>Maryuri Arguello</t>
-        </is>
-      </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Oportunidad de Maryuri Arguello</t>
+          <t>Oportunidad de REGENCY TECH SAS</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1632,10 +1614,10 @@
         </is>
       </c>
       <c r="G26" s="1" t="n">
-        <v>46125.71925925926</v>
+        <v>46141.59664351852</v>
       </c>
       <c r="I26" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J26" t="n">
         <v>2026</v>
@@ -1647,75 +1629,65 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>gabrielrodriguez@arrozsupremo.com</t>
-        </is>
-      </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Ganado</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>8000000</v>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>GABRIEL RODRIGUEZ</t>
-        </is>
+        <v>1200000</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Agente de Ventas</t>
+          <t>Oportunidad de EMCALI E.I.C.E ESP</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Richard Castaño</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G27" s="1" t="n">
-        <v>46119.62108796297</v>
+        <v>46141.59045138889</v>
       </c>
       <c r="H27" s="1" t="n">
-        <v>46141</v>
+        <v>46352</v>
       </c>
       <c r="I27" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="J27" t="n">
         <v>2026</v>
       </c>
       <c r="K27" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="L27" t="n">
         <v>2026</v>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Belkis.jimenez@agrauto.com.co</t>
+          <t>angie_feligrana@eficacia.com.co</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Negociación</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>0</v>
+        <v>6000000</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Oportunidad de AGRICOLA AUTOMOTRIZ SAS</t>
+          <t>Oportunidad de Eficacia sas / Angie Feligrana</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1724,24 +1696,33 @@
         </is>
       </c>
       <c r="G28" s="1" t="n">
-        <v>46119.38914351852</v>
+        <v>46126.63210648148</v>
+      </c>
+      <c r="H28" s="1" t="n">
+        <v>46150</v>
       </c>
       <c r="I28" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J28" t="n">
         <v>2026</v>
       </c>
+      <c r="K28" t="n">
+        <v>5</v>
+      </c>
+      <c r="L28" t="n">
+        <v>2026</v>
+      </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>anyela.aponza@cotel.com.co</t>
+          <t>Estrategiadigital@zuluagaysoto.com</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1752,9 +1733,14 @@
       <c r="C29" t="n">
         <v>0</v>
       </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Maryuri Arguello</t>
+        </is>
+      </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Oportunidad de COTEL SAL</t>
+          <t>Oportunidad de Maryuri Arguello</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1763,10 +1749,10 @@
         </is>
       </c>
       <c r="G29" s="1" t="n">
-        <v>46112.61271990741</v>
+        <v>46125.71925925926</v>
       </c>
       <c r="I29" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="J29" t="n">
         <v>2026</v>
@@ -1780,51 +1766,60 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>liliana.patino@quironsalud.com</t>
+          <t>gabrielrodriguez@arrozsupremo.com</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Ganado</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>0</v>
+        <v>8000000</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>CLINICA IMBANACO</t>
+          <t>GABRIEL RODRIGUEZ</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Oportunidad de Liliana Patiño Flórez</t>
+          <t>Agente de Ventas</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Richard Castaño</t>
         </is>
       </c>
       <c r="G30" s="1" t="n">
-        <v>46112.60853009259</v>
+        <v>46119.62108796297</v>
+      </c>
+      <c r="H30" s="1" t="n">
+        <v>46141</v>
       </c>
       <c r="I30" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="J30" t="n">
         <v>2026</v>
       </c>
+      <c r="K30" t="n">
+        <v>4</v>
+      </c>
+      <c r="L30" t="n">
+        <v>2026</v>
+      </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>casanchez@jgb.com.co</t>
+          <t>Belkis.jimenez@agrauto.com.co</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1837,7 +1832,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Oportunidad de JGB S.A.</t>
+          <t>Oportunidad de AGRICOLA AUTOMOTRIZ SAS</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1846,10 +1841,10 @@
         </is>
       </c>
       <c r="G31" s="1" t="n">
-        <v>46112.6052662037</v>
+        <v>46119.38914351852</v>
       </c>
       <c r="I31" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="J31" t="n">
         <v>2026</v>
@@ -1863,12 +1858,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>damaris.gomez@disfarma.com.co</t>
+          <t>anyela.aponza@cotel.com.co</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Seguimiento</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -1876,7 +1871,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Oportunidad de DISFARMA</t>
+          <t>Oportunidad de COTEL SAL</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1885,7 +1880,7 @@
         </is>
       </c>
       <c r="G32" s="1" t="n">
-        <v>46112.60325231482</v>
+        <v>46112.61271990741</v>
       </c>
       <c r="I32" t="n">
         <v>14</v>
@@ -1902,7 +1897,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>alergologosdeoccidente@gmail.com</t>
+          <t>liliana.patino@quironsalud.com</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1915,12 +1910,12 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Johana Gonzalez</t>
+          <t>CLINICA IMBANACO</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Oportunidad de Johana Gonzalez</t>
+          <t>Oportunidad de Liliana Patiño Flórez</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1929,10 +1924,10 @@
         </is>
       </c>
       <c r="G33" s="1" t="n">
-        <v>46107.51248842593</v>
+        <v>46112.60853009259</v>
       </c>
       <c r="I33" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J33" t="n">
         <v>2026</v>
@@ -1946,60 +1941,51 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>DavidEsteban.Porras@alfalaval.com</t>
+          <t>casanchez@jgb.com.co</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Ganado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>15000000</v>
+        <v>0</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Oportunidad de OPORTUNIDAD ENCUESTAS ALFALAVAL</t>
+          <t>Oportunidad de JGB S.A.</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G34" s="1" t="n">
-        <v>46101.72893518519</v>
-      </c>
-      <c r="H34" s="1" t="n">
-        <v>46141</v>
+        <v>46112.6052662037</v>
       </c>
       <c r="I34" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="J34" t="n">
         <v>2026</v>
       </c>
-      <c r="K34" t="n">
-        <v>4</v>
-      </c>
-      <c r="L34" t="n">
-        <v>2026</v>
-      </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Dr.arcarmona@gmail.com</t>
+          <t>damaris.gomez@disfarma.com.co</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Seguimiento</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -2007,7 +1993,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Oportunidad de GAMANUCLEAR LTDA - Dr Alberto Carmona</t>
+          <t>Oportunidad de DISFARMA</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -2016,10 +2002,10 @@
         </is>
       </c>
       <c r="G35" s="1" t="n">
-        <v>46098.65114583333</v>
+        <v>46112.60325231482</v>
       </c>
       <c r="I35" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="J35" t="n">
         <v>2026</v>
@@ -2033,7 +2019,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>cecilia.guevara@cosmitet.net / administracion.crd@cosmitet.net</t>
+          <t>alergologosdeoccidente@gmail.com</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2046,12 +2032,12 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Cecilia Guevara</t>
+          <t>Johana Gonzalez</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Oportunidad de CLINICA REY DAVID Walter Charria</t>
+          <t>Oportunidad de Johana Gonzalez</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -2060,10 +2046,10 @@
         </is>
       </c>
       <c r="G36" s="1" t="n">
-        <v>46094.69002314815</v>
+        <v>46107.51248842593</v>
       </c>
       <c r="I36" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="J36" t="n">
         <v>2026</v>
@@ -2077,104 +2063,94 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>vicerrectoriacademica@unicatolica.edu.co</t>
+          <t>DavidEsteban.Porras@alfalaval.com</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Ganado</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>0</v>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>Jorge Silva</t>
-        </is>
+        <v>15000000</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Oportunidad de Jorge Silva</t>
+          <t>Oportunidad de OPORTUNIDAD ENCUESTAS ALFALAVAL</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G37" s="1" t="n">
-        <v>46094.66880787037</v>
+        <v>46101.72893518519</v>
+      </c>
+      <c r="H37" s="1" t="n">
+        <v>46141</v>
       </c>
       <c r="I37" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J37" t="n">
         <v>2026</v>
       </c>
+      <c r="K37" t="n">
+        <v>4</v>
+      </c>
+      <c r="L37" t="n">
+        <v>2026</v>
+      </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>pedroperea02@gmail.com</t>
+          <t>Dr.arcarmona@gmail.com</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Ganado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>2160000</v>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>Pedro Pablo Perea Mafla</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Oportunidad de Encuestas</t>
+          <t>Oportunidad de GAMANUCLEAR LTDA - Dr Alberto Carmona</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G38" s="1" t="n">
-        <v>46094.65905092593</v>
-      </c>
-      <c r="H38" s="1" t="n">
-        <v>46141</v>
+        <v>46098.65114583333</v>
       </c>
       <c r="I38" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J38" t="n">
         <v>2026</v>
       </c>
-      <c r="K38" t="n">
-        <v>4</v>
-      </c>
-      <c r="L38" t="n">
-        <v>2026</v>
-      </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>cristina.papamija@bmm.com.co</t>
+          <t>cecilia.guevara@cosmitet.net / administracion.crd@cosmitet.net</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2183,20 +2159,25 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>8071000</v>
+        <v>0</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Cecilia Guevara</t>
+        </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Oportunidad de BANCO MUNDO MUJER</t>
+          <t>Oportunidad de CLINICA REY DAVID Walter Charria</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G39" s="1" t="n">
-        <v>46094.65019675926</v>
+        <v>46094.69002314815</v>
       </c>
       <c r="I39" t="n">
         <v>11</v>
@@ -2213,7 +2194,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>capacitacionvirtual@fundacionwwbcol.org</t>
+          <t>vicerrectoriacademica@unicatolica.edu.co</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2222,20 +2203,25 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>1600000</v>
+        <v>0</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Jorge Silva</t>
+        </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Licenciamiento y ajuste WhatsApp FUNDACIÓN WWB</t>
+          <t>Oportunidad de Jorge Silva</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G40" s="1" t="n">
-        <v>46094.64826388889</v>
+        <v>46094.66880787037</v>
       </c>
       <c r="I40" t="n">
         <v>11</v>
@@ -2252,7 +2238,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>carol.cuesta@cbolivar.com</t>
+          <t>pedroperea02@gmail.com</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2261,16 +2247,16 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>2900000</v>
+        <v>2160000</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>CAROL CUESTA</t>
+          <t>Pedro Pablo Perea Mafla</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Gestión de Subsidios CB Bogotá</t>
+          <t>Oportunidad de Encuestas</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2279,10 +2265,10 @@
         </is>
       </c>
       <c r="G41" s="1" t="n">
-        <v>46094.64454861111</v>
+        <v>46094.65905092593</v>
       </c>
       <c r="H41" s="1" t="n">
-        <v>46135</v>
+        <v>46141</v>
       </c>
       <c r="I41" t="n">
         <v>11</v>
@@ -2305,7 +2291,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>edwin.munoz.v@uniminuto.edu</t>
+          <t>cristina.papamija@bmm.com.co</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2314,20 +2300,20 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>0</v>
+        <v>8071000</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Oportunidad de UNIMINUTO</t>
+          <t>Oportunidad de BANCO MUNDO MUJER</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G42" s="1" t="n">
-        <v>46092.63626157407</v>
+        <v>46094.65019675926</v>
       </c>
       <c r="I42" t="n">
         <v>11</v>
@@ -2344,7 +2330,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>jaime_zuluaga@eficacia.com.co</t>
+          <t>capacitacionvirtual@fundacionwwbcol.org</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2353,25 +2339,20 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>0</v>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>Jaime Alberto</t>
-        </is>
+        <v>1600000</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Oportunidad de Jaime Alberto Zuluaga</t>
+          <t>Licenciamiento y ajuste WhatsApp FUNDACIÓN WWB</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G43" s="1" t="n">
-        <v>46092.63153935185</v>
+        <v>46094.64826388889</v>
       </c>
       <c r="I43" t="n">
         <v>11</v>
@@ -2388,34 +2369,37 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>comercial@isyscol.com</t>
+          <t>carol.cuesta@cbolivar.com</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Ganado</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>0</v>
+        <v>2900000</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Andres Nader</t>
+          <t>CAROL CUESTA</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Oportunidad de Andres Nader</t>
+          <t>Gestión de Subsidios CB Bogotá</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G44" s="1" t="n">
-        <v>46091.59211805555</v>
+        <v>46094.64454861111</v>
+      </c>
+      <c r="H44" s="1" t="n">
+        <v>46135</v>
       </c>
       <c r="I44" t="n">
         <v>11</v>
@@ -2423,16 +2407,22 @@
       <c r="J44" t="n">
         <v>2026</v>
       </c>
+      <c r="K44" t="n">
+        <v>4</v>
+      </c>
+      <c r="L44" t="n">
+        <v>2026</v>
+      </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>mercadeo@norteysur.co</t>
+          <t>edwin.munoz.v@uniminuto.edu</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2443,14 +2433,9 @@
       <c r="C45" t="n">
         <v>0</v>
       </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>Isabella Mesa</t>
-        </is>
-      </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Oportunidad de Isabella Mesa</t>
+          <t>Oportunidad de UNIMINUTO</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -2459,7 +2444,7 @@
         </is>
       </c>
       <c r="G45" s="1" t="n">
-        <v>46091.40078703704</v>
+        <v>46092.63626157407</v>
       </c>
       <c r="I45" t="n">
         <v>11</v>
@@ -2474,26 +2459,36 @@
       </c>
     </row>
     <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>jaime_zuluaga@eficacia.com.co</t>
+        </is>
+      </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Seguimiento</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C46" t="n">
         <v>0</v>
       </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Jaime Alberto</t>
+        </is>
+      </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Clasificación EMAIL Comfenalco Cartagena</t>
+          <t>Oportunidad de Jaime Alberto Zuluaga</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Maria Fernanda Gaviria</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G46" s="1" t="n">
-        <v>46091.3665625</v>
+        <v>46092.63153935185</v>
       </c>
       <c r="I46" t="n">
         <v>11</v>
@@ -2508,6 +2503,11 @@
       </c>
     </row>
     <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>comercial@isyscol.com</t>
+        </is>
+      </c>
       <c r="B47" t="inlineStr">
         <is>
           <t>Perdido</t>
@@ -2516,21 +2516,26 @@
       <c r="C47" t="n">
         <v>0</v>
       </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Andres Nader</t>
+        </is>
+      </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Oportunidad de ESE HOSPITAL LA MARIA</t>
+          <t>Oportunidad de Andres Nader</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Laura Alejandra Castañeda</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G47" s="1" t="n">
-        <v>46083.67605324074</v>
+        <v>46091.59211805555</v>
       </c>
       <c r="I47" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J47" t="n">
         <v>2026</v>
@@ -2542,6 +2547,11 @@
       </c>
     </row>
     <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>mercadeo@norteysur.co</t>
+        </is>
+      </c>
       <c r="B48" t="inlineStr">
         <is>
           <t>Perdido</t>
@@ -2550,21 +2560,26 @@
       <c r="C48" t="n">
         <v>0</v>
       </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Isabella Mesa</t>
+        </is>
+      </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Oportunidad de SUPER TRANSPORTE</t>
+          <t>Oportunidad de Isabella Mesa</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Laura Alejandra Castañeda</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G48" s="1" t="n">
-        <v>46083.6706712963</v>
+        <v>46091.40078703704</v>
       </c>
       <c r="I48" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J48" t="n">
         <v>2026</v>
@@ -2578,7 +2593,7 @@
     <row r="49">
       <c r="B49" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Seguimiento</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -2586,19 +2601,19 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Oportunidad de ENLACES IP S.A.S</t>
+          <t>Clasificación EMAIL Comfenalco Cartagena</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Laura Alejandra Castañeda</t>
+          <t>Maria Fernanda Gaviria</t>
         </is>
       </c>
       <c r="G49" s="1" t="n">
-        <v>46083.50145833333</v>
+        <v>46091.3665625</v>
       </c>
       <c r="I49" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J49" t="n">
         <v>2026</v>
@@ -2610,11 +2625,6 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>accounting@diaza.com</t>
-        </is>
-      </c>
       <c r="B50" t="inlineStr">
         <is>
           <t>Perdido</t>
@@ -2623,26 +2633,21 @@
       <c r="C50" t="n">
         <v>0</v>
       </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>JOHANA RODRIGUEZ</t>
-        </is>
-      </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Oportunidad de JOHANA RODRIGUEZ</t>
+          <t>Oportunidad de ESE HOSPITAL LA MARIA</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Laura Alejandra Castañeda</t>
         </is>
       </c>
       <c r="G50" s="1" t="n">
-        <v>46079.73486111111</v>
+        <v>46083.67605324074</v>
       </c>
       <c r="I50" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J50" t="n">
         <v>2026</v>
@@ -2654,11 +2659,6 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>mensajeriamyr@gmail.com</t>
-        </is>
-      </c>
       <c r="B51" t="inlineStr">
         <is>
           <t>Perdido</t>
@@ -2669,19 +2669,19 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Oportunidad de MENSAJERIA M&amp;R SAS</t>
+          <t>Oportunidad de SUPER TRANSPORTE</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Laura Alejandra Castañeda</t>
         </is>
       </c>
       <c r="G51" s="1" t="n">
-        <v>46079.72262731481</v>
+        <v>46083.6706712963</v>
       </c>
       <c r="I51" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J51" t="n">
         <v>2026</v>
@@ -2693,11 +2693,6 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>sistemaspanaderialeal@gmail.com</t>
-        </is>
-      </c>
       <c r="B52" t="inlineStr">
         <is>
           <t>Perdido</t>
@@ -2706,26 +2701,21 @@
       <c r="C52" t="n">
         <v>0</v>
       </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>Diego Rios</t>
-        </is>
-      </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>JAMDAC SAS, Diego Rios</t>
+          <t>Oportunidad de ENLACES IP S.A.S</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Laura Alejandra Castañeda</t>
         </is>
       </c>
       <c r="G52" s="1" t="n">
-        <v>46071.63706018519</v>
+        <v>46083.50145833333</v>
       </c>
       <c r="I52" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="J52" t="n">
         <v>2026</v>
@@ -2739,7 +2729,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>efernandez@unico.com.co</t>
+          <t>accounting@diaza.com</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2752,12 +2742,12 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Erick Fernandez</t>
+          <t>JOHANA RODRIGUEZ</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Oportunidad de Erick Fernandez</t>
+          <t>Oportunidad de JOHANA RODRIGUEZ</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -2766,10 +2756,10 @@
         </is>
       </c>
       <c r="G53" s="1" t="n">
-        <v>46064.3750462963</v>
+        <v>46079.73486111111</v>
       </c>
       <c r="I53" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="J53" t="n">
         <v>2026</v>
@@ -2783,7 +2773,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>kabenitez@icesi.edu.co</t>
+          <t>mensajeriamyr@gmail.com</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2792,28 +2782,23 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>10000000</v>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>KENI BENITEZ</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Oportunidad de KENI BENITEZ</t>
+          <t>Oportunidad de MENSAJERIA M&amp;R SAS</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G54" s="1" t="n">
-        <v>46059.34918981481</v>
+        <v>46079.72262731481</v>
       </c>
       <c r="I54" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J54" t="n">
         <v>2026</v>
@@ -2827,7 +2812,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>patovar@uao.edu.co</t>
+          <t>sistemaspanaderialeal@gmail.com</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2840,12 +2825,12 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Paula Tovar</t>
+          <t>Diego Rios</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Oportunidad de UNIVERSIDAD AUTONOMA DE OCCIDENTE</t>
+          <t>JAMDAC SAS, Diego Rios</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -2854,10 +2839,10 @@
         </is>
       </c>
       <c r="G55" s="1" t="n">
-        <v>46058.72516203704</v>
+        <v>46071.63706018519</v>
       </c>
       <c r="I55" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J55" t="n">
         <v>2026</v>
@@ -2871,7 +2856,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>comercial@isyscol.com</t>
+          <t>efernandez@unico.com.co</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2882,9 +2867,14 @@
       <c r="C56" t="n">
         <v>0</v>
       </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Erick Fernandez</t>
+        </is>
+      </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Oportunidad de TECNOLOGIAS ISYSCOL SAS</t>
+          <t>Oportunidad de Erick Fernandez</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -2893,10 +2883,10 @@
         </is>
       </c>
       <c r="G56" s="1" t="n">
-        <v>46057.58993055556</v>
+        <v>46064.3750462963</v>
       </c>
       <c r="I56" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J56" t="n">
         <v>2026</v>
@@ -2908,26 +2898,36 @@
       </c>
     </row>
     <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>kabenitez@icesi.edu.co</t>
+        </is>
+      </c>
       <c r="B57" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>15000000</v>
+        <v>10000000</v>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>KENI BENITEZ</t>
+        </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Oportunidad de VOICE IA EFICACIA</t>
+          <t>Oportunidad de KENI BENITEZ</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G57" s="1" t="n">
-        <v>46057.3409837963</v>
+        <v>46059.34918981481</v>
       </c>
       <c r="I57" t="n">
         <v>6</v>
@@ -2942,29 +2942,39 @@
       </c>
     </row>
     <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>patovar@uao.edu.co</t>
+        </is>
+      </c>
       <c r="B58" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>4000000</v>
+        <v>0</v>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Paula Tovar</t>
+        </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Oportunidad de Eficacia WhatsApp</t>
+          <t>Oportunidad de UNIVERSIDAD AUTONOMA DE OCCIDENTE</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G58" s="1" t="n">
-        <v>46049.67292824074</v>
+        <v>46058.72516203704</v>
       </c>
       <c r="I58" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J58" t="n">
         <v>2026</v>
@@ -2976,32 +2986,37 @@
       </c>
     </row>
     <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>comercial@isyscol.com</t>
+        </is>
+      </c>
       <c r="B59" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>20000000</v>
+        <v>0</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Oportunidad de CRUZ ROJA COLOMBIANA SECCIONAL VALLE DEL CAUCA</t>
+          <t>Oportunidad de TECNOLOGIAS ISYSCOL SAS</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G59" s="1" t="n">
-        <v>46006.49650462963</v>
+        <v>46057.58993055556</v>
       </c>
       <c r="I59" t="n">
-        <v>51</v>
+        <v>6</v>
       </c>
       <c r="J59" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="M59" t="inlineStr">
         <is>
@@ -3010,37 +3025,32 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>silvia.figueroa@neurithmedia.com</t>
-        </is>
-      </c>
       <c r="B60" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>25000000</v>
+        <v>15000000</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Contact center ventas España</t>
+          <t>Oportunidad de VOICE IA EFICACIA</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Richard Castaño</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G60" s="1" t="n">
-        <v>45960.61145833333</v>
+        <v>46057.3409837963</v>
       </c>
       <c r="I60" t="n">
-        <v>44</v>
+        <v>6</v>
       </c>
       <c r="J60" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="M60" t="inlineStr">
         <is>
@@ -3055,31 +3065,26 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>37000000</v>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>Mabel</t>
-        </is>
+        <v>4000000</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Masivos Licitacion</t>
+          <t>Oportunidad de Eficacia WhatsApp</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Richard Castaño</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G61" s="1" t="n">
-        <v>45940.49372685186</v>
+        <v>46049.67292824074</v>
       </c>
       <c r="I61" t="n">
-        <v>41</v>
+        <v>5</v>
       </c>
       <c r="J61" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="M61" t="inlineStr">
         <is>
@@ -3088,27 +3093,17 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>ana.zuniga@cbolivar.com</t>
-        </is>
-      </c>
       <c r="B62" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>4997000</v>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>Ana Lucia Zuñiga</t>
-        </is>
+        <v>20000000</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Constructora Bolivar Agente Redes</t>
+          <t>Oportunidad de CRUZ ROJA COLOMBIANA SECCIONAL VALLE DEL CAUCA</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -3117,10 +3112,10 @@
         </is>
       </c>
       <c r="G62" s="1" t="n">
-        <v>45940.49215277778</v>
+        <v>46006.49650462963</v>
       </c>
       <c r="I62" t="n">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="J62" t="n">
         <v>2025</v>
@@ -3134,7 +3129,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>julian_mendez@extras.com.co</t>
+          <t>silvia.figueroa@neurithmedia.com</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3143,28 +3138,23 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>15000000</v>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>Julian Mendez.</t>
-        </is>
+        <v>25000000</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Oportunidad de EFICACIA S A S</t>
+          <t>Contact center ventas España</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Richard Castaño</t>
         </is>
       </c>
       <c r="G63" s="1" t="n">
-        <v>45922.66201388889</v>
+        <v>45960.61145833333</v>
       </c>
       <c r="I63" t="n">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="J63" t="n">
         <v>2025</v>
@@ -3176,34 +3166,34 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>info@eficacia.com.co</t>
-        </is>
-      </c>
       <c r="B64" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>0</v>
+        <v>37000000</v>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Mabel</t>
+        </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Nutresa</t>
+          <t>Masivos Licitacion</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Richard Castaño</t>
         </is>
       </c>
       <c r="G64" s="1" t="n">
-        <v>45922.66199074074</v>
+        <v>45940.49372685186</v>
       </c>
       <c r="I64" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="J64" t="n">
         <v>2025</v>
@@ -3217,37 +3207,37 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>hrodriguez@jaramillomora.com</t>
+          <t>ana.zuniga@cbolivar.com</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Seguimiento</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>30000000</v>
+        <v>4997000</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>HANNA</t>
+          <t>Ana Lucia Zuñiga</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Oportunidad de JARAMILLO MORA CONSTRUCTORA S A</t>
+          <t>Constructora Bolivar Agente Redes</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Richard Castaño</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G65" s="1" t="n">
-        <v>45916.71618055556</v>
+        <v>45940.49215277778</v>
       </c>
       <c r="I65" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="J65" t="n">
         <v>2025</v>
@@ -3259,29 +3249,39 @@
       </c>
     </row>
     <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>julian_mendez@extras.com.co</t>
+        </is>
+      </c>
       <c r="B66" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>147000000</v>
+        <v>15000000</v>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Julian Mendez.</t>
+        </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Contact Center Agendamiento citas</t>
+          <t>Oportunidad de EFICACIA S A S</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Richard Castaño</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G66" s="1" t="n">
-        <v>45916.67502314815</v>
+        <v>45922.66201388889</v>
       </c>
       <c r="I66" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="J66" t="n">
         <v>2025</v>
@@ -3295,7 +3295,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>jaime_zuluaga@eficacia.com.co</t>
+          <t>info@eficacia.com.co</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3304,11 +3304,11 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>14700000</v>
+        <v>0</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Agentes contact center encuestas</t>
+          <t>Nutresa</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -3317,23 +3317,14 @@
         </is>
       </c>
       <c r="G67" s="1" t="n">
-        <v>45916.65275462963</v>
-      </c>
-      <c r="H67" s="1" t="n">
-        <v>45930</v>
+        <v>45922.66199074074</v>
       </c>
       <c r="I67" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="J67" t="n">
         <v>2025</v>
       </c>
-      <c r="K67" t="n">
-        <v>9</v>
-      </c>
-      <c r="L67" t="n">
-        <v>2025</v>
-      </c>
       <c r="M67" t="inlineStr">
         <is>
           <t>No calificado</t>
@@ -3341,31 +3332,36 @@
       </c>
     </row>
     <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>hrodriguez@jaramillomora.com</t>
+        </is>
+      </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Seguimiento</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>4796000</v>
+        <v>30000000</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Juan Grisales</t>
+          <t>HANNA</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Agente Call Center Outbound</t>
+          <t>Oportunidad de JARAMILLO MORA CONSTRUCTORA S A</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Richard Castaño</t>
         </is>
       </c>
       <c r="G68" s="1" t="n">
-        <v>45915.4809375</v>
+        <v>45916.71618055556</v>
       </c>
       <c r="I68" t="n">
         <v>38</v>
@@ -3380,39 +3376,26 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>gestormercadeo@lamontana.co</t>
-        </is>
-      </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Seguimiento</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>25000000</v>
-      </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>Alejandra Ossa</t>
-        </is>
+        <v>147000000</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Voice BOT</t>
+          <t>Contact Center Agendamiento citas</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Richard Castaño</t>
         </is>
       </c>
       <c r="G69" s="1" t="n">
-        <v>45915.48023148148</v>
-      </c>
-      <c r="H69" s="1" t="n">
-        <v>46150</v>
+        <v>45916.67502314815</v>
       </c>
       <c r="I69" t="n">
         <v>38</v>
@@ -3420,12 +3403,6 @@
       <c r="J69" t="n">
         <v>2025</v>
       </c>
-      <c r="K69" t="n">
-        <v>5</v>
-      </c>
-      <c r="L69" t="n">
-        <v>2026</v>
-      </c>
       <c r="M69" t="inlineStr">
         <is>
           <t>No calificado</t>
@@ -3435,7 +3412,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>elkinmarquezconsuegra@gmail.com</t>
+          <t>jaime_zuluaga@eficacia.com.co</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -3444,11 +3421,11 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>2500000</v>
+        <v>14700000</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Venta Masivos</t>
+          <t>Agentes contact center encuestas</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -3457,7 +3434,10 @@
         </is>
       </c>
       <c r="G70" s="1" t="n">
-        <v>45915.47924768519</v>
+        <v>45916.65275462963</v>
+      </c>
+      <c r="H70" s="1" t="n">
+        <v>45930</v>
       </c>
       <c r="I70" t="n">
         <v>38</v>
@@ -3465,6 +3445,12 @@
       <c r="J70" t="n">
         <v>2025</v>
       </c>
+      <c r="K70" t="n">
+        <v>9</v>
+      </c>
+      <c r="L70" t="n">
+        <v>2025</v>
+      </c>
       <c r="M70" t="inlineStr">
         <is>
           <t>No calificado</t>
@@ -3472,27 +3458,22 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>bladimir.munoz@uptc.edu.co</t>
-        </is>
-      </c>
       <c r="B71" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>22000000</v>
+        <v>4796000</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Bladimir Muñoz Forero</t>
+          <t>Juan Grisales</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Oportunidad Venta BPO</t>
+          <t>Agente Call Center Outbound</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -3501,7 +3482,7 @@
         </is>
       </c>
       <c r="G71" s="1" t="n">
-        <v>45915.47494212963</v>
+        <v>45915.4809375</v>
       </c>
       <c r="I71" t="n">
         <v>38</v>
@@ -3518,29 +3499,37 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>gerencia@alitasfactory.com</t>
+          <t>gestormercadeo@lamontana.co</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Seguimiento</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>40000000</v>
+        <v>25000000</v>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Alejandra Ossa</t>
+        </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>1 agente IA para ventas y asesoramiento</t>
+          <t>Voice BOT</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Richard Castaño</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G72" s="1" t="n">
-        <v>45915.47300925926</v>
+        <v>45915.48023148148</v>
+      </c>
+      <c r="H72" s="1" t="n">
+        <v>46150</v>
       </c>
       <c r="I72" t="n">
         <v>38</v>
@@ -3548,6 +3537,12 @@
       <c r="J72" t="n">
         <v>2025</v>
       </c>
+      <c r="K72" t="n">
+        <v>5</v>
+      </c>
+      <c r="L72" t="n">
+        <v>2026</v>
+      </c>
       <c r="M72" t="inlineStr">
         <is>
           <t>No calificado</t>
@@ -3557,7 +3552,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>mmonroy@falabella.com.co</t>
+          <t>elkinmarquezconsuegra@gmail.com</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -3566,20 +3561,20 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>60000000</v>
+        <v>2500000</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Agente IA Try and Buy Inbound y Outbound</t>
+          <t>Venta Masivos</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Richard Castaño</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G73" s="1" t="n">
-        <v>45915.46633101852</v>
+        <v>45915.47924768519</v>
       </c>
       <c r="I73" t="n">
         <v>38</v>
@@ -3596,7 +3591,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>gerencia@motosymotoselpaisa.com</t>
+          <t>bladimir.munoz@uptc.edu.co</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -3605,11 +3600,16 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>40000000</v>
+        <v>22000000</v>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Bladimir Muñoz Forero</t>
+        </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Oportunidad de MOTOS Y MOTOS EL PAISA S A S</t>
+          <t>Oportunidad Venta BPO</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -3618,7 +3618,7 @@
         </is>
       </c>
       <c r="G74" s="1" t="n">
-        <v>45915.46252314815</v>
+        <v>45915.47494212963</v>
       </c>
       <c r="I74" t="n">
         <v>38</v>
@@ -3635,7 +3635,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>isanchez@unico.com.co</t>
+          <t>gerencia@alitasfactory.com</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -3644,20 +3644,20 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>0</v>
+        <v>40000000</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>1 agente IA para relacionamiento con locatarios</t>
+          <t>1 agente IA para ventas y asesoramiento</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Richard Castaño</t>
         </is>
       </c>
       <c r="G75" s="1" t="n">
-        <v>45915.46157407408</v>
+        <v>45915.47300925926</v>
       </c>
       <c r="I75" t="n">
         <v>38</v>
@@ -3674,7 +3674,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>asantiago@stop.com.co</t>
+          <t>mmonroy@falabella.com.co</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -3683,20 +3683,20 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>30000000</v>
+        <v>60000000</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>1 Agente IA en cobranzas</t>
+          <t>Agente IA Try and Buy Inbound y Outbound</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Richard Castaño</t>
         </is>
       </c>
       <c r="G76" s="1" t="n">
-        <v>45915.46052083333</v>
+        <v>45915.46633101852</v>
       </c>
       <c r="I76" t="n">
         <v>38</v>
@@ -3713,7 +3713,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>jcastano@mercaldas.com.co</t>
+          <t>gerencia@motosymotoselpaisa.com</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -3722,11 +3722,11 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>30000000</v>
+        <v>40000000</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>1 agente IA para ventas y asesoramiento</t>
+          <t>Oportunidad de MOTOS Y MOTOS EL PAISA S A S</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -3735,7 +3735,7 @@
         </is>
       </c>
       <c r="G77" s="1" t="n">
-        <v>45915.35666666667</v>
+        <v>45915.46252314815</v>
       </c>
       <c r="I77" t="n">
         <v>38</v>
@@ -3752,7 +3752,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>calidad@cempac.com.co</t>
+          <t>isanchez@unico.com.co</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -3761,11 +3761,11 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>42000000</v>
+        <v>0</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>1 agente IA para ventas y asesoramiento</t>
+          <t>1 agente IA para relacionamiento con locatarios</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -3774,7 +3774,7 @@
         </is>
       </c>
       <c r="G78" s="1" t="n">
-        <v>45915.35537037037</v>
+        <v>45915.46157407408</v>
       </c>
       <c r="I78" t="n">
         <v>38</v>
@@ -3791,7 +3791,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>info@eficacia.com.co</t>
+          <t>asantiago@stop.com.co</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -3800,20 +3800,20 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>15000000</v>
+        <v>30000000</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Requieren IA para PQRS y exploran otras opciones</t>
+          <t>1 Agente IA en cobranzas</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G79" s="1" t="n">
-        <v>45915.35351851852</v>
+        <v>45915.46052083333</v>
       </c>
       <c r="I79" t="n">
         <v>38</v>
@@ -3830,7 +3830,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>orlandogomez@grupogiraldo.com</t>
+          <t>jcastano@mercaldas.com.co</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -3841,11 +3841,6 @@
       <c r="C80" t="n">
         <v>30000000</v>
       </c>
-      <c r="D80" t="inlineStr">
-        <is>
-          <t>Orlando Gomez</t>
-        </is>
-      </c>
       <c r="E80" t="inlineStr">
         <is>
           <t>1 agente IA para ventas y asesoramiento</t>
@@ -3857,7 +3852,7 @@
         </is>
       </c>
       <c r="G80" s="1" t="n">
-        <v>45915.34180555555</v>
+        <v>45915.35666666667</v>
       </c>
       <c r="I80" t="n">
         <v>38</v>
@@ -3874,7 +3869,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>c.roman@chipichape.com.co</t>
+          <t>calidad@cempac.com.co</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -3883,11 +3878,11 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>60000000</v>
+        <v>42000000</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>3 Agentes IA</t>
+          <t>1 agente IA para ventas y asesoramiento</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -3896,7 +3891,7 @@
         </is>
       </c>
       <c r="G81" s="1" t="n">
-        <v>45915.33471064815</v>
+        <v>45915.35537037037</v>
       </c>
       <c r="I81" t="n">
         <v>38</v>

</xml_diff>

<commit_message>
CRM actualizado — 20/05/2026 16:01
</commit_message>
<xml_diff>
--- a/CRM_PowerBI_BrendaLuna_actualizado.xlsx
+++ b/CRM_PowerBI_BrendaLuna_actualizado.xlsx
@@ -946,7 +946,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>asantiago@stop.com.co</t>
+          <t>mercadeo@lasevillana.com.co</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -957,9 +957,14 @@
       <c r="C11" t="n">
         <v>0</v>
       </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fabio AlbertoGallego García </t>
+        </is>
+      </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Oportunidad de STOP SAS</t>
+          <t xml:space="preserve">Oportunidad de Fabio AlbertoGallego García </t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -968,7 +973,7 @@
         </is>
       </c>
       <c r="G11" s="1" t="n">
-        <v>46161.63508101852</v>
+        <v>46162.64569444444</v>
       </c>
       <c r="I11" t="n">
         <v>21</v>
@@ -985,7 +990,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>aestrada@teker.co</t>
+          <t>asantiago@stop.com.co</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -996,14 +1001,9 @@
       <c r="C12" t="n">
         <v>0</v>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>TEKER SALUD SAS</t>
-        </is>
-      </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Oportunidad de TEKER SALUD SAS</t>
+          <t>Oportunidad de STOP SAS</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1012,7 +1012,7 @@
         </is>
       </c>
       <c r="G12" s="1" t="n">
-        <v>46161.62922453704</v>
+        <v>46161.63508101852</v>
       </c>
       <c r="I12" t="n">
         <v>21</v>
@@ -1027,6 +1027,11 @@
       </c>
     </row>
     <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>aestrada@teker.co</t>
+        </is>
+      </c>
       <c r="B13" t="inlineStr">
         <is>
           <t>Nuevo</t>
@@ -1035,9 +1040,14 @@
       <c r="C13" t="n">
         <v>0</v>
       </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>TEKER SALUD SAS</t>
+        </is>
+      </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Oportunidad de TIAN IPS SAS</t>
+          <t>Oportunidad de TEKER SALUD SAS</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1046,7 +1056,7 @@
         </is>
       </c>
       <c r="G13" s="1" t="n">
-        <v>46161.61643518518</v>
+        <v>46161.62922453704</v>
       </c>
       <c r="I13" t="n">
         <v>21</v>
@@ -1061,11 +1071,6 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>administración@fullredtotal.com</t>
-        </is>
-      </c>
       <c r="B14" t="inlineStr">
         <is>
           <t>Nuevo</t>
@@ -1074,14 +1079,9 @@
       <c r="C14" t="n">
         <v>0</v>
       </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Eivar Eñasco</t>
-        </is>
-      </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Oportunidad de Eivar Eñasco</t>
+          <t>Oportunidad de TIAN IPS SAS</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1090,10 +1090,10 @@
         </is>
       </c>
       <c r="G14" s="1" t="n">
-        <v>46154.67546296296</v>
+        <v>46161.61643518518</v>
       </c>
       <c r="I14" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J14" t="n">
         <v>2026</v>
@@ -1107,25 +1107,25 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>cserna@surtifamiliar.com.co</t>
+          <t>administración@fullredtotal.com</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Negociación</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1950000</v>
+        <v>0</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Claudia Patricia Serna</t>
+          <t>Eivar Eñasco</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Oportunidad de Claudia Patricia Serna</t>
+          <t>Oportunidad de Eivar Eñasco</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1134,7 +1134,7 @@
         </is>
       </c>
       <c r="G15" s="1" t="n">
-        <v>46154.66616898148</v>
+        <v>46154.67546296296</v>
       </c>
       <c r="I15" t="n">
         <v>20</v>
@@ -1144,32 +1144,32 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>coordmercadeo@pacificcenter.co</t>
+          <t>cserna@surtifamiliar.com.co</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Negociación</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0</v>
+        <v>1950000</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Claudia Castro</t>
+          <t>Claudia Patricia Serna</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Oportunidad de Claudia Castro</t>
+          <t>Oportunidad de Claudia Patricia Serna</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1178,7 +1178,7 @@
         </is>
       </c>
       <c r="G16" s="1" t="n">
-        <v>46154.66341435185</v>
+        <v>46154.66616898148</v>
       </c>
       <c r="I16" t="n">
         <v>20</v>
@@ -1188,14 +1188,14 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>isabellarengifo27@gmail.com</t>
+          <t>coordmercadeo@pacificcenter.co</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1204,16 +1204,16 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>16000000</v>
+        <v>0</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Isabella Rengifo</t>
+          <t>Claudia Castro</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Oportunidad de Isabella Rengifo</t>
+          <t>Oportunidad de Claudia Castro</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1222,7 +1222,7 @@
         </is>
       </c>
       <c r="G17" s="1" t="n">
-        <v>46154.65981481481</v>
+        <v>46154.66341435185</v>
       </c>
       <c r="I17" t="n">
         <v>20</v>
@@ -1237,34 +1237,36 @@
       </c>
     </row>
     <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>isabellarengifo27@gmail.com</t>
+        </is>
+      </c>
       <c r="B18" t="inlineStr">
         <is>
           <t>Propuesta</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>50000000</v>
+        <v>28190000</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Paola Gómez - Agente Inmobiliaria Independiente</t>
+          <t>Isabella Rengifo</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Puesto de Trabajo CC Medellin</t>
+          <t>Oportunidad de Isabella Rengifo</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Richard Castaño</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G18" s="1" t="n">
-        <v>46154.49104166667</v>
-      </c>
-      <c r="H18" s="1" t="n">
-        <v>46170</v>
+        <v>46154.65981481481</v>
       </c>
       <c r="I18" t="n">
         <v>20</v>
@@ -1272,12 +1274,6 @@
       <c r="J18" t="n">
         <v>2026</v>
       </c>
-      <c r="K18" t="n">
-        <v>5</v>
-      </c>
-      <c r="L18" t="n">
-        <v>2026</v>
-      </c>
       <c r="M18" t="inlineStr">
         <is>
           <t>Calificado</t>
@@ -1285,31 +1281,34 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>alberto.ramirez@constructorabolivar.com</t>
-        </is>
-      </c>
       <c r="B19" t="inlineStr">
         <is>
           <t>Propuesta</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>3000000</v>
+        <v>50000000</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Paola Gómez - Agente Inmobiliaria Independiente</t>
+        </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Oportunidad de NPS Relacional</t>
+          <t>Puesto de Trabajo CC Medellin</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Richard Castaño</t>
         </is>
       </c>
       <c r="G19" s="1" t="n">
-        <v>46154.44511574074</v>
+        <v>46154.49104166667</v>
+      </c>
+      <c r="H19" s="1" t="n">
+        <v>46170</v>
       </c>
       <c r="I19" t="n">
         <v>20</v>
@@ -1317,6 +1316,12 @@
       <c r="J19" t="n">
         <v>2026</v>
       </c>
+      <c r="K19" t="n">
+        <v>5</v>
+      </c>
+      <c r="L19" t="n">
+        <v>2026</v>
+      </c>
       <c r="M19" t="inlineStr">
         <is>
           <t>Calificado</t>
@@ -1324,75 +1329,70 @@
       </c>
     </row>
     <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>alberto.ramirez@constructorabolivar.com</t>
+        </is>
+      </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C20" t="n">
         <v>3000000</v>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Oportunidad de NPS Relacional</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Jennifer Hoyos Gallego</t>
+        </is>
+      </c>
+      <c r="G20" s="1" t="n">
+        <v>46154.44511574074</v>
+      </c>
+      <c r="I20" t="n">
+        <v>20</v>
+      </c>
+      <c r="J20" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>Calificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="D21" t="inlineStr">
         <is>
           <t>MADERKIT</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>Oportunidad de MADERKIT</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G20" s="1" t="n">
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G21" s="1" t="n">
         <v>46147.66540509259</v>
-      </c>
-      <c r="I20" t="n">
-        <v>19</v>
-      </c>
-      <c r="J20" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>No calificado</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>omer120395@gmail.com</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
-        <v>0</v>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Omer Peñaloza</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>Oportunidad de Omer Peñaloza</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G21" s="1" t="n">
-        <v>46147.66090277778</v>
       </c>
       <c r="I21" t="n">
         <v>19</v>
@@ -1409,7 +1409,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>directora.it@supermercadobelalcazar.com.co</t>
+          <t>omer120395@gmail.com</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1418,11 +1418,16 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>6000000</v>
+        <v>0</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Omer Peñaloza</t>
+        </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Oportunidad de ABASTECEMOS DE OCCIDENTE</t>
+          <t>Oportunidad de Omer Peñaloza</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1431,10 +1436,7 @@
         </is>
       </c>
       <c r="G22" s="1" t="n">
-        <v>46147.64170138889</v>
-      </c>
-      <c r="H22" s="1" t="n">
-        <v>46157</v>
+        <v>46147.66090277778</v>
       </c>
       <c r="I22" t="n">
         <v>19</v>
@@ -1442,12 +1444,6 @@
       <c r="J22" t="n">
         <v>2026</v>
       </c>
-      <c r="K22" t="n">
-        <v>5</v>
-      </c>
-      <c r="L22" t="n">
-        <v>2026</v>
-      </c>
       <c r="M22" t="inlineStr">
         <is>
           <t>No calificado</t>
@@ -1457,20 +1453,20 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>oscar.molina@terrenoshouston.com</t>
+          <t>directora.it@supermercadobelalcazar.com.co</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Negociación</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>37623040</v>
+        <v>6000000</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Oportunidad de COLONY RIDGE</t>
+          <t>Oportunidad de ABASTECEMOS DE OCCIDENTE</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1479,10 +1475,10 @@
         </is>
       </c>
       <c r="G23" s="1" t="n">
-        <v>46147.60297453704</v>
+        <v>46147.64170138889</v>
       </c>
       <c r="H23" s="1" t="n">
-        <v>46150</v>
+        <v>46157</v>
       </c>
       <c r="I23" t="n">
         <v>19</v>
@@ -1498,27 +1494,27 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>jsantacr@ccc.org.co</t>
+          <t>oscar.molina@terrenoshouston.com</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Negociación</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>55000000</v>
+        <v>37623040</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Oportunidad de CAMARA DE COMERCIO CALI</t>
+          <t>Oportunidad de COLONY RIDGE</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1527,33 +1523,33 @@
         </is>
       </c>
       <c r="G24" s="1" t="n">
-        <v>46141.62370370371</v>
+        <v>46147.60297453704</v>
       </c>
       <c r="H24" s="1" t="n">
-        <v>46289</v>
+        <v>46150</v>
       </c>
       <c r="I24" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J24" t="n">
         <v>2026</v>
       </c>
       <c r="K24" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="L24" t="n">
         <v>2026</v>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>exportaciones@laprovincia.com</t>
+          <t>jsantacr@ccc.org.co</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1562,11 +1558,11 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>6000000</v>
+        <v>55000000</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Oportunidad de PRODUCTOS LA PROVINCIA SAS</t>
+          <t>Oportunidad de CAMARA DE COMERCIO CALI</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1575,7 +1571,10 @@
         </is>
       </c>
       <c r="G25" s="1" t="n">
-        <v>46141.62021990741</v>
+        <v>46141.62370370371</v>
+      </c>
+      <c r="H25" s="1" t="n">
+        <v>46289</v>
       </c>
       <c r="I25" t="n">
         <v>18</v>
@@ -1583,6 +1582,12 @@
       <c r="J25" t="n">
         <v>2026</v>
       </c>
+      <c r="K25" t="n">
+        <v>9</v>
+      </c>
+      <c r="L25" t="n">
+        <v>2026</v>
+      </c>
       <c r="M25" t="inlineStr">
         <is>
           <t>No calificado</t>
@@ -1592,7 +1597,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>coordinador.mercadeo@regency.com.co</t>
+          <t>exportaciones@laprovincia.com</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1601,11 +1606,11 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>0</v>
+        <v>6000000</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Oportunidad de REGENCY TECH SAS</t>
+          <t>Oportunidad de PRODUCTOS LA PROVINCIA SAS</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1614,7 +1619,7 @@
         </is>
       </c>
       <c r="G26" s="1" t="n">
-        <v>46141.59664351852</v>
+        <v>46141.62021990741</v>
       </c>
       <c r="I26" t="n">
         <v>18</v>
@@ -1629,17 +1634,22 @@
       </c>
     </row>
     <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>coordinador.mercadeo@regency.com.co</t>
+        </is>
+      </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1200000</v>
+        <v>0</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Oportunidad de EMCALI E.I.C.E ESP</t>
+          <t>Oportunidad de REGENCY TECH SAS</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1648,10 +1658,7 @@
         </is>
       </c>
       <c r="G27" s="1" t="n">
-        <v>46141.59045138889</v>
-      </c>
-      <c r="H27" s="1" t="n">
-        <v>46352</v>
+        <v>46141.59664351852</v>
       </c>
       <c r="I27" t="n">
         <v>18</v>
@@ -1659,88 +1666,72 @@
       <c r="J27" t="n">
         <v>2026</v>
       </c>
-      <c r="K27" t="n">
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>No calificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Contactado</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>1200000</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Oportunidad de EMCALI E.I.C.E ESP</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G28" s="1" t="n">
+        <v>46141.59045138889</v>
+      </c>
+      <c r="H28" s="1" t="n">
+        <v>46352</v>
+      </c>
+      <c r="I28" t="n">
+        <v>18</v>
+      </c>
+      <c r="J28" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K28" t="n">
         <v>11</v>
       </c>
-      <c r="L27" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M27" t="inlineStr">
-        <is>
-          <t>No calificado</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>angie_feligrana@eficacia.com.co</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Negociación</t>
-        </is>
-      </c>
-      <c r="C28" t="n">
-        <v>6000000</v>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>Oportunidad de Eficacia sas / Angie Feligrana</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G28" s="1" t="n">
-        <v>46126.63210648148</v>
-      </c>
-      <c r="H28" s="1" t="n">
-        <v>46150</v>
-      </c>
-      <c r="I28" t="n">
-        <v>16</v>
-      </c>
-      <c r="J28" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K28" t="n">
-        <v>5</v>
-      </c>
       <c r="L28" t="n">
         <v>2026</v>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Estrategiadigital@zuluagaysoto.com</t>
+          <t>angie_feligrana@eficacia.com.co</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Seguimiento</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>0</v>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Maryuri Arguello</t>
-        </is>
+        <v>6000000</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Oportunidad de Maryuri Arguello</t>
+          <t>Oportunidad de Eficacia sas / Angie Feligrana</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1749,7 +1740,10 @@
         </is>
       </c>
       <c r="G29" s="1" t="n">
-        <v>46125.71925925926</v>
+        <v>46126.63210648148</v>
+      </c>
+      <c r="H29" s="1" t="n">
+        <v>46150</v>
       </c>
       <c r="I29" t="n">
         <v>16</v>
@@ -1757,6 +1751,12 @@
       <c r="J29" t="n">
         <v>2026</v>
       </c>
+      <c r="K29" t="n">
+        <v>5</v>
+      </c>
+      <c r="L29" t="n">
+        <v>2026</v>
+      </c>
       <c r="M29" t="inlineStr">
         <is>
           <t>No calificado</t>
@@ -1766,82 +1766,81 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>gabrielrodriguez@arrozsupremo.com</t>
+          <t>Estrategiadigital@zuluagaysoto.com</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Ganado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>8000000</v>
+        <v>0</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>GABRIEL RODRIGUEZ</t>
+          <t>Maryuri Arguello</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Agente de Ventas</t>
+          <t>Oportunidad de Maryuri Arguello</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Richard Castaño</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G30" s="1" t="n">
-        <v>46119.62108796297</v>
-      </c>
-      <c r="H30" s="1" t="n">
-        <v>46141</v>
+        <v>46125.71925925926</v>
       </c>
       <c r="I30" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J30" t="n">
         <v>2026</v>
       </c>
-      <c r="K30" t="n">
-        <v>4</v>
-      </c>
-      <c r="L30" t="n">
-        <v>2026</v>
-      </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Belkis.jimenez@agrauto.com.co</t>
+          <t>gabrielrodriguez@arrozsupremo.com</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Ganado</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>0</v>
+        <v>8000000</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>GABRIEL RODRIGUEZ</t>
+        </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Oportunidad de AGRICOLA AUTOMOTRIZ SAS</t>
+          <t>Agente de Ventas</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Richard Castaño</t>
         </is>
       </c>
       <c r="G31" s="1" t="n">
-        <v>46119.38914351852</v>
+        <v>46119.62108796297</v>
+      </c>
+      <c r="H31" s="1" t="n">
+        <v>46141</v>
       </c>
       <c r="I31" t="n">
         <v>15</v>
@@ -1849,16 +1848,22 @@
       <c r="J31" t="n">
         <v>2026</v>
       </c>
+      <c r="K31" t="n">
+        <v>4</v>
+      </c>
+      <c r="L31" t="n">
+        <v>2026</v>
+      </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>anyela.aponza@cotel.com.co</t>
+          <t>Belkis.jimenez@agrauto.com.co</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1871,7 +1876,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Oportunidad de COTEL SAL</t>
+          <t>Oportunidad de AGRICOLA AUTOMOTRIZ SAS</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1880,10 +1885,10 @@
         </is>
       </c>
       <c r="G32" s="1" t="n">
-        <v>46112.61271990741</v>
+        <v>46119.38914351852</v>
       </c>
       <c r="I32" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="J32" t="n">
         <v>2026</v>
@@ -1897,7 +1902,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>liliana.patino@quironsalud.com</t>
+          <t>anyela.aponza@cotel.com.co</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1908,14 +1913,9 @@
       <c r="C33" t="n">
         <v>0</v>
       </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>CLINICA IMBANACO</t>
-        </is>
-      </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Oportunidad de Liliana Patiño Flórez</t>
+          <t>Oportunidad de COTEL SAL</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1924,7 +1924,7 @@
         </is>
       </c>
       <c r="G33" s="1" t="n">
-        <v>46112.60853009259</v>
+        <v>46112.61271990741</v>
       </c>
       <c r="I33" t="n">
         <v>14</v>
@@ -1941,7 +1941,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>casanchez@jgb.com.co</t>
+          <t>liliana.patino@quironsalud.com</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1952,9 +1952,14 @@
       <c r="C34" t="n">
         <v>0</v>
       </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>CLINICA IMBANACO</t>
+        </is>
+      </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Oportunidad de JGB S.A.</t>
+          <t>Oportunidad de Liliana Patiño Flórez</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1963,7 +1968,7 @@
         </is>
       </c>
       <c r="G34" s="1" t="n">
-        <v>46112.6052662037</v>
+        <v>46112.60853009259</v>
       </c>
       <c r="I34" t="n">
         <v>14</v>
@@ -1980,12 +1985,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>damaris.gomez@disfarma.com.co</t>
+          <t>casanchez@jgb.com.co</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Seguimiento</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -1993,7 +1998,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Oportunidad de DISFARMA</t>
+          <t>Oportunidad de JGB S.A.</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -2002,7 +2007,7 @@
         </is>
       </c>
       <c r="G35" s="1" t="n">
-        <v>46112.60325231482</v>
+        <v>46112.6052662037</v>
       </c>
       <c r="I35" t="n">
         <v>14</v>
@@ -2019,25 +2024,20 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>alergologosdeoccidente@gmail.com</t>
+          <t>damaris.gomez@disfarma.com.co</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Seguimiento</t>
         </is>
       </c>
       <c r="C36" t="n">
         <v>0</v>
       </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>Johana Gonzalez</t>
-        </is>
-      </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Oportunidad de Johana Gonzalez</t>
+          <t>Oportunidad de DISFARMA</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -2046,10 +2046,10 @@
         </is>
       </c>
       <c r="G36" s="1" t="n">
-        <v>46107.51248842593</v>
+        <v>46112.60325231482</v>
       </c>
       <c r="I36" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J36" t="n">
         <v>2026</v>
@@ -2063,77 +2063,76 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>DavidEsteban.Porras@alfalaval.com</t>
+          <t>alergologosdeoccidente@gmail.com</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Ganado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>15000000</v>
+        <v>0</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Johana Gonzalez</t>
+        </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Oportunidad de OPORTUNIDAD ENCUESTAS ALFALAVAL</t>
+          <t>Oportunidad de Johana Gonzalez</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G37" s="1" t="n">
-        <v>46101.72893518519</v>
-      </c>
-      <c r="H37" s="1" t="n">
-        <v>46141</v>
+        <v>46107.51248842593</v>
       </c>
       <c r="I37" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J37" t="n">
         <v>2026</v>
       </c>
-      <c r="K37" t="n">
-        <v>4</v>
-      </c>
-      <c r="L37" t="n">
-        <v>2026</v>
-      </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Dr.arcarmona@gmail.com</t>
+          <t>DavidEsteban.Porras@alfalaval.com</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Ganado</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>0</v>
+        <v>15000000</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Oportunidad de GAMANUCLEAR LTDA - Dr Alberto Carmona</t>
+          <t>Oportunidad de OPORTUNIDAD ENCUESTAS ALFALAVAL</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G38" s="1" t="n">
-        <v>46098.65114583333</v>
+        <v>46101.72893518519</v>
+      </c>
+      <c r="H38" s="1" t="n">
+        <v>46141</v>
       </c>
       <c r="I38" t="n">
         <v>12</v>
@@ -2141,16 +2140,22 @@
       <c r="J38" t="n">
         <v>2026</v>
       </c>
+      <c r="K38" t="n">
+        <v>4</v>
+      </c>
+      <c r="L38" t="n">
+        <v>2026</v>
+      </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>cecilia.guevara@cosmitet.net / administracion.crd@cosmitet.net</t>
+          <t>Dr.arcarmona@gmail.com</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2161,14 +2166,9 @@
       <c r="C39" t="n">
         <v>0</v>
       </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>Cecilia Guevara</t>
-        </is>
-      </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Oportunidad de CLINICA REY DAVID Walter Charria</t>
+          <t>Oportunidad de GAMANUCLEAR LTDA - Dr Alberto Carmona</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2177,10 +2177,10 @@
         </is>
       </c>
       <c r="G39" s="1" t="n">
-        <v>46094.69002314815</v>
+        <v>46098.65114583333</v>
       </c>
       <c r="I39" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J39" t="n">
         <v>2026</v>
@@ -2194,7 +2194,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>vicerrectoriacademica@unicatolica.edu.co</t>
+          <t>cecilia.guevara@cosmitet.net / administracion.crd@cosmitet.net</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2207,12 +2207,12 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Jorge Silva</t>
+          <t>Cecilia Guevara</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Oportunidad de Jorge Silva</t>
+          <t>Oportunidad de CLINICA REY DAVID Walter Charria</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -2221,7 +2221,7 @@
         </is>
       </c>
       <c r="G40" s="1" t="n">
-        <v>46094.66880787037</v>
+        <v>46094.69002314815</v>
       </c>
       <c r="I40" t="n">
         <v>11</v>
@@ -2238,37 +2238,34 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>pedroperea02@gmail.com</t>
+          <t>vicerrectoriacademica@unicatolica.edu.co</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Ganado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>2160000</v>
+        <v>0</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Pedro Pablo Perea Mafla</t>
+          <t>Jorge Silva</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Oportunidad de Encuestas</t>
+          <t>Oportunidad de Jorge Silva</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G41" s="1" t="n">
-        <v>46094.65905092593</v>
-      </c>
-      <c r="H41" s="1" t="n">
-        <v>46141</v>
+        <v>46094.66880787037</v>
       </c>
       <c r="I41" t="n">
         <v>11</v>
@@ -2276,35 +2273,34 @@
       <c r="J41" t="n">
         <v>2026</v>
       </c>
-      <c r="K41" t="n">
-        <v>4</v>
-      </c>
-      <c r="L41" t="n">
-        <v>2026</v>
-      </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>cristina.papamija@bmm.com.co</t>
+          <t>pedroperea02@gmail.com</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Ganado</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>8071000</v>
+        <v>2160000</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Pedro Pablo Perea Mafla</t>
+        </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Oportunidad de BANCO MUNDO MUJER</t>
+          <t>Oportunidad de Encuestas</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -2313,7 +2309,10 @@
         </is>
       </c>
       <c r="G42" s="1" t="n">
-        <v>46094.65019675926</v>
+        <v>46094.65905092593</v>
+      </c>
+      <c r="H42" s="1" t="n">
+        <v>46141</v>
       </c>
       <c r="I42" t="n">
         <v>11</v>
@@ -2321,16 +2320,22 @@
       <c r="J42" t="n">
         <v>2026</v>
       </c>
+      <c r="K42" t="n">
+        <v>4</v>
+      </c>
+      <c r="L42" t="n">
+        <v>2026</v>
+      </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>capacitacionvirtual@fundacionwwbcol.org</t>
+          <t>cristina.papamija@bmm.com.co</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2339,11 +2344,11 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>1600000</v>
+        <v>8071000</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Licenciamiento y ajuste WhatsApp FUNDACIÓN WWB</t>
+          <t>Oportunidad de BANCO MUNDO MUJER</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2352,7 +2357,7 @@
         </is>
       </c>
       <c r="G43" s="1" t="n">
-        <v>46094.64826388889</v>
+        <v>46094.65019675926</v>
       </c>
       <c r="I43" t="n">
         <v>11</v>
@@ -2369,25 +2374,20 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>carol.cuesta@cbolivar.com</t>
+          <t>capacitacionvirtual@fundacionwwbcol.org</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Ganado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>2900000</v>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>CAROL CUESTA</t>
-        </is>
+        <v>1600000</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Gestión de Subsidios CB Bogotá</t>
+          <t>Licenciamiento y ajuste WhatsApp FUNDACIÓN WWB</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -2396,10 +2396,7 @@
         </is>
       </c>
       <c r="G44" s="1" t="n">
-        <v>46094.64454861111</v>
-      </c>
-      <c r="H44" s="1" t="n">
-        <v>46135</v>
+        <v>46094.64826388889</v>
       </c>
       <c r="I44" t="n">
         <v>11</v>
@@ -2407,44 +2404,46 @@
       <c r="J44" t="n">
         <v>2026</v>
       </c>
-      <c r="K44" t="n">
-        <v>4</v>
-      </c>
-      <c r="L44" t="n">
-        <v>2026</v>
-      </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>edwin.munoz.v@uniminuto.edu</t>
+          <t>carol.cuesta@cbolivar.com</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Ganado</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>0</v>
+        <v>2900000</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>CAROL CUESTA</t>
+        </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Oportunidad de UNIMINUTO</t>
+          <t>Gestión de Subsidios CB Bogotá</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G45" s="1" t="n">
-        <v>46092.63626157407</v>
+        <v>46094.64454861111</v>
+      </c>
+      <c r="H45" s="1" t="n">
+        <v>46135</v>
       </c>
       <c r="I45" t="n">
         <v>11</v>
@@ -2452,16 +2451,22 @@
       <c r="J45" t="n">
         <v>2026</v>
       </c>
+      <c r="K45" t="n">
+        <v>4</v>
+      </c>
+      <c r="L45" t="n">
+        <v>2026</v>
+      </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>jaime_zuluaga@eficacia.com.co</t>
+          <t>edwin.munoz.v@uniminuto.edu</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2472,14 +2477,9 @@
       <c r="C46" t="n">
         <v>0</v>
       </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>Jaime Alberto</t>
-        </is>
-      </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Oportunidad de Jaime Alberto Zuluaga</t>
+          <t>Oportunidad de UNIMINUTO</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2488,7 +2488,7 @@
         </is>
       </c>
       <c r="G46" s="1" t="n">
-        <v>46092.63153935185</v>
+        <v>46092.63626157407</v>
       </c>
       <c r="I46" t="n">
         <v>11</v>
@@ -2505,7 +2505,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>comercial@isyscol.com</t>
+          <t>jaime_zuluaga@eficacia.com.co</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2518,12 +2518,12 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Andres Nader</t>
+          <t>Jaime Alberto</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Oportunidad de Andres Nader</t>
+          <t>Oportunidad de Jaime Alberto Zuluaga</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -2532,7 +2532,7 @@
         </is>
       </c>
       <c r="G47" s="1" t="n">
-        <v>46091.59211805555</v>
+        <v>46092.63153935185</v>
       </c>
       <c r="I47" t="n">
         <v>11</v>
@@ -2549,7 +2549,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>mercadeo@norteysur.co</t>
+          <t>comercial@isyscol.com</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2562,12 +2562,12 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Isabella Mesa</t>
+          <t>Andres Nader</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Oportunidad de Isabella Mesa</t>
+          <t>Oportunidad de Andres Nader</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2576,7 +2576,7 @@
         </is>
       </c>
       <c r="G48" s="1" t="n">
-        <v>46091.40078703704</v>
+        <v>46091.59211805555</v>
       </c>
       <c r="I48" t="n">
         <v>11</v>
@@ -2591,26 +2591,36 @@
       </c>
     </row>
     <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>mercadeo@norteysur.co</t>
+        </is>
+      </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Seguimiento</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C49" t="n">
         <v>0</v>
       </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Isabella Mesa</t>
+        </is>
+      </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Clasificación EMAIL Comfenalco Cartagena</t>
+          <t>Oportunidad de Isabella Mesa</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Maria Fernanda Gaviria</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G49" s="1" t="n">
-        <v>46091.3665625</v>
+        <v>46091.40078703704</v>
       </c>
       <c r="I49" t="n">
         <v>11</v>
@@ -2627,7 +2637,7 @@
     <row r="50">
       <c r="B50" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Seguimiento</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -2635,19 +2645,19 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Oportunidad de ESE HOSPITAL LA MARIA</t>
+          <t>Clasificación EMAIL Comfenalco Cartagena</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Laura Alejandra Castañeda</t>
+          <t>Maria Fernanda Gaviria</t>
         </is>
       </c>
       <c r="G50" s="1" t="n">
-        <v>46083.67605324074</v>
+        <v>46091.3665625</v>
       </c>
       <c r="I50" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J50" t="n">
         <v>2026</v>
@@ -2669,7 +2679,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Oportunidad de SUPER TRANSPORTE</t>
+          <t>Oportunidad de ESE HOSPITAL LA MARIA</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -2678,7 +2688,7 @@
         </is>
       </c>
       <c r="G51" s="1" t="n">
-        <v>46083.6706712963</v>
+        <v>46083.67605324074</v>
       </c>
       <c r="I51" t="n">
         <v>10</v>
@@ -2703,7 +2713,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Oportunidad de ENLACES IP S.A.S</t>
+          <t>Oportunidad de SUPER TRANSPORTE</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -2712,7 +2722,7 @@
         </is>
       </c>
       <c r="G52" s="1" t="n">
-        <v>46083.50145833333</v>
+        <v>46083.6706712963</v>
       </c>
       <c r="I52" t="n">
         <v>10</v>
@@ -2727,11 +2737,6 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>accounting@diaza.com</t>
-        </is>
-      </c>
       <c r="B53" t="inlineStr">
         <is>
           <t>Perdido</t>
@@ -2740,26 +2745,21 @@
       <c r="C53" t="n">
         <v>0</v>
       </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>JOHANA RODRIGUEZ</t>
-        </is>
-      </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Oportunidad de JOHANA RODRIGUEZ</t>
+          <t>Oportunidad de ENLACES IP S.A.S</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Laura Alejandra Castañeda</t>
         </is>
       </c>
       <c r="G53" s="1" t="n">
-        <v>46079.73486111111</v>
+        <v>46083.50145833333</v>
       </c>
       <c r="I53" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J53" t="n">
         <v>2026</v>
@@ -2773,7 +2773,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>mensajeriamyr@gmail.com</t>
+          <t>accounting@diaza.com</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2784,9 +2784,14 @@
       <c r="C54" t="n">
         <v>0</v>
       </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>JOHANA RODRIGUEZ</t>
+        </is>
+      </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Oportunidad de MENSAJERIA M&amp;R SAS</t>
+          <t>Oportunidad de JOHANA RODRIGUEZ</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -2795,7 +2800,7 @@
         </is>
       </c>
       <c r="G54" s="1" t="n">
-        <v>46079.72262731481</v>
+        <v>46079.73486111111</v>
       </c>
       <c r="I54" t="n">
         <v>9</v>
@@ -2812,7 +2817,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>sistemaspanaderialeal@gmail.com</t>
+          <t>mensajeriamyr@gmail.com</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2823,14 +2828,9 @@
       <c r="C55" t="n">
         <v>0</v>
       </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>Diego Rios</t>
-        </is>
-      </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>JAMDAC SAS, Diego Rios</t>
+          <t>Oportunidad de MENSAJERIA M&amp;R SAS</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -2839,10 +2839,10 @@
         </is>
       </c>
       <c r="G55" s="1" t="n">
-        <v>46071.63706018519</v>
+        <v>46079.72262731481</v>
       </c>
       <c r="I55" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J55" t="n">
         <v>2026</v>
@@ -2856,7 +2856,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>efernandez@unico.com.co</t>
+          <t>sistemaspanaderialeal@gmail.com</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2869,12 +2869,12 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Erick Fernandez</t>
+          <t>Diego Rios</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Oportunidad de Erick Fernandez</t>
+          <t>JAMDAC SAS, Diego Rios</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -2883,10 +2883,10 @@
         </is>
       </c>
       <c r="G56" s="1" t="n">
-        <v>46064.3750462963</v>
+        <v>46071.63706018519</v>
       </c>
       <c r="I56" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J56" t="n">
         <v>2026</v>
@@ -2900,7 +2900,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>kabenitez@icesi.edu.co</t>
+          <t>efernandez@unico.com.co</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2909,28 +2909,28 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>10000000</v>
+        <v>0</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>KENI BENITEZ</t>
+          <t>Erick Fernandez</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Oportunidad de KENI BENITEZ</t>
+          <t>Oportunidad de Erick Fernandez</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G57" s="1" t="n">
-        <v>46059.34918981481</v>
+        <v>46064.3750462963</v>
       </c>
       <c r="I57" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J57" t="n">
         <v>2026</v>
@@ -2944,7 +2944,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>patovar@uao.edu.co</t>
+          <t>kabenitez@icesi.edu.co</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2953,25 +2953,25 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>0</v>
+        <v>10000000</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Paula Tovar</t>
+          <t>KENI BENITEZ</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Oportunidad de UNIVERSIDAD AUTONOMA DE OCCIDENTE</t>
+          <t>Oportunidad de KENI BENITEZ</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G58" s="1" t="n">
-        <v>46058.72516203704</v>
+        <v>46059.34918981481</v>
       </c>
       <c r="I58" t="n">
         <v>6</v>
@@ -2988,7 +2988,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>comercial@isyscol.com</t>
+          <t>patovar@uao.edu.co</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2999,9 +2999,14 @@
       <c r="C59" t="n">
         <v>0</v>
       </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Paula Tovar</t>
+        </is>
+      </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Oportunidad de TECNOLOGIAS ISYSCOL SAS</t>
+          <t>Oportunidad de UNIVERSIDAD AUTONOMA DE OCCIDENTE</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -3010,7 +3015,7 @@
         </is>
       </c>
       <c r="G59" s="1" t="n">
-        <v>46057.58993055556</v>
+        <v>46058.72516203704</v>
       </c>
       <c r="I59" t="n">
         <v>6</v>
@@ -3025,17 +3030,22 @@
       </c>
     </row>
     <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>comercial@isyscol.com</t>
+        </is>
+      </c>
       <c r="B60" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>15000000</v>
+        <v>0</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Oportunidad de VOICE IA EFICACIA</t>
+          <t>Oportunidad de TECNOLOGIAS ISYSCOL SAS</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -3044,7 +3054,7 @@
         </is>
       </c>
       <c r="G60" s="1" t="n">
-        <v>46057.3409837963</v>
+        <v>46057.58993055556</v>
       </c>
       <c r="I60" t="n">
         <v>6</v>
@@ -3065,23 +3075,23 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>4000000</v>
+        <v>15000000</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Oportunidad de Eficacia WhatsApp</t>
+          <t>Oportunidad de VOICE IA EFICACIA</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G61" s="1" t="n">
-        <v>46049.67292824074</v>
+        <v>46057.3409837963</v>
       </c>
       <c r="I61" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J61" t="n">
         <v>2026</v>
@@ -3099,62 +3109,57 @@
         </is>
       </c>
       <c r="C62" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Oportunidad de Eficacia WhatsApp</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Jennifer Hoyos Gallego</t>
+        </is>
+      </c>
+      <c r="G62" s="1" t="n">
+        <v>46049.67292824074</v>
+      </c>
+      <c r="I62" t="n">
+        <v>5</v>
+      </c>
+      <c r="J62" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>No calificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
         <v>20000000</v>
       </c>
-      <c r="E62" t="inlineStr">
+      <c r="E63" t="inlineStr">
         <is>
           <t>Oportunidad de CRUZ ROJA COLOMBIANA SECCIONAL VALLE DEL CAUCA</t>
         </is>
       </c>
-      <c r="F62" t="inlineStr">
+      <c r="F63" t="inlineStr">
         <is>
           <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
-      <c r="G62" s="1" t="n">
+      <c r="G63" s="1" t="n">
         <v>46006.49650462963</v>
       </c>
-      <c r="I62" t="n">
+      <c r="I63" t="n">
         <v>51</v>
-      </c>
-      <c r="J62" t="n">
-        <v>2025</v>
-      </c>
-      <c r="M62" t="inlineStr">
-        <is>
-          <t>No calificado</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>silvia.figueroa@neurithmedia.com</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C63" t="n">
-        <v>25000000</v>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>Contact center ventas España</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>Richard Castaño</t>
-        </is>
-      </c>
-      <c r="G63" s="1" t="n">
-        <v>45960.61145833333</v>
-      </c>
-      <c r="I63" t="n">
-        <v>44</v>
       </c>
       <c r="J63" t="n">
         <v>2025</v>
@@ -3166,22 +3171,22 @@
       </c>
     </row>
     <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>silvia.figueroa@neurithmedia.com</t>
+        </is>
+      </c>
       <c r="B64" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>37000000</v>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>Mabel</t>
-        </is>
+        <v>25000000</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Masivos Licitacion</t>
+          <t>Contact center ventas España</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -3190,10 +3195,10 @@
         </is>
       </c>
       <c r="G64" s="1" t="n">
-        <v>45940.49372685186</v>
+        <v>45960.61145833333</v>
       </c>
       <c r="I64" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="J64" t="n">
         <v>2025</v>
@@ -3205,36 +3210,31 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>ana.zuniga@cbolivar.com</t>
-        </is>
-      </c>
       <c r="B65" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>4997000</v>
+        <v>37000000</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Ana Lucia Zuñiga</t>
+          <t>Mabel</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Constructora Bolivar Agente Redes</t>
+          <t>Masivos Licitacion</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Richard Castaño</t>
         </is>
       </c>
       <c r="G65" s="1" t="n">
-        <v>45940.49215277778</v>
+        <v>45940.49372685186</v>
       </c>
       <c r="I65" t="n">
         <v>41</v>
@@ -3251,7 +3251,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>julian_mendez@extras.com.co</t>
+          <t>ana.zuniga@cbolivar.com</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -3260,28 +3260,28 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>15000000</v>
+        <v>4997000</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Julian Mendez.</t>
+          <t>Ana Lucia Zuñiga</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Oportunidad de EFICACIA S A S</t>
+          <t>Constructora Bolivar Agente Redes</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G66" s="1" t="n">
-        <v>45922.66201388889</v>
+        <v>45940.49215277778</v>
       </c>
       <c r="I66" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="J66" t="n">
         <v>2025</v>
@@ -3295,7 +3295,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>info@eficacia.com.co</t>
+          <t>julian_mendez@extras.com.co</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3304,11 +3304,16 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>0</v>
+        <v>15000000</v>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Julian Mendez.</t>
+        </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Nutresa</t>
+          <t>Oportunidad de EFICACIA S A S</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -3317,7 +3322,7 @@
         </is>
       </c>
       <c r="G67" s="1" t="n">
-        <v>45922.66199074074</v>
+        <v>45922.66201388889</v>
       </c>
       <c r="I67" t="n">
         <v>39</v>
@@ -3334,37 +3339,32 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>hrodriguez@jaramillomora.com</t>
+          <t>info@eficacia.com.co</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Seguimiento</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>30000000</v>
-      </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>HANNA</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Oportunidad de JARAMILLO MORA CONSTRUCTORA S A</t>
+          <t>Nutresa</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Richard Castaño</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G68" s="1" t="n">
-        <v>45916.71618055556</v>
+        <v>45922.66199074074</v>
       </c>
       <c r="I68" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="J68" t="n">
         <v>2025</v>
@@ -3376,17 +3376,27 @@
       </c>
     </row>
     <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>hrodriguez@jaramillomora.com</t>
+        </is>
+      </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Seguimiento</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>147000000</v>
+        <v>30000000</v>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>HANNA</t>
+        </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Contact Center Agendamiento citas</t>
+          <t>Oportunidad de JARAMILLO MORA CONSTRUCTORA S A</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -3395,7 +3405,7 @@
         </is>
       </c>
       <c r="G69" s="1" t="n">
-        <v>45916.67502314815</v>
+        <v>45916.71618055556</v>
       </c>
       <c r="I69" t="n">
         <v>38</v>
@@ -3410,34 +3420,26 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>jaime_zuluaga@eficacia.com.co</t>
-        </is>
-      </c>
       <c r="B70" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>14700000</v>
+        <v>147000000</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Agentes contact center encuestas</t>
+          <t>Contact Center Agendamiento citas</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Richard Castaño</t>
         </is>
       </c>
       <c r="G70" s="1" t="n">
-        <v>45916.65275462963</v>
-      </c>
-      <c r="H70" s="1" t="n">
-        <v>45930</v>
+        <v>45916.67502314815</v>
       </c>
       <c r="I70" t="n">
         <v>38</v>
@@ -3445,12 +3447,6 @@
       <c r="J70" t="n">
         <v>2025</v>
       </c>
-      <c r="K70" t="n">
-        <v>9</v>
-      </c>
-      <c r="L70" t="n">
-        <v>2025</v>
-      </c>
       <c r="M70" t="inlineStr">
         <is>
           <t>No calificado</t>
@@ -3458,22 +3454,22 @@
       </c>
     </row>
     <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>jaime_zuluaga@eficacia.com.co</t>
+        </is>
+      </c>
       <c r="B71" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>4796000</v>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>Juan Grisales</t>
-        </is>
+        <v>14700000</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Agente Call Center Outbound</t>
+          <t>Agentes contact center encuestas</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -3482,7 +3478,10 @@
         </is>
       </c>
       <c r="G71" s="1" t="n">
-        <v>45915.4809375</v>
+        <v>45916.65275462963</v>
+      </c>
+      <c r="H71" s="1" t="n">
+        <v>45930</v>
       </c>
       <c r="I71" t="n">
         <v>38</v>
@@ -3490,6 +3489,12 @@
       <c r="J71" t="n">
         <v>2025</v>
       </c>
+      <c r="K71" t="n">
+        <v>9</v>
+      </c>
+      <c r="L71" t="n">
+        <v>2025</v>
+      </c>
       <c r="M71" t="inlineStr">
         <is>
           <t>No calificado</t>
@@ -3497,27 +3502,22 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>gestormercadeo@lamontana.co</t>
-        </is>
-      </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Seguimiento</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>25000000</v>
+        <v>4796000</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Alejandra Ossa</t>
+          <t>Juan Grisales</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Voice BOT</t>
+          <t>Agente Call Center Outbound</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -3526,10 +3526,7 @@
         </is>
       </c>
       <c r="G72" s="1" t="n">
-        <v>45915.48023148148</v>
-      </c>
-      <c r="H72" s="1" t="n">
-        <v>46150</v>
+        <v>45915.4809375</v>
       </c>
       <c r="I72" t="n">
         <v>38</v>
@@ -3537,12 +3534,6 @@
       <c r="J72" t="n">
         <v>2025</v>
       </c>
-      <c r="K72" t="n">
-        <v>5</v>
-      </c>
-      <c r="L72" t="n">
-        <v>2026</v>
-      </c>
       <c r="M72" t="inlineStr">
         <is>
           <t>No calificado</t>
@@ -3552,20 +3543,25 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>elkinmarquezconsuegra@gmail.com</t>
+          <t>gestormercadeo@lamontana.co</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Seguimiento</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>2500000</v>
+        <v>25000000</v>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Alejandra Ossa</t>
+        </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Venta Masivos</t>
+          <t>Voice BOT</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -3574,7 +3570,10 @@
         </is>
       </c>
       <c r="G73" s="1" t="n">
-        <v>45915.47924768519</v>
+        <v>45915.48023148148</v>
+      </c>
+      <c r="H73" s="1" t="n">
+        <v>46150</v>
       </c>
       <c r="I73" t="n">
         <v>38</v>
@@ -3582,6 +3581,12 @@
       <c r="J73" t="n">
         <v>2025</v>
       </c>
+      <c r="K73" t="n">
+        <v>5</v>
+      </c>
+      <c r="L73" t="n">
+        <v>2026</v>
+      </c>
       <c r="M73" t="inlineStr">
         <is>
           <t>No calificado</t>
@@ -3591,7 +3596,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>bladimir.munoz@uptc.edu.co</t>
+          <t>elkinmarquezconsuegra@gmail.com</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -3600,16 +3605,11 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>22000000</v>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>Bladimir Muñoz Forero</t>
-        </is>
+        <v>2500000</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Oportunidad Venta BPO</t>
+          <t>Venta Masivos</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -3618,7 +3618,7 @@
         </is>
       </c>
       <c r="G74" s="1" t="n">
-        <v>45915.47494212963</v>
+        <v>45915.47924768519</v>
       </c>
       <c r="I74" t="n">
         <v>38</v>
@@ -3635,7 +3635,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>gerencia@alitasfactory.com</t>
+          <t>bladimir.munoz@uptc.edu.co</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -3644,20 +3644,25 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>40000000</v>
+        <v>22000000</v>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Bladimir Muñoz Forero</t>
+        </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>1 agente IA para ventas y asesoramiento</t>
+          <t>Oportunidad Venta BPO</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Richard Castaño</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G75" s="1" t="n">
-        <v>45915.47300925926</v>
+        <v>45915.47494212963</v>
       </c>
       <c r="I75" t="n">
         <v>38</v>
@@ -3674,7 +3679,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>mmonroy@falabella.com.co</t>
+          <t>gerencia@alitasfactory.com</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -3683,11 +3688,11 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>60000000</v>
+        <v>40000000</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Agente IA Try and Buy Inbound y Outbound</t>
+          <t>1 agente IA para ventas y asesoramiento</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -3696,7 +3701,7 @@
         </is>
       </c>
       <c r="G76" s="1" t="n">
-        <v>45915.46633101852</v>
+        <v>45915.47300925926</v>
       </c>
       <c r="I76" t="n">
         <v>38</v>
@@ -3713,7 +3718,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>gerencia@motosymotoselpaisa.com</t>
+          <t>mmonroy@falabella.com.co</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -3722,20 +3727,20 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>40000000</v>
+        <v>60000000</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Oportunidad de MOTOS Y MOTOS EL PAISA S A S</t>
+          <t>Agente IA Try and Buy Inbound y Outbound</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Richard Castaño</t>
         </is>
       </c>
       <c r="G77" s="1" t="n">
-        <v>45915.46252314815</v>
+        <v>45915.46633101852</v>
       </c>
       <c r="I77" t="n">
         <v>38</v>
@@ -3752,7 +3757,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>isanchez@unico.com.co</t>
+          <t>gerencia@motosymotoselpaisa.com</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -3761,11 +3766,11 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>0</v>
+        <v>40000000</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>1 agente IA para relacionamiento con locatarios</t>
+          <t>Oportunidad de MOTOS Y MOTOS EL PAISA S A S</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -3774,7 +3779,7 @@
         </is>
       </c>
       <c r="G78" s="1" t="n">
-        <v>45915.46157407408</v>
+        <v>45915.46252314815</v>
       </c>
       <c r="I78" t="n">
         <v>38</v>
@@ -3791,7 +3796,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>asantiago@stop.com.co</t>
+          <t>isanchez@unico.com.co</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -3800,11 +3805,11 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>30000000</v>
+        <v>0</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>1 Agente IA en cobranzas</t>
+          <t>1 agente IA para relacionamiento con locatarios</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -3813,7 +3818,7 @@
         </is>
       </c>
       <c r="G79" s="1" t="n">
-        <v>45915.46052083333</v>
+        <v>45915.46157407408</v>
       </c>
       <c r="I79" t="n">
         <v>38</v>
@@ -3830,7 +3835,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>jcastano@mercaldas.com.co</t>
+          <t>asantiago@stop.com.co</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -3843,7 +3848,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>1 agente IA para ventas y asesoramiento</t>
+          <t>1 Agente IA en cobranzas</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -3852,7 +3857,7 @@
         </is>
       </c>
       <c r="G80" s="1" t="n">
-        <v>45915.35666666667</v>
+        <v>45915.46052083333</v>
       </c>
       <c r="I80" t="n">
         <v>38</v>
@@ -3869,7 +3874,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>calidad@cempac.com.co</t>
+          <t>jcastano@mercaldas.com.co</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -3878,7 +3883,7 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>42000000</v>
+        <v>30000000</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -3891,7 +3896,7 @@
         </is>
       </c>
       <c r="G81" s="1" t="n">
-        <v>45915.35537037037</v>
+        <v>45915.35666666667</v>
       </c>
       <c r="I81" t="n">
         <v>38</v>

</xml_diff>

<commit_message>
CRM actualizado — 22/05/2026 09:06
</commit_message>
<xml_diff>
--- a/CRM_PowerBI_BrendaLuna_actualizado.xlsx
+++ b/CRM_PowerBI_BrendaLuna_actualizado.xlsx
@@ -946,25 +946,20 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>mercadeo@lasevillana.com.co</t>
+          <t>comercial2@felsyn.com</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fabio AlbertoGallego García </t>
-        </is>
+        <v>713400</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Oportunidad de Fabio AlbertoGallego García </t>
+          <t>Oportunidad de FONDO DE EMPLEADOS FELSYN</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -973,7 +968,7 @@
         </is>
       </c>
       <c r="G11" s="1" t="n">
-        <v>46162.64569444444</v>
+        <v>46163.49130787037</v>
       </c>
       <c r="I11" t="n">
         <v>21</v>
@@ -983,27 +978,32 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>asantiago@stop.com.co</t>
+          <t>mercadeo@lasevillana.com.co</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C12" t="n">
         <v>0</v>
       </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fabio AlbertoGallego García </t>
+        </is>
+      </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Oportunidad de STOP SAS</t>
+          <t xml:space="preserve">Oportunidad de Fabio AlbertoGallego García </t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1012,7 +1012,7 @@
         </is>
       </c>
       <c r="G12" s="1" t="n">
-        <v>46161.63508101852</v>
+        <v>46162.64569444444</v>
       </c>
       <c r="I12" t="n">
         <v>21</v>
@@ -1029,7 +1029,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>aestrada@teker.co</t>
+          <t>asantiago@stop.com.co</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1040,14 +1040,9 @@
       <c r="C13" t="n">
         <v>0</v>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>TEKER SALUD SAS</t>
-        </is>
-      </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Oportunidad de TEKER SALUD SAS</t>
+          <t>Oportunidad de STOP SAS</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1056,7 +1051,7 @@
         </is>
       </c>
       <c r="G13" s="1" t="n">
-        <v>46161.62922453704</v>
+        <v>46161.63508101852</v>
       </c>
       <c r="I13" t="n">
         <v>21</v>
@@ -1071,17 +1066,27 @@
       </c>
     </row>
     <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>aestrada@teker.co</t>
+        </is>
+      </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0</v>
+        <v>16914000</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>TEKER SALUD SAS</t>
+        </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Oportunidad de TIAN IPS SAS</t>
+          <t>Oportunidad de TEKER SALUD SAS</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1090,7 +1095,7 @@
         </is>
       </c>
       <c r="G14" s="1" t="n">
-        <v>46161.61643518518</v>
+        <v>46161.62922453704</v>
       </c>
       <c r="I14" t="n">
         <v>21</v>
@@ -1100,16 +1105,11 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>administración@fullredtotal.com</t>
-        </is>
-      </c>
       <c r="B15" t="inlineStr">
         <is>
           <t>Nuevo</t>
@@ -1118,14 +1118,9 @@
       <c r="C15" t="n">
         <v>0</v>
       </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Eivar Eñasco</t>
-        </is>
-      </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Oportunidad de Eivar Eñasco</t>
+          <t>Oportunidad de TIAN IPS SAS</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1134,10 +1129,10 @@
         </is>
       </c>
       <c r="G15" s="1" t="n">
-        <v>46154.67546296296</v>
+        <v>46161.61643518518</v>
       </c>
       <c r="I15" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J15" t="n">
         <v>2026</v>
@@ -1151,25 +1146,25 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>cserna@surtifamiliar.com.co</t>
+          <t>administración@fullredtotal.com</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Negociación</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>1950000</v>
+        <v>14000000</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Claudia Patricia Serna</t>
+          <t>Eivar Eñasco</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Oportunidad de Claudia Patricia Serna</t>
+          <t>Oportunidad de Eivar Eñasco</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1178,7 +1173,7 @@
         </is>
       </c>
       <c r="G16" s="1" t="n">
-        <v>46154.66616898148</v>
+        <v>46154.67546296296</v>
       </c>
       <c r="I16" t="n">
         <v>20</v>
@@ -1195,25 +1190,25 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>coordmercadeo@pacificcenter.co</t>
+          <t>cserna@surtifamiliar.com.co</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Negociación</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0</v>
+        <v>1950000</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Claudia Castro</t>
+          <t>Claudia Patricia Serna</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Oportunidad de Claudia Castro</t>
+          <t>Oportunidad de Claudia Patricia Serna</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1222,7 +1217,7 @@
         </is>
       </c>
       <c r="G17" s="1" t="n">
-        <v>46154.66341435185</v>
+        <v>46154.66616898148</v>
       </c>
       <c r="I17" t="n">
         <v>20</v>
@@ -1232,14 +1227,14 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>isabellarengifo27@gmail.com</t>
+          <t>coordmercadeo@pacificcenter.co</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1248,16 +1243,16 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>28190000</v>
+        <v>5600000</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Isabella Rengifo</t>
+          <t>Claudia Castro</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Oportunidad de Isabella Rengifo</t>
+          <t>Oportunidad de Claudia Castro</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1266,7 +1261,7 @@
         </is>
       </c>
       <c r="G18" s="1" t="n">
-        <v>46154.65981481481</v>
+        <v>46154.66341435185</v>
       </c>
       <c r="I18" t="n">
         <v>20</v>
@@ -1281,34 +1276,36 @@
       </c>
     </row>
     <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>isabellarengifo27@gmail.com</t>
+        </is>
+      </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>50000000</v>
+        <v>28190000</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Paola Gómez - Agente Inmobiliaria Independiente</t>
+          <t>Isabella Rengifo</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Puesto de Trabajo CC Medellin</t>
+          <t>Oportunidad de Isabella Rengifo</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Richard Castaño</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G19" s="1" t="n">
-        <v>46154.49104166667</v>
-      </c>
-      <c r="H19" s="1" t="n">
-        <v>46170</v>
+        <v>46154.65981481481</v>
       </c>
       <c r="I19" t="n">
         <v>20</v>
@@ -1316,44 +1313,41 @@
       <c r="J19" t="n">
         <v>2026</v>
       </c>
-      <c r="K19" t="n">
-        <v>5</v>
-      </c>
-      <c r="L19" t="n">
-        <v>2026</v>
-      </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>alberto.ramirez@constructorabolivar.com</t>
-        </is>
-      </c>
       <c r="B20" t="inlineStr">
         <is>
           <t>Propuesta</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>3000000</v>
+        <v>50000000</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Paola Gómez - Agente Inmobiliaria Independiente</t>
+        </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Oportunidad de NPS Relacional</t>
+          <t>Puesto de Trabajo CC Medellin</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Richard Castaño</t>
         </is>
       </c>
       <c r="G20" s="1" t="n">
-        <v>46154.44511574074</v>
+        <v>46154.49104166667</v>
+      </c>
+      <c r="H20" s="1" t="n">
+        <v>46170</v>
       </c>
       <c r="I20" t="n">
         <v>20</v>
@@ -1361,6 +1355,12 @@
       <c r="J20" t="n">
         <v>2026</v>
       </c>
+      <c r="K20" t="n">
+        <v>5</v>
+      </c>
+      <c r="L20" t="n">
+        <v>2026</v>
+      </c>
       <c r="M20" t="inlineStr">
         <is>
           <t>Calificado</t>
@@ -1368,75 +1368,70 @@
       </c>
     </row>
     <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>alberto.ramirez@constructorabolivar.com</t>
+        </is>
+      </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C21" t="n">
         <v>3000000</v>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Oportunidad de NPS Relacional</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Jennifer Hoyos Gallego</t>
+        </is>
+      </c>
+      <c r="G21" s="1" t="n">
+        <v>46154.44511574074</v>
+      </c>
+      <c r="I21" t="n">
+        <v>20</v>
+      </c>
+      <c r="J21" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>Calificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="D22" t="inlineStr">
         <is>
           <t>MADERKIT</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>Oportunidad de MADERKIT</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G21" s="1" t="n">
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G22" s="1" t="n">
         <v>46147.66540509259</v>
-      </c>
-      <c r="I21" t="n">
-        <v>19</v>
-      </c>
-      <c r="J21" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>No calificado</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>omer120395@gmail.com</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C22" t="n">
-        <v>0</v>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Omer Peñaloza</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>Oportunidad de Omer Peñaloza</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G22" s="1" t="n">
-        <v>46147.66090277778</v>
       </c>
       <c r="I22" t="n">
         <v>19</v>
@@ -1453,7 +1448,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>directora.it@supermercadobelalcazar.com.co</t>
+          <t>omer120395@gmail.com</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1462,11 +1457,16 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>6000000</v>
+        <v>0</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Omer Peñaloza</t>
+        </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Oportunidad de ABASTECEMOS DE OCCIDENTE</t>
+          <t>Oportunidad de Omer Peñaloza</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1475,10 +1475,7 @@
         </is>
       </c>
       <c r="G23" s="1" t="n">
-        <v>46147.64170138889</v>
-      </c>
-      <c r="H23" s="1" t="n">
-        <v>46157</v>
+        <v>46147.66090277778</v>
       </c>
       <c r="I23" t="n">
         <v>19</v>
@@ -1486,12 +1483,6 @@
       <c r="J23" t="n">
         <v>2026</v>
       </c>
-      <c r="K23" t="n">
-        <v>5</v>
-      </c>
-      <c r="L23" t="n">
-        <v>2026</v>
-      </c>
       <c r="M23" t="inlineStr">
         <is>
           <t>No calificado</t>
@@ -1501,20 +1492,20 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>oscar.molina@terrenoshouston.com</t>
+          <t>directora.it@supermercadobelalcazar.com.co</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Negociación</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>37623040</v>
+        <v>6000000</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Oportunidad de COLONY RIDGE</t>
+          <t>Oportunidad de ABASTECEMOS DE OCCIDENTE</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1523,10 +1514,10 @@
         </is>
       </c>
       <c r="G24" s="1" t="n">
-        <v>46147.60297453704</v>
+        <v>46147.64170138889</v>
       </c>
       <c r="H24" s="1" t="n">
-        <v>46150</v>
+        <v>46157</v>
       </c>
       <c r="I24" t="n">
         <v>19</v>
@@ -1542,27 +1533,27 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>jsantacr@ccc.org.co</t>
+          <t>oscar.molina@terrenoshouston.com</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Negociación</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>55000000</v>
+        <v>37623040</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Oportunidad de CAMARA DE COMERCIO CALI</t>
+          <t>Oportunidad de COLONY RIDGE</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1571,46 +1562,46 @@
         </is>
       </c>
       <c r="G25" s="1" t="n">
-        <v>46141.62370370371</v>
+        <v>46147.60297453704</v>
       </c>
       <c r="H25" s="1" t="n">
-        <v>46289</v>
+        <v>46150</v>
       </c>
       <c r="I25" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J25" t="n">
         <v>2026</v>
       </c>
       <c r="K25" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="L25" t="n">
         <v>2026</v>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>exportaciones@laprovincia.com</t>
+          <t>jsantacr@ccc.org.co</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>6000000</v>
+        <v>55000000</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Oportunidad de PRODUCTOS LA PROVINCIA SAS</t>
+          <t>Oportunidad de CAMARA DE COMERCIO CALI</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1619,7 +1610,10 @@
         </is>
       </c>
       <c r="G26" s="1" t="n">
-        <v>46141.62021990741</v>
+        <v>46141.62370370371</v>
+      </c>
+      <c r="H26" s="1" t="n">
+        <v>46289</v>
       </c>
       <c r="I26" t="n">
         <v>18</v>
@@ -1627,6 +1621,12 @@
       <c r="J26" t="n">
         <v>2026</v>
       </c>
+      <c r="K26" t="n">
+        <v>9</v>
+      </c>
+      <c r="L26" t="n">
+        <v>2026</v>
+      </c>
       <c r="M26" t="inlineStr">
         <is>
           <t>No calificado</t>
@@ -1636,7 +1636,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>coordinador.mercadeo@regency.com.co</t>
+          <t>exportaciones@laprovincia.com</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1645,11 +1645,11 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>0</v>
+        <v>6000000</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Oportunidad de REGENCY TECH SAS</t>
+          <t>Oportunidad de PRODUCTOS LA PROVINCIA SAS</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1658,7 +1658,7 @@
         </is>
       </c>
       <c r="G27" s="1" t="n">
-        <v>46141.59664351852</v>
+        <v>46141.62021990741</v>
       </c>
       <c r="I27" t="n">
         <v>18</v>
@@ -1673,17 +1673,22 @@
       </c>
     </row>
     <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>coordinador.mercadeo@regency.com.co</t>
+        </is>
+      </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1200000</v>
+        <v>0</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Oportunidad de EMCALI E.I.C.E ESP</t>
+          <t>Oportunidad de REGENCY TECH SAS</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1692,10 +1697,7 @@
         </is>
       </c>
       <c r="G28" s="1" t="n">
-        <v>46141.59045138889</v>
-      </c>
-      <c r="H28" s="1" t="n">
-        <v>46352</v>
+        <v>46141.59664351852</v>
       </c>
       <c r="I28" t="n">
         <v>18</v>
@@ -1703,56 +1705,45 @@
       <c r="J28" t="n">
         <v>2026</v>
       </c>
-      <c r="K28" t="n">
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>No calificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Contactado</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>1200000</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Oportunidad de EMCALI E.I.C.E ESP</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G29" s="1" t="n">
+        <v>46141.59045138889</v>
+      </c>
+      <c r="H29" s="1" t="n">
+        <v>46352</v>
+      </c>
+      <c r="I29" t="n">
+        <v>18</v>
+      </c>
+      <c r="J29" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K29" t="n">
         <v>11</v>
-      </c>
-      <c r="L28" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M28" t="inlineStr">
-        <is>
-          <t>No calificado</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>angie_feligrana@eficacia.com.co</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Seguimiento</t>
-        </is>
-      </c>
-      <c r="C29" t="n">
-        <v>6000000</v>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>Oportunidad de Eficacia sas / Angie Feligrana</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G29" s="1" t="n">
-        <v>46126.63210648148</v>
-      </c>
-      <c r="H29" s="1" t="n">
-        <v>46150</v>
-      </c>
-      <c r="I29" t="n">
-        <v>16</v>
-      </c>
-      <c r="J29" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K29" t="n">
-        <v>5</v>
       </c>
       <c r="L29" t="n">
         <v>2026</v>
@@ -1766,25 +1757,20 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Estrategiadigital@zuluagaysoto.com</t>
+          <t>angie_feligrana@eficacia.com.co</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Seguimiento</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>0</v>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Maryuri Arguello</t>
-        </is>
+        <v>6000000</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Oportunidad de Maryuri Arguello</t>
+          <t>Oportunidad de Eficacia sas / Angie Feligrana</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1793,7 +1779,10 @@
         </is>
       </c>
       <c r="G30" s="1" t="n">
-        <v>46125.71925925926</v>
+        <v>46126.63210648148</v>
+      </c>
+      <c r="H30" s="1" t="n">
+        <v>46150</v>
       </c>
       <c r="I30" t="n">
         <v>16</v>
@@ -1801,6 +1790,12 @@
       <c r="J30" t="n">
         <v>2026</v>
       </c>
+      <c r="K30" t="n">
+        <v>5</v>
+      </c>
+      <c r="L30" t="n">
+        <v>2026</v>
+      </c>
       <c r="M30" t="inlineStr">
         <is>
           <t>No calificado</t>
@@ -1810,82 +1805,81 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>gabrielrodriguez@arrozsupremo.com</t>
+          <t>Estrategiadigital@zuluagaysoto.com</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Ganado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>8000000</v>
+        <v>0</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>GABRIEL RODRIGUEZ</t>
+          <t>Maryuri Arguello</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Agente de Ventas</t>
+          <t>Oportunidad de Maryuri Arguello</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Richard Castaño</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G31" s="1" t="n">
-        <v>46119.62108796297</v>
-      </c>
-      <c r="H31" s="1" t="n">
-        <v>46141</v>
+        <v>46125.71925925926</v>
       </c>
       <c r="I31" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J31" t="n">
         <v>2026</v>
       </c>
-      <c r="K31" t="n">
-        <v>4</v>
-      </c>
-      <c r="L31" t="n">
-        <v>2026</v>
-      </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Belkis.jimenez@agrauto.com.co</t>
+          <t>gabrielrodriguez@arrozsupremo.com</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Ganado</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>0</v>
+        <v>8000000</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>GABRIEL RODRIGUEZ</t>
+        </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Oportunidad de AGRICOLA AUTOMOTRIZ SAS</t>
+          <t>Agente de Ventas</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Richard Castaño</t>
         </is>
       </c>
       <c r="G32" s="1" t="n">
-        <v>46119.38914351852</v>
+        <v>46119.62108796297</v>
+      </c>
+      <c r="H32" s="1" t="n">
+        <v>46141</v>
       </c>
       <c r="I32" t="n">
         <v>15</v>
@@ -1893,16 +1887,22 @@
       <c r="J32" t="n">
         <v>2026</v>
       </c>
+      <c r="K32" t="n">
+        <v>4</v>
+      </c>
+      <c r="L32" t="n">
+        <v>2026</v>
+      </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>anyela.aponza@cotel.com.co</t>
+          <t>Belkis.jimenez@agrauto.com.co</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1915,7 +1915,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Oportunidad de COTEL SAL</t>
+          <t>Oportunidad de AGRICOLA AUTOMOTRIZ SAS</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1924,10 +1924,10 @@
         </is>
       </c>
       <c r="G33" s="1" t="n">
-        <v>46112.61271990741</v>
+        <v>46119.38914351852</v>
       </c>
       <c r="I33" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="J33" t="n">
         <v>2026</v>
@@ -1941,7 +1941,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>liliana.patino@quironsalud.com</t>
+          <t>anyela.aponza@cotel.com.co</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1952,14 +1952,9 @@
       <c r="C34" t="n">
         <v>0</v>
       </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>CLINICA IMBANACO</t>
-        </is>
-      </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Oportunidad de Liliana Patiño Flórez</t>
+          <t>Oportunidad de COTEL SAL</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1968,7 +1963,7 @@
         </is>
       </c>
       <c r="G34" s="1" t="n">
-        <v>46112.60853009259</v>
+        <v>46112.61271990741</v>
       </c>
       <c r="I34" t="n">
         <v>14</v>
@@ -1985,7 +1980,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>casanchez@jgb.com.co</t>
+          <t>liliana.patino@quironsalud.com</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1996,9 +1991,14 @@
       <c r="C35" t="n">
         <v>0</v>
       </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>CLINICA IMBANACO</t>
+        </is>
+      </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Oportunidad de JGB S.A.</t>
+          <t>Oportunidad de Liliana Patiño Flórez</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -2007,7 +2007,7 @@
         </is>
       </c>
       <c r="G35" s="1" t="n">
-        <v>46112.6052662037</v>
+        <v>46112.60853009259</v>
       </c>
       <c r="I35" t="n">
         <v>14</v>
@@ -2024,12 +2024,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>damaris.gomez@disfarma.com.co</t>
+          <t>casanchez@jgb.com.co</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Seguimiento</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -2037,7 +2037,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Oportunidad de DISFARMA</t>
+          <t>Oportunidad de JGB S.A.</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -2046,7 +2046,7 @@
         </is>
       </c>
       <c r="G36" s="1" t="n">
-        <v>46112.60325231482</v>
+        <v>46112.6052662037</v>
       </c>
       <c r="I36" t="n">
         <v>14</v>
@@ -2063,25 +2063,20 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>alergologosdeoccidente@gmail.com</t>
+          <t>damaris.gomez@disfarma.com.co</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Seguimiento</t>
         </is>
       </c>
       <c r="C37" t="n">
         <v>0</v>
       </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>Johana Gonzalez</t>
-        </is>
-      </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Oportunidad de Johana Gonzalez</t>
+          <t>Oportunidad de DISFARMA</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -2090,10 +2085,10 @@
         </is>
       </c>
       <c r="G37" s="1" t="n">
-        <v>46107.51248842593</v>
+        <v>46112.60325231482</v>
       </c>
       <c r="I37" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J37" t="n">
         <v>2026</v>
@@ -2107,77 +2102,76 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>DavidEsteban.Porras@alfalaval.com</t>
+          <t>alergologosdeoccidente@gmail.com</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Ganado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>15000000</v>
+        <v>0</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Johana Gonzalez</t>
+        </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Oportunidad de OPORTUNIDAD ENCUESTAS ALFALAVAL</t>
+          <t>Oportunidad de Johana Gonzalez</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G38" s="1" t="n">
-        <v>46101.72893518519</v>
-      </c>
-      <c r="H38" s="1" t="n">
-        <v>46141</v>
+        <v>46107.51248842593</v>
       </c>
       <c r="I38" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J38" t="n">
         <v>2026</v>
       </c>
-      <c r="K38" t="n">
-        <v>4</v>
-      </c>
-      <c r="L38" t="n">
-        <v>2026</v>
-      </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Dr.arcarmona@gmail.com</t>
+          <t>DavidEsteban.Porras@alfalaval.com</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Ganado</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>0</v>
+        <v>15000000</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Oportunidad de GAMANUCLEAR LTDA - Dr Alberto Carmona</t>
+          <t>Oportunidad de OPORTUNIDAD ENCUESTAS ALFALAVAL</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G39" s="1" t="n">
-        <v>46098.65114583333</v>
+        <v>46101.72893518519</v>
+      </c>
+      <c r="H39" s="1" t="n">
+        <v>46141</v>
       </c>
       <c r="I39" t="n">
         <v>12</v>
@@ -2185,16 +2179,22 @@
       <c r="J39" t="n">
         <v>2026</v>
       </c>
+      <c r="K39" t="n">
+        <v>4</v>
+      </c>
+      <c r="L39" t="n">
+        <v>2026</v>
+      </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>cecilia.guevara@cosmitet.net / administracion.crd@cosmitet.net</t>
+          <t>Dr.arcarmona@gmail.com</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2205,14 +2205,9 @@
       <c r="C40" t="n">
         <v>0</v>
       </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>Cecilia Guevara</t>
-        </is>
-      </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Oportunidad de CLINICA REY DAVID Walter Charria</t>
+          <t>Oportunidad de GAMANUCLEAR LTDA - Dr Alberto Carmona</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -2221,10 +2216,10 @@
         </is>
       </c>
       <c r="G40" s="1" t="n">
-        <v>46094.69002314815</v>
+        <v>46098.65114583333</v>
       </c>
       <c r="I40" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J40" t="n">
         <v>2026</v>
@@ -2238,7 +2233,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>vicerrectoriacademica@unicatolica.edu.co</t>
+          <t>cecilia.guevara@cosmitet.net / administracion.crd@cosmitet.net</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2251,12 +2246,12 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Jorge Silva</t>
+          <t>Cecilia Guevara</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Oportunidad de Jorge Silva</t>
+          <t>Oportunidad de CLINICA REY DAVID Walter Charria</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2265,7 +2260,7 @@
         </is>
       </c>
       <c r="G41" s="1" t="n">
-        <v>46094.66880787037</v>
+        <v>46094.69002314815</v>
       </c>
       <c r="I41" t="n">
         <v>11</v>
@@ -2282,37 +2277,34 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>pedroperea02@gmail.com</t>
+          <t>vicerrectoriacademica@unicatolica.edu.co</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Ganado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>2160000</v>
+        <v>0</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Pedro Pablo Perea Mafla</t>
+          <t>Jorge Silva</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Oportunidad de Encuestas</t>
+          <t>Oportunidad de Jorge Silva</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G42" s="1" t="n">
-        <v>46094.65905092593</v>
-      </c>
-      <c r="H42" s="1" t="n">
-        <v>46141</v>
+        <v>46094.66880787037</v>
       </c>
       <c r="I42" t="n">
         <v>11</v>
@@ -2320,35 +2312,34 @@
       <c r="J42" t="n">
         <v>2026</v>
       </c>
-      <c r="K42" t="n">
-        <v>4</v>
-      </c>
-      <c r="L42" t="n">
-        <v>2026</v>
-      </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>cristina.papamija@bmm.com.co</t>
+          <t>pedroperea02@gmail.com</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Ganado</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>8071000</v>
+        <v>2160000</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Pedro Pablo Perea Mafla</t>
+        </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Oportunidad de BANCO MUNDO MUJER</t>
+          <t>Oportunidad de Encuestas</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2357,7 +2348,10 @@
         </is>
       </c>
       <c r="G43" s="1" t="n">
-        <v>46094.65019675926</v>
+        <v>46094.65905092593</v>
+      </c>
+      <c r="H43" s="1" t="n">
+        <v>46141</v>
       </c>
       <c r="I43" t="n">
         <v>11</v>
@@ -2365,16 +2359,22 @@
       <c r="J43" t="n">
         <v>2026</v>
       </c>
+      <c r="K43" t="n">
+        <v>4</v>
+      </c>
+      <c r="L43" t="n">
+        <v>2026</v>
+      </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>capacitacionvirtual@fundacionwwbcol.org</t>
+          <t>cristina.papamija@bmm.com.co</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2383,11 +2383,11 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>1600000</v>
+        <v>8071000</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Licenciamiento y ajuste WhatsApp FUNDACIÓN WWB</t>
+          <t>Oportunidad de BANCO MUNDO MUJER</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -2396,7 +2396,7 @@
         </is>
       </c>
       <c r="G44" s="1" t="n">
-        <v>46094.64826388889</v>
+        <v>46094.65019675926</v>
       </c>
       <c r="I44" t="n">
         <v>11</v>
@@ -2413,25 +2413,20 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>carol.cuesta@cbolivar.com</t>
+          <t>capacitacionvirtual@fundacionwwbcol.org</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Ganado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>2900000</v>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>CAROL CUESTA</t>
-        </is>
+        <v>1600000</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Gestión de Subsidios CB Bogotá</t>
+          <t>Licenciamiento y ajuste WhatsApp FUNDACIÓN WWB</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -2440,10 +2435,7 @@
         </is>
       </c>
       <c r="G45" s="1" t="n">
-        <v>46094.64454861111</v>
-      </c>
-      <c r="H45" s="1" t="n">
-        <v>46135</v>
+        <v>46094.64826388889</v>
       </c>
       <c r="I45" t="n">
         <v>11</v>
@@ -2451,44 +2443,46 @@
       <c r="J45" t="n">
         <v>2026</v>
       </c>
-      <c r="K45" t="n">
-        <v>4</v>
-      </c>
-      <c r="L45" t="n">
-        <v>2026</v>
-      </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>edwin.munoz.v@uniminuto.edu</t>
+          <t>carol.cuesta@cbolivar.com</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Ganado</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>0</v>
+        <v>2900000</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>CAROL CUESTA</t>
+        </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Oportunidad de UNIMINUTO</t>
+          <t>Gestión de Subsidios CB Bogotá</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G46" s="1" t="n">
-        <v>46092.63626157407</v>
+        <v>46094.64454861111</v>
+      </c>
+      <c r="H46" s="1" t="n">
+        <v>46135</v>
       </c>
       <c r="I46" t="n">
         <v>11</v>
@@ -2496,16 +2490,22 @@
       <c r="J46" t="n">
         <v>2026</v>
       </c>
+      <c r="K46" t="n">
+        <v>4</v>
+      </c>
+      <c r="L46" t="n">
+        <v>2026</v>
+      </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>jaime_zuluaga@eficacia.com.co</t>
+          <t>edwin.munoz.v@uniminuto.edu</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2516,14 +2516,9 @@
       <c r="C47" t="n">
         <v>0</v>
       </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>Jaime Alberto</t>
-        </is>
-      </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Oportunidad de Jaime Alberto Zuluaga</t>
+          <t>Oportunidad de UNIMINUTO</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -2532,7 +2527,7 @@
         </is>
       </c>
       <c r="G47" s="1" t="n">
-        <v>46092.63153935185</v>
+        <v>46092.63626157407</v>
       </c>
       <c r="I47" t="n">
         <v>11</v>
@@ -2549,7 +2544,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>comercial@isyscol.com</t>
+          <t>jaime_zuluaga@eficacia.com.co</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2562,12 +2557,12 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Andres Nader</t>
+          <t>Jaime Alberto</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Oportunidad de Andres Nader</t>
+          <t>Oportunidad de Jaime Alberto Zuluaga</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2576,7 +2571,7 @@
         </is>
       </c>
       <c r="G48" s="1" t="n">
-        <v>46091.59211805555</v>
+        <v>46092.63153935185</v>
       </c>
       <c r="I48" t="n">
         <v>11</v>
@@ -2593,7 +2588,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>mercadeo@norteysur.co</t>
+          <t>comercial@isyscol.com</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2606,12 +2601,12 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Isabella Mesa</t>
+          <t>Andres Nader</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Oportunidad de Isabella Mesa</t>
+          <t>Oportunidad de Andres Nader</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -2620,7 +2615,7 @@
         </is>
       </c>
       <c r="G49" s="1" t="n">
-        <v>46091.40078703704</v>
+        <v>46091.59211805555</v>
       </c>
       <c r="I49" t="n">
         <v>11</v>
@@ -2635,26 +2630,36 @@
       </c>
     </row>
     <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>mercadeo@norteysur.co</t>
+        </is>
+      </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Seguimiento</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C50" t="n">
         <v>0</v>
       </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Isabella Mesa</t>
+        </is>
+      </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Clasificación EMAIL Comfenalco Cartagena</t>
+          <t>Oportunidad de Isabella Mesa</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Maria Fernanda Gaviria</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G50" s="1" t="n">
-        <v>46091.3665625</v>
+        <v>46091.40078703704</v>
       </c>
       <c r="I50" t="n">
         <v>11</v>
@@ -2671,7 +2676,7 @@
     <row r="51">
       <c r="B51" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Seguimiento</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -2679,19 +2684,19 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Oportunidad de ESE HOSPITAL LA MARIA</t>
+          <t>Clasificación EMAIL Comfenalco Cartagena</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Laura Alejandra Castañeda</t>
+          <t>Maria Fernanda Gaviria</t>
         </is>
       </c>
       <c r="G51" s="1" t="n">
-        <v>46083.67605324074</v>
+        <v>46091.3665625</v>
       </c>
       <c r="I51" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J51" t="n">
         <v>2026</v>
@@ -2713,7 +2718,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Oportunidad de SUPER TRANSPORTE</t>
+          <t>Oportunidad de ESE HOSPITAL LA MARIA</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -2722,7 +2727,7 @@
         </is>
       </c>
       <c r="G52" s="1" t="n">
-        <v>46083.6706712963</v>
+        <v>46083.67605324074</v>
       </c>
       <c r="I52" t="n">
         <v>10</v>
@@ -2747,7 +2752,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Oportunidad de ENLACES IP S.A.S</t>
+          <t>Oportunidad de SUPER TRANSPORTE</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -2756,7 +2761,7 @@
         </is>
       </c>
       <c r="G53" s="1" t="n">
-        <v>46083.50145833333</v>
+        <v>46083.6706712963</v>
       </c>
       <c r="I53" t="n">
         <v>10</v>
@@ -2771,11 +2776,6 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>accounting@diaza.com</t>
-        </is>
-      </c>
       <c r="B54" t="inlineStr">
         <is>
           <t>Perdido</t>
@@ -2784,26 +2784,21 @@
       <c r="C54" t="n">
         <v>0</v>
       </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>JOHANA RODRIGUEZ</t>
-        </is>
-      </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Oportunidad de JOHANA RODRIGUEZ</t>
+          <t>Oportunidad de ENLACES IP S.A.S</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Laura Alejandra Castañeda</t>
         </is>
       </c>
       <c r="G54" s="1" t="n">
-        <v>46079.73486111111</v>
+        <v>46083.50145833333</v>
       </c>
       <c r="I54" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J54" t="n">
         <v>2026</v>
@@ -2817,7 +2812,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>mensajeriamyr@gmail.com</t>
+          <t>accounting@diaza.com</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2828,9 +2823,14 @@
       <c r="C55" t="n">
         <v>0</v>
       </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>JOHANA RODRIGUEZ</t>
+        </is>
+      </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Oportunidad de MENSAJERIA M&amp;R SAS</t>
+          <t>Oportunidad de JOHANA RODRIGUEZ</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -2839,7 +2839,7 @@
         </is>
       </c>
       <c r="G55" s="1" t="n">
-        <v>46079.72262731481</v>
+        <v>46079.73486111111</v>
       </c>
       <c r="I55" t="n">
         <v>9</v>
@@ -2856,7 +2856,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>sistemaspanaderialeal@gmail.com</t>
+          <t>mensajeriamyr@gmail.com</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2867,14 +2867,9 @@
       <c r="C56" t="n">
         <v>0</v>
       </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>Diego Rios</t>
-        </is>
-      </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>JAMDAC SAS, Diego Rios</t>
+          <t>Oportunidad de MENSAJERIA M&amp;R SAS</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -2883,10 +2878,10 @@
         </is>
       </c>
       <c r="G56" s="1" t="n">
-        <v>46071.63706018519</v>
+        <v>46079.72262731481</v>
       </c>
       <c r="I56" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J56" t="n">
         <v>2026</v>
@@ -2900,7 +2895,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>efernandez@unico.com.co</t>
+          <t>sistemaspanaderialeal@gmail.com</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2913,12 +2908,12 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Erick Fernandez</t>
+          <t>Diego Rios</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Oportunidad de Erick Fernandez</t>
+          <t>JAMDAC SAS, Diego Rios</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -2927,10 +2922,10 @@
         </is>
       </c>
       <c r="G57" s="1" t="n">
-        <v>46064.3750462963</v>
+        <v>46071.63706018519</v>
       </c>
       <c r="I57" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J57" t="n">
         <v>2026</v>
@@ -2944,7 +2939,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>kabenitez@icesi.edu.co</t>
+          <t>efernandez@unico.com.co</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2953,28 +2948,28 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>10000000</v>
+        <v>0</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>KENI BENITEZ</t>
+          <t>Erick Fernandez</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Oportunidad de KENI BENITEZ</t>
+          <t>Oportunidad de Erick Fernandez</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G58" s="1" t="n">
-        <v>46059.34918981481</v>
+        <v>46064.3750462963</v>
       </c>
       <c r="I58" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J58" t="n">
         <v>2026</v>
@@ -2988,7 +2983,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>patovar@uao.edu.co</t>
+          <t>kabenitez@icesi.edu.co</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2997,25 +2992,25 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>0</v>
+        <v>10000000</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Paula Tovar</t>
+          <t>KENI BENITEZ</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Oportunidad de UNIVERSIDAD AUTONOMA DE OCCIDENTE</t>
+          <t>Oportunidad de KENI BENITEZ</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G59" s="1" t="n">
-        <v>46058.72516203704</v>
+        <v>46059.34918981481</v>
       </c>
       <c r="I59" t="n">
         <v>6</v>
@@ -3032,7 +3027,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>comercial@isyscol.com</t>
+          <t>patovar@uao.edu.co</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -3043,9 +3038,14 @@
       <c r="C60" t="n">
         <v>0</v>
       </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Paula Tovar</t>
+        </is>
+      </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Oportunidad de TECNOLOGIAS ISYSCOL SAS</t>
+          <t>Oportunidad de UNIVERSIDAD AUTONOMA DE OCCIDENTE</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -3054,7 +3054,7 @@
         </is>
       </c>
       <c r="G60" s="1" t="n">
-        <v>46057.58993055556</v>
+        <v>46058.72516203704</v>
       </c>
       <c r="I60" t="n">
         <v>6</v>
@@ -3069,17 +3069,22 @@
       </c>
     </row>
     <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>comercial@isyscol.com</t>
+        </is>
+      </c>
       <c r="B61" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>15000000</v>
+        <v>0</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Oportunidad de VOICE IA EFICACIA</t>
+          <t>Oportunidad de TECNOLOGIAS ISYSCOL SAS</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -3088,7 +3093,7 @@
         </is>
       </c>
       <c r="G61" s="1" t="n">
-        <v>46057.3409837963</v>
+        <v>46057.58993055556</v>
       </c>
       <c r="I61" t="n">
         <v>6</v>
@@ -3109,23 +3114,23 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>4000000</v>
+        <v>15000000</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Oportunidad de Eficacia WhatsApp</t>
+          <t>Oportunidad de VOICE IA EFICACIA</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G62" s="1" t="n">
-        <v>46049.67292824074</v>
+        <v>46057.3409837963</v>
       </c>
       <c r="I62" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J62" t="n">
         <v>2026</v>
@@ -3143,62 +3148,57 @@
         </is>
       </c>
       <c r="C63" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Oportunidad de Eficacia WhatsApp</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Jennifer Hoyos Gallego</t>
+        </is>
+      </c>
+      <c r="G63" s="1" t="n">
+        <v>46049.67292824074</v>
+      </c>
+      <c r="I63" t="n">
+        <v>5</v>
+      </c>
+      <c r="J63" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>No calificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
         <v>20000000</v>
       </c>
-      <c r="E63" t="inlineStr">
+      <c r="E64" t="inlineStr">
         <is>
           <t>Oportunidad de CRUZ ROJA COLOMBIANA SECCIONAL VALLE DEL CAUCA</t>
         </is>
       </c>
-      <c r="F63" t="inlineStr">
+      <c r="F64" t="inlineStr">
         <is>
           <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
-      <c r="G63" s="1" t="n">
+      <c r="G64" s="1" t="n">
         <v>46006.49650462963</v>
       </c>
-      <c r="I63" t="n">
+      <c r="I64" t="n">
         <v>51</v>
-      </c>
-      <c r="J63" t="n">
-        <v>2025</v>
-      </c>
-      <c r="M63" t="inlineStr">
-        <is>
-          <t>No calificado</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>silvia.figueroa@neurithmedia.com</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C64" t="n">
-        <v>25000000</v>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>Contact center ventas España</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>Richard Castaño</t>
-        </is>
-      </c>
-      <c r="G64" s="1" t="n">
-        <v>45960.61145833333</v>
-      </c>
-      <c r="I64" t="n">
-        <v>44</v>
       </c>
       <c r="J64" t="n">
         <v>2025</v>
@@ -3210,22 +3210,22 @@
       </c>
     </row>
     <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>silvia.figueroa@neurithmedia.com</t>
+        </is>
+      </c>
       <c r="B65" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>37000000</v>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>Mabel</t>
-        </is>
+        <v>25000000</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Masivos Licitacion</t>
+          <t>Contact center ventas España</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -3234,10 +3234,10 @@
         </is>
       </c>
       <c r="G65" s="1" t="n">
-        <v>45940.49372685186</v>
+        <v>45960.61145833333</v>
       </c>
       <c r="I65" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="J65" t="n">
         <v>2025</v>
@@ -3249,36 +3249,31 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>ana.zuniga@cbolivar.com</t>
-        </is>
-      </c>
       <c r="B66" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>4997000</v>
+        <v>37000000</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Ana Lucia Zuñiga</t>
+          <t>Mabel</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Constructora Bolivar Agente Redes</t>
+          <t>Masivos Licitacion</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Richard Castaño</t>
         </is>
       </c>
       <c r="G66" s="1" t="n">
-        <v>45940.49215277778</v>
+        <v>45940.49372685186</v>
       </c>
       <c r="I66" t="n">
         <v>41</v>
@@ -3295,7 +3290,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>julian_mendez@extras.com.co</t>
+          <t>ana.zuniga@cbolivar.com</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3304,28 +3299,28 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>15000000</v>
+        <v>4997000</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Julian Mendez.</t>
+          <t>Ana Lucia Zuñiga</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Oportunidad de EFICACIA S A S</t>
+          <t>Constructora Bolivar Agente Redes</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G67" s="1" t="n">
-        <v>45922.66201388889</v>
+        <v>45940.49215277778</v>
       </c>
       <c r="I67" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="J67" t="n">
         <v>2025</v>
@@ -3339,7 +3334,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>info@eficacia.com.co</t>
+          <t>julian_mendez@extras.com.co</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -3348,11 +3343,16 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>0</v>
+        <v>15000000</v>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Julian Mendez.</t>
+        </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Nutresa</t>
+          <t>Oportunidad de EFICACIA S A S</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -3361,7 +3361,7 @@
         </is>
       </c>
       <c r="G68" s="1" t="n">
-        <v>45922.66199074074</v>
+        <v>45922.66201388889</v>
       </c>
       <c r="I68" t="n">
         <v>39</v>
@@ -3378,37 +3378,32 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>hrodriguez@jaramillomora.com</t>
+          <t>info@eficacia.com.co</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Seguimiento</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>30000000</v>
-      </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>HANNA</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Oportunidad de JARAMILLO MORA CONSTRUCTORA S A</t>
+          <t>Nutresa</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Richard Castaño</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G69" s="1" t="n">
-        <v>45916.71618055556</v>
+        <v>45922.66199074074</v>
       </c>
       <c r="I69" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="J69" t="n">
         <v>2025</v>
@@ -3420,17 +3415,27 @@
       </c>
     </row>
     <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>hrodriguez@jaramillomora.com</t>
+        </is>
+      </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Seguimiento</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>147000000</v>
+        <v>30000000</v>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>HANNA</t>
+        </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Contact Center Agendamiento citas</t>
+          <t>Oportunidad de JARAMILLO MORA CONSTRUCTORA S A</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -3439,7 +3444,7 @@
         </is>
       </c>
       <c r="G70" s="1" t="n">
-        <v>45916.67502314815</v>
+        <v>45916.71618055556</v>
       </c>
       <c r="I70" t="n">
         <v>38</v>
@@ -3454,34 +3459,26 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>jaime_zuluaga@eficacia.com.co</t>
-        </is>
-      </c>
       <c r="B71" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>14700000</v>
+        <v>147000000</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Agentes contact center encuestas</t>
+          <t>Contact Center Agendamiento citas</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Richard Castaño</t>
         </is>
       </c>
       <c r="G71" s="1" t="n">
-        <v>45916.65275462963</v>
-      </c>
-      <c r="H71" s="1" t="n">
-        <v>45930</v>
+        <v>45916.67502314815</v>
       </c>
       <c r="I71" t="n">
         <v>38</v>
@@ -3489,12 +3486,6 @@
       <c r="J71" t="n">
         <v>2025</v>
       </c>
-      <c r="K71" t="n">
-        <v>9</v>
-      </c>
-      <c r="L71" t="n">
-        <v>2025</v>
-      </c>
       <c r="M71" t="inlineStr">
         <is>
           <t>No calificado</t>
@@ -3502,22 +3493,22 @@
       </c>
     </row>
     <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>jaime_zuluaga@eficacia.com.co</t>
+        </is>
+      </c>
       <c r="B72" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>4796000</v>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>Juan Grisales</t>
-        </is>
+        <v>14700000</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Agente Call Center Outbound</t>
+          <t>Agentes contact center encuestas</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -3526,7 +3517,10 @@
         </is>
       </c>
       <c r="G72" s="1" t="n">
-        <v>45915.4809375</v>
+        <v>45916.65275462963</v>
+      </c>
+      <c r="H72" s="1" t="n">
+        <v>45930</v>
       </c>
       <c r="I72" t="n">
         <v>38</v>
@@ -3534,6 +3528,12 @@
       <c r="J72" t="n">
         <v>2025</v>
       </c>
+      <c r="K72" t="n">
+        <v>9</v>
+      </c>
+      <c r="L72" t="n">
+        <v>2025</v>
+      </c>
       <c r="M72" t="inlineStr">
         <is>
           <t>No calificado</t>
@@ -3541,27 +3541,22 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>gestormercadeo@lamontana.co</t>
-        </is>
-      </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Seguimiento</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>25000000</v>
+        <v>4796000</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Alejandra Ossa</t>
+          <t>Juan Grisales</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Voice BOT</t>
+          <t>Agente Call Center Outbound</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -3570,10 +3565,7 @@
         </is>
       </c>
       <c r="G73" s="1" t="n">
-        <v>45915.48023148148</v>
-      </c>
-      <c r="H73" s="1" t="n">
-        <v>46150</v>
+        <v>45915.4809375</v>
       </c>
       <c r="I73" t="n">
         <v>38</v>
@@ -3581,12 +3573,6 @@
       <c r="J73" t="n">
         <v>2025</v>
       </c>
-      <c r="K73" t="n">
-        <v>5</v>
-      </c>
-      <c r="L73" t="n">
-        <v>2026</v>
-      </c>
       <c r="M73" t="inlineStr">
         <is>
           <t>No calificado</t>
@@ -3596,20 +3582,25 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>elkinmarquezconsuegra@gmail.com</t>
+          <t>gestormercadeo@lamontana.co</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Seguimiento</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>2500000</v>
+        <v>25000000</v>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Alejandra Ossa</t>
+        </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Venta Masivos</t>
+          <t>Voice BOT</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -3618,7 +3609,10 @@
         </is>
       </c>
       <c r="G74" s="1" t="n">
-        <v>45915.47924768519</v>
+        <v>45915.48023148148</v>
+      </c>
+      <c r="H74" s="1" t="n">
+        <v>46150</v>
       </c>
       <c r="I74" t="n">
         <v>38</v>
@@ -3626,6 +3620,12 @@
       <c r="J74" t="n">
         <v>2025</v>
       </c>
+      <c r="K74" t="n">
+        <v>5</v>
+      </c>
+      <c r="L74" t="n">
+        <v>2026</v>
+      </c>
       <c r="M74" t="inlineStr">
         <is>
           <t>No calificado</t>
@@ -3635,7 +3635,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>bladimir.munoz@uptc.edu.co</t>
+          <t>elkinmarquezconsuegra@gmail.com</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -3644,16 +3644,11 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>22000000</v>
-      </c>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>Bladimir Muñoz Forero</t>
-        </is>
+        <v>2500000</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Oportunidad Venta BPO</t>
+          <t>Venta Masivos</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -3662,7 +3657,7 @@
         </is>
       </c>
       <c r="G75" s="1" t="n">
-        <v>45915.47494212963</v>
+        <v>45915.47924768519</v>
       </c>
       <c r="I75" t="n">
         <v>38</v>
@@ -3679,7 +3674,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>gerencia@alitasfactory.com</t>
+          <t>bladimir.munoz@uptc.edu.co</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -3688,20 +3683,25 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>40000000</v>
+        <v>22000000</v>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Bladimir Muñoz Forero</t>
+        </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>1 agente IA para ventas y asesoramiento</t>
+          <t>Oportunidad Venta BPO</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Richard Castaño</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G76" s="1" t="n">
-        <v>45915.47300925926</v>
+        <v>45915.47494212963</v>
       </c>
       <c r="I76" t="n">
         <v>38</v>
@@ -3718,7 +3718,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>mmonroy@falabella.com.co</t>
+          <t>gerencia@alitasfactory.com</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -3727,11 +3727,11 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>60000000</v>
+        <v>40000000</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Agente IA Try and Buy Inbound y Outbound</t>
+          <t>1 agente IA para ventas y asesoramiento</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -3740,7 +3740,7 @@
         </is>
       </c>
       <c r="G77" s="1" t="n">
-        <v>45915.46633101852</v>
+        <v>45915.47300925926</v>
       </c>
       <c r="I77" t="n">
         <v>38</v>
@@ -3757,7 +3757,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>gerencia@motosymotoselpaisa.com</t>
+          <t>mmonroy@falabella.com.co</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -3766,20 +3766,20 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>40000000</v>
+        <v>60000000</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Oportunidad de MOTOS Y MOTOS EL PAISA S A S</t>
+          <t>Agente IA Try and Buy Inbound y Outbound</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Richard Castaño</t>
         </is>
       </c>
       <c r="G78" s="1" t="n">
-        <v>45915.46252314815</v>
+        <v>45915.46633101852</v>
       </c>
       <c r="I78" t="n">
         <v>38</v>
@@ -3796,7 +3796,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>isanchez@unico.com.co</t>
+          <t>gerencia@motosymotoselpaisa.com</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -3805,11 +3805,11 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>0</v>
+        <v>40000000</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>1 agente IA para relacionamiento con locatarios</t>
+          <t>Oportunidad de MOTOS Y MOTOS EL PAISA S A S</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -3818,7 +3818,7 @@
         </is>
       </c>
       <c r="G79" s="1" t="n">
-        <v>45915.46157407408</v>
+        <v>45915.46252314815</v>
       </c>
       <c r="I79" t="n">
         <v>38</v>
@@ -3835,7 +3835,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>asantiago@stop.com.co</t>
+          <t>isanchez@unico.com.co</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -3844,11 +3844,11 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>30000000</v>
+        <v>0</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>1 Agente IA en cobranzas</t>
+          <t>1 agente IA para relacionamiento con locatarios</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -3857,7 +3857,7 @@
         </is>
       </c>
       <c r="G80" s="1" t="n">
-        <v>45915.46052083333</v>
+        <v>45915.46157407408</v>
       </c>
       <c r="I80" t="n">
         <v>38</v>
@@ -3874,7 +3874,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>jcastano@mercaldas.com.co</t>
+          <t>asantiago@stop.com.co</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -3887,7 +3887,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>1 agente IA para ventas y asesoramiento</t>
+          <t>1 Agente IA en cobranzas</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -3896,7 +3896,7 @@
         </is>
       </c>
       <c r="G81" s="1" t="n">
-        <v>45915.35666666667</v>
+        <v>45915.46052083333</v>
       </c>
       <c r="I81" t="n">
         <v>38</v>

</xml_diff>

<commit_message>
CRM actualizado — 26/05/2026 14:45
</commit_message>
<xml_diff>
--- a/CRM_PowerBI_BrendaLuna_actualizado.xlsx
+++ b/CRM_PowerBI_BrendaLuna_actualizado.xlsx
@@ -944,22 +944,22 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>comercial2@felsyn.com</t>
-        </is>
-      </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>713400</v>
+        <v>0</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Olga Lucia Hurtado</t>
+        </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Oportunidad de FONDO DE EMPLEADOS FELSYN</t>
+          <t>Oportunidad de Olga Lucia Hurtado</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -968,42 +968,37 @@
         </is>
       </c>
       <c r="G11" s="1" t="n">
-        <v>46163.49130787037</v>
+        <v>46168.49854166667</v>
       </c>
       <c r="I11" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="J11" t="n">
         <v>2026</v>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>mercadeo@lasevillana.com.co</t>
+          <t>comercial2@felsyn.com</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0</v>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fabio AlbertoGallego García </t>
-        </is>
+        <v>713400</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Oportunidad de Fabio AlbertoGallego García </t>
+          <t>Oportunidad de FONDO DE EMPLEADOS FELSYN</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1012,7 +1007,7 @@
         </is>
       </c>
       <c r="G12" s="1" t="n">
-        <v>46162.64569444444</v>
+        <v>46163.49130787037</v>
       </c>
       <c r="I12" t="n">
         <v>21</v>
@@ -1022,27 +1017,32 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>asantiago@stop.com.co</t>
+          <t>mercadeo@lasevillana.com.co</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C13" t="n">
         <v>0</v>
       </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fabio AlbertoGallego García </t>
+        </is>
+      </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Oportunidad de STOP SAS</t>
+          <t xml:space="preserve">Oportunidad de Fabio AlbertoGallego García </t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1051,7 +1051,7 @@
         </is>
       </c>
       <c r="G13" s="1" t="n">
-        <v>46161.63508101852</v>
+        <v>46162.64569444444</v>
       </c>
       <c r="I13" t="n">
         <v>21</v>
@@ -1068,25 +1068,20 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>aestrada@teker.co</t>
+          <t>asantiago@stop.com.co</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>16914000</v>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>TEKER SALUD SAS</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Oportunidad de TEKER SALUD SAS</t>
+          <t>Oportunidad de STOP SAS</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1095,7 +1090,7 @@
         </is>
       </c>
       <c r="G14" s="1" t="n">
-        <v>46161.62922453704</v>
+        <v>46161.63508101852</v>
       </c>
       <c r="I14" t="n">
         <v>21</v>
@@ -1105,22 +1100,32 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>aestrada@teker.co</t>
+        </is>
+      </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0</v>
+        <v>16914000</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>TEKER SALUD SAS</t>
+        </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Oportunidad de TIAN IPS SAS</t>
+          <t>Oportunidad de TEKER SALUD SAS</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1129,7 +1134,7 @@
         </is>
       </c>
       <c r="G15" s="1" t="n">
-        <v>46161.61643518518</v>
+        <v>46161.62922453704</v>
       </c>
       <c r="I15" t="n">
         <v>21</v>
@@ -1139,32 +1144,22 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>administración@fullredtotal.com</t>
-        </is>
-      </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>14000000</v>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Eivar Eñasco</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Oportunidad de Eivar Eñasco</t>
+          <t>Oportunidad de TIAN IPS SAS</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1173,42 +1168,42 @@
         </is>
       </c>
       <c r="G16" s="1" t="n">
-        <v>46154.67546296296</v>
+        <v>46161.61643518518</v>
       </c>
       <c r="I16" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J16" t="n">
         <v>2026</v>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>cserna@surtifamiliar.com.co</t>
+          <t>administración@fullredtotal.com</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Negociación</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1950000</v>
+        <v>14000000</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Claudia Patricia Serna</t>
+          <t>Eivar Eñasco</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Oportunidad de Claudia Patricia Serna</t>
+          <t>Oportunidad de Eivar Eñasco</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1217,7 +1212,7 @@
         </is>
       </c>
       <c r="G17" s="1" t="n">
-        <v>46154.66616898148</v>
+        <v>46154.67546296296</v>
       </c>
       <c r="I17" t="n">
         <v>20</v>
@@ -1234,25 +1229,25 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>coordmercadeo@pacificcenter.co</t>
+          <t>cserna@surtifamiliar.com.co</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Negociación</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>5600000</v>
+        <v>1950000</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Claudia Castro</t>
+          <t>Claudia Patricia Serna</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Oportunidad de Claudia Castro</t>
+          <t>Oportunidad de Claudia Patricia Serna</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1261,7 +1256,7 @@
         </is>
       </c>
       <c r="G18" s="1" t="n">
-        <v>46154.66341435185</v>
+        <v>46154.66616898148</v>
       </c>
       <c r="I18" t="n">
         <v>20</v>
@@ -1278,25 +1273,25 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>isabellarengifo27@gmail.com</t>
+          <t>coordmercadeo@pacificcenter.co</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>28190000</v>
+        <v>5600000</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Isabella Rengifo</t>
+          <t>Claudia Castro</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Oportunidad de Isabella Rengifo</t>
+          <t>Oportunidad de Claudia Castro</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1305,7 +1300,7 @@
         </is>
       </c>
       <c r="G19" s="1" t="n">
-        <v>46154.65981481481</v>
+        <v>46154.66341435185</v>
       </c>
       <c r="I19" t="n">
         <v>20</v>
@@ -1315,39 +1310,41 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>isabellarengifo27@gmail.com</t>
+        </is>
+      </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>50000000</v>
+        <v>28190000</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Paola Gómez - Agente Inmobiliaria Independiente</t>
+          <t>Isabella Rengifo</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Puesto de Trabajo CC Medellin</t>
+          <t>Oportunidad de Isabella Rengifo</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Richard Castaño</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G20" s="1" t="n">
-        <v>46154.49104166667</v>
-      </c>
-      <c r="H20" s="1" t="n">
-        <v>46170</v>
+        <v>46154.65981481481</v>
       </c>
       <c r="I20" t="n">
         <v>20</v>
@@ -1355,44 +1352,41 @@
       <c r="J20" t="n">
         <v>2026</v>
       </c>
-      <c r="K20" t="n">
-        <v>5</v>
-      </c>
-      <c r="L20" t="n">
-        <v>2026</v>
-      </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>alberto.ramirez@constructorabolivar.com</t>
-        </is>
-      </c>
       <c r="B21" t="inlineStr">
         <is>
           <t>Propuesta</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>3000000</v>
+        <v>50000000</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Paola Gómez - Agente Inmobiliaria Independiente</t>
+        </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Oportunidad de NPS Relacional</t>
+          <t>Puesto de Trabajo CC Medellin</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Richard Castaño</t>
         </is>
       </c>
       <c r="G21" s="1" t="n">
-        <v>46154.44511574074</v>
+        <v>46154.49104166667</v>
+      </c>
+      <c r="H21" s="1" t="n">
+        <v>46170</v>
       </c>
       <c r="I21" t="n">
         <v>20</v>
@@ -1400,6 +1394,12 @@
       <c r="J21" t="n">
         <v>2026</v>
       </c>
+      <c r="K21" t="n">
+        <v>5</v>
+      </c>
+      <c r="L21" t="n">
+        <v>2026</v>
+      </c>
       <c r="M21" t="inlineStr">
         <is>
           <t>Calificado</t>
@@ -1407,75 +1407,70 @@
       </c>
     </row>
     <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>alberto.ramirez@constructorabolivar.com</t>
+        </is>
+      </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C22" t="n">
         <v>3000000</v>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Oportunidad de NPS Relacional</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Jennifer Hoyos Gallego</t>
+        </is>
+      </c>
+      <c r="G22" s="1" t="n">
+        <v>46154.44511574074</v>
+      </c>
+      <c r="I22" t="n">
+        <v>20</v>
+      </c>
+      <c r="J22" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>Calificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="D23" t="inlineStr">
         <is>
           <t>MADERKIT</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>Oportunidad de MADERKIT</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G22" s="1" t="n">
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G23" s="1" t="n">
         <v>46147.66540509259</v>
-      </c>
-      <c r="I22" t="n">
-        <v>19</v>
-      </c>
-      <c r="J22" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t>No calificado</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>omer120395@gmail.com</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C23" t="n">
-        <v>0</v>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Omer Peñaloza</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>Oportunidad de Omer Peñaloza</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G23" s="1" t="n">
-        <v>46147.66090277778</v>
       </c>
       <c r="I23" t="n">
         <v>19</v>
@@ -1492,7 +1487,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>directora.it@supermercadobelalcazar.com.co</t>
+          <t>omer120395@gmail.com</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1501,11 +1496,16 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>6000000</v>
+        <v>0</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Omer Peñaloza</t>
+        </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Oportunidad de ABASTECEMOS DE OCCIDENTE</t>
+          <t>Oportunidad de Omer Peñaloza</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1514,10 +1514,7 @@
         </is>
       </c>
       <c r="G24" s="1" t="n">
-        <v>46147.64170138889</v>
-      </c>
-      <c r="H24" s="1" t="n">
-        <v>46157</v>
+        <v>46147.66090277778</v>
       </c>
       <c r="I24" t="n">
         <v>19</v>
@@ -1525,12 +1522,6 @@
       <c r="J24" t="n">
         <v>2026</v>
       </c>
-      <c r="K24" t="n">
-        <v>5</v>
-      </c>
-      <c r="L24" t="n">
-        <v>2026</v>
-      </c>
       <c r="M24" t="inlineStr">
         <is>
           <t>No calificado</t>
@@ -1540,20 +1531,20 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>oscar.molina@terrenoshouston.com</t>
+          <t>directora.it@supermercadobelalcazar.com.co</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Negociación</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>37623040</v>
+        <v>6000000</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Oportunidad de COLONY RIDGE</t>
+          <t>Oportunidad de ABASTECEMOS DE OCCIDENTE</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1562,10 +1553,10 @@
         </is>
       </c>
       <c r="G25" s="1" t="n">
-        <v>46147.60297453704</v>
+        <v>46147.64170138889</v>
       </c>
       <c r="H25" s="1" t="n">
-        <v>46150</v>
+        <v>46157</v>
       </c>
       <c r="I25" t="n">
         <v>19</v>
@@ -1581,27 +1572,27 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>jsantacr@ccc.org.co</t>
+          <t>oscar.molina@terrenoshouston.com</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Negociación</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>55000000</v>
+        <v>37623040</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Oportunidad de CAMARA DE COMERCIO CALI</t>
+          <t>Oportunidad de COLONY RIDGE</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1610,46 +1601,46 @@
         </is>
       </c>
       <c r="G26" s="1" t="n">
-        <v>46141.62370370371</v>
+        <v>46147.60297453704</v>
       </c>
       <c r="H26" s="1" t="n">
-        <v>46289</v>
+        <v>46150</v>
       </c>
       <c r="I26" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J26" t="n">
         <v>2026</v>
       </c>
       <c r="K26" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="L26" t="n">
         <v>2026</v>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>exportaciones@laprovincia.com</t>
+          <t>jsantacr@ccc.org.co</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>6000000</v>
+        <v>55000000</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Oportunidad de PRODUCTOS LA PROVINCIA SAS</t>
+          <t>Oportunidad de CAMARA DE COMERCIO CALI</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1658,7 +1649,10 @@
         </is>
       </c>
       <c r="G27" s="1" t="n">
-        <v>46141.62021990741</v>
+        <v>46141.62370370371</v>
+      </c>
+      <c r="H27" s="1" t="n">
+        <v>46289</v>
       </c>
       <c r="I27" t="n">
         <v>18</v>
@@ -1666,6 +1660,12 @@
       <c r="J27" t="n">
         <v>2026</v>
       </c>
+      <c r="K27" t="n">
+        <v>9</v>
+      </c>
+      <c r="L27" t="n">
+        <v>2026</v>
+      </c>
       <c r="M27" t="inlineStr">
         <is>
           <t>No calificado</t>
@@ -1675,7 +1675,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>coordinador.mercadeo@regency.com.co</t>
+          <t>exportaciones@laprovincia.com</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1684,11 +1684,11 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>0</v>
+        <v>6000000</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Oportunidad de REGENCY TECH SAS</t>
+          <t>Oportunidad de PRODUCTOS LA PROVINCIA SAS</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1697,7 +1697,7 @@
         </is>
       </c>
       <c r="G28" s="1" t="n">
-        <v>46141.59664351852</v>
+        <v>46141.62021990741</v>
       </c>
       <c r="I28" t="n">
         <v>18</v>
@@ -1712,17 +1712,22 @@
       </c>
     </row>
     <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>coordinador.mercadeo@regency.com.co</t>
+        </is>
+      </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1200000</v>
+        <v>0</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Oportunidad de EMCALI E.I.C.E ESP</t>
+          <t>Oportunidad de REGENCY TECH SAS</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1731,10 +1736,7 @@
         </is>
       </c>
       <c r="G29" s="1" t="n">
-        <v>46141.59045138889</v>
-      </c>
-      <c r="H29" s="1" t="n">
-        <v>46352</v>
+        <v>46141.59664351852</v>
       </c>
       <c r="I29" t="n">
         <v>18</v>
@@ -1742,56 +1744,45 @@
       <c r="J29" t="n">
         <v>2026</v>
       </c>
-      <c r="K29" t="n">
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>No calificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Contactado</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>1200000</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Oportunidad de EMCALI E.I.C.E ESP</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G30" s="1" t="n">
+        <v>46141.59045138889</v>
+      </c>
+      <c r="H30" s="1" t="n">
+        <v>46352</v>
+      </c>
+      <c r="I30" t="n">
+        <v>18</v>
+      </c>
+      <c r="J30" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K30" t="n">
         <v>11</v>
-      </c>
-      <c r="L29" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M29" t="inlineStr">
-        <is>
-          <t>No calificado</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>angie_feligrana@eficacia.com.co</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Seguimiento</t>
-        </is>
-      </c>
-      <c r="C30" t="n">
-        <v>6000000</v>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>Oportunidad de Eficacia sas / Angie Feligrana</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G30" s="1" t="n">
-        <v>46126.63210648148</v>
-      </c>
-      <c r="H30" s="1" t="n">
-        <v>46150</v>
-      </c>
-      <c r="I30" t="n">
-        <v>16</v>
-      </c>
-      <c r="J30" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K30" t="n">
-        <v>5</v>
       </c>
       <c r="L30" t="n">
         <v>2026</v>
@@ -1805,25 +1796,20 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Estrategiadigital@zuluagaysoto.com</t>
+          <t>angie_feligrana@eficacia.com.co</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Seguimiento</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>0</v>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>Maryuri Arguello</t>
-        </is>
+        <v>6000000</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Oportunidad de Maryuri Arguello</t>
+          <t>Oportunidad de Eficacia sas / Angie Feligrana</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1832,7 +1818,10 @@
         </is>
       </c>
       <c r="G31" s="1" t="n">
-        <v>46125.71925925926</v>
+        <v>46126.63210648148</v>
+      </c>
+      <c r="H31" s="1" t="n">
+        <v>46150</v>
       </c>
       <c r="I31" t="n">
         <v>16</v>
@@ -1840,6 +1829,12 @@
       <c r="J31" t="n">
         <v>2026</v>
       </c>
+      <c r="K31" t="n">
+        <v>5</v>
+      </c>
+      <c r="L31" t="n">
+        <v>2026</v>
+      </c>
       <c r="M31" t="inlineStr">
         <is>
           <t>No calificado</t>
@@ -1849,82 +1844,81 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>gabrielrodriguez@arrozsupremo.com</t>
+          <t>Estrategiadigital@zuluagaysoto.com</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Ganado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>8000000</v>
+        <v>0</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>GABRIEL RODRIGUEZ</t>
+          <t>Maryuri Arguello</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Agente de Ventas</t>
+          <t>Oportunidad de Maryuri Arguello</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Richard Castaño</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G32" s="1" t="n">
-        <v>46119.62108796297</v>
-      </c>
-      <c r="H32" s="1" t="n">
-        <v>46141</v>
+        <v>46125.71925925926</v>
       </c>
       <c r="I32" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J32" t="n">
         <v>2026</v>
       </c>
-      <c r="K32" t="n">
-        <v>4</v>
-      </c>
-      <c r="L32" t="n">
-        <v>2026</v>
-      </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Belkis.jimenez@agrauto.com.co</t>
+          <t>gabrielrodriguez@arrozsupremo.com</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Ganado</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>0</v>
+        <v>8000000</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>GABRIEL RODRIGUEZ</t>
+        </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Oportunidad de AGRICOLA AUTOMOTRIZ SAS</t>
+          <t>Agente de Ventas</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Richard Castaño</t>
         </is>
       </c>
       <c r="G33" s="1" t="n">
-        <v>46119.38914351852</v>
+        <v>46119.62108796297</v>
+      </c>
+      <c r="H33" s="1" t="n">
+        <v>46141</v>
       </c>
       <c r="I33" t="n">
         <v>15</v>
@@ -1932,16 +1926,22 @@
       <c r="J33" t="n">
         <v>2026</v>
       </c>
+      <c r="K33" t="n">
+        <v>4</v>
+      </c>
+      <c r="L33" t="n">
+        <v>2026</v>
+      </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>anyela.aponza@cotel.com.co</t>
+          <t>Belkis.jimenez@agrauto.com.co</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1954,7 +1954,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Oportunidad de COTEL SAL</t>
+          <t>Oportunidad de AGRICOLA AUTOMOTRIZ SAS</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1963,10 +1963,10 @@
         </is>
       </c>
       <c r="G34" s="1" t="n">
-        <v>46112.61271990741</v>
+        <v>46119.38914351852</v>
       </c>
       <c r="I34" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="J34" t="n">
         <v>2026</v>
@@ -1980,7 +1980,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>liliana.patino@quironsalud.com</t>
+          <t>anyela.aponza@cotel.com.co</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1991,14 +1991,9 @@
       <c r="C35" t="n">
         <v>0</v>
       </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>CLINICA IMBANACO</t>
-        </is>
-      </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Oportunidad de Liliana Patiño Flórez</t>
+          <t>Oportunidad de COTEL SAL</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -2007,7 +2002,7 @@
         </is>
       </c>
       <c r="G35" s="1" t="n">
-        <v>46112.60853009259</v>
+        <v>46112.61271990741</v>
       </c>
       <c r="I35" t="n">
         <v>14</v>
@@ -2024,7 +2019,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>casanchez@jgb.com.co</t>
+          <t>liliana.patino@quironsalud.com</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2035,9 +2030,14 @@
       <c r="C36" t="n">
         <v>0</v>
       </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>CLINICA IMBANACO</t>
+        </is>
+      </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Oportunidad de JGB S.A.</t>
+          <t>Oportunidad de Liliana Patiño Flórez</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -2046,7 +2046,7 @@
         </is>
       </c>
       <c r="G36" s="1" t="n">
-        <v>46112.6052662037</v>
+        <v>46112.60853009259</v>
       </c>
       <c r="I36" t="n">
         <v>14</v>
@@ -2063,12 +2063,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>damaris.gomez@disfarma.com.co</t>
+          <t>casanchez@jgb.com.co</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Seguimiento</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -2076,7 +2076,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Oportunidad de DISFARMA</t>
+          <t>Oportunidad de JGB S.A.</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -2085,7 +2085,7 @@
         </is>
       </c>
       <c r="G37" s="1" t="n">
-        <v>46112.60325231482</v>
+        <v>46112.6052662037</v>
       </c>
       <c r="I37" t="n">
         <v>14</v>
@@ -2102,25 +2102,20 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>alergologosdeoccidente@gmail.com</t>
+          <t>damaris.gomez@disfarma.com.co</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Seguimiento</t>
         </is>
       </c>
       <c r="C38" t="n">
         <v>0</v>
       </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>Johana Gonzalez</t>
-        </is>
-      </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Oportunidad de Johana Gonzalez</t>
+          <t>Oportunidad de DISFARMA</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2129,10 +2124,10 @@
         </is>
       </c>
       <c r="G38" s="1" t="n">
-        <v>46107.51248842593</v>
+        <v>46112.60325231482</v>
       </c>
       <c r="I38" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J38" t="n">
         <v>2026</v>
@@ -2146,77 +2141,76 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>DavidEsteban.Porras@alfalaval.com</t>
+          <t>alergologosdeoccidente@gmail.com</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Ganado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>15000000</v>
+        <v>0</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Johana Gonzalez</t>
+        </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Oportunidad de OPORTUNIDAD ENCUESTAS ALFALAVAL</t>
+          <t>Oportunidad de Johana Gonzalez</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G39" s="1" t="n">
-        <v>46101.72893518519</v>
-      </c>
-      <c r="H39" s="1" t="n">
-        <v>46141</v>
+        <v>46107.51248842593</v>
       </c>
       <c r="I39" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J39" t="n">
         <v>2026</v>
       </c>
-      <c r="K39" t="n">
-        <v>4</v>
-      </c>
-      <c r="L39" t="n">
-        <v>2026</v>
-      </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Dr.arcarmona@gmail.com</t>
+          <t>DavidEsteban.Porras@alfalaval.com</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Ganado</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>0</v>
+        <v>15000000</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Oportunidad de GAMANUCLEAR LTDA - Dr Alberto Carmona</t>
+          <t>Oportunidad de OPORTUNIDAD ENCUESTAS ALFALAVAL</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G40" s="1" t="n">
-        <v>46098.65114583333</v>
+        <v>46101.72893518519</v>
+      </c>
+      <c r="H40" s="1" t="n">
+        <v>46141</v>
       </c>
       <c r="I40" t="n">
         <v>12</v>
@@ -2224,16 +2218,22 @@
       <c r="J40" t="n">
         <v>2026</v>
       </c>
+      <c r="K40" t="n">
+        <v>4</v>
+      </c>
+      <c r="L40" t="n">
+        <v>2026</v>
+      </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>cecilia.guevara@cosmitet.net / administracion.crd@cosmitet.net</t>
+          <t>Dr.arcarmona@gmail.com</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2244,14 +2244,9 @@
       <c r="C41" t="n">
         <v>0</v>
       </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>Cecilia Guevara</t>
-        </is>
-      </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Oportunidad de CLINICA REY DAVID Walter Charria</t>
+          <t>Oportunidad de GAMANUCLEAR LTDA - Dr Alberto Carmona</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2260,10 +2255,10 @@
         </is>
       </c>
       <c r="G41" s="1" t="n">
-        <v>46094.69002314815</v>
+        <v>46098.65114583333</v>
       </c>
       <c r="I41" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J41" t="n">
         <v>2026</v>
@@ -2277,7 +2272,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>vicerrectoriacademica@unicatolica.edu.co</t>
+          <t>cecilia.guevara@cosmitet.net / administracion.crd@cosmitet.net</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2290,12 +2285,12 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Jorge Silva</t>
+          <t>Cecilia Guevara</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Oportunidad de Jorge Silva</t>
+          <t>Oportunidad de CLINICA REY DAVID Walter Charria</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -2304,7 +2299,7 @@
         </is>
       </c>
       <c r="G42" s="1" t="n">
-        <v>46094.66880787037</v>
+        <v>46094.69002314815</v>
       </c>
       <c r="I42" t="n">
         <v>11</v>
@@ -2321,37 +2316,34 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>pedroperea02@gmail.com</t>
+          <t>vicerrectoriacademica@unicatolica.edu.co</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Ganado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>2160000</v>
+        <v>0</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Pedro Pablo Perea Mafla</t>
+          <t>Jorge Silva</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Oportunidad de Encuestas</t>
+          <t>Oportunidad de Jorge Silva</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G43" s="1" t="n">
-        <v>46094.65905092593</v>
-      </c>
-      <c r="H43" s="1" t="n">
-        <v>46141</v>
+        <v>46094.66880787037</v>
       </c>
       <c r="I43" t="n">
         <v>11</v>
@@ -2359,35 +2351,34 @@
       <c r="J43" t="n">
         <v>2026</v>
       </c>
-      <c r="K43" t="n">
-        <v>4</v>
-      </c>
-      <c r="L43" t="n">
-        <v>2026</v>
-      </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>cristina.papamija@bmm.com.co</t>
+          <t>pedroperea02@gmail.com</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Ganado</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>8071000</v>
+        <v>2160000</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Pedro Pablo Perea Mafla</t>
+        </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Oportunidad de BANCO MUNDO MUJER</t>
+          <t>Oportunidad de Encuestas</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -2396,7 +2387,10 @@
         </is>
       </c>
       <c r="G44" s="1" t="n">
-        <v>46094.65019675926</v>
+        <v>46094.65905092593</v>
+      </c>
+      <c r="H44" s="1" t="n">
+        <v>46141</v>
       </c>
       <c r="I44" t="n">
         <v>11</v>
@@ -2404,16 +2398,22 @@
       <c r="J44" t="n">
         <v>2026</v>
       </c>
+      <c r="K44" t="n">
+        <v>4</v>
+      </c>
+      <c r="L44" t="n">
+        <v>2026</v>
+      </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>capacitacionvirtual@fundacionwwbcol.org</t>
+          <t>cristina.papamija@bmm.com.co</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2422,11 +2422,11 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>1600000</v>
+        <v>8071000</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Licenciamiento y ajuste WhatsApp FUNDACIÓN WWB</t>
+          <t>Oportunidad de BANCO MUNDO MUJER</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -2435,7 +2435,7 @@
         </is>
       </c>
       <c r="G45" s="1" t="n">
-        <v>46094.64826388889</v>
+        <v>46094.65019675926</v>
       </c>
       <c r="I45" t="n">
         <v>11</v>
@@ -2452,25 +2452,20 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>carol.cuesta@cbolivar.com</t>
+          <t>capacitacionvirtual@fundacionwwbcol.org</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Ganado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>2900000</v>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>CAROL CUESTA</t>
-        </is>
+        <v>1600000</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Gestión de Subsidios CB Bogotá</t>
+          <t>Licenciamiento y ajuste WhatsApp FUNDACIÓN WWB</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2479,10 +2474,7 @@
         </is>
       </c>
       <c r="G46" s="1" t="n">
-        <v>46094.64454861111</v>
-      </c>
-      <c r="H46" s="1" t="n">
-        <v>46135</v>
+        <v>46094.64826388889</v>
       </c>
       <c r="I46" t="n">
         <v>11</v>
@@ -2490,44 +2482,46 @@
       <c r="J46" t="n">
         <v>2026</v>
       </c>
-      <c r="K46" t="n">
-        <v>4</v>
-      </c>
-      <c r="L46" t="n">
-        <v>2026</v>
-      </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>edwin.munoz.v@uniminuto.edu</t>
+          <t>carol.cuesta@cbolivar.com</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Ganado</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>0</v>
+        <v>2900000</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>CAROL CUESTA</t>
+        </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Oportunidad de UNIMINUTO</t>
+          <t>Gestión de Subsidios CB Bogotá</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G47" s="1" t="n">
-        <v>46092.63626157407</v>
+        <v>46094.64454861111</v>
+      </c>
+      <c r="H47" s="1" t="n">
+        <v>46135</v>
       </c>
       <c r="I47" t="n">
         <v>11</v>
@@ -2535,16 +2529,22 @@
       <c r="J47" t="n">
         <v>2026</v>
       </c>
+      <c r="K47" t="n">
+        <v>4</v>
+      </c>
+      <c r="L47" t="n">
+        <v>2026</v>
+      </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>jaime_zuluaga@eficacia.com.co</t>
+          <t>edwin.munoz.v@uniminuto.edu</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2555,14 +2555,9 @@
       <c r="C48" t="n">
         <v>0</v>
       </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>Jaime Alberto</t>
-        </is>
-      </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Oportunidad de Jaime Alberto Zuluaga</t>
+          <t>Oportunidad de UNIMINUTO</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2571,7 +2566,7 @@
         </is>
       </c>
       <c r="G48" s="1" t="n">
-        <v>46092.63153935185</v>
+        <v>46092.63626157407</v>
       </c>
       <c r="I48" t="n">
         <v>11</v>
@@ -2588,7 +2583,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>comercial@isyscol.com</t>
+          <t>jaime_zuluaga@eficacia.com.co</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2601,12 +2596,12 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Andres Nader</t>
+          <t>Jaime Alberto</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Oportunidad de Andres Nader</t>
+          <t>Oportunidad de Jaime Alberto Zuluaga</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -2615,7 +2610,7 @@
         </is>
       </c>
       <c r="G49" s="1" t="n">
-        <v>46091.59211805555</v>
+        <v>46092.63153935185</v>
       </c>
       <c r="I49" t="n">
         <v>11</v>
@@ -2632,7 +2627,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>mercadeo@norteysur.co</t>
+          <t>comercial@isyscol.com</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2645,12 +2640,12 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Isabella Mesa</t>
+          <t>Andres Nader</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Oportunidad de Isabella Mesa</t>
+          <t>Oportunidad de Andres Nader</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -2659,7 +2654,7 @@
         </is>
       </c>
       <c r="G50" s="1" t="n">
-        <v>46091.40078703704</v>
+        <v>46091.59211805555</v>
       </c>
       <c r="I50" t="n">
         <v>11</v>
@@ -2674,26 +2669,36 @@
       </c>
     </row>
     <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>mercadeo@norteysur.co</t>
+        </is>
+      </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Seguimiento</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C51" t="n">
         <v>0</v>
       </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Isabella Mesa</t>
+        </is>
+      </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Clasificación EMAIL Comfenalco Cartagena</t>
+          <t>Oportunidad de Isabella Mesa</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Maria Fernanda Gaviria</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G51" s="1" t="n">
-        <v>46091.3665625</v>
+        <v>46091.40078703704</v>
       </c>
       <c r="I51" t="n">
         <v>11</v>
@@ -2710,7 +2715,7 @@
     <row r="52">
       <c r="B52" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Seguimiento</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -2718,19 +2723,19 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Oportunidad de ESE HOSPITAL LA MARIA</t>
+          <t>Clasificación EMAIL Comfenalco Cartagena</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Laura Alejandra Castañeda</t>
+          <t>Maria Fernanda Gaviria</t>
         </is>
       </c>
       <c r="G52" s="1" t="n">
-        <v>46083.67605324074</v>
+        <v>46091.3665625</v>
       </c>
       <c r="I52" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J52" t="n">
         <v>2026</v>
@@ -2752,7 +2757,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Oportunidad de SUPER TRANSPORTE</t>
+          <t>Oportunidad de ESE HOSPITAL LA MARIA</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -2761,7 +2766,7 @@
         </is>
       </c>
       <c r="G53" s="1" t="n">
-        <v>46083.6706712963</v>
+        <v>46083.67605324074</v>
       </c>
       <c r="I53" t="n">
         <v>10</v>
@@ -2786,7 +2791,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Oportunidad de ENLACES IP S.A.S</t>
+          <t>Oportunidad de SUPER TRANSPORTE</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -2795,7 +2800,7 @@
         </is>
       </c>
       <c r="G54" s="1" t="n">
-        <v>46083.50145833333</v>
+        <v>46083.6706712963</v>
       </c>
       <c r="I54" t="n">
         <v>10</v>
@@ -2810,11 +2815,6 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>accounting@diaza.com</t>
-        </is>
-      </c>
       <c r="B55" t="inlineStr">
         <is>
           <t>Perdido</t>
@@ -2823,26 +2823,21 @@
       <c r="C55" t="n">
         <v>0</v>
       </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>JOHANA RODRIGUEZ</t>
-        </is>
-      </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Oportunidad de JOHANA RODRIGUEZ</t>
+          <t>Oportunidad de ENLACES IP S.A.S</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Laura Alejandra Castañeda</t>
         </is>
       </c>
       <c r="G55" s="1" t="n">
-        <v>46079.73486111111</v>
+        <v>46083.50145833333</v>
       </c>
       <c r="I55" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J55" t="n">
         <v>2026</v>
@@ -2856,7 +2851,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>mensajeriamyr@gmail.com</t>
+          <t>accounting@diaza.com</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2867,9 +2862,14 @@
       <c r="C56" t="n">
         <v>0</v>
       </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>JOHANA RODRIGUEZ</t>
+        </is>
+      </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Oportunidad de MENSAJERIA M&amp;R SAS</t>
+          <t>Oportunidad de JOHANA RODRIGUEZ</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -2878,7 +2878,7 @@
         </is>
       </c>
       <c r="G56" s="1" t="n">
-        <v>46079.72262731481</v>
+        <v>46079.73486111111</v>
       </c>
       <c r="I56" t="n">
         <v>9</v>
@@ -2895,7 +2895,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>sistemaspanaderialeal@gmail.com</t>
+          <t>mensajeriamyr@gmail.com</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2906,14 +2906,9 @@
       <c r="C57" t="n">
         <v>0</v>
       </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>Diego Rios</t>
-        </is>
-      </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>JAMDAC SAS, Diego Rios</t>
+          <t>Oportunidad de MENSAJERIA M&amp;R SAS</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -2922,10 +2917,10 @@
         </is>
       </c>
       <c r="G57" s="1" t="n">
-        <v>46071.63706018519</v>
+        <v>46079.72262731481</v>
       </c>
       <c r="I57" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J57" t="n">
         <v>2026</v>
@@ -2939,7 +2934,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>efernandez@unico.com.co</t>
+          <t>sistemaspanaderialeal@gmail.com</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2952,12 +2947,12 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Erick Fernandez</t>
+          <t>Diego Rios</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Oportunidad de Erick Fernandez</t>
+          <t>JAMDAC SAS, Diego Rios</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -2966,10 +2961,10 @@
         </is>
       </c>
       <c r="G58" s="1" t="n">
-        <v>46064.3750462963</v>
+        <v>46071.63706018519</v>
       </c>
       <c r="I58" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J58" t="n">
         <v>2026</v>
@@ -2983,7 +2978,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>kabenitez@icesi.edu.co</t>
+          <t>efernandez@unico.com.co</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2992,28 +2987,28 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>10000000</v>
+        <v>0</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>KENI BENITEZ</t>
+          <t>Erick Fernandez</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Oportunidad de KENI BENITEZ</t>
+          <t>Oportunidad de Erick Fernandez</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G59" s="1" t="n">
-        <v>46059.34918981481</v>
+        <v>46064.3750462963</v>
       </c>
       <c r="I59" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J59" t="n">
         <v>2026</v>
@@ -3027,7 +3022,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>patovar@uao.edu.co</t>
+          <t>kabenitez@icesi.edu.co</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -3036,25 +3031,25 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>0</v>
+        <v>10000000</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Paula Tovar</t>
+          <t>KENI BENITEZ</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Oportunidad de UNIVERSIDAD AUTONOMA DE OCCIDENTE</t>
+          <t>Oportunidad de KENI BENITEZ</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G60" s="1" t="n">
-        <v>46058.72516203704</v>
+        <v>46059.34918981481</v>
       </c>
       <c r="I60" t="n">
         <v>6</v>
@@ -3071,7 +3066,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>comercial@isyscol.com</t>
+          <t>patovar@uao.edu.co</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -3082,9 +3077,14 @@
       <c r="C61" t="n">
         <v>0</v>
       </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Paula Tovar</t>
+        </is>
+      </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Oportunidad de TECNOLOGIAS ISYSCOL SAS</t>
+          <t>Oportunidad de UNIVERSIDAD AUTONOMA DE OCCIDENTE</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -3093,7 +3093,7 @@
         </is>
       </c>
       <c r="G61" s="1" t="n">
-        <v>46057.58993055556</v>
+        <v>46058.72516203704</v>
       </c>
       <c r="I61" t="n">
         <v>6</v>
@@ -3108,17 +3108,22 @@
       </c>
     </row>
     <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>comercial@isyscol.com</t>
+        </is>
+      </c>
       <c r="B62" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>15000000</v>
+        <v>0</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Oportunidad de VOICE IA EFICACIA</t>
+          <t>Oportunidad de TECNOLOGIAS ISYSCOL SAS</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -3127,7 +3132,7 @@
         </is>
       </c>
       <c r="G62" s="1" t="n">
-        <v>46057.3409837963</v>
+        <v>46057.58993055556</v>
       </c>
       <c r="I62" t="n">
         <v>6</v>
@@ -3148,23 +3153,23 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>4000000</v>
+        <v>15000000</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Oportunidad de Eficacia WhatsApp</t>
+          <t>Oportunidad de VOICE IA EFICACIA</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G63" s="1" t="n">
-        <v>46049.67292824074</v>
+        <v>46057.3409837963</v>
       </c>
       <c r="I63" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J63" t="n">
         <v>2026</v>
@@ -3182,62 +3187,57 @@
         </is>
       </c>
       <c r="C64" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Oportunidad de Eficacia WhatsApp</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Jennifer Hoyos Gallego</t>
+        </is>
+      </c>
+      <c r="G64" s="1" t="n">
+        <v>46049.67292824074</v>
+      </c>
+      <c r="I64" t="n">
+        <v>5</v>
+      </c>
+      <c r="J64" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>No calificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
         <v>20000000</v>
       </c>
-      <c r="E64" t="inlineStr">
+      <c r="E65" t="inlineStr">
         <is>
           <t>Oportunidad de CRUZ ROJA COLOMBIANA SECCIONAL VALLE DEL CAUCA</t>
         </is>
       </c>
-      <c r="F64" t="inlineStr">
+      <c r="F65" t="inlineStr">
         <is>
           <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
-      <c r="G64" s="1" t="n">
+      <c r="G65" s="1" t="n">
         <v>46006.49650462963</v>
       </c>
-      <c r="I64" t="n">
+      <c r="I65" t="n">
         <v>51</v>
-      </c>
-      <c r="J64" t="n">
-        <v>2025</v>
-      </c>
-      <c r="M64" t="inlineStr">
-        <is>
-          <t>No calificado</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>silvia.figueroa@neurithmedia.com</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C65" t="n">
-        <v>25000000</v>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>Contact center ventas España</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>Richard Castaño</t>
-        </is>
-      </c>
-      <c r="G65" s="1" t="n">
-        <v>45960.61145833333</v>
-      </c>
-      <c r="I65" t="n">
-        <v>44</v>
       </c>
       <c r="J65" t="n">
         <v>2025</v>
@@ -3249,22 +3249,22 @@
       </c>
     </row>
     <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>silvia.figueroa@neurithmedia.com</t>
+        </is>
+      </c>
       <c r="B66" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>37000000</v>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>Mabel</t>
-        </is>
+        <v>25000000</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Masivos Licitacion</t>
+          <t>Contact center ventas España</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -3273,10 +3273,10 @@
         </is>
       </c>
       <c r="G66" s="1" t="n">
-        <v>45940.49372685186</v>
+        <v>45960.61145833333</v>
       </c>
       <c r="I66" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="J66" t="n">
         <v>2025</v>
@@ -3288,36 +3288,31 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>ana.zuniga@cbolivar.com</t>
-        </is>
-      </c>
       <c r="B67" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>4997000</v>
+        <v>37000000</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Ana Lucia Zuñiga</t>
+          <t>Mabel</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Constructora Bolivar Agente Redes</t>
+          <t>Masivos Licitacion</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Richard Castaño</t>
         </is>
       </c>
       <c r="G67" s="1" t="n">
-        <v>45940.49215277778</v>
+        <v>45940.49372685186</v>
       </c>
       <c r="I67" t="n">
         <v>41</v>
@@ -3334,7 +3329,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>julian_mendez@extras.com.co</t>
+          <t>ana.zuniga@cbolivar.com</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -3343,28 +3338,28 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>15000000</v>
+        <v>4997000</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Julian Mendez.</t>
+          <t>Ana Lucia Zuñiga</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Oportunidad de EFICACIA S A S</t>
+          <t>Constructora Bolivar Agente Redes</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G68" s="1" t="n">
-        <v>45922.66201388889</v>
+        <v>45940.49215277778</v>
       </c>
       <c r="I68" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="J68" t="n">
         <v>2025</v>
@@ -3378,7 +3373,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>info@eficacia.com.co</t>
+          <t>julian_mendez@extras.com.co</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -3387,11 +3382,16 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>0</v>
+        <v>15000000</v>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Julian Mendez.</t>
+        </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Nutresa</t>
+          <t>Oportunidad de EFICACIA S A S</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -3400,7 +3400,7 @@
         </is>
       </c>
       <c r="G69" s="1" t="n">
-        <v>45922.66199074074</v>
+        <v>45922.66201388889</v>
       </c>
       <c r="I69" t="n">
         <v>39</v>
@@ -3417,37 +3417,32 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>hrodriguez@jaramillomora.com</t>
+          <t>info@eficacia.com.co</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Seguimiento</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>30000000</v>
-      </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>HANNA</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Oportunidad de JARAMILLO MORA CONSTRUCTORA S A</t>
+          <t>Nutresa</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Richard Castaño</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G70" s="1" t="n">
-        <v>45916.71618055556</v>
+        <v>45922.66199074074</v>
       </c>
       <c r="I70" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="J70" t="n">
         <v>2025</v>
@@ -3459,17 +3454,27 @@
       </c>
     </row>
     <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>hrodriguez@jaramillomora.com</t>
+        </is>
+      </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Seguimiento</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>147000000</v>
+        <v>30000000</v>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>HANNA</t>
+        </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Contact Center Agendamiento citas</t>
+          <t>Oportunidad de JARAMILLO MORA CONSTRUCTORA S A</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -3478,7 +3483,7 @@
         </is>
       </c>
       <c r="G71" s="1" t="n">
-        <v>45916.67502314815</v>
+        <v>45916.71618055556</v>
       </c>
       <c r="I71" t="n">
         <v>38</v>
@@ -3493,34 +3498,26 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>jaime_zuluaga@eficacia.com.co</t>
-        </is>
-      </c>
       <c r="B72" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>14700000</v>
+        <v>147000000</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Agentes contact center encuestas</t>
+          <t>Contact Center Agendamiento citas</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Richard Castaño</t>
         </is>
       </c>
       <c r="G72" s="1" t="n">
-        <v>45916.65275462963</v>
-      </c>
-      <c r="H72" s="1" t="n">
-        <v>45930</v>
+        <v>45916.67502314815</v>
       </c>
       <c r="I72" t="n">
         <v>38</v>
@@ -3528,12 +3525,6 @@
       <c r="J72" t="n">
         <v>2025</v>
       </c>
-      <c r="K72" t="n">
-        <v>9</v>
-      </c>
-      <c r="L72" t="n">
-        <v>2025</v>
-      </c>
       <c r="M72" t="inlineStr">
         <is>
           <t>No calificado</t>
@@ -3541,22 +3532,22 @@
       </c>
     </row>
     <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>jaime_zuluaga@eficacia.com.co</t>
+        </is>
+      </c>
       <c r="B73" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>4796000</v>
-      </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>Juan Grisales</t>
-        </is>
+        <v>14700000</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Agente Call Center Outbound</t>
+          <t>Agentes contact center encuestas</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -3565,7 +3556,10 @@
         </is>
       </c>
       <c r="G73" s="1" t="n">
-        <v>45915.4809375</v>
+        <v>45916.65275462963</v>
+      </c>
+      <c r="H73" s="1" t="n">
+        <v>45930</v>
       </c>
       <c r="I73" t="n">
         <v>38</v>
@@ -3573,6 +3567,12 @@
       <c r="J73" t="n">
         <v>2025</v>
       </c>
+      <c r="K73" t="n">
+        <v>9</v>
+      </c>
+      <c r="L73" t="n">
+        <v>2025</v>
+      </c>
       <c r="M73" t="inlineStr">
         <is>
           <t>No calificado</t>
@@ -3580,27 +3580,22 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>gestormercadeo@lamontana.co</t>
-        </is>
-      </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Seguimiento</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>25000000</v>
+        <v>4796000</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Alejandra Ossa</t>
+          <t>Juan Grisales</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Voice BOT</t>
+          <t>Agente Call Center Outbound</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -3609,10 +3604,7 @@
         </is>
       </c>
       <c r="G74" s="1" t="n">
-        <v>45915.48023148148</v>
-      </c>
-      <c r="H74" s="1" t="n">
-        <v>46150</v>
+        <v>45915.4809375</v>
       </c>
       <c r="I74" t="n">
         <v>38</v>
@@ -3620,12 +3612,6 @@
       <c r="J74" t="n">
         <v>2025</v>
       </c>
-      <c r="K74" t="n">
-        <v>5</v>
-      </c>
-      <c r="L74" t="n">
-        <v>2026</v>
-      </c>
       <c r="M74" t="inlineStr">
         <is>
           <t>No calificado</t>
@@ -3635,20 +3621,25 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>elkinmarquezconsuegra@gmail.com</t>
+          <t>gestormercadeo@lamontana.co</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Seguimiento</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>2500000</v>
+        <v>25000000</v>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Alejandra Ossa</t>
+        </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Venta Masivos</t>
+          <t>Voice BOT</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -3657,7 +3648,10 @@
         </is>
       </c>
       <c r="G75" s="1" t="n">
-        <v>45915.47924768519</v>
+        <v>45915.48023148148</v>
+      </c>
+      <c r="H75" s="1" t="n">
+        <v>46150</v>
       </c>
       <c r="I75" t="n">
         <v>38</v>
@@ -3665,6 +3659,12 @@
       <c r="J75" t="n">
         <v>2025</v>
       </c>
+      <c r="K75" t="n">
+        <v>5</v>
+      </c>
+      <c r="L75" t="n">
+        <v>2026</v>
+      </c>
       <c r="M75" t="inlineStr">
         <is>
           <t>No calificado</t>
@@ -3674,7 +3674,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>bladimir.munoz@uptc.edu.co</t>
+          <t>elkinmarquezconsuegra@gmail.com</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -3683,16 +3683,11 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>22000000</v>
-      </c>
-      <c r="D76" t="inlineStr">
-        <is>
-          <t>Bladimir Muñoz Forero</t>
-        </is>
+        <v>2500000</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Oportunidad Venta BPO</t>
+          <t>Venta Masivos</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -3701,7 +3696,7 @@
         </is>
       </c>
       <c r="G76" s="1" t="n">
-        <v>45915.47494212963</v>
+        <v>45915.47924768519</v>
       </c>
       <c r="I76" t="n">
         <v>38</v>
@@ -3718,7 +3713,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>gerencia@alitasfactory.com</t>
+          <t>bladimir.munoz@uptc.edu.co</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -3727,20 +3722,25 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>40000000</v>
+        <v>22000000</v>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Bladimir Muñoz Forero</t>
+        </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>1 agente IA para ventas y asesoramiento</t>
+          <t>Oportunidad Venta BPO</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Richard Castaño</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G77" s="1" t="n">
-        <v>45915.47300925926</v>
+        <v>45915.47494212963</v>
       </c>
       <c r="I77" t="n">
         <v>38</v>
@@ -3757,7 +3757,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>mmonroy@falabella.com.co</t>
+          <t>gerencia@alitasfactory.com</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -3766,11 +3766,11 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>60000000</v>
+        <v>40000000</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Agente IA Try and Buy Inbound y Outbound</t>
+          <t>1 agente IA para ventas y asesoramiento</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -3779,7 +3779,7 @@
         </is>
       </c>
       <c r="G78" s="1" t="n">
-        <v>45915.46633101852</v>
+        <v>45915.47300925926</v>
       </c>
       <c r="I78" t="n">
         <v>38</v>
@@ -3796,7 +3796,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>gerencia@motosymotoselpaisa.com</t>
+          <t>mmonroy@falabella.com.co</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -3805,20 +3805,20 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>40000000</v>
+        <v>60000000</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Oportunidad de MOTOS Y MOTOS EL PAISA S A S</t>
+          <t>Agente IA Try and Buy Inbound y Outbound</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Richard Castaño</t>
         </is>
       </c>
       <c r="G79" s="1" t="n">
-        <v>45915.46252314815</v>
+        <v>45915.46633101852</v>
       </c>
       <c r="I79" t="n">
         <v>38</v>
@@ -3835,7 +3835,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>isanchez@unico.com.co</t>
+          <t>gerencia@motosymotoselpaisa.com</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -3844,11 +3844,11 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>0</v>
+        <v>40000000</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>1 agente IA para relacionamiento con locatarios</t>
+          <t>Oportunidad de MOTOS Y MOTOS EL PAISA S A S</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -3857,7 +3857,7 @@
         </is>
       </c>
       <c r="G80" s="1" t="n">
-        <v>45915.46157407408</v>
+        <v>45915.46252314815</v>
       </c>
       <c r="I80" t="n">
         <v>38</v>
@@ -3874,7 +3874,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>asantiago@stop.com.co</t>
+          <t>isanchez@unico.com.co</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -3883,11 +3883,11 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>30000000</v>
+        <v>0</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>1 Agente IA en cobranzas</t>
+          <t>1 agente IA para relacionamiento con locatarios</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -3896,7 +3896,7 @@
         </is>
       </c>
       <c r="G81" s="1" t="n">
-        <v>45915.46052083333</v>
+        <v>45915.46157407408</v>
       </c>
       <c r="I81" t="n">
         <v>38</v>

</xml_diff>

<commit_message>
CRM actualizado — 29/05/2026 14:43
</commit_message>
<xml_diff>
--- a/CRM_PowerBI_BrendaLuna_actualizado.xlsx
+++ b/CRM_PowerBI_BrendaLuna_actualizado.xlsx
@@ -494,7 +494,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Negociación</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -535,7 +535,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
@@ -990,7 +990,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1017,7 +1017,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
CRM actualizado — 02/06/2026 16:01
</commit_message>
<xml_diff>
--- a/CRM_PowerBI_BrendaLuna_actualizado.xlsx
+++ b/CRM_PowerBI_BrendaLuna_actualizado.xlsx
@@ -944,6 +944,11 @@
       </c>
     </row>
     <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>dgamoneda@productosdrogam.com</t>
+        </is>
+      </c>
       <c r="B11" t="inlineStr">
         <is>
           <t>Nuevo</t>
@@ -954,12 +959,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Olga Lucia Hurtado</t>
+          <t xml:space="preserve">Diego Mauricio Gamoneda </t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Oportunidad de Olga Lucia Hurtado</t>
+          <t xml:space="preserve">Oportunidad de Diego Mauricio Gamoneda </t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -968,10 +973,10 @@
         </is>
       </c>
       <c r="G11" s="1" t="n">
-        <v>46168.49854166667</v>
+        <v>46175.66417824074</v>
       </c>
       <c r="I11" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="J11" t="n">
         <v>2026</v>
@@ -985,7 +990,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>comercial2@felsyn.com</t>
+          <t>alexander.rojas@friogan.com</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -994,11 +999,11 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>713400</v>
+        <v>0</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Oportunidad de FONDO DE EMPLEADOS FELSYN</t>
+          <t>Oportunidad de FRIOGAN S.A</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1007,10 +1012,10 @@
         </is>
       </c>
       <c r="G12" s="1" t="n">
-        <v>46163.49130787037</v>
+        <v>46175.63597222222</v>
       </c>
       <c r="I12" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="J12" t="n">
         <v>2026</v>
@@ -1022,27 +1027,17 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>mercadeo@lasevillana.com.co</t>
-        </is>
-      </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C13" t="n">
         <v>0</v>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fabio AlbertoGallego García </t>
-        </is>
-      </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Oportunidad de Fabio AlbertoGallego García </t>
+          <t>Oportunidad de Agromercados la Montaña</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1051,10 +1046,10 @@
         </is>
       </c>
       <c r="G13" s="1" t="n">
-        <v>46162.64569444444</v>
+        <v>46175.62239583334</v>
       </c>
       <c r="I13" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="J13" t="n">
         <v>2026</v>
@@ -1068,7 +1063,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>asantiago@stop.com.co</t>
+          <t>juand.rios@alkosto.com.co</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1081,7 +1076,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Oportunidad de STOP SAS</t>
+          <t>Oportunidad de ALKOSTO</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1090,10 +1085,10 @@
         </is>
       </c>
       <c r="G14" s="1" t="n">
-        <v>46161.63508101852</v>
+        <v>46175.62055555556</v>
       </c>
       <c r="I14" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="J14" t="n">
         <v>2026</v>
@@ -1107,25 +1102,25 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>aestrada@teker.co</t>
+          <t>gerencia4087@grupo-exito.com</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>16914000</v>
+        <v>0</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>TEKER SALUD SAS</t>
+          <t>Grupo exito ‒ 1007386172 - Sneider Quirama</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Oportunidad de TEKER SALUD SAS</t>
+          <t>Oportunidad de Grupo exito</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1134,32 +1129,42 @@
         </is>
       </c>
       <c r="G15" s="1" t="n">
-        <v>46161.62922453704</v>
+        <v>46175.61638888889</v>
       </c>
       <c r="I15" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="J15" t="n">
         <v>2026</v>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>ldgomez@supertiendascanaveral.com</t>
+        </is>
+      </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C16" t="n">
         <v>0</v>
       </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Luis David Gomez</t>
+        </is>
+      </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Oportunidad de TIAN IPS SAS</t>
+          <t>Oportunidad de Luis David Gomez</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1168,10 +1173,10 @@
         </is>
       </c>
       <c r="G16" s="1" t="n">
-        <v>46161.61643518518</v>
+        <v>46175.60493055556</v>
       </c>
       <c r="I16" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="J16" t="n">
         <v>2026</v>
@@ -1185,25 +1190,20 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>administración@fullredtotal.com</t>
+          <t>davida_vanegas@coomeva.com.co</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>14000000</v>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Eivar Eñasco</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Oportunidad de Eivar Eñasco</t>
+          <t>Oportunidad de BANCOOMEVA</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1212,42 +1212,42 @@
         </is>
       </c>
       <c r="G17" s="1" t="n">
-        <v>46154.67546296296</v>
+        <v>46175.47109953704</v>
       </c>
       <c r="I17" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="J17" t="n">
         <v>2026</v>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>cserna@surtifamiliar.com.co</t>
+          <t>alejandro.delgado@filedesk.com.co</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Negociación</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>1950000</v>
+        <v>0</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Claudia Patricia Serna</t>
+          <t>AlejandroDelgado</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Oportunidad de Claudia Patricia Serna</t>
+          <t>Oportunidad de AlejandroDelgado</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1256,42 +1256,37 @@
         </is>
       </c>
       <c r="G18" s="1" t="n">
-        <v>46154.66616898148</v>
+        <v>46174.71665509259</v>
       </c>
       <c r="I18" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="J18" t="n">
         <v>2026</v>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>coordmercadeo@pacificcenter.co</t>
-        </is>
-      </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>5600000</v>
+        <v>0</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Claudia Castro</t>
+          <t>Olga Lucia Hurtado</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Oportunidad de Claudia Castro</t>
+          <t>Oportunidad de Olga Lucia Hurtado</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1300,42 +1295,37 @@
         </is>
       </c>
       <c r="G19" s="1" t="n">
-        <v>46154.66341435185</v>
+        <v>46168.49854166667</v>
       </c>
       <c r="I19" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="J19" t="n">
         <v>2026</v>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>isabellarengifo27@gmail.com</t>
+          <t>comercial2@felsyn.com</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>28190000</v>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Isabella Rengifo</t>
-        </is>
+        <v>713400</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Oportunidad de Isabella Rengifo</t>
+          <t>Oportunidad de FONDO DE EMPLEADOS FELSYN</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1344,10 +1334,10 @@
         </is>
       </c>
       <c r="G20" s="1" t="n">
-        <v>46154.65981481481</v>
+        <v>46163.49130787037</v>
       </c>
       <c r="I20" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J20" t="n">
         <v>2026</v>
@@ -1359,153 +1349,144 @@
       </c>
     </row>
     <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>mercadeo@lasevillana.com.co</t>
+        </is>
+      </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>50000000</v>
+        <v>0</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Paola Gómez - Agente Inmobiliaria Independiente</t>
+          <t xml:space="preserve">Fabio AlbertoGallego García </t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Puesto de Trabajo CC Medellin</t>
+          <t xml:space="preserve">Oportunidad de Fabio AlbertoGallego García </t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Richard Castaño</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G21" s="1" t="n">
-        <v>46154.49104166667</v>
-      </c>
-      <c r="H21" s="1" t="n">
-        <v>46170</v>
+        <v>46162.64569444444</v>
       </c>
       <c r="I21" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J21" t="n">
         <v>2026</v>
       </c>
-      <c r="K21" t="n">
-        <v>5</v>
-      </c>
-      <c r="L21" t="n">
-        <v>2026</v>
-      </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>alberto.ramirez@constructorabolivar.com</t>
+          <t>asantiago@stop.com.co</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
+          <t>Contactado</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Oportunidad de STOP SAS</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G22" s="1" t="n">
+        <v>46161.63508101852</v>
+      </c>
+      <c r="I22" t="n">
+        <v>21</v>
+      </c>
+      <c r="J22" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>No calificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>aestrada@teker.co</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
           <t>Propuesta</t>
         </is>
       </c>
-      <c r="C22" t="n">
-        <v>3000000</v>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>Oportunidad de NPS Relacional</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Jennifer Hoyos Gallego</t>
-        </is>
-      </c>
-      <c r="G22" s="1" t="n">
-        <v>46154.44511574074</v>
-      </c>
-      <c r="I22" t="n">
-        <v>20</v>
-      </c>
-      <c r="J22" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M22" t="inlineStr">
+      <c r="C23" t="n">
+        <v>16914000</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>TEKER SALUD SAS</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Oportunidad de TEKER SALUD SAS</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G23" s="1" t="n">
+        <v>46161.62922453704</v>
+      </c>
+      <c r="I23" t="n">
+        <v>21</v>
+      </c>
+      <c r="J23" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M23" t="inlineStr">
         <is>
           <t>Calificado</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C23" t="n">
-        <v>3000000</v>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>MADERKIT</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>Oportunidad de MADERKIT</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G23" s="1" t="n">
-        <v>46147.66540509259</v>
-      </c>
-      <c r="I23" t="n">
-        <v>19</v>
-      </c>
-      <c r="J23" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>No calificado</t>
-        </is>
-      </c>
-    </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>omer120395@gmail.com</t>
-        </is>
-      </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C24" t="n">
         <v>0</v>
       </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>Omer Peñaloza</t>
-        </is>
-      </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Oportunidad de Omer Peñaloza</t>
+          <t>Oportunidad de TIAN IPS SAS</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1514,10 +1495,10 @@
         </is>
       </c>
       <c r="G24" s="1" t="n">
-        <v>46147.66090277778</v>
+        <v>46161.61643518518</v>
       </c>
       <c r="I24" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="J24" t="n">
         <v>2026</v>
@@ -1531,20 +1512,25 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>directora.it@supermercadobelalcazar.com.co</t>
+          <t>administración@fullredtotal.com</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>6000000</v>
+        <v>14000000</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Eivar Eñasco</t>
+        </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Oportunidad de ABASTECEMOS DE OCCIDENTE</t>
+          <t>Oportunidad de Eivar Eñasco</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1553,33 +1539,24 @@
         </is>
       </c>
       <c r="G25" s="1" t="n">
-        <v>46147.64170138889</v>
-      </c>
-      <c r="H25" s="1" t="n">
-        <v>46157</v>
+        <v>46154.67546296296</v>
       </c>
       <c r="I25" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J25" t="n">
         <v>2026</v>
       </c>
-      <c r="K25" t="n">
-        <v>5</v>
-      </c>
-      <c r="L25" t="n">
-        <v>2026</v>
-      </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>oscar.molina@terrenoshouston.com</t>
+          <t>cserna@surtifamiliar.com.co</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1588,11 +1565,16 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>37623040</v>
+        <v>1950000</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Claudia Patricia Serna</t>
+        </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Oportunidad de COLONY RIDGE</t>
+          <t>Oportunidad de Claudia Patricia Serna</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1601,21 +1583,12 @@
         </is>
       </c>
       <c r="G26" s="1" t="n">
-        <v>46147.60297453704</v>
-      </c>
-      <c r="H26" s="1" t="n">
-        <v>46150</v>
+        <v>46154.66616898148</v>
       </c>
       <c r="I26" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J26" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K26" t="n">
-        <v>5</v>
-      </c>
-      <c r="L26" t="n">
         <v>2026</v>
       </c>
       <c r="M26" t="inlineStr">
@@ -1627,20 +1600,25 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>jsantacr@ccc.org.co</t>
+          <t>coordmercadeo@pacificcenter.co</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>55000000</v>
+        <v>5600000</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Claudia Castro</t>
+        </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Oportunidad de CAMARA DE COMERCIO CALI</t>
+          <t>Oportunidad de Claudia Castro</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1649,33 +1627,24 @@
         </is>
       </c>
       <c r="G27" s="1" t="n">
-        <v>46141.62370370371</v>
-      </c>
-      <c r="H27" s="1" t="n">
-        <v>46289</v>
+        <v>46154.66341435185</v>
       </c>
       <c r="I27" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="J27" t="n">
         <v>2026</v>
       </c>
-      <c r="K27" t="n">
-        <v>9</v>
-      </c>
-      <c r="L27" t="n">
-        <v>2026</v>
-      </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>exportaciones@laprovincia.com</t>
+          <t>isabellarengifo27@gmail.com</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1684,11 +1653,16 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>6000000</v>
+        <v>28190000</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Isabella Rengifo</t>
+        </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Oportunidad de PRODUCTOS LA PROVINCIA SAS</t>
+          <t>Oportunidad de Isabella Rengifo</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1697,10 +1671,10 @@
         </is>
       </c>
       <c r="G28" s="1" t="n">
-        <v>46141.62021990741</v>
+        <v>46154.65981481481</v>
       </c>
       <c r="I28" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="J28" t="n">
         <v>2026</v>
@@ -1712,104 +1686,109 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>coordinador.mercadeo@regency.com.co</t>
-        </is>
-      </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>0</v>
+        <v>50000000</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Paola Gómez - Agente Inmobiliaria Independiente</t>
+        </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Oportunidad de REGENCY TECH SAS</t>
+          <t>Puesto de Trabajo CC Medellin</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Richard Castaño</t>
         </is>
       </c>
       <c r="G29" s="1" t="n">
-        <v>46141.59664351852</v>
+        <v>46154.49104166667</v>
+      </c>
+      <c r="H29" s="1" t="n">
+        <v>46170</v>
       </c>
       <c r="I29" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="J29" t="n">
         <v>2026</v>
       </c>
+      <c r="K29" t="n">
+        <v>5</v>
+      </c>
+      <c r="L29" t="n">
+        <v>2026</v>
+      </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>alberto.ramirez@constructorabolivar.com</t>
+        </is>
+      </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>1200000</v>
+        <v>3000000</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Oportunidad de EMCALI E.I.C.E ESP</t>
+          <t>Oportunidad de NPS Relacional</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G30" s="1" t="n">
-        <v>46141.59045138889</v>
-      </c>
-      <c r="H30" s="1" t="n">
-        <v>46352</v>
+        <v>46154.44511574074</v>
       </c>
       <c r="I30" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="J30" t="n">
         <v>2026</v>
       </c>
-      <c r="K30" t="n">
-        <v>11</v>
-      </c>
-      <c r="L30" t="n">
-        <v>2026</v>
-      </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>angie_feligrana@eficacia.com.co</t>
-        </is>
-      </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Seguimiento</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>6000000</v>
+        <v>3000000</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>MADERKIT</t>
+        </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Oportunidad de Eficacia sas / Angie Feligrana</t>
+          <t>Oportunidad de MADERKIT</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1818,21 +1797,12 @@
         </is>
       </c>
       <c r="G31" s="1" t="n">
-        <v>46126.63210648148</v>
-      </c>
-      <c r="H31" s="1" t="n">
-        <v>46150</v>
+        <v>46147.66540509259</v>
       </c>
       <c r="I31" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="J31" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K31" t="n">
-        <v>5</v>
-      </c>
-      <c r="L31" t="n">
         <v>2026</v>
       </c>
       <c r="M31" t="inlineStr">
@@ -1844,7 +1814,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Estrategiadigital@zuluagaysoto.com</t>
+          <t>omer120395@gmail.com</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1857,12 +1827,12 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Maryuri Arguello</t>
+          <t>Omer Peñaloza</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Oportunidad de Maryuri Arguello</t>
+          <t>Oportunidad de Omer Peñaloza</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1871,10 +1841,10 @@
         </is>
       </c>
       <c r="G32" s="1" t="n">
-        <v>46125.71925925926</v>
+        <v>46147.66090277778</v>
       </c>
       <c r="I32" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="J32" t="n">
         <v>2026</v>
@@ -1888,73 +1858,68 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>gabrielrodriguez@arrozsupremo.com</t>
+          <t>directora.it@supermercadobelalcazar.com.co</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Ganado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>8000000</v>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>GABRIEL RODRIGUEZ</t>
-        </is>
+        <v>6000000</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Agente de Ventas</t>
+          <t>Oportunidad de ABASTECEMOS DE OCCIDENTE</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Richard Castaño</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G33" s="1" t="n">
-        <v>46119.62108796297</v>
+        <v>46147.64170138889</v>
       </c>
       <c r="H33" s="1" t="n">
-        <v>46141</v>
+        <v>46157</v>
       </c>
       <c r="I33" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="J33" t="n">
         <v>2026</v>
       </c>
       <c r="K33" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L33" t="n">
         <v>2026</v>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Belkis.jimenez@agrauto.com.co</t>
+          <t>oscar.molina@terrenoshouston.com</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Negociación</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>0</v>
+        <v>37623040</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Oportunidad de AGRICOLA AUTOMOTRIZ SAS</t>
+          <t>Oportunidad de COLONY RIDGE</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1963,37 +1928,46 @@
         </is>
       </c>
       <c r="G34" s="1" t="n">
-        <v>46119.38914351852</v>
+        <v>46147.60297453704</v>
+      </c>
+      <c r="H34" s="1" t="n">
+        <v>46150</v>
       </c>
       <c r="I34" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="J34" t="n">
         <v>2026</v>
       </c>
+      <c r="K34" t="n">
+        <v>5</v>
+      </c>
+      <c r="L34" t="n">
+        <v>2026</v>
+      </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>anyela.aponza@cotel.com.co</t>
+          <t>jsantacr@ccc.org.co</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>0</v>
+        <v>55000000</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Oportunidad de COTEL SAL</t>
+          <t>Oportunidad de CAMARA DE COMERCIO CALI</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -2002,12 +1976,21 @@
         </is>
       </c>
       <c r="G35" s="1" t="n">
-        <v>46112.61271990741</v>
+        <v>46141.62370370371</v>
+      </c>
+      <c r="H35" s="1" t="n">
+        <v>46289</v>
       </c>
       <c r="I35" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="J35" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K35" t="n">
+        <v>9</v>
+      </c>
+      <c r="L35" t="n">
         <v>2026</v>
       </c>
       <c r="M35" t="inlineStr">
@@ -2019,7 +2002,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>liliana.patino@quironsalud.com</t>
+          <t>exportaciones@laprovincia.com</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2028,16 +2011,11 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>0</v>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>CLINICA IMBANACO</t>
-        </is>
+        <v>6000000</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Oportunidad de Liliana Patiño Flórez</t>
+          <t>Oportunidad de PRODUCTOS LA PROVINCIA SAS</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -2046,10 +2024,10 @@
         </is>
       </c>
       <c r="G36" s="1" t="n">
-        <v>46112.60853009259</v>
+        <v>46141.62021990741</v>
       </c>
       <c r="I36" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="J36" t="n">
         <v>2026</v>
@@ -2063,7 +2041,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>casanchez@jgb.com.co</t>
+          <t>coordinador.mercadeo@regency.com.co</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2076,7 +2054,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Oportunidad de JGB S.A.</t>
+          <t>Oportunidad de REGENCY TECH SAS</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -2085,10 +2063,10 @@
         </is>
       </c>
       <c r="G37" s="1" t="n">
-        <v>46112.6052662037</v>
+        <v>46141.59664351852</v>
       </c>
       <c r="I37" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="J37" t="n">
         <v>2026</v>
@@ -2100,22 +2078,17 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>damaris.gomez@disfarma.com.co</t>
-        </is>
-      </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Seguimiento</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>0</v>
+        <v>1200000</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Oportunidad de DISFARMA</t>
+          <t>Oportunidad de EMCALI E.I.C.E ESP</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2124,12 +2097,21 @@
         </is>
       </c>
       <c r="G38" s="1" t="n">
-        <v>46112.60325231482</v>
+        <v>46141.59045138889</v>
+      </c>
+      <c r="H38" s="1" t="n">
+        <v>46352</v>
       </c>
       <c r="I38" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="J38" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K38" t="n">
+        <v>11</v>
+      </c>
+      <c r="L38" t="n">
         <v>2026</v>
       </c>
       <c r="M38" t="inlineStr">
@@ -2141,25 +2123,20 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>alergologosdeoccidente@gmail.com</t>
+          <t>angie_feligrana@eficacia.com.co</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Seguimiento</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>0</v>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>Johana Gonzalez</t>
-        </is>
+        <v>6000000</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Oportunidad de Johana Gonzalez</t>
+          <t>Oportunidad de Eficacia sas / Angie Feligrana</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2168,12 +2145,21 @@
         </is>
       </c>
       <c r="G39" s="1" t="n">
-        <v>46107.51248842593</v>
+        <v>46126.63210648148</v>
+      </c>
+      <c r="H39" s="1" t="n">
+        <v>46150</v>
       </c>
       <c r="I39" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="J39" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K39" t="n">
+        <v>5</v>
+      </c>
+      <c r="L39" t="n">
         <v>2026</v>
       </c>
       <c r="M39" t="inlineStr">
@@ -2185,94 +2171,104 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>DavidEsteban.Porras@alfalaval.com</t>
+          <t>Estrategiadigital@zuluagaysoto.com</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Ganado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>15000000</v>
+        <v>0</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Maryuri Arguello</t>
+        </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Oportunidad de OPORTUNIDAD ENCUESTAS ALFALAVAL</t>
+          <t>Oportunidad de Maryuri Arguello</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G40" s="1" t="n">
-        <v>46101.72893518519</v>
-      </c>
-      <c r="H40" s="1" t="n">
-        <v>46141</v>
+        <v>46125.71925925926</v>
       </c>
       <c r="I40" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="J40" t="n">
         <v>2026</v>
       </c>
-      <c r="K40" t="n">
-        <v>4</v>
-      </c>
-      <c r="L40" t="n">
-        <v>2026</v>
-      </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Dr.arcarmona@gmail.com</t>
+          <t>gabrielrodriguez@arrozsupremo.com</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Ganado</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>0</v>
+        <v>8000000</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>GABRIEL RODRIGUEZ</t>
+        </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Oportunidad de GAMANUCLEAR LTDA - Dr Alberto Carmona</t>
+          <t>Agente de Ventas</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Richard Castaño</t>
         </is>
       </c>
       <c r="G41" s="1" t="n">
-        <v>46098.65114583333</v>
+        <v>46119.62108796297</v>
+      </c>
+      <c r="H41" s="1" t="n">
+        <v>46141</v>
       </c>
       <c r="I41" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="J41" t="n">
         <v>2026</v>
       </c>
+      <c r="K41" t="n">
+        <v>4</v>
+      </c>
+      <c r="L41" t="n">
+        <v>2026</v>
+      </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>cecilia.guevara@cosmitet.net / administracion.crd@cosmitet.net</t>
+          <t>Belkis.jimenez@agrauto.com.co</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2283,14 +2279,9 @@
       <c r="C42" t="n">
         <v>0</v>
       </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>Cecilia Guevara</t>
-        </is>
-      </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Oportunidad de CLINICA REY DAVID Walter Charria</t>
+          <t>Oportunidad de AGRICOLA AUTOMOTRIZ SAS</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -2299,10 +2290,10 @@
         </is>
       </c>
       <c r="G42" s="1" t="n">
-        <v>46094.69002314815</v>
+        <v>46119.38914351852</v>
       </c>
       <c r="I42" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="J42" t="n">
         <v>2026</v>
@@ -2316,7 +2307,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>vicerrectoriacademica@unicatolica.edu.co</t>
+          <t>anyela.aponza@cotel.com.co</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2327,14 +2318,9 @@
       <c r="C43" t="n">
         <v>0</v>
       </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>Jorge Silva</t>
-        </is>
-      </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Oportunidad de Jorge Silva</t>
+          <t>Oportunidad de COTEL SAL</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2343,10 +2329,10 @@
         </is>
       </c>
       <c r="G43" s="1" t="n">
-        <v>46094.66880787037</v>
+        <v>46112.61271990741</v>
       </c>
       <c r="I43" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="J43" t="n">
         <v>2026</v>
@@ -2360,60 +2346,51 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>pedroperea02@gmail.com</t>
+          <t>liliana.patino@quironsalud.com</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Ganado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>2160000</v>
+        <v>0</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Pedro Pablo Perea Mafla</t>
+          <t>CLINICA IMBANACO</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Oportunidad de Encuestas</t>
+          <t>Oportunidad de Liliana Patiño Flórez</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G44" s="1" t="n">
-        <v>46094.65905092593</v>
-      </c>
-      <c r="H44" s="1" t="n">
-        <v>46141</v>
+        <v>46112.60853009259</v>
       </c>
       <c r="I44" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="J44" t="n">
         <v>2026</v>
       </c>
-      <c r="K44" t="n">
-        <v>4</v>
-      </c>
-      <c r="L44" t="n">
-        <v>2026</v>
-      </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>cristina.papamija@bmm.com.co</t>
+          <t>casanchez@jgb.com.co</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2422,23 +2399,23 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>8071000</v>
+        <v>0</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Oportunidad de BANCO MUNDO MUJER</t>
+          <t>Oportunidad de JGB S.A.</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G45" s="1" t="n">
-        <v>46094.65019675926</v>
+        <v>46112.6052662037</v>
       </c>
       <c r="I45" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="J45" t="n">
         <v>2026</v>
@@ -2452,32 +2429,32 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>capacitacionvirtual@fundacionwwbcol.org</t>
+          <t>damaris.gomez@disfarma.com.co</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Seguimiento</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>1600000</v>
+        <v>0</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Licenciamiento y ajuste WhatsApp FUNDACIÓN WWB</t>
+          <t>Oportunidad de DISFARMA</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G46" s="1" t="n">
-        <v>46094.64826388889</v>
+        <v>46112.60325231482</v>
       </c>
       <c r="I46" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="J46" t="n">
         <v>2026</v>
@@ -2491,99 +2468,99 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>carol.cuesta@cbolivar.com</t>
+          <t>alergologosdeoccidente@gmail.com</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Ganado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>2900000</v>
+        <v>0</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>CAROL CUESTA</t>
+          <t>Johana Gonzalez</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Gestión de Subsidios CB Bogotá</t>
+          <t>Oportunidad de Johana Gonzalez</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G47" s="1" t="n">
-        <v>46094.64454861111</v>
-      </c>
-      <c r="H47" s="1" t="n">
-        <v>46135</v>
+        <v>46107.51248842593</v>
       </c>
       <c r="I47" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="J47" t="n">
         <v>2026</v>
       </c>
-      <c r="K47" t="n">
-        <v>4</v>
-      </c>
-      <c r="L47" t="n">
-        <v>2026</v>
-      </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>edwin.munoz.v@uniminuto.edu</t>
+          <t>DavidEsteban.Porras@alfalaval.com</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Ganado</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>0</v>
+        <v>15000000</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Oportunidad de UNIMINUTO</t>
+          <t>Oportunidad de OPORTUNIDAD ENCUESTAS ALFALAVAL</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G48" s="1" t="n">
-        <v>46092.63626157407</v>
+        <v>46101.72893518519</v>
+      </c>
+      <c r="H48" s="1" t="n">
+        <v>46141</v>
       </c>
       <c r="I48" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J48" t="n">
         <v>2026</v>
       </c>
+      <c r="K48" t="n">
+        <v>4</v>
+      </c>
+      <c r="L48" t="n">
+        <v>2026</v>
+      </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>jaime_zuluaga@eficacia.com.co</t>
+          <t>Dr.arcarmona@gmail.com</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2594,14 +2571,9 @@
       <c r="C49" t="n">
         <v>0</v>
       </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>Jaime Alberto</t>
-        </is>
-      </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Oportunidad de Jaime Alberto Zuluaga</t>
+          <t>Oportunidad de GAMANUCLEAR LTDA - Dr Alberto Carmona</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -2610,10 +2582,10 @@
         </is>
       </c>
       <c r="G49" s="1" t="n">
-        <v>46092.63153935185</v>
+        <v>46098.65114583333</v>
       </c>
       <c r="I49" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J49" t="n">
         <v>2026</v>
@@ -2627,7 +2599,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>comercial@isyscol.com</t>
+          <t>cecilia.guevara@cosmitet.net / administracion.crd@cosmitet.net</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2640,12 +2612,12 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Andres Nader</t>
+          <t>Cecilia Guevara</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Oportunidad de Andres Nader</t>
+          <t>Oportunidad de CLINICA REY DAVID Walter Charria</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -2654,7 +2626,7 @@
         </is>
       </c>
       <c r="G50" s="1" t="n">
-        <v>46091.59211805555</v>
+        <v>46094.69002314815</v>
       </c>
       <c r="I50" t="n">
         <v>11</v>
@@ -2671,7 +2643,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>mercadeo@norteysur.co</t>
+          <t>vicerrectoriacademica@unicatolica.edu.co</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2684,12 +2656,12 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Isabella Mesa</t>
+          <t>Jorge Silva</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Oportunidad de Isabella Mesa</t>
+          <t>Oportunidad de Jorge Silva</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -2698,7 +2670,7 @@
         </is>
       </c>
       <c r="G51" s="1" t="n">
-        <v>46091.40078703704</v>
+        <v>46094.66880787037</v>
       </c>
       <c r="I51" t="n">
         <v>11</v>
@@ -2713,26 +2685,39 @@
       </c>
     </row>
     <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>pedroperea02@gmail.com</t>
+        </is>
+      </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Seguimiento</t>
+          <t>Ganado</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>0</v>
+        <v>2160000</v>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Pedro Pablo Perea Mafla</t>
+        </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Clasificación EMAIL Comfenalco Cartagena</t>
+          <t>Oportunidad de Encuestas</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Maria Fernanda Gaviria</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G52" s="1" t="n">
-        <v>46091.3665625</v>
+        <v>46094.65905092593</v>
+      </c>
+      <c r="H52" s="1" t="n">
+        <v>46141</v>
       </c>
       <c r="I52" t="n">
         <v>11</v>
@@ -2740,36 +2725,47 @@
       <c r="J52" t="n">
         <v>2026</v>
       </c>
+      <c r="K52" t="n">
+        <v>4</v>
+      </c>
+      <c r="L52" t="n">
+        <v>2026</v>
+      </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>cristina.papamija@bmm.com.co</t>
+        </is>
+      </c>
       <c r="B53" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>0</v>
+        <v>8071000</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Oportunidad de ESE HOSPITAL LA MARIA</t>
+          <t>Oportunidad de BANCO MUNDO MUJER</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Laura Alejandra Castañeda</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G53" s="1" t="n">
-        <v>46083.67605324074</v>
+        <v>46094.65019675926</v>
       </c>
       <c r="I53" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J53" t="n">
         <v>2026</v>
@@ -2781,29 +2777,34 @@
       </c>
     </row>
     <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>capacitacionvirtual@fundacionwwbcol.org</t>
+        </is>
+      </c>
       <c r="B54" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>0</v>
+        <v>1600000</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Oportunidad de SUPER TRANSPORTE</t>
+          <t>Licenciamiento y ajuste WhatsApp FUNDACIÓN WWB</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Laura Alejandra Castañeda</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G54" s="1" t="n">
-        <v>46083.6706712963</v>
+        <v>46094.64826388889</v>
       </c>
       <c r="I54" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J54" t="n">
         <v>2026</v>
@@ -2815,43 +2816,62 @@
       </c>
     </row>
     <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>carol.cuesta@cbolivar.com</t>
+        </is>
+      </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Ganado</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>0</v>
+        <v>2900000</v>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>CAROL CUESTA</t>
+        </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Oportunidad de ENLACES IP S.A.S</t>
+          <t>Gestión de Subsidios CB Bogotá</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Laura Alejandra Castañeda</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G55" s="1" t="n">
-        <v>46083.50145833333</v>
+        <v>46094.64454861111</v>
+      </c>
+      <c r="H55" s="1" t="n">
+        <v>46135</v>
       </c>
       <c r="I55" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J55" t="n">
         <v>2026</v>
       </c>
+      <c r="K55" t="n">
+        <v>4</v>
+      </c>
+      <c r="L55" t="n">
+        <v>2026</v>
+      </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>accounting@diaza.com</t>
+          <t>edwin.munoz.v@uniminuto.edu</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2862,14 +2882,9 @@
       <c r="C56" t="n">
         <v>0</v>
       </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>JOHANA RODRIGUEZ</t>
-        </is>
-      </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Oportunidad de JOHANA RODRIGUEZ</t>
+          <t>Oportunidad de UNIMINUTO</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -2878,10 +2893,10 @@
         </is>
       </c>
       <c r="G56" s="1" t="n">
-        <v>46079.73486111111</v>
+        <v>46092.63626157407</v>
       </c>
       <c r="I56" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="J56" t="n">
         <v>2026</v>
@@ -2895,7 +2910,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>mensajeriamyr@gmail.com</t>
+          <t>jaime_zuluaga@eficacia.com.co</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2906,9 +2921,14 @@
       <c r="C57" t="n">
         <v>0</v>
       </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Jaime Alberto</t>
+        </is>
+      </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Oportunidad de MENSAJERIA M&amp;R SAS</t>
+          <t>Oportunidad de Jaime Alberto Zuluaga</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -2917,10 +2937,10 @@
         </is>
       </c>
       <c r="G57" s="1" t="n">
-        <v>46079.72262731481</v>
+        <v>46092.63153935185</v>
       </c>
       <c r="I57" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="J57" t="n">
         <v>2026</v>
@@ -2934,7 +2954,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>sistemaspanaderialeal@gmail.com</t>
+          <t>comercial@isyscol.com</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2947,12 +2967,12 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Diego Rios</t>
+          <t>Andres Nader</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>JAMDAC SAS, Diego Rios</t>
+          <t>Oportunidad de Andres Nader</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -2961,10 +2981,10 @@
         </is>
       </c>
       <c r="G58" s="1" t="n">
-        <v>46071.63706018519</v>
+        <v>46091.59211805555</v>
       </c>
       <c r="I58" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="J58" t="n">
         <v>2026</v>
@@ -2978,7 +2998,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>efernandez@unico.com.co</t>
+          <t>mercadeo@norteysur.co</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2991,12 +3011,12 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Erick Fernandez</t>
+          <t>Isabella Mesa</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Oportunidad de Erick Fernandez</t>
+          <t>Oportunidad de Isabella Mesa</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -3005,10 +3025,10 @@
         </is>
       </c>
       <c r="G59" s="1" t="n">
-        <v>46064.3750462963</v>
+        <v>46091.40078703704</v>
       </c>
       <c r="I59" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="J59" t="n">
         <v>2026</v>
@@ -3020,39 +3040,29 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>kabenitez@icesi.edu.co</t>
-        </is>
-      </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Seguimiento</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>10000000</v>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>KENI BENITEZ</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Oportunidad de KENI BENITEZ</t>
+          <t>Clasificación EMAIL Comfenalco Cartagena</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Maria Fernanda Gaviria</t>
         </is>
       </c>
       <c r="G60" s="1" t="n">
-        <v>46059.34918981481</v>
+        <v>46091.3665625</v>
       </c>
       <c r="I60" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="J60" t="n">
         <v>2026</v>
@@ -3064,11 +3074,6 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>patovar@uao.edu.co</t>
-        </is>
-      </c>
       <c r="B61" t="inlineStr">
         <is>
           <t>Perdido</t>
@@ -3077,26 +3082,21 @@
       <c r="C61" t="n">
         <v>0</v>
       </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>Paula Tovar</t>
-        </is>
-      </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Oportunidad de UNIVERSIDAD AUTONOMA DE OCCIDENTE</t>
+          <t>Oportunidad de ESE HOSPITAL LA MARIA</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Laura Alejandra Castañeda</t>
         </is>
       </c>
       <c r="G61" s="1" t="n">
-        <v>46058.72516203704</v>
+        <v>46083.67605324074</v>
       </c>
       <c r="I61" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="J61" t="n">
         <v>2026</v>
@@ -3108,11 +3108,6 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>comercial@isyscol.com</t>
-        </is>
-      </c>
       <c r="B62" t="inlineStr">
         <is>
           <t>Perdido</t>
@@ -3123,19 +3118,19 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Oportunidad de TECNOLOGIAS ISYSCOL SAS</t>
+          <t>Oportunidad de SUPER TRANSPORTE</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Laura Alejandra Castañeda</t>
         </is>
       </c>
       <c r="G62" s="1" t="n">
-        <v>46057.58993055556</v>
+        <v>46083.6706712963</v>
       </c>
       <c r="I62" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="J62" t="n">
         <v>2026</v>
@@ -3153,23 +3148,23 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>15000000</v>
+        <v>0</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Oportunidad de VOICE IA EFICACIA</t>
+          <t>Oportunidad de ENLACES IP S.A.S</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Laura Alejandra Castañeda</t>
         </is>
       </c>
       <c r="G63" s="1" t="n">
-        <v>46057.3409837963</v>
+        <v>46083.50145833333</v>
       </c>
       <c r="I63" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="J63" t="n">
         <v>2026</v>
@@ -3181,29 +3176,39 @@
       </c>
     </row>
     <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>accounting@diaza.com</t>
+        </is>
+      </c>
       <c r="B64" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>4000000</v>
+        <v>0</v>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>JOHANA RODRIGUEZ</t>
+        </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Oportunidad de Eficacia WhatsApp</t>
+          <t>Oportunidad de JOHANA RODRIGUEZ</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G64" s="1" t="n">
-        <v>46049.67292824074</v>
+        <v>46079.73486111111</v>
       </c>
       <c r="I64" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="J64" t="n">
         <v>2026</v>
@@ -3215,32 +3220,37 @@
       </c>
     </row>
     <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>mensajeriamyr@gmail.com</t>
+        </is>
+      </c>
       <c r="B65" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>20000000</v>
+        <v>0</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Oportunidad de CRUZ ROJA COLOMBIANA SECCIONAL VALLE DEL CAUCA</t>
+          <t>Oportunidad de MENSAJERIA M&amp;R SAS</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G65" s="1" t="n">
-        <v>46006.49650462963</v>
+        <v>46079.72262731481</v>
       </c>
       <c r="I65" t="n">
-        <v>51</v>
+        <v>9</v>
       </c>
       <c r="J65" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="M65" t="inlineStr">
         <is>
@@ -3251,7 +3261,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>silvia.figueroa@neurithmedia.com</t>
+          <t>sistemaspanaderialeal@gmail.com</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -3260,26 +3270,31 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>25000000</v>
+        <v>0</v>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Diego Rios</t>
+        </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Contact center ventas España</t>
+          <t>JAMDAC SAS, Diego Rios</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Richard Castaño</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G66" s="1" t="n">
-        <v>45960.61145833333</v>
+        <v>46071.63706018519</v>
       </c>
       <c r="I66" t="n">
-        <v>44</v>
+        <v>8</v>
       </c>
       <c r="J66" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="M66" t="inlineStr">
         <is>
@@ -3288,37 +3303,42 @@
       </c>
     </row>
     <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>efernandez@unico.com.co</t>
+        </is>
+      </c>
       <c r="B67" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>37000000</v>
+        <v>0</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Mabel</t>
+          <t>Erick Fernandez</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Masivos Licitacion</t>
+          <t>Oportunidad de Erick Fernandez</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Richard Castaño</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G67" s="1" t="n">
-        <v>45940.49372685186</v>
+        <v>46064.3750462963</v>
       </c>
       <c r="I67" t="n">
-        <v>41</v>
+        <v>7</v>
       </c>
       <c r="J67" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="M67" t="inlineStr">
         <is>
@@ -3329,7 +3349,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>ana.zuniga@cbolivar.com</t>
+          <t>kabenitez@icesi.edu.co</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -3338,16 +3358,16 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>4997000</v>
+        <v>10000000</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Ana Lucia Zuñiga</t>
+          <t>KENI BENITEZ</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Constructora Bolivar Agente Redes</t>
+          <t>Oportunidad de KENI BENITEZ</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -3356,13 +3376,13 @@
         </is>
       </c>
       <c r="G68" s="1" t="n">
-        <v>45940.49215277778</v>
+        <v>46059.34918981481</v>
       </c>
       <c r="I68" t="n">
-        <v>41</v>
+        <v>6</v>
       </c>
       <c r="J68" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="M68" t="inlineStr">
         <is>
@@ -3373,7 +3393,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>julian_mendez@extras.com.co</t>
+          <t>patovar@uao.edu.co</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -3382,16 +3402,16 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>15000000</v>
+        <v>0</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Julian Mendez.</t>
+          <t>Paula Tovar</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Oportunidad de EFICACIA S A S</t>
+          <t>Oportunidad de UNIVERSIDAD AUTONOMA DE OCCIDENTE</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -3400,13 +3420,13 @@
         </is>
       </c>
       <c r="G69" s="1" t="n">
-        <v>45922.66201388889</v>
+        <v>46058.72516203704</v>
       </c>
       <c r="I69" t="n">
-        <v>39</v>
+        <v>6</v>
       </c>
       <c r="J69" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="M69" t="inlineStr">
         <is>
@@ -3417,7 +3437,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>info@eficacia.com.co</t>
+          <t>comercial@isyscol.com</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -3430,7 +3450,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Nutresa</t>
+          <t>Oportunidad de TECNOLOGIAS ISYSCOL SAS</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -3439,13 +3459,13 @@
         </is>
       </c>
       <c r="G70" s="1" t="n">
-        <v>45922.66199074074</v>
+        <v>46057.58993055556</v>
       </c>
       <c r="I70" t="n">
-        <v>39</v>
+        <v>6</v>
       </c>
       <c r="J70" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="M70" t="inlineStr">
         <is>
@@ -3454,42 +3474,32 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>hrodriguez@jaramillomora.com</t>
-        </is>
-      </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Seguimiento</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>30000000</v>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>HANNA</t>
-        </is>
+        <v>15000000</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Oportunidad de JARAMILLO MORA CONSTRUCTORA S A</t>
+          <t>Oportunidad de VOICE IA EFICACIA</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Richard Castaño</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G71" s="1" t="n">
-        <v>45916.71618055556</v>
+        <v>46057.3409837963</v>
       </c>
       <c r="I71" t="n">
-        <v>38</v>
+        <v>6</v>
       </c>
       <c r="J71" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="M71" t="inlineStr">
         <is>
@@ -3504,26 +3514,26 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>147000000</v>
+        <v>4000000</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Contact Center Agendamiento citas</t>
+          <t>Oportunidad de Eficacia WhatsApp</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Richard Castaño</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G72" s="1" t="n">
-        <v>45916.67502314815</v>
+        <v>46049.67292824074</v>
       </c>
       <c r="I72" t="n">
-        <v>38</v>
+        <v>5</v>
       </c>
       <c r="J72" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="M72" t="inlineStr">
         <is>
@@ -3532,47 +3542,33 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>jaime_zuluaga@eficacia.com.co</t>
-        </is>
-      </c>
       <c r="B73" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>14700000</v>
+        <v>20000000</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Agentes contact center encuestas</t>
+          <t>Oportunidad de CRUZ ROJA COLOMBIANA SECCIONAL VALLE DEL CAUCA</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G73" s="1" t="n">
-        <v>45916.65275462963</v>
-      </c>
-      <c r="H73" s="1" t="n">
-        <v>45930</v>
+        <v>46006.49650462963</v>
       </c>
       <c r="I73" t="n">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="J73" t="n">
         <v>2025</v>
       </c>
-      <c r="K73" t="n">
-        <v>9</v>
-      </c>
-      <c r="L73" t="n">
-        <v>2025</v>
-      </c>
       <c r="M73" t="inlineStr">
         <is>
           <t>No calificado</t>
@@ -3580,34 +3576,34 @@
       </c>
     </row>
     <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>silvia.figueroa@neurithmedia.com</t>
+        </is>
+      </c>
       <c r="B74" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>4796000</v>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>Juan Grisales</t>
-        </is>
+        <v>25000000</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Agente Call Center Outbound</t>
+          <t>Contact center ventas España</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Richard Castaño</t>
         </is>
       </c>
       <c r="G74" s="1" t="n">
-        <v>45915.4809375</v>
+        <v>45960.61145833333</v>
       </c>
       <c r="I74" t="n">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="J74" t="n">
         <v>2025</v>
@@ -3619,52 +3615,38 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>gestormercadeo@lamontana.co</t>
-        </is>
-      </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Seguimiento</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>25000000</v>
+        <v>37000000</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Alejandra Ossa</t>
+          <t>Mabel</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Voice BOT</t>
+          <t>Masivos Licitacion</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Richard Castaño</t>
         </is>
       </c>
       <c r="G75" s="1" t="n">
-        <v>45915.48023148148</v>
-      </c>
-      <c r="H75" s="1" t="n">
-        <v>46150</v>
+        <v>45940.49372685186</v>
       </c>
       <c r="I75" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="J75" t="n">
         <v>2025</v>
       </c>
-      <c r="K75" t="n">
-        <v>5</v>
-      </c>
-      <c r="L75" t="n">
-        <v>2026</v>
-      </c>
       <c r="M75" t="inlineStr">
         <is>
           <t>No calificado</t>
@@ -3674,7 +3656,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>elkinmarquezconsuegra@gmail.com</t>
+          <t>ana.zuniga@cbolivar.com</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -3683,23 +3665,28 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>2500000</v>
+        <v>4997000</v>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Ana Lucia Zuñiga</t>
+        </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Venta Masivos</t>
+          <t>Constructora Bolivar Agente Redes</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G76" s="1" t="n">
-        <v>45915.47924768519</v>
+        <v>45940.49215277778</v>
       </c>
       <c r="I76" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="J76" t="n">
         <v>2025</v>
@@ -3713,7 +3700,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>bladimir.munoz@uptc.edu.co</t>
+          <t>julian_mendez@extras.com.co</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -3722,16 +3709,16 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>22000000</v>
+        <v>15000000</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Bladimir Muñoz Forero</t>
+          <t>Julian Mendez.</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Oportunidad Venta BPO</t>
+          <t>Oportunidad de EFICACIA S A S</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -3740,10 +3727,10 @@
         </is>
       </c>
       <c r="G77" s="1" t="n">
-        <v>45915.47494212963</v>
+        <v>45922.66201388889</v>
       </c>
       <c r="I77" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="J77" t="n">
         <v>2025</v>
@@ -3757,7 +3744,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>gerencia@alitasfactory.com</t>
+          <t>info@eficacia.com.co</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -3766,23 +3753,23 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>40000000</v>
+        <v>0</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>1 agente IA para ventas y asesoramiento</t>
+          <t>Nutresa</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Richard Castaño</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G78" s="1" t="n">
-        <v>45915.47300925926</v>
+        <v>45922.66199074074</v>
       </c>
       <c r="I78" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="J78" t="n">
         <v>2025</v>
@@ -3796,20 +3783,25 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>mmonroy@falabella.com.co</t>
+          <t>hrodriguez@jaramillomora.com</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Seguimiento</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>60000000</v>
+        <v>30000000</v>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>HANNA</t>
+        </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Agente IA Try and Buy Inbound y Outbound</t>
+          <t>Oportunidad de JARAMILLO MORA CONSTRUCTORA S A</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -3818,7 +3810,7 @@
         </is>
       </c>
       <c r="G79" s="1" t="n">
-        <v>45915.46633101852</v>
+        <v>45916.71618055556</v>
       </c>
       <c r="I79" t="n">
         <v>38</v>
@@ -3833,31 +3825,26 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t>gerencia@motosymotoselpaisa.com</t>
-        </is>
-      </c>
       <c r="B80" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>40000000</v>
+        <v>147000000</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Oportunidad de MOTOS Y MOTOS EL PAISA S A S</t>
+          <t>Contact Center Agendamiento citas</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Richard Castaño</t>
         </is>
       </c>
       <c r="G80" s="1" t="n">
-        <v>45915.46252314815</v>
+        <v>45916.67502314815</v>
       </c>
       <c r="I80" t="n">
         <v>38</v>
@@ -3874,7 +3861,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>isanchez@unico.com.co</t>
+          <t>jaime_zuluaga@eficacia.com.co</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -3883,11 +3870,11 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>0</v>
+        <v>14700000</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>1 agente IA para relacionamiento con locatarios</t>
+          <t>Agentes contact center encuestas</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -3896,12 +3883,21 @@
         </is>
       </c>
       <c r="G81" s="1" t="n">
-        <v>45915.46157407408</v>
+        <v>45916.65275462963</v>
+      </c>
+      <c r="H81" s="1" t="n">
+        <v>45930</v>
       </c>
       <c r="I81" t="n">
         <v>38</v>
       </c>
       <c r="J81" t="n">
+        <v>2025</v>
+      </c>
+      <c r="K81" t="n">
+        <v>9</v>
+      </c>
+      <c r="L81" t="n">
         <v>2025</v>
       </c>
       <c r="M81" t="inlineStr">

</xml_diff>

<commit_message>
CRM actualizado — 09/06/2026 09:47
</commit_message>
<xml_diff>
--- a/CRM_PowerBI_BrendaLuna_actualizado.xlsx
+++ b/CRM_PowerBI_BrendaLuna_actualizado.xlsx
@@ -951,7 +951,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1273,11 +1273,11 @@
     <row r="19">
       <c r="B19" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0</v>
+        <v>35000000</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -1439,7 +1439,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -1471,7 +1471,7 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
@@ -1688,7 +1688,7 @@
     <row r="29">
       <c r="B29" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -1729,7 +1729,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
@@ -1741,7 +1741,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Ganado</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -1911,7 +1911,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Negociación</t>
+          <t>Seguimiento</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -1947,7 +1947,7 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
@@ -3042,7 +3042,7 @@
     <row r="60">
       <c r="B60" t="inlineStr">
         <is>
-          <t>Seguimiento</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C60" t="n">

</xml_diff>

<commit_message>
CRM actualizado — 16/06/2026 14:12
</commit_message>
<xml_diff>
--- a/CRM_PowerBI_BrendaLuna_actualizado.xlsx
+++ b/CRM_PowerBI_BrendaLuna_actualizado.xlsx
@@ -946,25 +946,20 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>dgamoneda@productosdrogam.com</t>
+          <t>directoradjunto@dclass.edu.co</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C11" t="n">
         <v>0</v>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Diego Mauricio Gamoneda </t>
-        </is>
-      </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Oportunidad de Diego Mauricio Gamoneda </t>
+          <t>Oportunidad de DCLASS ACADEMIA SAS</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -973,10 +968,10 @@
         </is>
       </c>
       <c r="G11" s="1" t="n">
-        <v>46175.66417824074</v>
+        <v>46189.49674768518</v>
       </c>
       <c r="I11" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="J11" t="n">
         <v>2026</v>
@@ -990,54 +985,64 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>alexander.rojas@friogan.com</t>
+          <t>Belkis.jimenez@agrauto.com.co</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
+          <t>Propuesta</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Oportunidad de AGRICOLA AUTOMOTRIZ SAS / BELKYS JIMENEZ</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G12" s="1" t="n">
+        <v>46182.67912037037</v>
+      </c>
+      <c r="I12" t="n">
+        <v>24</v>
+      </c>
+      <c r="J12" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Calificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>luisa.baena@automarcali.com</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
           <t>Nuevo</t>
         </is>
       </c>
-      <c r="C12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Oportunidad de FRIOGAN S.A</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G12" s="1" t="n">
-        <v>46175.63597222222</v>
-      </c>
-      <c r="I12" t="n">
-        <v>23</v>
-      </c>
-      <c r="J12" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>No calificado</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
       <c r="C13" t="n">
         <v>0</v>
       </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>luisa.baena@automarcali.com</t>
+        </is>
+      </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Oportunidad de Agromercados la Montaña</t>
+          <t>Oportunidad de luisa.baena@automarcali.com</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1046,10 +1051,10 @@
         </is>
       </c>
       <c r="G13" s="1" t="n">
-        <v>46175.62239583334</v>
+        <v>46182.67809027778</v>
       </c>
       <c r="I13" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J13" t="n">
         <v>2026</v>
@@ -1063,20 +1068,25 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>juand.rios@alkosto.com.co</t>
+          <t>directormercadeo@almotores.com</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C14" t="n">
         <v>0</v>
       </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Viviana Vanegas</t>
+        </is>
+      </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Oportunidad de ALKOSTO</t>
+          <t>Oportunidad de Viviana Vanegas</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1085,42 +1095,37 @@
         </is>
       </c>
       <c r="G14" s="1" t="n">
-        <v>46175.62055555556</v>
+        <v>46182.67621527778</v>
       </c>
       <c r="I14" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J14" t="n">
         <v>2026</v>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>gerencia4087@grupo-exito.com</t>
+          <t>xiomara.duran@autopacifico.com.co</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C15" t="n">
         <v>0</v>
       </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Grupo exito ‒ 1007386172 - Sneider Quirama</t>
-        </is>
-      </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Oportunidad de Grupo exito</t>
+          <t>Oportunidad de xiomara.duran@autopacifico.com.co</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1129,10 +1134,10 @@
         </is>
       </c>
       <c r="G15" s="1" t="n">
-        <v>46175.61638888889</v>
+        <v>46182.65815972222</v>
       </c>
       <c r="I15" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J15" t="n">
         <v>2026</v>
@@ -1146,7 +1151,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ldgomez@supertiendascanaveral.com</t>
+          <t>alejandrosaavedraconde@comfandi.com.co</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1159,12 +1164,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Luis David Gomez</t>
+          <t>ALEJANDRO</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Oportunidad de Luis David Gomez</t>
+          <t>Oportunidad de ALEJANDRO</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1173,10 +1178,10 @@
         </is>
       </c>
       <c r="G16" s="1" t="n">
-        <v>46175.60493055556</v>
+        <v>46182.64278935185</v>
       </c>
       <c r="I16" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J16" t="n">
         <v>2026</v>
@@ -1190,12 +1195,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>davida_vanegas@coomeva.com.co</t>
+          <t>administracion@fiando.com.co</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -1203,7 +1208,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Oportunidad de BANCOOMEVA</t>
+          <t>Oportunidad de FIANDO LTDA</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1212,10 +1217,10 @@
         </is>
       </c>
       <c r="G17" s="1" t="n">
-        <v>46175.47109953704</v>
+        <v>46182.61304398148</v>
       </c>
       <c r="I17" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J17" t="n">
         <v>2026</v>
@@ -1229,12 +1234,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>alejandro.delgado@filedesk.com.co</t>
+          <t>dgamoneda@productosdrogam.com</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -1242,12 +1247,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>AlejandroDelgado</t>
+          <t xml:space="preserve">Diego Mauricio Gamoneda </t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Oportunidad de AlejandroDelgado</t>
+          <t xml:space="preserve">Oportunidad de Diego Mauricio Gamoneda </t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1256,7 +1261,7 @@
         </is>
       </c>
       <c r="G18" s="1" t="n">
-        <v>46174.71665509259</v>
+        <v>46175.66417824074</v>
       </c>
       <c r="I18" t="n">
         <v>23</v>
@@ -1271,22 +1276,22 @@
       </c>
     </row>
     <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>alexander.rojas@friogan.com</t>
+        </is>
+      </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>35000000</v>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Olga Lucia Hurtado</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Oportunidad de Olga Lucia Hurtado</t>
+          <t>Oportunidad de FRIOGAN S.A</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1295,10 +1300,10 @@
         </is>
       </c>
       <c r="G19" s="1" t="n">
-        <v>46168.49854166667</v>
+        <v>46175.63597222222</v>
       </c>
       <c r="I19" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="J19" t="n">
         <v>2026</v>
@@ -1310,22 +1315,17 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>comercial2@felsyn.com</t>
-        </is>
-      </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>713400</v>
+        <v>0</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Oportunidad de FONDO DE EMPLEADOS FELSYN</t>
+          <t>Oportunidad de Agromercados la Montaña</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1334,10 +1334,10 @@
         </is>
       </c>
       <c r="G20" s="1" t="n">
-        <v>46163.49130787037</v>
+        <v>46175.62239583334</v>
       </c>
       <c r="I20" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="J20" t="n">
         <v>2026</v>
@@ -1351,25 +1351,20 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>mercadeo@lasevillana.com.co</t>
+          <t>juand.rios@alkosto.com.co</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C21" t="n">
         <v>0</v>
       </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fabio AlbertoGallego García </t>
-        </is>
-      </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Oportunidad de Fabio AlbertoGallego García </t>
+          <t>Oportunidad de ALKOSTO</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1378,10 +1373,10 @@
         </is>
       </c>
       <c r="G21" s="1" t="n">
-        <v>46162.64569444444</v>
+        <v>46175.62055555556</v>
       </c>
       <c r="I21" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="J21" t="n">
         <v>2026</v>
@@ -1395,20 +1390,25 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>asantiago@stop.com.co</t>
+          <t>gerencia4087@grupo-exito.com</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C22" t="n">
         <v>0</v>
       </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Grupo exito ‒ 1007386172 - Sneider Quirama</t>
+        </is>
+      </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Oportunidad de STOP SAS</t>
+          <t>Oportunidad de Grupo exito</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1417,10 +1417,10 @@
         </is>
       </c>
       <c r="G22" s="1" t="n">
-        <v>46161.63508101852</v>
+        <v>46175.61638888889</v>
       </c>
       <c r="I22" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="J22" t="n">
         <v>2026</v>
@@ -1434,25 +1434,25 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>aestrada@teker.co</t>
+          <t>ldgomez@supertiendascanaveral.com</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>16914000</v>
+        <v>0</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>TEKER SALUD SAS</t>
+          <t>Luis David Gomez</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Oportunidad de TEKER SALUD SAS</t>
+          <t>Oportunidad de Luis David Gomez</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1461,10 +1461,10 @@
         </is>
       </c>
       <c r="G23" s="1" t="n">
-        <v>46161.62922453704</v>
+        <v>46175.60493055556</v>
       </c>
       <c r="I23" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="J23" t="n">
         <v>2026</v>
@@ -1476,6 +1476,11 @@
       </c>
     </row>
     <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>davida_vanegas@coomeva.com.co</t>
+        </is>
+      </c>
       <c r="B24" t="inlineStr">
         <is>
           <t>Contactado</t>
@@ -1486,7 +1491,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Oportunidad de TIAN IPS SAS</t>
+          <t>Oportunidad de BANCOOMEVA</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1495,10 +1500,10 @@
         </is>
       </c>
       <c r="G24" s="1" t="n">
-        <v>46161.61643518518</v>
+        <v>46175.47109953704</v>
       </c>
       <c r="I24" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="J24" t="n">
         <v>2026</v>
@@ -1512,25 +1517,25 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>administración@fullredtotal.com</t>
+          <t>alejandro.delgado@filedesk.com.co</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>14000000</v>
+        <v>0</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Eivar Eñasco</t>
+          <t>AlejandroDelgado</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Oportunidad de Eivar Eñasco</t>
+          <t>Oportunidad de AlejandroDelgado</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1539,42 +1544,37 @@
         </is>
       </c>
       <c r="G25" s="1" t="n">
-        <v>46154.67546296296</v>
+        <v>46174.71665509259</v>
       </c>
       <c r="I25" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="J25" t="n">
         <v>2026</v>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>cserna@surtifamiliar.com.co</t>
-        </is>
-      </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Negociación</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>1950000</v>
+        <v>35000000</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Claudia Patricia Serna</t>
+          <t>Olga Lucia Hurtado</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Oportunidad de Claudia Patricia Serna</t>
+          <t>Oportunidad de Olga Lucia Hurtado</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1583,42 +1583,37 @@
         </is>
       </c>
       <c r="G26" s="1" t="n">
-        <v>46154.66616898148</v>
+        <v>46168.49854166667</v>
       </c>
       <c r="I26" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="J26" t="n">
         <v>2026</v>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>coordmercadeo@pacificcenter.co</t>
+          <t>comercial2@felsyn.com</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>5600000</v>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Claudia Castro</t>
-        </is>
+        <v>713400</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Oportunidad de Claudia Castro</t>
+          <t>Oportunidad de FONDO DE EMPLEADOS FELSYN</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1627,42 +1622,42 @@
         </is>
       </c>
       <c r="G27" s="1" t="n">
-        <v>46154.66341435185</v>
+        <v>46163.49130787037</v>
       </c>
       <c r="I27" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J27" t="n">
         <v>2026</v>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>isabellarengifo27@gmail.com</t>
+          <t>mercadeo@lasevillana.com.co</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>28190000</v>
+        <v>0</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Isabella Rengifo</t>
+          <t xml:space="preserve">Fabio AlbertoGallego García </t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Oportunidad de Isabella Rengifo</t>
+          <t xml:space="preserve">Oportunidad de Fabio AlbertoGallego García </t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1671,10 +1666,10 @@
         </is>
       </c>
       <c r="G28" s="1" t="n">
-        <v>46154.65981481481</v>
+        <v>46162.64569444444</v>
       </c>
       <c r="I28" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J28" t="n">
         <v>2026</v>
@@ -1686,45 +1681,36 @@
       </c>
     </row>
     <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>asantiago@stop.com.co</t>
+        </is>
+      </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>50000000</v>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Paola Gómez - Agente Inmobiliaria Independiente</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Puesto de Trabajo CC Medellin</t>
+          <t>Oportunidad de STOP SAS</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Richard Castaño</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G29" s="1" t="n">
-        <v>46154.49104166667</v>
-      </c>
-      <c r="H29" s="1" t="n">
-        <v>46170</v>
+        <v>46161.63508101852</v>
       </c>
       <c r="I29" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J29" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K29" t="n">
-        <v>5</v>
-      </c>
-      <c r="L29" t="n">
         <v>2026</v>
       </c>
       <c r="M29" t="inlineStr">
@@ -1736,59 +1722,59 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>alberto.ramirez@constructorabolivar.com</t>
+          <t>aestrada@teker.co</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Ganado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>3000000</v>
+        <v>16914000</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>TEKER SALUD SAS</t>
+        </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Oportunidad de NPS Relacional</t>
+          <t>Oportunidad de TEKER SALUD SAS</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G30" s="1" t="n">
-        <v>46154.44511574074</v>
+        <v>46161.62922453704</v>
       </c>
       <c r="I30" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J30" t="n">
         <v>2026</v>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="B31" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>3000000</v>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>MADERKIT</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Oportunidad de MADERKIT</t>
+          <t>Oportunidad de TIAN IPS SAS</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1797,10 +1783,10 @@
         </is>
       </c>
       <c r="G31" s="1" t="n">
-        <v>46147.66540509259</v>
+        <v>46161.61643518518</v>
       </c>
       <c r="I31" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="J31" t="n">
         <v>2026</v>
@@ -1814,25 +1800,25 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>omer120395@gmail.com</t>
+          <t>administración@fullredtotal.com</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>0</v>
+        <v>14000000</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Omer Peñaloza</t>
+          <t>Eivar Eñasco</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Oportunidad de Omer Peñaloza</t>
+          <t>Oportunidad de Eivar Eñasco</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1841,37 +1827,42 @@
         </is>
       </c>
       <c r="G32" s="1" t="n">
-        <v>46147.66090277778</v>
+        <v>46154.67546296296</v>
       </c>
       <c r="I32" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J32" t="n">
         <v>2026</v>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>directora.it@supermercadobelalcazar.com.co</t>
+          <t>cserna@surtifamiliar.com.co</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Negociación</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>6000000</v>
+        <v>1950000</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Claudia Patricia Serna</t>
+        </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Oportunidad de ABASTECEMOS DE OCCIDENTE</t>
+          <t>Oportunidad de Claudia Patricia Serna</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1880,46 +1871,42 @@
         </is>
       </c>
       <c r="G33" s="1" t="n">
-        <v>46147.64170138889</v>
-      </c>
-      <c r="H33" s="1" t="n">
-        <v>46157</v>
+        <v>46154.66616898148</v>
       </c>
       <c r="I33" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J33" t="n">
         <v>2026</v>
       </c>
-      <c r="K33" t="n">
-        <v>5</v>
-      </c>
-      <c r="L33" t="n">
-        <v>2026</v>
-      </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>oscar.molina@terrenoshouston.com</t>
+          <t>coordmercadeo@pacificcenter.co</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Seguimiento</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>37623040</v>
+        <v>5600000</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Claudia Castro</t>
+        </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Oportunidad de COLONY RIDGE</t>
+          <t>Oportunidad de Claudia Castro</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1928,46 +1915,42 @@
         </is>
       </c>
       <c r="G34" s="1" t="n">
-        <v>46147.60297453704</v>
-      </c>
-      <c r="H34" s="1" t="n">
-        <v>46150</v>
+        <v>46154.66341435185</v>
       </c>
       <c r="I34" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J34" t="n">
         <v>2026</v>
       </c>
-      <c r="K34" t="n">
-        <v>5</v>
-      </c>
-      <c r="L34" t="n">
-        <v>2026</v>
-      </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>jsantacr@ccc.org.co</t>
+          <t>isabellarengifo27@gmail.com</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>55000000</v>
+        <v>28190000</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Isabella Rengifo</t>
+        </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Oportunidad de CAMARA DE COMERCIO CALI</t>
+          <t>Oportunidad de Isabella Rengifo</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1976,23 +1959,14 @@
         </is>
       </c>
       <c r="G35" s="1" t="n">
-        <v>46141.62370370371</v>
-      </c>
-      <c r="H35" s="1" t="n">
-        <v>46289</v>
+        <v>46154.65981481481</v>
       </c>
       <c r="I35" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="J35" t="n">
         <v>2026</v>
       </c>
-      <c r="K35" t="n">
-        <v>9</v>
-      </c>
-      <c r="L35" t="n">
-        <v>2026</v>
-      </c>
       <c r="M35" t="inlineStr">
         <is>
           <t>No calificado</t>
@@ -2000,36 +1974,45 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>exportaciones@laprovincia.com</t>
-        </is>
-      </c>
       <c r="B36" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>6000000</v>
+        <v>50000000</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Paola Gómez - Agente Inmobiliaria Independiente</t>
+        </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Oportunidad de PRODUCTOS LA PROVINCIA SAS</t>
+          <t>Puesto de Trabajo CC Medellin</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Richard Castaño</t>
         </is>
       </c>
       <c r="G36" s="1" t="n">
-        <v>46141.62021990741</v>
+        <v>46154.49104166667</v>
+      </c>
+      <c r="H36" s="1" t="n">
+        <v>46170</v>
       </c>
       <c r="I36" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="J36" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K36" t="n">
+        <v>5</v>
+      </c>
+      <c r="L36" t="n">
         <v>2026</v>
       </c>
       <c r="M36" t="inlineStr">
@@ -2041,54 +2024,59 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>coordinador.mercadeo@regency.com.co</t>
+          <t>alberto.ramirez@constructorabolivar.com</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Ganado</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>0</v>
+        <v>3000000</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Oportunidad de REGENCY TECH SAS</t>
+          <t>Oportunidad de NPS Relacional</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G37" s="1" t="n">
-        <v>46141.59664351852</v>
+        <v>46154.44511574074</v>
       </c>
       <c r="I37" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="J37" t="n">
         <v>2026</v>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="B38" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>1200000</v>
+        <v>3000000</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>MADERKIT</t>
+        </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Oportunidad de EMCALI E.I.C.E ESP</t>
+          <t>Oportunidad de MADERKIT</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2097,21 +2085,12 @@
         </is>
       </c>
       <c r="G38" s="1" t="n">
-        <v>46141.59045138889</v>
-      </c>
-      <c r="H38" s="1" t="n">
-        <v>46352</v>
+        <v>46147.66540509259</v>
       </c>
       <c r="I38" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J38" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K38" t="n">
-        <v>11</v>
-      </c>
-      <c r="L38" t="n">
         <v>2026</v>
       </c>
       <c r="M38" t="inlineStr">
@@ -2123,20 +2102,25 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>angie_feligrana@eficacia.com.co</t>
+          <t>omer120395@gmail.com</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Seguimiento</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>6000000</v>
+        <v>0</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Omer Peñaloza</t>
+        </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Oportunidad de Eficacia sas / Angie Feligrana</t>
+          <t>Oportunidad de Omer Peñaloza</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2145,21 +2129,12 @@
         </is>
       </c>
       <c r="G39" s="1" t="n">
-        <v>46126.63210648148</v>
-      </c>
-      <c r="H39" s="1" t="n">
-        <v>46150</v>
+        <v>46147.66090277778</v>
       </c>
       <c r="I39" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="J39" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K39" t="n">
-        <v>5</v>
-      </c>
-      <c r="L39" t="n">
         <v>2026</v>
       </c>
       <c r="M39" t="inlineStr">
@@ -2171,7 +2146,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Estrategiadigital@zuluagaysoto.com</t>
+          <t>directora.it@supermercadobelalcazar.com.co</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2180,16 +2155,11 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>0</v>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>Maryuri Arguello</t>
-        </is>
+        <v>6000000</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Oportunidad de Maryuri Arguello</t>
+          <t>Oportunidad de ABASTECEMOS DE OCCIDENTE</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -2198,12 +2168,21 @@
         </is>
       </c>
       <c r="G40" s="1" t="n">
-        <v>46125.71925925926</v>
+        <v>46147.64170138889</v>
+      </c>
+      <c r="H40" s="1" t="n">
+        <v>46157</v>
       </c>
       <c r="I40" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="J40" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K40" t="n">
+        <v>5</v>
+      </c>
+      <c r="L40" t="n">
         <v>2026</v>
       </c>
       <c r="M40" t="inlineStr">
@@ -2215,73 +2194,68 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>gabrielrodriguez@arrozsupremo.com</t>
+          <t>oscar.molina@terrenoshouston.com</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Ganado</t>
+          <t>Seguimiento</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>8000000</v>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>GABRIEL RODRIGUEZ</t>
-        </is>
+        <v>37623040</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Agente de Ventas</t>
+          <t>Oportunidad de COLONY RIDGE</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Richard Castaño</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G41" s="1" t="n">
-        <v>46119.62108796297</v>
+        <v>46147.60297453704</v>
       </c>
       <c r="H41" s="1" t="n">
-        <v>46141</v>
+        <v>46150</v>
       </c>
       <c r="I41" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="J41" t="n">
         <v>2026</v>
       </c>
       <c r="K41" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L41" t="n">
         <v>2026</v>
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Belkis.jimenez@agrauto.com.co</t>
+          <t>jsantacr@ccc.org.co</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>0</v>
+        <v>55000000</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Oportunidad de AGRICOLA AUTOMOTRIZ SAS</t>
+          <t>Oportunidad de CAMARA DE COMERCIO CALI</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -2290,12 +2264,21 @@
         </is>
       </c>
       <c r="G42" s="1" t="n">
-        <v>46119.38914351852</v>
+        <v>46141.62370370371</v>
+      </c>
+      <c r="H42" s="1" t="n">
+        <v>46289</v>
       </c>
       <c r="I42" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="J42" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K42" t="n">
+        <v>9</v>
+      </c>
+      <c r="L42" t="n">
         <v>2026</v>
       </c>
       <c r="M42" t="inlineStr">
@@ -2307,7 +2290,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>anyela.aponza@cotel.com.co</t>
+          <t>exportaciones@laprovincia.com</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2316,11 +2299,11 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>0</v>
+        <v>6000000</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Oportunidad de COTEL SAL</t>
+          <t>Oportunidad de PRODUCTOS LA PROVINCIA SAS</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2329,10 +2312,10 @@
         </is>
       </c>
       <c r="G43" s="1" t="n">
-        <v>46112.61271990741</v>
+        <v>46141.62021990741</v>
       </c>
       <c r="I43" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="J43" t="n">
         <v>2026</v>
@@ -2346,7 +2329,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>liliana.patino@quironsalud.com</t>
+          <t>coordinador.mercadeo@regency.com.co</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2357,14 +2340,9 @@
       <c r="C44" t="n">
         <v>0</v>
       </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>CLINICA IMBANACO</t>
-        </is>
-      </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Oportunidad de Liliana Patiño Flórez</t>
+          <t>Oportunidad de REGENCY TECH SAS</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -2373,10 +2351,10 @@
         </is>
       </c>
       <c r="G44" s="1" t="n">
-        <v>46112.60853009259</v>
+        <v>46141.59664351852</v>
       </c>
       <c r="I44" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="J44" t="n">
         <v>2026</v>
@@ -2388,22 +2366,17 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>casanchez@jgb.com.co</t>
-        </is>
-      </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>0</v>
+        <v>1200000</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Oportunidad de JGB S.A.</t>
+          <t>Oportunidad de EMCALI E.I.C.E ESP</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -2412,12 +2385,21 @@
         </is>
       </c>
       <c r="G45" s="1" t="n">
-        <v>46112.6052662037</v>
+        <v>46141.59045138889</v>
+      </c>
+      <c r="H45" s="1" t="n">
+        <v>46352</v>
       </c>
       <c r="I45" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="J45" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K45" t="n">
+        <v>11</v>
+      </c>
+      <c r="L45" t="n">
         <v>2026</v>
       </c>
       <c r="M45" t="inlineStr">
@@ -2429,7 +2411,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>damaris.gomez@disfarma.com.co</t>
+          <t>angie_feligrana@eficacia.com.co</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2438,11 +2420,11 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>0</v>
+        <v>6000000</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Oportunidad de DISFARMA</t>
+          <t>Oportunidad de Eficacia sas / Angie Feligrana</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2451,12 +2433,21 @@
         </is>
       </c>
       <c r="G46" s="1" t="n">
-        <v>46112.60325231482</v>
+        <v>46126.63210648148</v>
+      </c>
+      <c r="H46" s="1" t="n">
+        <v>46150</v>
       </c>
       <c r="I46" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="J46" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K46" t="n">
+        <v>5</v>
+      </c>
+      <c r="L46" t="n">
         <v>2026</v>
       </c>
       <c r="M46" t="inlineStr">
@@ -2468,7 +2459,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>alergologosdeoccidente@gmail.com</t>
+          <t>Estrategiadigital@zuluagaysoto.com</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2481,12 +2472,12 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Johana Gonzalez</t>
+          <t>Maryuri Arguello</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Oportunidad de Johana Gonzalez</t>
+          <t>Oportunidad de Maryuri Arguello</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -2495,10 +2486,10 @@
         </is>
       </c>
       <c r="G47" s="1" t="n">
-        <v>46107.51248842593</v>
+        <v>46125.71925925926</v>
       </c>
       <c r="I47" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="J47" t="n">
         <v>2026</v>
@@ -2512,7 +2503,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>DavidEsteban.Porras@alfalaval.com</t>
+          <t>gabrielrodriguez@arrozsupremo.com</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2521,26 +2512,31 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>15000000</v>
+        <v>8000000</v>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>GABRIEL RODRIGUEZ</t>
+        </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Oportunidad de OPORTUNIDAD ENCUESTAS ALFALAVAL</t>
+          <t>Agente de Ventas</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Richard Castaño</t>
         </is>
       </c>
       <c r="G48" s="1" t="n">
-        <v>46101.72893518519</v>
+        <v>46119.62108796297</v>
       </c>
       <c r="H48" s="1" t="n">
         <v>46141</v>
       </c>
       <c r="I48" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="J48" t="n">
         <v>2026</v>
@@ -2560,7 +2556,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Dr.arcarmona@gmail.com</t>
+          <t>Belkis.jimenez@agrauto.com.co</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2573,7 +2569,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Oportunidad de GAMANUCLEAR LTDA - Dr Alberto Carmona</t>
+          <t>Oportunidad de AGRICOLA AUTOMOTRIZ SAS</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -2582,10 +2578,10 @@
         </is>
       </c>
       <c r="G49" s="1" t="n">
-        <v>46098.65114583333</v>
+        <v>46119.38914351852</v>
       </c>
       <c r="I49" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="J49" t="n">
         <v>2026</v>
@@ -2599,7 +2595,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>cecilia.guevara@cosmitet.net / administracion.crd@cosmitet.net</t>
+          <t>anyela.aponza@cotel.com.co</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2610,14 +2606,9 @@
       <c r="C50" t="n">
         <v>0</v>
       </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>Cecilia Guevara</t>
-        </is>
-      </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Oportunidad de CLINICA REY DAVID Walter Charria</t>
+          <t>Oportunidad de COTEL SAL</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -2626,10 +2617,10 @@
         </is>
       </c>
       <c r="G50" s="1" t="n">
-        <v>46094.69002314815</v>
+        <v>46112.61271990741</v>
       </c>
       <c r="I50" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="J50" t="n">
         <v>2026</v>
@@ -2643,7 +2634,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>vicerrectoriacademica@unicatolica.edu.co</t>
+          <t>liliana.patino@quironsalud.com</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2656,12 +2647,12 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Jorge Silva</t>
+          <t>CLINICA IMBANACO</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Oportunidad de Jorge Silva</t>
+          <t>Oportunidad de Liliana Patiño Flórez</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -2670,10 +2661,10 @@
         </is>
       </c>
       <c r="G51" s="1" t="n">
-        <v>46094.66880787037</v>
+        <v>46112.60853009259</v>
       </c>
       <c r="I51" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="J51" t="n">
         <v>2026</v>
@@ -2687,85 +2678,71 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>pedroperea02@gmail.com</t>
+          <t>casanchez@jgb.com.co</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Ganado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>2160000</v>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>Pedro Pablo Perea Mafla</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Oportunidad de Encuestas</t>
+          <t>Oportunidad de JGB S.A.</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G52" s="1" t="n">
-        <v>46094.65905092593</v>
-      </c>
-      <c r="H52" s="1" t="n">
-        <v>46141</v>
+        <v>46112.6052662037</v>
       </c>
       <c r="I52" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="J52" t="n">
         <v>2026</v>
       </c>
-      <c r="K52" t="n">
-        <v>4</v>
-      </c>
-      <c r="L52" t="n">
-        <v>2026</v>
-      </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>cristina.papamija@bmm.com.co</t>
+          <t>damaris.gomez@disfarma.com.co</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Seguimiento</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>8071000</v>
+        <v>0</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Oportunidad de BANCO MUNDO MUJER</t>
+          <t>Oportunidad de DISFARMA</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G53" s="1" t="n">
-        <v>46094.65019675926</v>
+        <v>46112.60325231482</v>
       </c>
       <c r="I53" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="J53" t="n">
         <v>2026</v>
@@ -2779,7 +2756,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>capacitacionvirtual@fundacionwwbcol.org</t>
+          <t>alergologosdeoccidente@gmail.com</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2788,23 +2765,28 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>1600000</v>
+        <v>0</v>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Johana Gonzalez</t>
+        </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Licenciamiento y ajuste WhatsApp FUNDACIÓN WWB</t>
+          <t>Oportunidad de Johana Gonzalez</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G54" s="1" t="n">
-        <v>46094.64826388889</v>
+        <v>46107.51248842593</v>
       </c>
       <c r="I54" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="J54" t="n">
         <v>2026</v>
@@ -2818,7 +2800,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>carol.cuesta@cbolivar.com</t>
+          <t>DavidEsteban.Porras@alfalaval.com</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2827,16 +2809,11 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>2900000</v>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>CAROL CUESTA</t>
-        </is>
+        <v>15000000</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Gestión de Subsidios CB Bogotá</t>
+          <t>Oportunidad de OPORTUNIDAD ENCUESTAS ALFALAVAL</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -2845,13 +2822,13 @@
         </is>
       </c>
       <c r="G55" s="1" t="n">
-        <v>46094.64454861111</v>
+        <v>46101.72893518519</v>
       </c>
       <c r="H55" s="1" t="n">
-        <v>46135</v>
+        <v>46141</v>
       </c>
       <c r="I55" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J55" t="n">
         <v>2026</v>
@@ -2871,7 +2848,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>edwin.munoz.v@uniminuto.edu</t>
+          <t>Dr.arcarmona@gmail.com</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2884,7 +2861,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Oportunidad de UNIMINUTO</t>
+          <t>Oportunidad de GAMANUCLEAR LTDA - Dr Alberto Carmona</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -2893,10 +2870,10 @@
         </is>
       </c>
       <c r="G56" s="1" t="n">
-        <v>46092.63626157407</v>
+        <v>46098.65114583333</v>
       </c>
       <c r="I56" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J56" t="n">
         <v>2026</v>
@@ -2910,7 +2887,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>jaime_zuluaga@eficacia.com.co</t>
+          <t>cecilia.guevara@cosmitet.net / administracion.crd@cosmitet.net</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2923,12 +2900,12 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Jaime Alberto</t>
+          <t>Cecilia Guevara</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Oportunidad de Jaime Alberto Zuluaga</t>
+          <t>Oportunidad de CLINICA REY DAVID Walter Charria</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -2937,7 +2914,7 @@
         </is>
       </c>
       <c r="G57" s="1" t="n">
-        <v>46092.63153935185</v>
+        <v>46094.69002314815</v>
       </c>
       <c r="I57" t="n">
         <v>11</v>
@@ -2954,7 +2931,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>comercial@isyscol.com</t>
+          <t>vicerrectoriacademica@unicatolica.edu.co</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2967,12 +2944,12 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Andres Nader</t>
+          <t>Jorge Silva</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Oportunidad de Andres Nader</t>
+          <t>Oportunidad de Jorge Silva</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -2981,7 +2958,7 @@
         </is>
       </c>
       <c r="G58" s="1" t="n">
-        <v>46091.59211805555</v>
+        <v>46094.66880787037</v>
       </c>
       <c r="I58" t="n">
         <v>11</v>
@@ -2998,34 +2975,37 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>mercadeo@norteysur.co</t>
+          <t>pedroperea02@gmail.com</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Ganado</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>0</v>
+        <v>2160000</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Isabella Mesa</t>
+          <t>Pedro Pablo Perea Mafla</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Oportunidad de Isabella Mesa</t>
+          <t>Oportunidad de Encuestas</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G59" s="1" t="n">
-        <v>46091.40078703704</v>
+        <v>46094.65905092593</v>
+      </c>
+      <c r="H59" s="1" t="n">
+        <v>46141</v>
       </c>
       <c r="I59" t="n">
         <v>11</v>
@@ -3033,33 +3013,44 @@
       <c r="J59" t="n">
         <v>2026</v>
       </c>
+      <c r="K59" t="n">
+        <v>4</v>
+      </c>
+      <c r="L59" t="n">
+        <v>2026</v>
+      </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>cristina.papamija@bmm.com.co</t>
+        </is>
+      </c>
       <c r="B60" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>0</v>
+        <v>8071000</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Clasificación EMAIL Comfenalco Cartagena</t>
+          <t>Oportunidad de BANCO MUNDO MUJER</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Maria Fernanda Gaviria</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G60" s="1" t="n">
-        <v>46091.3665625</v>
+        <v>46094.65019675926</v>
       </c>
       <c r="I60" t="n">
         <v>11</v>
@@ -3074,29 +3065,34 @@
       </c>
     </row>
     <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>capacitacionvirtual@fundacionwwbcol.org</t>
+        </is>
+      </c>
       <c r="B61" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>0</v>
+        <v>1600000</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Oportunidad de ESE HOSPITAL LA MARIA</t>
+          <t>Licenciamiento y ajuste WhatsApp FUNDACIÓN WWB</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Laura Alejandra Castañeda</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G61" s="1" t="n">
-        <v>46083.67605324074</v>
+        <v>46094.64826388889</v>
       </c>
       <c r="I61" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J61" t="n">
         <v>2026</v>
@@ -3108,63 +3104,87 @@
       </c>
     </row>
     <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>carol.cuesta@cbolivar.com</t>
+        </is>
+      </c>
       <c r="B62" t="inlineStr">
         <is>
+          <t>Ganado</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>2900000</v>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>CAROL CUESTA</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Gestión de Subsidios CB Bogotá</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Jennifer Hoyos Gallego</t>
+        </is>
+      </c>
+      <c r="G62" s="1" t="n">
+        <v>46094.64454861111</v>
+      </c>
+      <c r="H62" s="1" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I62" t="n">
+        <v>11</v>
+      </c>
+      <c r="J62" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K62" t="n">
+        <v>4</v>
+      </c>
+      <c r="L62" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>Calificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>edwin.munoz.v@uniminuto.edu</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
           <t>Perdido</t>
         </is>
       </c>
-      <c r="C62" t="n">
-        <v>0</v>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>Oportunidad de SUPER TRANSPORTE</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>Laura Alejandra Castañeda</t>
-        </is>
-      </c>
-      <c r="G62" s="1" t="n">
-        <v>46083.6706712963</v>
-      </c>
-      <c r="I62" t="n">
-        <v>10</v>
-      </c>
-      <c r="J62" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M62" t="inlineStr">
-        <is>
-          <t>No calificado</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
       <c r="C63" t="n">
         <v>0</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Oportunidad de ENLACES IP S.A.S</t>
+          <t>Oportunidad de UNIMINUTO</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Laura Alejandra Castañeda</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G63" s="1" t="n">
-        <v>46083.50145833333</v>
+        <v>46092.63626157407</v>
       </c>
       <c r="I63" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J63" t="n">
         <v>2026</v>
@@ -3178,7 +3198,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>accounting@diaza.com</t>
+          <t>jaime_zuluaga@eficacia.com.co</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3191,12 +3211,12 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>JOHANA RODRIGUEZ</t>
+          <t>Jaime Alberto</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Oportunidad de JOHANA RODRIGUEZ</t>
+          <t>Oportunidad de Jaime Alberto Zuluaga</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -3205,10 +3225,10 @@
         </is>
       </c>
       <c r="G64" s="1" t="n">
-        <v>46079.73486111111</v>
+        <v>46092.63153935185</v>
       </c>
       <c r="I64" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="J64" t="n">
         <v>2026</v>
@@ -3222,7 +3242,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>mensajeriamyr@gmail.com</t>
+          <t>comercial@isyscol.com</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -3233,9 +3253,14 @@
       <c r="C65" t="n">
         <v>0</v>
       </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Andres Nader</t>
+        </is>
+      </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Oportunidad de MENSAJERIA M&amp;R SAS</t>
+          <t>Oportunidad de Andres Nader</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -3244,10 +3269,10 @@
         </is>
       </c>
       <c r="G65" s="1" t="n">
-        <v>46079.72262731481</v>
+        <v>46091.59211805555</v>
       </c>
       <c r="I65" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="J65" t="n">
         <v>2026</v>
@@ -3261,313 +3286,303 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
+          <t>mercadeo@norteysur.co</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>0</v>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Isabella Mesa</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Oportunidad de Isabella Mesa</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G66" s="1" t="n">
+        <v>46091.40078703704</v>
+      </c>
+      <c r="I66" t="n">
+        <v>11</v>
+      </c>
+      <c r="J66" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>No calificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>0</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Clasificación EMAIL Comfenalco Cartagena</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Maria Fernanda Gaviria</t>
+        </is>
+      </c>
+      <c r="G67" s="1" t="n">
+        <v>46091.3665625</v>
+      </c>
+      <c r="I67" t="n">
+        <v>11</v>
+      </c>
+      <c r="J67" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>No calificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>0</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Oportunidad de ESE HOSPITAL LA MARIA</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Laura Alejandra Castañeda</t>
+        </is>
+      </c>
+      <c r="G68" s="1" t="n">
+        <v>46083.67605324074</v>
+      </c>
+      <c r="I68" t="n">
+        <v>10</v>
+      </c>
+      <c r="J68" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>No calificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>0</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Oportunidad de SUPER TRANSPORTE</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Laura Alejandra Castañeda</t>
+        </is>
+      </c>
+      <c r="G69" s="1" t="n">
+        <v>46083.6706712963</v>
+      </c>
+      <c r="I69" t="n">
+        <v>10</v>
+      </c>
+      <c r="J69" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>No calificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>0</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Oportunidad de ENLACES IP S.A.S</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Laura Alejandra Castañeda</t>
+        </is>
+      </c>
+      <c r="G70" s="1" t="n">
+        <v>46083.50145833333</v>
+      </c>
+      <c r="I70" t="n">
+        <v>10</v>
+      </c>
+      <c r="J70" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>No calificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>accounting@diaza.com</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>0</v>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>JOHANA RODRIGUEZ</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Oportunidad de JOHANA RODRIGUEZ</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G71" s="1" t="n">
+        <v>46079.73486111111</v>
+      </c>
+      <c r="I71" t="n">
+        <v>9</v>
+      </c>
+      <c r="J71" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>No calificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>mensajeriamyr@gmail.com</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>0</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Oportunidad de MENSAJERIA M&amp;R SAS</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G72" s="1" t="n">
+        <v>46079.72262731481</v>
+      </c>
+      <c r="I72" t="n">
+        <v>9</v>
+      </c>
+      <c r="J72" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>No calificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
           <t>sistemaspanaderialeal@gmail.com</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr">
+      <c r="B73" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
-      <c r="C66" t="n">
-        <v>0</v>
-      </c>
-      <c r="D66" t="inlineStr">
+      <c r="C73" t="n">
+        <v>0</v>
+      </c>
+      <c r="D73" t="inlineStr">
         <is>
           <t>Diego Rios</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr">
+      <c r="E73" t="inlineStr">
         <is>
           <t>JAMDAC SAS, Diego Rios</t>
         </is>
       </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G66" s="1" t="n">
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G73" s="1" t="n">
         <v>46071.63706018519</v>
       </c>
-      <c r="I66" t="n">
+      <c r="I73" t="n">
         <v>8</v>
       </c>
-      <c r="J66" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M66" t="inlineStr">
-        <is>
-          <t>No calificado</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>efernandez@unico.com.co</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C67" t="n">
-        <v>0</v>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>Erick Fernandez</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>Oportunidad de Erick Fernandez</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G67" s="1" t="n">
-        <v>46064.3750462963</v>
-      </c>
-      <c r="I67" t="n">
-        <v>7</v>
-      </c>
-      <c r="J67" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M67" t="inlineStr">
-        <is>
-          <t>No calificado</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>kabenitez@icesi.edu.co</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C68" t="n">
-        <v>10000000</v>
-      </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>KENI BENITEZ</t>
-        </is>
-      </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>Oportunidad de KENI BENITEZ</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t>Jennifer Hoyos Gallego</t>
-        </is>
-      </c>
-      <c r="G68" s="1" t="n">
-        <v>46059.34918981481</v>
-      </c>
-      <c r="I68" t="n">
-        <v>6</v>
-      </c>
-      <c r="J68" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M68" t="inlineStr">
-        <is>
-          <t>No calificado</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>patovar@uao.edu.co</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C69" t="n">
-        <v>0</v>
-      </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>Paula Tovar</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>Oportunidad de UNIVERSIDAD AUTONOMA DE OCCIDENTE</t>
-        </is>
-      </c>
-      <c r="F69" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G69" s="1" t="n">
-        <v>46058.72516203704</v>
-      </c>
-      <c r="I69" t="n">
-        <v>6</v>
-      </c>
-      <c r="J69" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M69" t="inlineStr">
-        <is>
-          <t>No calificado</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>comercial@isyscol.com</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C70" t="n">
-        <v>0</v>
-      </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>Oportunidad de TECNOLOGIAS ISYSCOL SAS</t>
-        </is>
-      </c>
-      <c r="F70" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G70" s="1" t="n">
-        <v>46057.58993055556</v>
-      </c>
-      <c r="I70" t="n">
-        <v>6</v>
-      </c>
-      <c r="J70" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M70" t="inlineStr">
-        <is>
-          <t>No calificado</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C71" t="n">
-        <v>15000000</v>
-      </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>Oportunidad de VOICE IA EFICACIA</t>
-        </is>
-      </c>
-      <c r="F71" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G71" s="1" t="n">
-        <v>46057.3409837963</v>
-      </c>
-      <c r="I71" t="n">
-        <v>6</v>
-      </c>
-      <c r="J71" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M71" t="inlineStr">
-        <is>
-          <t>No calificado</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C72" t="n">
-        <v>4000000</v>
-      </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>Oportunidad de Eficacia WhatsApp</t>
-        </is>
-      </c>
-      <c r="F72" t="inlineStr">
-        <is>
-          <t>Jennifer Hoyos Gallego</t>
-        </is>
-      </c>
-      <c r="G72" s="1" t="n">
-        <v>46049.67292824074</v>
-      </c>
-      <c r="I72" t="n">
-        <v>5</v>
-      </c>
-      <c r="J72" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M72" t="inlineStr">
-        <is>
-          <t>No calificado</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C73" t="n">
-        <v>20000000</v>
-      </c>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>Oportunidad de CRUZ ROJA COLOMBIANA SECCIONAL VALLE DEL CAUCA</t>
-        </is>
-      </c>
-      <c r="F73" t="inlineStr">
-        <is>
-          <t>Jennifer Hoyos Gallego</t>
-        </is>
-      </c>
-      <c r="G73" s="1" t="n">
-        <v>46006.49650462963</v>
-      </c>
-      <c r="I73" t="n">
-        <v>51</v>
-      </c>
       <c r="J73" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="M73" t="inlineStr">
         <is>
@@ -3578,7 +3593,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>silvia.figueroa@neurithmedia.com</t>
+          <t>efernandez@unico.com.co</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -3587,26 +3602,31 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>25000000</v>
+        <v>0</v>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Erick Fernandez</t>
+        </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Contact center ventas España</t>
+          <t>Oportunidad de Erick Fernandez</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Richard Castaño</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G74" s="1" t="n">
-        <v>45960.61145833333</v>
+        <v>46064.3750462963</v>
       </c>
       <c r="I74" t="n">
-        <v>44</v>
+        <v>7</v>
       </c>
       <c r="J74" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="M74" t="inlineStr">
         <is>
@@ -3615,37 +3635,42 @@
       </c>
     </row>
     <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>kabenitez@icesi.edu.co</t>
+        </is>
+      </c>
       <c r="B75" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>37000000</v>
+        <v>10000000</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Mabel</t>
+          <t>KENI BENITEZ</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Masivos Licitacion</t>
+          <t>Oportunidad de KENI BENITEZ</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Richard Castaño</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G75" s="1" t="n">
-        <v>45940.49372685186</v>
+        <v>46059.34918981481</v>
       </c>
       <c r="I75" t="n">
-        <v>41</v>
+        <v>6</v>
       </c>
       <c r="J75" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="M75" t="inlineStr">
         <is>
@@ -3656,7 +3681,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>ana.zuniga@cbolivar.com</t>
+          <t>patovar@uao.edu.co</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -3665,31 +3690,31 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>4997000</v>
+        <v>0</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Ana Lucia Zuñiga</t>
+          <t>Paula Tovar</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Constructora Bolivar Agente Redes</t>
+          <t>Oportunidad de UNIVERSIDAD AUTONOMA DE OCCIDENTE</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G76" s="1" t="n">
-        <v>45940.49215277778</v>
+        <v>46058.72516203704</v>
       </c>
       <c r="I76" t="n">
-        <v>41</v>
+        <v>6</v>
       </c>
       <c r="J76" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="M76" t="inlineStr">
         <is>
@@ -3700,7 +3725,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>julian_mendez@extras.com.co</t>
+          <t>comercial@isyscol.com</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -3709,114 +3734,94 @@
         </is>
       </c>
       <c r="C77" t="n">
+        <v>0</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Oportunidad de TECNOLOGIAS ISYSCOL SAS</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G77" s="1" t="n">
+        <v>46057.58993055556</v>
+      </c>
+      <c r="I77" t="n">
+        <v>6</v>
+      </c>
+      <c r="J77" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M77" t="inlineStr">
+        <is>
+          <t>No calificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
         <v>15000000</v>
       </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>Julian Mendez.</t>
-        </is>
-      </c>
-      <c r="E77" t="inlineStr">
-        <is>
-          <t>Oportunidad de EFICACIA S A S</t>
-        </is>
-      </c>
-      <c r="F77" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G77" s="1" t="n">
-        <v>45922.66201388889</v>
-      </c>
-      <c r="I77" t="n">
-        <v>39</v>
-      </c>
-      <c r="J77" t="n">
-        <v>2025</v>
-      </c>
-      <c r="M77" t="inlineStr">
-        <is>
-          <t>No calificado</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="inlineStr">
-        <is>
-          <t>info@eficacia.com.co</t>
-        </is>
-      </c>
-      <c r="B78" t="inlineStr">
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Oportunidad de VOICE IA EFICACIA</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G78" s="1" t="n">
+        <v>46057.3409837963</v>
+      </c>
+      <c r="I78" t="n">
+        <v>6</v>
+      </c>
+      <c r="J78" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M78" t="inlineStr">
+        <is>
+          <t>No calificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="B79" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
-      <c r="C78" t="n">
-        <v>0</v>
-      </c>
-      <c r="E78" t="inlineStr">
-        <is>
-          <t>Nutresa</t>
-        </is>
-      </c>
-      <c r="F78" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G78" s="1" t="n">
-        <v>45922.66199074074</v>
-      </c>
-      <c r="I78" t="n">
-        <v>39</v>
-      </c>
-      <c r="J78" t="n">
-        <v>2025</v>
-      </c>
-      <c r="M78" t="inlineStr">
-        <is>
-          <t>No calificado</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t>hrodriguez@jaramillomora.com</t>
-        </is>
-      </c>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>Seguimiento</t>
-        </is>
-      </c>
       <c r="C79" t="n">
-        <v>30000000</v>
-      </c>
-      <c r="D79" t="inlineStr">
-        <is>
-          <t>HANNA</t>
-        </is>
+        <v>4000000</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Oportunidad de JARAMILLO MORA CONSTRUCTORA S A</t>
+          <t>Oportunidad de Eficacia WhatsApp</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Richard Castaño</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G79" s="1" t="n">
-        <v>45916.71618055556</v>
+        <v>46049.67292824074</v>
       </c>
       <c r="I79" t="n">
-        <v>38</v>
+        <v>5</v>
       </c>
       <c r="J79" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="M79" t="inlineStr">
         <is>
@@ -3831,23 +3836,23 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>147000000</v>
+        <v>20000000</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Contact Center Agendamiento citas</t>
+          <t>Oportunidad de CRUZ ROJA COLOMBIANA SECCIONAL VALLE DEL CAUCA</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Richard Castaño</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G80" s="1" t="n">
-        <v>45916.67502314815</v>
+        <v>46006.49650462963</v>
       </c>
       <c r="I80" t="n">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="J80" t="n">
         <v>2025</v>
@@ -3861,7 +3866,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>jaime_zuluaga@eficacia.com.co</t>
+          <t>silvia.figueroa@neurithmedia.com</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -3870,34 +3875,25 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>14700000</v>
+        <v>25000000</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Agentes contact center encuestas</t>
+          <t>Contact center ventas España</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Richard Castaño</t>
         </is>
       </c>
       <c r="G81" s="1" t="n">
-        <v>45916.65275462963</v>
-      </c>
-      <c r="H81" s="1" t="n">
-        <v>45930</v>
+        <v>45960.61145833333</v>
       </c>
       <c r="I81" t="n">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="J81" t="n">
-        <v>2025</v>
-      </c>
-      <c r="K81" t="n">
-        <v>9</v>
-      </c>
-      <c r="L81" t="n">
         <v>2025</v>
       </c>
       <c r="M81" t="inlineStr">

</xml_diff>

<commit_message>
CRM actualizado — 25/06/2026 09:39
</commit_message>
<xml_diff>
--- a/CRM_PowerBI_BrendaLuna_actualizado.xlsx
+++ b/CRM_PowerBI_BrendaLuna_actualizado.xlsx
@@ -946,20 +946,25 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>directoradjunto@dclass.edu.co</t>
+          <t>mercadeo@norteysur.co</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0</v>
+        <v>28190000</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Isabella Mesa</t>
+        </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Oportunidad de DCLASS ACADEMIA SAS</t>
+          <t>Oportunidad de Isabella Mesa</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -968,7 +973,7 @@
         </is>
       </c>
       <c r="G11" s="1" t="n">
-        <v>46189.49674768518</v>
+        <v>46191.70076388889</v>
       </c>
       <c r="I11" t="n">
         <v>25</v>
@@ -978,19 +983,19 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Belkis.jimenez@agrauto.com.co</t>
+          <t>comercial@asertis.com.co</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -998,7 +1003,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Oportunidad de AGRICOLA AUTOMOTRIZ SAS / BELKYS JIMENEZ</t>
+          <t>Oportunidad de IMPORTADORA CALI S.A.</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1007,24 +1012,24 @@
         </is>
       </c>
       <c r="G12" s="1" t="n">
-        <v>46182.67912037037</v>
+        <v>46189.67539351852</v>
       </c>
       <c r="I12" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J12" t="n">
         <v>2026</v>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>luisa.baena@automarcali.com</t>
+          <t>educacion@360forma.edu.co</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1037,12 +1042,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>luisa.baena@automarcali.com</t>
+          <t>Jorge Sanchez / jefe Comercial</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Oportunidad de luisa.baena@automarcali.com</t>
+          <t>Oportunidad de Jorge Sanchez / jefe Comercial</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1051,10 +1056,10 @@
         </is>
       </c>
       <c r="G13" s="1" t="n">
-        <v>46182.67809027778</v>
+        <v>46189.65077546296</v>
       </c>
       <c r="I13" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J13" t="n">
         <v>2026</v>
@@ -1068,25 +1073,20 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>directormercadeo@almotores.com</t>
+          <t>directoradjunto@dclass.edu.co</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C14" t="n">
         <v>0</v>
       </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Viviana Vanegas</t>
-        </is>
-      </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Oportunidad de Viviana Vanegas</t>
+          <t>Oportunidad de DCLASS ACADEMIA SAS</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1095,29 +1095,29 @@
         </is>
       </c>
       <c r="G14" s="1" t="n">
-        <v>46182.67621527778</v>
+        <v>46189.49674768518</v>
       </c>
       <c r="I14" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J14" t="n">
         <v>2026</v>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>xiomara.duran@autopacifico.com.co</t>
+          <t>Belkis.jimenez@agrauto.com.co</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -1125,7 +1125,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Oportunidad de xiomara.duran@autopacifico.com.co</t>
+          <t>Oportunidad de AGRICOLA AUTOMOTRIZ SAS / BELKYS JIMENEZ</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1134,7 +1134,7 @@
         </is>
       </c>
       <c r="G15" s="1" t="n">
-        <v>46182.65815972222</v>
+        <v>46182.67912037037</v>
       </c>
       <c r="I15" t="n">
         <v>24</v>
@@ -1144,14 +1144,14 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>alejandrosaavedraconde@comfandi.com.co</t>
+          <t>luisa.baena@automarcali.com</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1164,12 +1164,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>ALEJANDRO</t>
+          <t>luisa.baena@automarcali.com</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Oportunidad de ALEJANDRO</t>
+          <t>Oportunidad de luisa.baena@automarcali.com</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1178,7 +1178,7 @@
         </is>
       </c>
       <c r="G16" s="1" t="n">
-        <v>46182.64278935185</v>
+        <v>46182.67809027778</v>
       </c>
       <c r="I16" t="n">
         <v>24</v>
@@ -1195,20 +1195,25 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>administracion@fiando.com.co</t>
+          <t>directormercadeo@almotores.com</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C17" t="n">
         <v>0</v>
       </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Viviana Vanegas</t>
+        </is>
+      </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Oportunidad de FIANDO LTDA</t>
+          <t>Oportunidad de Viviana Vanegas</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1217,7 +1222,7 @@
         </is>
       </c>
       <c r="G17" s="1" t="n">
-        <v>46182.61304398148</v>
+        <v>46182.67621527778</v>
       </c>
       <c r="I17" t="n">
         <v>24</v>
@@ -1227,14 +1232,14 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>dgamoneda@productosdrogam.com</t>
+          <t>xiomara.duran@autopacifico.com.co</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1245,14 +1250,9 @@
       <c r="C18" t="n">
         <v>0</v>
       </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Diego Mauricio Gamoneda </t>
-        </is>
-      </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Oportunidad de Diego Mauricio Gamoneda </t>
+          <t>Oportunidad de xiomara.duran@autopacifico.com.co</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1261,10 +1261,10 @@
         </is>
       </c>
       <c r="G18" s="1" t="n">
-        <v>46175.66417824074</v>
+        <v>46182.65815972222</v>
       </c>
       <c r="I18" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J18" t="n">
         <v>2026</v>
@@ -1278,7 +1278,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>alexander.rojas@friogan.com</t>
+          <t>alejandrosaavedraconde@comfandi.com.co</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1289,9 +1289,14 @@
       <c r="C19" t="n">
         <v>0</v>
       </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>ALEJANDRO</t>
+        </is>
+      </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Oportunidad de FRIOGAN S.A</t>
+          <t>Oportunidad de ALEJANDRO</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1300,10 +1305,10 @@
         </is>
       </c>
       <c r="G19" s="1" t="n">
-        <v>46175.63597222222</v>
+        <v>46182.64278935185</v>
       </c>
       <c r="I19" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J19" t="n">
         <v>2026</v>
@@ -1315,9 +1320,14 @@
       </c>
     </row>
     <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>administracion@fiando.com.co</t>
+        </is>
+      </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -1325,7 +1335,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Oportunidad de Agromercados la Montaña</t>
+          <t>Oportunidad de FIANDO LTDA</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1334,10 +1344,10 @@
         </is>
       </c>
       <c r="G20" s="1" t="n">
-        <v>46175.62239583334</v>
+        <v>46182.61304398148</v>
       </c>
       <c r="I20" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J20" t="n">
         <v>2026</v>
@@ -1351,20 +1361,25 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>juand.rios@alkosto.com.co</t>
+          <t>dgamoneda@productosdrogam.com</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C21" t="n">
         <v>0</v>
       </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Diego Mauricio Gamoneda </t>
+        </is>
+      </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Oportunidad de ALKOSTO</t>
+          <t xml:space="preserve">Oportunidad de Diego Mauricio Gamoneda </t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1373,7 +1388,7 @@
         </is>
       </c>
       <c r="G21" s="1" t="n">
-        <v>46175.62055555556</v>
+        <v>46175.66417824074</v>
       </c>
       <c r="I21" t="n">
         <v>23</v>
@@ -1390,7 +1405,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>gerencia4087@grupo-exito.com</t>
+          <t>alexander.rojas@friogan.com</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1401,14 +1416,9 @@
       <c r="C22" t="n">
         <v>0</v>
       </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Grupo exito ‒ 1007386172 - Sneider Quirama</t>
-        </is>
-      </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Oportunidad de Grupo exito</t>
+          <t>Oportunidad de FRIOGAN S.A</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1417,7 +1427,7 @@
         </is>
       </c>
       <c r="G22" s="1" t="n">
-        <v>46175.61638888889</v>
+        <v>46175.63597222222</v>
       </c>
       <c r="I22" t="n">
         <v>23</v>
@@ -1432,11 +1442,6 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>ldgomez@supertiendascanaveral.com</t>
-        </is>
-      </c>
       <c r="B23" t="inlineStr">
         <is>
           <t>Nuevo</t>
@@ -1445,14 +1450,9 @@
       <c r="C23" t="n">
         <v>0</v>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Luis David Gomez</t>
-        </is>
-      </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Oportunidad de Luis David Gomez</t>
+          <t>Oportunidad de Agromercados la Montaña</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1461,7 +1461,7 @@
         </is>
       </c>
       <c r="G23" s="1" t="n">
-        <v>46175.60493055556</v>
+        <v>46175.62239583334</v>
       </c>
       <c r="I23" t="n">
         <v>23</v>
@@ -1478,12 +1478,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>davida_vanegas@coomeva.com.co</t>
+          <t>juand.rios@alkosto.com.co</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -1491,7 +1491,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Oportunidad de BANCOOMEVA</t>
+          <t>Oportunidad de ALKOSTO</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1500,7 +1500,7 @@
         </is>
       </c>
       <c r="G24" s="1" t="n">
-        <v>46175.47109953704</v>
+        <v>46175.62055555556</v>
       </c>
       <c r="I24" t="n">
         <v>23</v>
@@ -1517,12 +1517,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>alejandro.delgado@filedesk.com.co</t>
+          <t>gerencia4087@grupo-exito.com</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -1530,12 +1530,12 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>AlejandroDelgado</t>
+          <t>Grupo exito ‒ 1007386172 - Sneider Quirama</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Oportunidad de AlejandroDelgado</t>
+          <t>Oportunidad de Grupo exito</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1544,7 +1544,7 @@
         </is>
       </c>
       <c r="G25" s="1" t="n">
-        <v>46174.71665509259</v>
+        <v>46175.61638888889</v>
       </c>
       <c r="I25" t="n">
         <v>23</v>
@@ -1559,22 +1559,27 @@
       </c>
     </row>
     <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>ldgomez@supertiendascanaveral.com</t>
+        </is>
+      </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>35000000</v>
+        <v>0</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Olga Lucia Hurtado</t>
+          <t>Luis David Gomez</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Oportunidad de Olga Lucia Hurtado</t>
+          <t>Oportunidad de Luis David Gomez</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1583,10 +1588,10 @@
         </is>
       </c>
       <c r="G26" s="1" t="n">
-        <v>46168.49854166667</v>
+        <v>46175.60493055556</v>
       </c>
       <c r="I26" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="J26" t="n">
         <v>2026</v>
@@ -1600,7 +1605,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>comercial2@felsyn.com</t>
+          <t>davida_vanegas@coomeva.com.co</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1609,11 +1614,11 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>713400</v>
+        <v>0</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Oportunidad de FONDO DE EMPLEADOS FELSYN</t>
+          <t>Oportunidad de BANCOOMEVA</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1622,10 +1627,10 @@
         </is>
       </c>
       <c r="G27" s="1" t="n">
-        <v>46163.49130787037</v>
+        <v>46175.47109953704</v>
       </c>
       <c r="I27" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="J27" t="n">
         <v>2026</v>
@@ -1639,7 +1644,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>mercadeo@lasevillana.com.co</t>
+          <t>alejandro.delgado@filedesk.com.co</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1652,12 +1657,12 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fabio AlbertoGallego García </t>
+          <t>AlejandroDelgado</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Oportunidad de Fabio AlbertoGallego García </t>
+          <t>Oportunidad de AlejandroDelgado</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1666,10 +1671,10 @@
         </is>
       </c>
       <c r="G28" s="1" t="n">
-        <v>46162.64569444444</v>
+        <v>46174.71665509259</v>
       </c>
       <c r="I28" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="J28" t="n">
         <v>2026</v>
@@ -1681,22 +1686,22 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>asantiago@stop.com.co</t>
-        </is>
-      </c>
       <c r="B29" t="inlineStr">
         <is>
           <t>Contactado</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>0</v>
+        <v>35000000</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Olga Lucia Hurtado</t>
+        </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Oportunidad de STOP SAS</t>
+          <t>Oportunidad de Olga Lucia Hurtado</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1705,10 +1710,10 @@
         </is>
       </c>
       <c r="G29" s="1" t="n">
-        <v>46161.63508101852</v>
+        <v>46168.49854166667</v>
       </c>
       <c r="I29" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="J29" t="n">
         <v>2026</v>
@@ -1722,25 +1727,20 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>aestrada@teker.co</t>
+          <t>comercial2@felsyn.com</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>16914000</v>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>TEKER SALUD SAS</t>
-        </is>
+        <v>713400</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Oportunidad de TEKER SALUD SAS</t>
+          <t>Oportunidad de FONDO DE EMPLEADOS FELSYN</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1749,7 +1749,7 @@
         </is>
       </c>
       <c r="G30" s="1" t="n">
-        <v>46161.62922453704</v>
+        <v>46163.49130787037</v>
       </c>
       <c r="I30" t="n">
         <v>21</v>
@@ -1764,6 +1764,11 @@
       </c>
     </row>
     <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>mercadeo@lasevillana.com.co</t>
+        </is>
+      </c>
       <c r="B31" t="inlineStr">
         <is>
           <t>Contactado</t>
@@ -1772,9 +1777,14 @@
       <c r="C31" t="n">
         <v>0</v>
       </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fabio AlbertoGallego García </t>
+        </is>
+      </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Oportunidad de TIAN IPS SAS</t>
+          <t xml:space="preserve">Oportunidad de Fabio AlbertoGallego García </t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1783,7 +1793,7 @@
         </is>
       </c>
       <c r="G31" s="1" t="n">
-        <v>46161.61643518518</v>
+        <v>46162.64569444444</v>
       </c>
       <c r="I31" t="n">
         <v>21</v>
@@ -1800,25 +1810,20 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>administración@fullredtotal.com</t>
+          <t>asantiago@stop.com.co</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>14000000</v>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Eivar Eñasco</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Oportunidad de Eivar Eñasco</t>
+          <t>Oportunidad de STOP SAS</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1827,42 +1832,42 @@
         </is>
       </c>
       <c r="G32" s="1" t="n">
-        <v>46154.67546296296</v>
+        <v>46161.63508101852</v>
       </c>
       <c r="I32" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J32" t="n">
         <v>2026</v>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>cserna@surtifamiliar.com.co</t>
+          <t>aestrada@teker.co</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Negociación</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>1950000</v>
+        <v>16914000</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Claudia Patricia Serna</t>
+          <t>TEKER SALUD SAS</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Oportunidad de Claudia Patricia Serna</t>
+          <t>Oportunidad de TEKER SALUD SAS</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1871,42 +1876,32 @@
         </is>
       </c>
       <c r="G33" s="1" t="n">
-        <v>46154.66616898148</v>
+        <v>46161.62922453704</v>
       </c>
       <c r="I33" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J33" t="n">
         <v>2026</v>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>coordmercadeo@pacificcenter.co</t>
-        </is>
-      </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>5600000</v>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Claudia Castro</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Oportunidad de Claudia Castro</t>
+          <t>Oportunidad de TIAN IPS SAS</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1915,24 +1910,24 @@
         </is>
       </c>
       <c r="G34" s="1" t="n">
-        <v>46154.66341435185</v>
+        <v>46161.61643518518</v>
       </c>
       <c r="I34" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J34" t="n">
         <v>2026</v>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>isabellarengifo27@gmail.com</t>
+          <t>administración@fullredtotal.com</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1941,16 +1936,16 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>28190000</v>
+        <v>14000000</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Isabella Rengifo</t>
+          <t>Eivar Eñasco</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Oportunidad de Isabella Rengifo</t>
+          <t>Oportunidad de Eivar Eñasco</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1959,7 +1954,7 @@
         </is>
       </c>
       <c r="G35" s="1" t="n">
-        <v>46154.65981481481</v>
+        <v>46154.67546296296</v>
       </c>
       <c r="I35" t="n">
         <v>20</v>
@@ -1974,34 +1969,36 @@
       </c>
     </row>
     <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>cserna@surtifamiliar.com.co</t>
+        </is>
+      </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Negociación</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>50000000</v>
+        <v>1950000</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Paola Gómez - Agente Inmobiliaria Independiente</t>
+          <t>Claudia Patricia Serna</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Puesto de Trabajo CC Medellin</t>
+          <t>Oportunidad de Claudia Patricia Serna</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Richard Castaño</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G36" s="1" t="n">
-        <v>46154.49104166667</v>
-      </c>
-      <c r="H36" s="1" t="n">
-        <v>46170</v>
+        <v>46154.66616898148</v>
       </c>
       <c r="I36" t="n">
         <v>20</v>
@@ -2009,44 +2006,43 @@
       <c r="J36" t="n">
         <v>2026</v>
       </c>
-      <c r="K36" t="n">
-        <v>5</v>
-      </c>
-      <c r="L36" t="n">
-        <v>2026</v>
-      </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>alberto.ramirez@constructorabolivar.com</t>
+          <t>coordmercadeo@pacificcenter.co</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Ganado</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>3000000</v>
+        <v>5600000</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Claudia Castro</t>
+        </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Oportunidad de NPS Relacional</t>
+          <t>Oportunidad de Claudia Castro</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G37" s="1" t="n">
-        <v>46154.44511574074</v>
+        <v>46154.66341435185</v>
       </c>
       <c r="I37" t="n">
         <v>20</v>
@@ -2061,22 +2057,27 @@
       </c>
     </row>
     <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>isabellarengifo27@gmail.com</t>
+        </is>
+      </c>
       <c r="B38" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>3000000</v>
+        <v>28190000</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>MADERKIT</t>
+          <t>Isabella Rengifo</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Oportunidad de MADERKIT</t>
+          <t>Oportunidad de Isabella Rengifo</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2085,10 +2086,10 @@
         </is>
       </c>
       <c r="G38" s="1" t="n">
-        <v>46147.66540509259</v>
+        <v>46154.65981481481</v>
       </c>
       <c r="I38" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J38" t="n">
         <v>2026</v>
@@ -2100,41 +2101,45 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>omer120395@gmail.com</t>
-        </is>
-      </c>
       <c r="B39" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>0</v>
+        <v>50000000</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Omer Peñaloza</t>
+          <t>Paola Gómez - Agente Inmobiliaria Independiente</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Oportunidad de Omer Peñaloza</t>
+          <t>Puesto de Trabajo CC Medellin</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Richard Castaño</t>
         </is>
       </c>
       <c r="G39" s="1" t="n">
-        <v>46147.66090277778</v>
+        <v>46154.49104166667</v>
+      </c>
+      <c r="H39" s="1" t="n">
+        <v>46170</v>
       </c>
       <c r="I39" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J39" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K39" t="n">
+        <v>5</v>
+      </c>
+      <c r="L39" t="n">
         <v>2026</v>
       </c>
       <c r="M39" t="inlineStr">
@@ -2146,68 +2151,59 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>directora.it@supermercadobelalcazar.com.co</t>
+          <t>alberto.ramirez@constructorabolivar.com</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
+          <t>Ganado</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Oportunidad de NPS Relacional</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Jennifer Hoyos Gallego</t>
+        </is>
+      </c>
+      <c r="G40" s="1" t="n">
+        <v>46154.44511574074</v>
+      </c>
+      <c r="I40" t="n">
+        <v>20</v>
+      </c>
+      <c r="J40" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>Calificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" t="inlineStr">
+        <is>
           <t>Perdido</t>
         </is>
       </c>
-      <c r="C40" t="n">
-        <v>6000000</v>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>Oportunidad de ABASTECEMOS DE OCCIDENTE</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G40" s="1" t="n">
-        <v>46147.64170138889</v>
-      </c>
-      <c r="H40" s="1" t="n">
-        <v>46157</v>
-      </c>
-      <c r="I40" t="n">
-        <v>19</v>
-      </c>
-      <c r="J40" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K40" t="n">
-        <v>5</v>
-      </c>
-      <c r="L40" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M40" t="inlineStr">
-        <is>
-          <t>No calificado</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>oscar.molina@terrenoshouston.com</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>Seguimiento</t>
-        </is>
-      </c>
       <c r="C41" t="n">
-        <v>37623040</v>
+        <v>3000000</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>MADERKIT</t>
+        </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Oportunidad de COLONY RIDGE</t>
+          <t>Oportunidad de MADERKIT</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2216,10 +2212,7 @@
         </is>
       </c>
       <c r="G41" s="1" t="n">
-        <v>46147.60297453704</v>
-      </c>
-      <c r="H41" s="1" t="n">
-        <v>46150</v>
+        <v>46147.66540509259</v>
       </c>
       <c r="I41" t="n">
         <v>19</v>
@@ -2227,12 +2220,6 @@
       <c r="J41" t="n">
         <v>2026</v>
       </c>
-      <c r="K41" t="n">
-        <v>5</v>
-      </c>
-      <c r="L41" t="n">
-        <v>2026</v>
-      </c>
       <c r="M41" t="inlineStr">
         <is>
           <t>No calificado</t>
@@ -2242,20 +2229,25 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>jsantacr@ccc.org.co</t>
+          <t>omer120395@gmail.com</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>55000000</v>
+        <v>0</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Omer Peñaloza</t>
+        </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Oportunidad de CAMARA DE COMERCIO CALI</t>
+          <t>Oportunidad de Omer Peñaloza</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -2264,21 +2256,12 @@
         </is>
       </c>
       <c r="G42" s="1" t="n">
-        <v>46141.62370370371</v>
-      </c>
-      <c r="H42" s="1" t="n">
-        <v>46289</v>
+        <v>46147.66090277778</v>
       </c>
       <c r="I42" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J42" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K42" t="n">
-        <v>9</v>
-      </c>
-      <c r="L42" t="n">
         <v>2026</v>
       </c>
       <c r="M42" t="inlineStr">
@@ -2290,7 +2273,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>exportaciones@laprovincia.com</t>
+          <t>directora.it@supermercadobelalcazar.com.co</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2303,7 +2286,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Oportunidad de PRODUCTOS LA PROVINCIA SAS</t>
+          <t>Oportunidad de ABASTECEMOS DE OCCIDENTE</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2312,12 +2295,21 @@
         </is>
       </c>
       <c r="G43" s="1" t="n">
-        <v>46141.62021990741</v>
+        <v>46147.64170138889</v>
+      </c>
+      <c r="H43" s="1" t="n">
+        <v>46157</v>
       </c>
       <c r="I43" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J43" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K43" t="n">
+        <v>5</v>
+      </c>
+      <c r="L43" t="n">
         <v>2026</v>
       </c>
       <c r="M43" t="inlineStr">
@@ -2329,20 +2321,20 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>coordinador.mercadeo@regency.com.co</t>
+          <t>oscar.molina@terrenoshouston.com</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Seguimiento</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>0</v>
+        <v>37623040</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Oportunidad de REGENCY TECH SAS</t>
+          <t>Oportunidad de COLONY RIDGE</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -2351,14 +2343,23 @@
         </is>
       </c>
       <c r="G44" s="1" t="n">
-        <v>46141.59664351852</v>
+        <v>46147.60297453704</v>
+      </c>
+      <c r="H44" s="1" t="n">
+        <v>46150</v>
       </c>
       <c r="I44" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J44" t="n">
         <v>2026</v>
       </c>
+      <c r="K44" t="n">
+        <v>5</v>
+      </c>
+      <c r="L44" t="n">
+        <v>2026</v>
+      </c>
       <c r="M44" t="inlineStr">
         <is>
           <t>No calificado</t>
@@ -2366,17 +2367,22 @@
       </c>
     </row>
     <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>jsantacr@ccc.org.co</t>
+        </is>
+      </c>
       <c r="B45" t="inlineStr">
         <is>
           <t>Contactado</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>1200000</v>
+        <v>55000000</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Oportunidad de EMCALI E.I.C.E ESP</t>
+          <t>Oportunidad de CAMARA DE COMERCIO CALI</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -2385,10 +2391,10 @@
         </is>
       </c>
       <c r="G45" s="1" t="n">
-        <v>46141.59045138889</v>
+        <v>46141.62370370371</v>
       </c>
       <c r="H45" s="1" t="n">
-        <v>46352</v>
+        <v>46289</v>
       </c>
       <c r="I45" t="n">
         <v>18</v>
@@ -2397,7 +2403,7 @@
         <v>2026</v>
       </c>
       <c r="K45" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="L45" t="n">
         <v>2026</v>
@@ -2411,12 +2417,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>angie_feligrana@eficacia.com.co</t>
+          <t>exportaciones@laprovincia.com</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Seguimiento</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -2424,7 +2430,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Oportunidad de Eficacia sas / Angie Feligrana</t>
+          <t>Oportunidad de PRODUCTOS LA PROVINCIA SAS</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2433,21 +2439,12 @@
         </is>
       </c>
       <c r="G46" s="1" t="n">
-        <v>46126.63210648148</v>
-      </c>
-      <c r="H46" s="1" t="n">
-        <v>46150</v>
+        <v>46141.62021990741</v>
       </c>
       <c r="I46" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J46" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K46" t="n">
-        <v>5</v>
-      </c>
-      <c r="L46" t="n">
         <v>2026</v>
       </c>
       <c r="M46" t="inlineStr">
@@ -2459,7 +2456,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Estrategiadigital@zuluagaysoto.com</t>
+          <t>coordinador.mercadeo@regency.com.co</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2470,14 +2467,9 @@
       <c r="C47" t="n">
         <v>0</v>
       </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>Maryuri Arguello</t>
-        </is>
-      </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Oportunidad de Maryuri Arguello</t>
+          <t>Oportunidad de REGENCY TECH SAS</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -2486,10 +2478,10 @@
         </is>
       </c>
       <c r="G47" s="1" t="n">
-        <v>46125.71925925926</v>
+        <v>46141.59664351852</v>
       </c>
       <c r="I47" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J47" t="n">
         <v>2026</v>
@@ -2501,75 +2493,65 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>gabrielrodriguez@arrozsupremo.com</t>
-        </is>
-      </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Ganado</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>8000000</v>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>GABRIEL RODRIGUEZ</t>
-        </is>
+        <v>1200000</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Agente de Ventas</t>
+          <t>Oportunidad de EMCALI E.I.C.E ESP</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Richard Castaño</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G48" s="1" t="n">
-        <v>46119.62108796297</v>
+        <v>46141.59045138889</v>
       </c>
       <c r="H48" s="1" t="n">
-        <v>46141</v>
+        <v>46352</v>
       </c>
       <c r="I48" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="J48" t="n">
         <v>2026</v>
       </c>
       <c r="K48" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="L48" t="n">
         <v>2026</v>
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Belkis.jimenez@agrauto.com.co</t>
+          <t>angie_feligrana@eficacia.com.co</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Seguimiento</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>0</v>
+        <v>6000000</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Oportunidad de AGRICOLA AUTOMOTRIZ SAS</t>
+          <t>Oportunidad de Eficacia sas / Angie Feligrana</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -2578,12 +2560,21 @@
         </is>
       </c>
       <c r="G49" s="1" t="n">
-        <v>46119.38914351852</v>
+        <v>46126.63210648148</v>
+      </c>
+      <c r="H49" s="1" t="n">
+        <v>46150</v>
       </c>
       <c r="I49" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J49" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K49" t="n">
+        <v>5</v>
+      </c>
+      <c r="L49" t="n">
         <v>2026</v>
       </c>
       <c r="M49" t="inlineStr">
@@ -2595,7 +2586,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>anyela.aponza@cotel.com.co</t>
+          <t>Estrategiadigital@zuluagaysoto.com</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2606,9 +2597,14 @@
       <c r="C50" t="n">
         <v>0</v>
       </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Maryuri Arguello</t>
+        </is>
+      </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Oportunidad de COTEL SAL</t>
+          <t>Oportunidad de Maryuri Arguello</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -2617,10 +2613,10 @@
         </is>
       </c>
       <c r="G50" s="1" t="n">
-        <v>46112.61271990741</v>
+        <v>46125.71925925926</v>
       </c>
       <c r="I50" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="J50" t="n">
         <v>2026</v>
@@ -2634,51 +2630,60 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>liliana.patino@quironsalud.com</t>
+          <t>gabrielrodriguez@arrozsupremo.com</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Ganado</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>0</v>
+        <v>8000000</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>CLINICA IMBANACO</t>
+          <t>GABRIEL RODRIGUEZ</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Oportunidad de Liliana Patiño Flórez</t>
+          <t>Agente de Ventas</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Richard Castaño</t>
         </is>
       </c>
       <c r="G51" s="1" t="n">
-        <v>46112.60853009259</v>
+        <v>46119.62108796297</v>
+      </c>
+      <c r="H51" s="1" t="n">
+        <v>46141</v>
       </c>
       <c r="I51" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="J51" t="n">
         <v>2026</v>
       </c>
+      <c r="K51" t="n">
+        <v>4</v>
+      </c>
+      <c r="L51" t="n">
+        <v>2026</v>
+      </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>casanchez@jgb.com.co</t>
+          <t>Belkis.jimenez@agrauto.com.co</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2691,7 +2696,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Oportunidad de JGB S.A.</t>
+          <t>Oportunidad de AGRICOLA AUTOMOTRIZ SAS</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -2700,10 +2705,10 @@
         </is>
       </c>
       <c r="G52" s="1" t="n">
-        <v>46112.6052662037</v>
+        <v>46119.38914351852</v>
       </c>
       <c r="I52" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="J52" t="n">
         <v>2026</v>
@@ -2717,12 +2722,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>damaris.gomez@disfarma.com.co</t>
+          <t>anyela.aponza@cotel.com.co</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Seguimiento</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -2730,7 +2735,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Oportunidad de DISFARMA</t>
+          <t>Oportunidad de COTEL SAL</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -2739,7 +2744,7 @@
         </is>
       </c>
       <c r="G53" s="1" t="n">
-        <v>46112.60325231482</v>
+        <v>46112.61271990741</v>
       </c>
       <c r="I53" t="n">
         <v>14</v>
@@ -2756,7 +2761,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>alergologosdeoccidente@gmail.com</t>
+          <t>liliana.patino@quironsalud.com</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2769,12 +2774,12 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Johana Gonzalez</t>
+          <t>CLINICA IMBANACO</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Oportunidad de Johana Gonzalez</t>
+          <t>Oportunidad de Liliana Patiño Flórez</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -2783,10 +2788,10 @@
         </is>
       </c>
       <c r="G54" s="1" t="n">
-        <v>46107.51248842593</v>
+        <v>46112.60853009259</v>
       </c>
       <c r="I54" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J54" t="n">
         <v>2026</v>
@@ -2800,60 +2805,51 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>DavidEsteban.Porras@alfalaval.com</t>
+          <t>casanchez@jgb.com.co</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Ganado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>15000000</v>
+        <v>0</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Oportunidad de OPORTUNIDAD ENCUESTAS ALFALAVAL</t>
+          <t>Oportunidad de JGB S.A.</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G55" s="1" t="n">
-        <v>46101.72893518519</v>
-      </c>
-      <c r="H55" s="1" t="n">
-        <v>46141</v>
+        <v>46112.6052662037</v>
       </c>
       <c r="I55" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="J55" t="n">
         <v>2026</v>
       </c>
-      <c r="K55" t="n">
-        <v>4</v>
-      </c>
-      <c r="L55" t="n">
-        <v>2026</v>
-      </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Dr.arcarmona@gmail.com</t>
+          <t>damaris.gomez@disfarma.com.co</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Seguimiento</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -2861,7 +2857,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Oportunidad de GAMANUCLEAR LTDA - Dr Alberto Carmona</t>
+          <t>Oportunidad de DISFARMA</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -2870,10 +2866,10 @@
         </is>
       </c>
       <c r="G56" s="1" t="n">
-        <v>46098.65114583333</v>
+        <v>46112.60325231482</v>
       </c>
       <c r="I56" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="J56" t="n">
         <v>2026</v>
@@ -2887,7 +2883,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>cecilia.guevara@cosmitet.net / administracion.crd@cosmitet.net</t>
+          <t>alergologosdeoccidente@gmail.com</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2900,12 +2896,12 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Cecilia Guevara</t>
+          <t>Johana Gonzalez</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Oportunidad de CLINICA REY DAVID Walter Charria</t>
+          <t>Oportunidad de Johana Gonzalez</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -2914,10 +2910,10 @@
         </is>
       </c>
       <c r="G57" s="1" t="n">
-        <v>46094.69002314815</v>
+        <v>46107.51248842593</v>
       </c>
       <c r="I57" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="J57" t="n">
         <v>2026</v>
@@ -2931,104 +2927,94 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>vicerrectoriacademica@unicatolica.edu.co</t>
+          <t>DavidEsteban.Porras@alfalaval.com</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Ganado</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>0</v>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>Jorge Silva</t>
-        </is>
+        <v>15000000</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Oportunidad de Jorge Silva</t>
+          <t>Oportunidad de OPORTUNIDAD ENCUESTAS ALFALAVAL</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G58" s="1" t="n">
-        <v>46094.66880787037</v>
+        <v>46101.72893518519</v>
+      </c>
+      <c r="H58" s="1" t="n">
+        <v>46141</v>
       </c>
       <c r="I58" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J58" t="n">
         <v>2026</v>
       </c>
+      <c r="K58" t="n">
+        <v>4</v>
+      </c>
+      <c r="L58" t="n">
+        <v>2026</v>
+      </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>pedroperea02@gmail.com</t>
+          <t>Dr.arcarmona@gmail.com</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Ganado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>2160000</v>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>Pedro Pablo Perea Mafla</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Oportunidad de Encuestas</t>
+          <t>Oportunidad de GAMANUCLEAR LTDA - Dr Alberto Carmona</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G59" s="1" t="n">
-        <v>46094.65905092593</v>
-      </c>
-      <c r="H59" s="1" t="n">
-        <v>46141</v>
+        <v>46098.65114583333</v>
       </c>
       <c r="I59" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J59" t="n">
         <v>2026</v>
       </c>
-      <c r="K59" t="n">
-        <v>4</v>
-      </c>
-      <c r="L59" t="n">
-        <v>2026</v>
-      </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>cristina.papamija@bmm.com.co</t>
+          <t>cecilia.guevara@cosmitet.net / administracion.crd@cosmitet.net</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -3037,20 +3023,25 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>8071000</v>
+        <v>0</v>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Cecilia Guevara</t>
+        </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Oportunidad de BANCO MUNDO MUJER</t>
+          <t>Oportunidad de CLINICA REY DAVID Walter Charria</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G60" s="1" t="n">
-        <v>46094.65019675926</v>
+        <v>46094.69002314815</v>
       </c>
       <c r="I60" t="n">
         <v>11</v>
@@ -3067,7 +3058,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>capacitacionvirtual@fundacionwwbcol.org</t>
+          <t>vicerrectoriacademica@unicatolica.edu.co</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -3076,20 +3067,25 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>1600000</v>
+        <v>0</v>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Jorge Silva</t>
+        </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Licenciamiento y ajuste WhatsApp FUNDACIÓN WWB</t>
+          <t>Oportunidad de Jorge Silva</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G61" s="1" t="n">
-        <v>46094.64826388889</v>
+        <v>46094.66880787037</v>
       </c>
       <c r="I61" t="n">
         <v>11</v>
@@ -3106,7 +3102,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>carol.cuesta@cbolivar.com</t>
+          <t>pedroperea02@gmail.com</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -3115,16 +3111,16 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>2900000</v>
+        <v>2160000</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>CAROL CUESTA</t>
+          <t>Pedro Pablo Perea Mafla</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Gestión de Subsidios CB Bogotá</t>
+          <t>Oportunidad de Encuestas</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -3133,10 +3129,10 @@
         </is>
       </c>
       <c r="G62" s="1" t="n">
-        <v>46094.64454861111</v>
+        <v>46094.65905092593</v>
       </c>
       <c r="H62" s="1" t="n">
-        <v>46135</v>
+        <v>46141</v>
       </c>
       <c r="I62" t="n">
         <v>11</v>
@@ -3159,7 +3155,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>edwin.munoz.v@uniminuto.edu</t>
+          <t>cristina.papamija@bmm.com.co</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3168,20 +3164,20 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>0</v>
+        <v>8071000</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Oportunidad de UNIMINUTO</t>
+          <t>Oportunidad de BANCO MUNDO MUJER</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G63" s="1" t="n">
-        <v>46092.63626157407</v>
+        <v>46094.65019675926</v>
       </c>
       <c r="I63" t="n">
         <v>11</v>
@@ -3198,7 +3194,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>jaime_zuluaga@eficacia.com.co</t>
+          <t>capacitacionvirtual@fundacionwwbcol.org</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3207,25 +3203,20 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>0</v>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>Jaime Alberto</t>
-        </is>
+        <v>1600000</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Oportunidad de Jaime Alberto Zuluaga</t>
+          <t>Licenciamiento y ajuste WhatsApp FUNDACIÓN WWB</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G64" s="1" t="n">
-        <v>46092.63153935185</v>
+        <v>46094.64826388889</v>
       </c>
       <c r="I64" t="n">
         <v>11</v>
@@ -3242,34 +3233,37 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>comercial@isyscol.com</t>
+          <t>carol.cuesta@cbolivar.com</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Ganado</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>0</v>
+        <v>2900000</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Andres Nader</t>
+          <t>CAROL CUESTA</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Oportunidad de Andres Nader</t>
+          <t>Gestión de Subsidios CB Bogotá</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G65" s="1" t="n">
-        <v>46091.59211805555</v>
+        <v>46094.64454861111</v>
+      </c>
+      <c r="H65" s="1" t="n">
+        <v>46135</v>
       </c>
       <c r="I65" t="n">
         <v>11</v>
@@ -3277,16 +3271,22 @@
       <c r="J65" t="n">
         <v>2026</v>
       </c>
+      <c r="K65" t="n">
+        <v>4</v>
+      </c>
+      <c r="L65" t="n">
+        <v>2026</v>
+      </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>mercadeo@norteysur.co</t>
+          <t>edwin.munoz.v@uniminuto.edu</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -3297,14 +3297,9 @@
       <c r="C66" t="n">
         <v>0</v>
       </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>Isabella Mesa</t>
-        </is>
-      </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Oportunidad de Isabella Mesa</t>
+          <t>Oportunidad de UNIMINUTO</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -3313,7 +3308,7 @@
         </is>
       </c>
       <c r="G66" s="1" t="n">
-        <v>46091.40078703704</v>
+        <v>46092.63626157407</v>
       </c>
       <c r="I66" t="n">
         <v>11</v>
@@ -3328,6 +3323,11 @@
       </c>
     </row>
     <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>jaime_zuluaga@eficacia.com.co</t>
+        </is>
+      </c>
       <c r="B67" t="inlineStr">
         <is>
           <t>Perdido</t>
@@ -3336,18 +3336,23 @@
       <c r="C67" t="n">
         <v>0</v>
       </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Jaime Alberto</t>
+        </is>
+      </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Clasificación EMAIL Comfenalco Cartagena</t>
+          <t>Oportunidad de Jaime Alberto Zuluaga</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Maria Fernanda Gaviria</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G67" s="1" t="n">
-        <v>46091.3665625</v>
+        <v>46092.63153935185</v>
       </c>
       <c r="I67" t="n">
         <v>11</v>
@@ -3362,6 +3367,11 @@
       </c>
     </row>
     <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>comercial@isyscol.com</t>
+        </is>
+      </c>
       <c r="B68" t="inlineStr">
         <is>
           <t>Perdido</t>
@@ -3370,21 +3380,26 @@
       <c r="C68" t="n">
         <v>0</v>
       </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Andres Nader</t>
+        </is>
+      </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Oportunidad de ESE HOSPITAL LA MARIA</t>
+          <t>Oportunidad de Andres Nader</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Laura Alejandra Castañeda</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G68" s="1" t="n">
-        <v>46083.67605324074</v>
+        <v>46091.59211805555</v>
       </c>
       <c r="I68" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J68" t="n">
         <v>2026</v>
@@ -3396,6 +3411,11 @@
       </c>
     </row>
     <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>mercadeo@norteysur.co</t>
+        </is>
+      </c>
       <c r="B69" t="inlineStr">
         <is>
           <t>Perdido</t>
@@ -3404,21 +3424,26 @@
       <c r="C69" t="n">
         <v>0</v>
       </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Isabella Mesa</t>
+        </is>
+      </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Oportunidad de SUPER TRANSPORTE</t>
+          <t>Oportunidad de Isabella Mesa</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Laura Alejandra Castañeda</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G69" s="1" t="n">
-        <v>46083.6706712963</v>
+        <v>46091.40078703704</v>
       </c>
       <c r="I69" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J69" t="n">
         <v>2026</v>
@@ -3440,146 +3465,121 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
+          <t>Clasificación EMAIL Comfenalco Cartagena</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Maria Fernanda Gaviria</t>
+        </is>
+      </c>
+      <c r="G70" s="1" t="n">
+        <v>46091.3665625</v>
+      </c>
+      <c r="I70" t="n">
+        <v>11</v>
+      </c>
+      <c r="J70" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>No calificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>0</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Oportunidad de ESE HOSPITAL LA MARIA</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Laura Alejandra Castañeda</t>
+        </is>
+      </c>
+      <c r="G71" s="1" t="n">
+        <v>46083.67605324074</v>
+      </c>
+      <c r="I71" t="n">
+        <v>10</v>
+      </c>
+      <c r="J71" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>No calificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>0</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Oportunidad de SUPER TRANSPORTE</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Laura Alejandra Castañeda</t>
+        </is>
+      </c>
+      <c r="G72" s="1" t="n">
+        <v>46083.6706712963</v>
+      </c>
+      <c r="I72" t="n">
+        <v>10</v>
+      </c>
+      <c r="J72" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>No calificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>0</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
           <t>Oportunidad de ENLACES IP S.A.S</t>
         </is>
       </c>
-      <c r="F70" t="inlineStr">
+      <c r="F73" t="inlineStr">
         <is>
           <t>Laura Alejandra Castañeda</t>
         </is>
       </c>
-      <c r="G70" s="1" t="n">
+      <c r="G73" s="1" t="n">
         <v>46083.50145833333</v>
       </c>
-      <c r="I70" t="n">
+      <c r="I73" t="n">
         <v>10</v>
-      </c>
-      <c r="J70" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M70" t="inlineStr">
-        <is>
-          <t>No calificado</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>accounting@diaza.com</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C71" t="n">
-        <v>0</v>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>JOHANA RODRIGUEZ</t>
-        </is>
-      </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>Oportunidad de JOHANA RODRIGUEZ</t>
-        </is>
-      </c>
-      <c r="F71" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G71" s="1" t="n">
-        <v>46079.73486111111</v>
-      </c>
-      <c r="I71" t="n">
-        <v>9</v>
-      </c>
-      <c r="J71" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M71" t="inlineStr">
-        <is>
-          <t>No calificado</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>mensajeriamyr@gmail.com</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C72" t="n">
-        <v>0</v>
-      </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>Oportunidad de MENSAJERIA M&amp;R SAS</t>
-        </is>
-      </c>
-      <c r="F72" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G72" s="1" t="n">
-        <v>46079.72262731481</v>
-      </c>
-      <c r="I72" t="n">
-        <v>9</v>
-      </c>
-      <c r="J72" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M72" t="inlineStr">
-        <is>
-          <t>No calificado</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>sistemaspanaderialeal@gmail.com</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C73" t="n">
-        <v>0</v>
-      </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>Diego Rios</t>
-        </is>
-      </c>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>JAMDAC SAS, Diego Rios</t>
-        </is>
-      </c>
-      <c r="F73" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G73" s="1" t="n">
-        <v>46071.63706018519</v>
-      </c>
-      <c r="I73" t="n">
-        <v>8</v>
       </c>
       <c r="J73" t="n">
         <v>2026</v>
@@ -3593,7 +3593,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>efernandez@unico.com.co</t>
+          <t>accounting@diaza.com</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -3606,12 +3606,12 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Erick Fernandez</t>
+          <t>JOHANA RODRIGUEZ</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Oportunidad de Erick Fernandez</t>
+          <t>Oportunidad de JOHANA RODRIGUEZ</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -3620,10 +3620,10 @@
         </is>
       </c>
       <c r="G74" s="1" t="n">
-        <v>46064.3750462963</v>
+        <v>46079.73486111111</v>
       </c>
       <c r="I74" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="J74" t="n">
         <v>2026</v>
@@ -3637,7 +3637,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>kabenitez@icesi.edu.co</t>
+          <t>mensajeriamyr@gmail.com</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -3646,28 +3646,23 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>10000000</v>
-      </c>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>KENI BENITEZ</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Oportunidad de KENI BENITEZ</t>
+          <t>Oportunidad de MENSAJERIA M&amp;R SAS</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G75" s="1" t="n">
-        <v>46059.34918981481</v>
+        <v>46079.72262731481</v>
       </c>
       <c r="I75" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J75" t="n">
         <v>2026</v>
@@ -3681,7 +3676,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>patovar@uao.edu.co</t>
+          <t>sistemaspanaderialeal@gmail.com</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -3694,12 +3689,12 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Paula Tovar</t>
+          <t>Diego Rios</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Oportunidad de UNIVERSIDAD AUTONOMA DE OCCIDENTE</t>
+          <t>JAMDAC SAS, Diego Rios</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -3708,10 +3703,10 @@
         </is>
       </c>
       <c r="G76" s="1" t="n">
-        <v>46058.72516203704</v>
+        <v>46071.63706018519</v>
       </c>
       <c r="I76" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J76" t="n">
         <v>2026</v>
@@ -3725,7 +3720,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>comercial@isyscol.com</t>
+          <t>efernandez@unico.com.co</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -3736,9 +3731,14 @@
       <c r="C77" t="n">
         <v>0</v>
       </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Erick Fernandez</t>
+        </is>
+      </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Oportunidad de TECNOLOGIAS ISYSCOL SAS</t>
+          <t>Oportunidad de Erick Fernandez</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -3747,10 +3747,10 @@
         </is>
       </c>
       <c r="G77" s="1" t="n">
-        <v>46057.58993055556</v>
+        <v>46064.3750462963</v>
       </c>
       <c r="I77" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J77" t="n">
         <v>2026</v>
@@ -3762,26 +3762,36 @@
       </c>
     </row>
     <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>kabenitez@icesi.edu.co</t>
+        </is>
+      </c>
       <c r="B78" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>15000000</v>
+        <v>10000000</v>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>KENI BENITEZ</t>
+        </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Oportunidad de VOICE IA EFICACIA</t>
+          <t>Oportunidad de KENI BENITEZ</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G78" s="1" t="n">
-        <v>46057.3409837963</v>
+        <v>46059.34918981481</v>
       </c>
       <c r="I78" t="n">
         <v>6</v>
@@ -3796,29 +3806,39 @@
       </c>
     </row>
     <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>patovar@uao.edu.co</t>
+        </is>
+      </c>
       <c r="B79" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>4000000</v>
+        <v>0</v>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Paula Tovar</t>
+        </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Oportunidad de Eficacia WhatsApp</t>
+          <t>Oportunidad de UNIVERSIDAD AUTONOMA DE OCCIDENTE</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G79" s="1" t="n">
-        <v>46049.67292824074</v>
+        <v>46058.72516203704</v>
       </c>
       <c r="I79" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J79" t="n">
         <v>2026</v>
@@ -3830,32 +3850,37 @@
       </c>
     </row>
     <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>comercial@isyscol.com</t>
+        </is>
+      </c>
       <c r="B80" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>20000000</v>
+        <v>0</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Oportunidad de CRUZ ROJA COLOMBIANA SECCIONAL VALLE DEL CAUCA</t>
+          <t>Oportunidad de TECNOLOGIAS ISYSCOL SAS</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G80" s="1" t="n">
-        <v>46006.49650462963</v>
+        <v>46057.58993055556</v>
       </c>
       <c r="I80" t="n">
-        <v>51</v>
+        <v>6</v>
       </c>
       <c r="J80" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="M80" t="inlineStr">
         <is>
@@ -3864,37 +3889,32 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t>silvia.figueroa@neurithmedia.com</t>
-        </is>
-      </c>
       <c r="B81" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>25000000</v>
+        <v>15000000</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Contact center ventas España</t>
+          <t>Oportunidad de VOICE IA EFICACIA</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Richard Castaño</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G81" s="1" t="n">
-        <v>45960.61145833333</v>
+        <v>46057.3409837963</v>
       </c>
       <c r="I81" t="n">
-        <v>44</v>
+        <v>6</v>
       </c>
       <c r="J81" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="M81" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
CRM actualizado — 14/07/2026 15:28
</commit_message>
<xml_diff>
--- a/CRM_PowerBI_BrendaLuna_actualizado.xlsx
+++ b/CRM_PowerBI_BrendaLuna_actualizado.xlsx
@@ -946,25 +946,20 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>mercadeo@norteysur.co</t>
+          <t>Servicios@procana.oeg</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Ganado</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>28190000</v>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Isabella Mesa</t>
-        </is>
+        <v>9000000</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Oportunidad de Isabella Mesa</t>
+          <t>Oportunidad de PROCAÑA</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -973,12 +968,21 @@
         </is>
       </c>
       <c r="G11" s="1" t="n">
-        <v>46191.70076388889</v>
+        <v>46198.45984953704</v>
+      </c>
+      <c r="H11" s="1" t="n">
+        <v>46217</v>
       </c>
       <c r="I11" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="J11" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K11" t="n">
+        <v>7</v>
+      </c>
+      <c r="L11" t="n">
         <v>2026</v>
       </c>
       <c r="M11" t="inlineStr">
@@ -990,7 +994,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>comercial@asertis.com.co</t>
+          <t>coor.calidad@clinicamedical.com.co</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1003,7 +1007,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Oportunidad de IMPORTADORA CALI S.A.</t>
+          <t>Oportunidad de Clínica Medical S.A.S.</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1012,10 +1016,10 @@
         </is>
       </c>
       <c r="G12" s="1" t="n">
-        <v>46189.67539351852</v>
+        <v>46217.62244212963</v>
       </c>
       <c r="I12" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="J12" t="n">
         <v>2026</v>
@@ -1029,7 +1033,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>educacion@360forma.edu.co</t>
+          <t>calidad@institutodelcorazon.com</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1040,14 +1044,9 @@
       <c r="C13" t="n">
         <v>0</v>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Jorge Sanchez / jefe Comercial</t>
-        </is>
-      </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Oportunidad de Jorge Sanchez / jefe Comercial</t>
+          <t>Oportunidad de Instituto del Corazón de Bogotá</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1056,10 +1055,10 @@
         </is>
       </c>
       <c r="G13" s="1" t="n">
-        <v>46189.65077546296</v>
+        <v>46217.62072916667</v>
       </c>
       <c r="I13" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="J13" t="n">
         <v>2026</v>
@@ -1073,7 +1072,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>directoradjunto@dclass.edu.co</t>
+          <t>ana.ulloa@mederi.com.co</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1086,7 +1085,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Oportunidad de DCLASS ACADEMIA SAS</t>
+          <t>Oportunidad de Hospital Universitario Mayor - Mederi</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1095,10 +1094,10 @@
         </is>
       </c>
       <c r="G14" s="1" t="n">
-        <v>46189.49674768518</v>
+        <v>46217.61866898148</v>
       </c>
       <c r="I14" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="J14" t="n">
         <v>2026</v>
@@ -1112,12 +1111,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Belkis.jimenez@agrauto.com.co</t>
+          <t>ayudantia@homil.gov.co</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -1125,7 +1124,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Oportunidad de AGRICOLA AUTOMOTRIZ SAS / BELKYS JIMENEZ</t>
+          <t>Oportunidad de Hospital Militar Central</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1134,24 +1133,24 @@
         </is>
       </c>
       <c r="G15" s="1" t="n">
-        <v>46182.67912037037</v>
+        <v>46217.61708333333</v>
       </c>
       <c r="I15" t="n">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="J15" t="n">
         <v>2026</v>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>luisa.baena@automarcali.com</t>
+          <t>direccion.general@hospitalinfantildesanjose.org.co</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1162,14 +1161,9 @@
       <c r="C16" t="n">
         <v>0</v>
       </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>luisa.baena@automarcali.com</t>
-        </is>
-      </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Oportunidad de luisa.baena@automarcali.com</t>
+          <t>Oportunidad de Fundación Hospital Infantil Universitario de San José</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1178,10 +1172,10 @@
         </is>
       </c>
       <c r="G16" s="1" t="n">
-        <v>46182.67809027778</v>
+        <v>46217.6153587963</v>
       </c>
       <c r="I16" t="n">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="J16" t="n">
         <v>2026</v>
@@ -1195,25 +1189,20 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>directormercadeo@almotores.com</t>
+          <t>calidad@clinicadeloccidente.com</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C17" t="n">
         <v>0</v>
       </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Viviana Vanegas</t>
-        </is>
-      </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Oportunidad de Viviana Vanegas</t>
+          <t>Oportunidad de Clínica del Occidente S.A.</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1222,29 +1211,29 @@
         </is>
       </c>
       <c r="G17" s="1" t="n">
-        <v>46182.67621527778</v>
+        <v>46217.61388888889</v>
       </c>
       <c r="I17" t="n">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="J17" t="n">
         <v>2026</v>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>xiomara.duran@autopacifico.com.co</t>
+          <t>calidad@husi.org.co</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -1252,7 +1241,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Oportunidad de xiomara.duran@autopacifico.com.co</t>
+          <t>Oportunidad de Hospital Universitario San Ignacio</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1261,10 +1250,10 @@
         </is>
       </c>
       <c r="G18" s="1" t="n">
-        <v>46182.65815972222</v>
+        <v>46217.61174768519</v>
       </c>
       <c r="I18" t="n">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="J18" t="n">
         <v>2026</v>
@@ -1278,7 +1267,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>alejandrosaavedraconde@comfandi.com.co</t>
+          <t>cmarly@clinicademarly.com.co</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1289,14 +1278,9 @@
       <c r="C19" t="n">
         <v>0</v>
       </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>ALEJANDRO</t>
-        </is>
-      </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Oportunidad de ALEJANDRO</t>
+          <t>Oportunidad de Clínica de Marly</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1305,10 +1289,10 @@
         </is>
       </c>
       <c r="G19" s="1" t="n">
-        <v>46182.64278935185</v>
+        <v>46217.60430555556</v>
       </c>
       <c r="I19" t="n">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="J19" t="n">
         <v>2026</v>
@@ -1322,12 +1306,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>administracion@fiando.com.co</t>
+          <t>gerencia@hus.org.co</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -1335,7 +1319,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Oportunidad de FIANDO LTDA</t>
+          <t>Oportunidad de Hospital Universitario de la Samaritana</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1344,10 +1328,10 @@
         </is>
       </c>
       <c r="G20" s="1" t="n">
-        <v>46182.61304398148</v>
+        <v>46217.60261574074</v>
       </c>
       <c r="I20" t="n">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="J20" t="n">
         <v>2026</v>
@@ -1361,25 +1345,20 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>dgamoneda@productosdrogam.com</t>
+          <t>nomorales@colsanitas.com</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C21" t="n">
         <v>0</v>
       </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Diego Mauricio Gamoneda </t>
-        </is>
-      </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Oportunidad de Diego Mauricio Gamoneda </t>
+          <t>Oportunidad de Clínica Colsanitas Reina Sofía Pediátrica y Mujer</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1388,10 +1367,10 @@
         </is>
       </c>
       <c r="G21" s="1" t="n">
-        <v>46175.66417824074</v>
+        <v>46217.60097222222</v>
       </c>
       <c r="I21" t="n">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="J21" t="n">
         <v>2026</v>
@@ -1405,7 +1384,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>alexander.rojas@friogan.com</t>
+          <t>nomorales@colsanitas.com</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1418,7 +1397,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Oportunidad de FRIOGAN S.A</t>
+          <t>Oportunidad de Clínica Universitaria Colombia (Colsanitas)</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1427,10 +1406,10 @@
         </is>
       </c>
       <c r="G22" s="1" t="n">
-        <v>46175.63597222222</v>
+        <v>46217.59863425926</v>
       </c>
       <c r="I22" t="n">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="J22" t="n">
         <v>2026</v>
@@ -1442,6 +1421,11 @@
       </c>
     </row>
     <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>zayda.rodriguez@cpolaya.com.co</t>
+        </is>
+      </c>
       <c r="B23" t="inlineStr">
         <is>
           <t>Nuevo</t>
@@ -1452,7 +1436,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Oportunidad de Agromercados la Montaña</t>
+          <t>Oportunidad de Centro Policlínico del Olaya</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1461,10 +1445,10 @@
         </is>
       </c>
       <c r="G23" s="1" t="n">
-        <v>46175.62239583334</v>
+        <v>46217.59719907407</v>
       </c>
       <c r="I23" t="n">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="J23" t="n">
         <v>2026</v>
@@ -1478,12 +1462,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>juand.rios@alkosto.com.co</t>
+          <t>pcasallas@lacardiol.org</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -1491,7 +1475,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Oportunidad de ALKOSTO</t>
+          <t>Oportunidad de Fundación Cardioinfantil - Instituto de Cardiología</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1500,10 +1484,10 @@
         </is>
       </c>
       <c r="G24" s="1" t="n">
-        <v>46175.62055555556</v>
+        <v>46217.59630787037</v>
       </c>
       <c r="I24" t="n">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="J24" t="n">
         <v>2026</v>
@@ -1517,7 +1501,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>gerencia4087@grupo-exito.com</t>
+          <t>dir_calidad@clinicajuanncorpas.com</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1528,14 +1512,9 @@
       <c r="C25" t="n">
         <v>0</v>
       </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>Grupo exito ‒ 1007386172 - Sneider Quirama</t>
-        </is>
-      </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Oportunidad de Grupo exito</t>
+          <t>Oportunidad de Clínica Juan N Corpas Ltda</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1544,10 +1523,10 @@
         </is>
       </c>
       <c r="G25" s="1" t="n">
-        <v>46175.61638888889</v>
+        <v>46217.52333333333</v>
       </c>
       <c r="I25" t="n">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="J25" t="n">
         <v>2026</v>
@@ -1561,7 +1540,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ldgomez@supertiendascanaveral.com</t>
+          <t>dianaespinosanarvaez@gmail.com</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1572,14 +1551,9 @@
       <c r="C26" t="n">
         <v>0</v>
       </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>Luis David Gomez</t>
-        </is>
-      </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Oportunidad de Luis David Gomez</t>
+          <t>Oportunidad de Clínica Onkos</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1588,10 +1562,10 @@
         </is>
       </c>
       <c r="G26" s="1" t="n">
-        <v>46175.60493055556</v>
+        <v>46217.52202546296</v>
       </c>
       <c r="I26" t="n">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="J26" t="n">
         <v>2026</v>
@@ -1605,12 +1579,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>davida_vanegas@coomeva.com.co</t>
+          <t>gestiondecalidad@clinicapalermo.com.co</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -1618,7 +1592,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Oportunidad de BANCOOMEVA</t>
+          <t>Oportunidad de Clínica Palermo</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1627,10 +1601,10 @@
         </is>
       </c>
       <c r="G27" s="1" t="n">
-        <v>46175.47109953704</v>
+        <v>46217.51743055556</v>
       </c>
       <c r="I27" t="n">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="J27" t="n">
         <v>2026</v>
@@ -1644,25 +1618,20 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>alejandro.delgado@filedesk.com.co</t>
+          <t>calidad@hospitaldesanjose.org.co</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C28" t="n">
         <v>0</v>
       </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>AlejandroDelgado</t>
-        </is>
-      </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Oportunidad de AlejandroDelgado</t>
+          <t>Oportunidad de Hospital San José - Sociedad de Cirugía de Bogotá</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1671,10 +1640,10 @@
         </is>
       </c>
       <c r="G28" s="1" t="n">
-        <v>46174.71665509259</v>
+        <v>46217.51425925926</v>
       </c>
       <c r="I28" t="n">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="J28" t="n">
         <v>2026</v>
@@ -1686,22 +1655,22 @@
       </c>
     </row>
     <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>jzapata@ioir.org.co</t>
+        </is>
+      </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>35000000</v>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Olga Lucia Hurtado</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Oportunidad de Olga Lucia Hurtado</t>
+          <t>Oportunidad de Instituto de Ortopedia Infantil Roosevelt</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1710,10 +1679,10 @@
         </is>
       </c>
       <c r="G29" s="1" t="n">
-        <v>46168.49854166667</v>
+        <v>46217.51231481481</v>
       </c>
       <c r="I29" t="n">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="J29" t="n">
         <v>2026</v>
@@ -1727,20 +1696,20 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>comercial2@felsyn.com</t>
+          <t>diana.potesno@colsubsidio.com</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>713400</v>
+        <v>0</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Oportunidad de FONDO DE EMPLEADOS FELSYN</t>
+          <t>Oportunidad de Clínica Colsubsidio Calle 100</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1749,10 +1718,10 @@
         </is>
       </c>
       <c r="G30" s="1" t="n">
-        <v>46163.49130787037</v>
+        <v>46217.51116898148</v>
       </c>
       <c r="I30" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="J30" t="n">
         <v>2026</v>
@@ -1766,25 +1735,20 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>mercadeo@lasevillana.com.co</t>
+          <t>diana.potesno@colsubsidio.com</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C31" t="n">
         <v>0</v>
       </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fabio AlbertoGallego García </t>
-        </is>
-      </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Oportunidad de Fabio AlbertoGallego García </t>
+          <t>Oportunidad de Clínica Colsubsidio Calle 100</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1793,10 +1757,10 @@
         </is>
       </c>
       <c r="G31" s="1" t="n">
-        <v>46162.64569444444</v>
+        <v>46217.50983796296</v>
       </c>
       <c r="I31" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="J31" t="n">
         <v>2026</v>
@@ -1810,12 +1774,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>asantiago@stop.com.co</t>
+          <t>jose.chaves@colsubsidio.com</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -1823,7 +1787,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Oportunidad de STOP SAS</t>
+          <t>Oportunidad de Clínica Colsubsidio Ciudad Roma</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1832,10 +1796,10 @@
         </is>
       </c>
       <c r="G32" s="1" t="n">
-        <v>46161.63508101852</v>
+        <v>46217.50767361111</v>
       </c>
       <c r="I32" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="J32" t="n">
         <v>2026</v>
@@ -1849,25 +1813,20 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>aestrada@teker.co</t>
+          <t>carlos.artetamo@colsubsidio.com</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>16914000</v>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>TEKER SALUD SAS</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Oportunidad de TEKER SALUD SAS</t>
+          <t>Oportunidad de Clínica Infantil Colsubsidio</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1876,10 +1835,10 @@
         </is>
       </c>
       <c r="G33" s="1" t="n">
-        <v>46161.62922453704</v>
+        <v>46217.50050925926</v>
       </c>
       <c r="I33" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="J33" t="n">
         <v>2026</v>
@@ -1891,9 +1850,14 @@
       </c>
     </row>
     <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>notificacionescdc@clinicadelcountry.com</t>
+        </is>
+      </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -1901,7 +1865,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Oportunidad de TIAN IPS SAS</t>
+          <t>Oportunidad de Clínica del Country IPS</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1910,10 +1874,10 @@
         </is>
       </c>
       <c r="G34" s="1" t="n">
-        <v>46161.61643518518</v>
+        <v>46217.49881944444</v>
       </c>
       <c r="I34" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="J34" t="n">
         <v>2026</v>
@@ -1927,25 +1891,20 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>administración@fullredtotal.com</t>
+          <t>direcciongeneral@shaio.org</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>14000000</v>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>Eivar Eñasco</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Oportunidad de Eivar Eñasco</t>
+          <t>Oportunidad de Fundación Abood Shaio</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1954,10 +1913,10 @@
         </is>
       </c>
       <c r="G35" s="1" t="n">
-        <v>46154.67546296296</v>
+        <v>46217.49715277777</v>
       </c>
       <c r="I35" t="n">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="J35" t="n">
         <v>2026</v>
@@ -1971,25 +1930,20 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>cserna@surtifamiliar.com.co</t>
+          <t>direccion@cancer.gov.co</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Negociación</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>1950000</v>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>Claudia Patricia Serna</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Oportunidad de Claudia Patricia Serna</t>
+          <t>Oportunidad de Instituto Nacional de Cancerología</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -1998,42 +1952,37 @@
         </is>
       </c>
       <c r="G36" s="1" t="n">
-        <v>46154.66616898148</v>
+        <v>46217.47924768519</v>
       </c>
       <c r="I36" t="n">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="J36" t="n">
         <v>2026</v>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>coordmercadeo@pacificcenter.co</t>
+          <t>sdirmedica@clinicadelamujer.com.co</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>5600000</v>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>Claudia Castro</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Oportunidad de Claudia Castro</t>
+          <t>Oportunidad de Clínica de la Mujer</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -2042,42 +1991,37 @@
         </is>
       </c>
       <c r="G37" s="1" t="n">
-        <v>46154.66341435185</v>
+        <v>46217.47585648148</v>
       </c>
       <c r="I37" t="n">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="J37" t="n">
         <v>2026</v>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>isabellarengifo27@gmail.com</t>
+          <t>lidercalidad@homifundacion.org.co</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>28190000</v>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>Isabella Rengifo</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Oportunidad de Isabella Rengifo</t>
+          <t>Oportunidad de Fundación Hospital de la Misericordia (HOMI)</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2086,10 +2030,10 @@
         </is>
       </c>
       <c r="G38" s="1" t="n">
-        <v>46154.65981481481</v>
+        <v>46217.47246527778</v>
       </c>
       <c r="I38" t="n">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="J38" t="n">
         <v>2026</v>
@@ -2101,45 +2045,36 @@
       </c>
     </row>
     <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>direcciongeneral1@stewardcolombia.org</t>
+        </is>
+      </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>50000000</v>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>Paola Gómez - Agente Inmobiliaria Independiente</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Puesto de Trabajo CC Medellin</t>
+          <t>Oportunidad de Hospital Universitario Clínica San Rafael</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Richard Castaño</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G39" s="1" t="n">
-        <v>46154.49104166667</v>
-      </c>
-      <c r="H39" s="1" t="n">
-        <v>46170</v>
+        <v>46217.00748842592</v>
       </c>
       <c r="I39" t="n">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="J39" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K39" t="n">
-        <v>5</v>
-      </c>
-      <c r="L39" t="n">
         <v>2026</v>
       </c>
       <c r="M39" t="inlineStr">
@@ -2151,59 +2086,59 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>alberto.ramirez@constructorabolivar.com</t>
+          <t>adriana.urrego@fsfb.org.co</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Ganado</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>3000000</v>
+        <v>0</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Oportunidad de NPS Relacional</t>
+          <t>Oportunidad de FUNDACION SANTA FE DE BOGOTA</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G40" s="1" t="n">
-        <v>46154.44511574074</v>
+        <v>46217.00381944444</v>
       </c>
       <c r="I40" t="n">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="J40" t="n">
         <v>2026</v>
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>calidadsalud@cafam.com.co</t>
+        </is>
+      </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>3000000</v>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>MADERKIT</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Oportunidad de MADERKIT</t>
+          <t>Oportunidad de Centro de Atención en Salud CAFAM Clínica Calle 51</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2212,10 +2147,10 @@
         </is>
       </c>
       <c r="G41" s="1" t="n">
-        <v>46147.66540509259</v>
+        <v>46216.99954861111</v>
       </c>
       <c r="I41" t="n">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="J41" t="n">
         <v>2026</v>
@@ -2229,25 +2164,20 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>omer120395@gmail.com</t>
+          <t>notificacionesjudiciales@fhsc.org.co</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C42" t="n">
         <v>0</v>
       </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>Omer Peñaloza</t>
-        </is>
-      </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Oportunidad de Omer Peñaloza</t>
+          <t>Oportunidad de Fundación Hospital San Carlos</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -2256,10 +2186,10 @@
         </is>
       </c>
       <c r="G42" s="1" t="n">
-        <v>46147.66090277778</v>
+        <v>46216.99548611111</v>
       </c>
       <c r="I42" t="n">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="J42" t="n">
         <v>2026</v>
@@ -2273,20 +2203,20 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>directora.it@supermercadobelalcazar.com.co</t>
+          <t>calidad@proseguir.org</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>6000000</v>
+        <v>0</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Oportunidad de ABASTECEMOS DE OCCIDENTE</t>
+          <t>Oportunidad de PROSEGUIR SEDE 3</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2295,21 +2225,12 @@
         </is>
       </c>
       <c r="G43" s="1" t="n">
-        <v>46147.64170138889</v>
-      </c>
-      <c r="H43" s="1" t="n">
-        <v>46157</v>
+        <v>46216.99299768519</v>
       </c>
       <c r="I43" t="n">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="J43" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K43" t="n">
-        <v>5</v>
-      </c>
-      <c r="L43" t="n">
         <v>2026</v>
       </c>
       <c r="M43" t="inlineStr">
@@ -2321,55 +2242,46 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>oscar.molina@terrenoshouston.com</t>
+          <t>centrodecontacto@uao.edu.co</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Seguimiento</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>37623040</v>
+        <v>10000000</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Oportunidad de COLONY RIDGE</t>
+          <t>Oportunidad de UNIVERSIDAD AUTONOMA DE OCCIDENTE</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G44" s="1" t="n">
-        <v>46147.60297453704</v>
-      </c>
-      <c r="H44" s="1" t="n">
-        <v>46150</v>
+        <v>46213.49821759259</v>
       </c>
       <c r="I44" t="n">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="J44" t="n">
         <v>2026</v>
       </c>
-      <c r="K44" t="n">
-        <v>5</v>
-      </c>
-      <c r="L44" t="n">
-        <v>2026</v>
-      </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>jsantacr@ccc.org.co</t>
+          <t>carlos.segovia@warena.co</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2378,34 +2290,25 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>55000000</v>
+        <v>35000000</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Oportunidad de CAMARA DE COMERCIO CALI</t>
+          <t>Oportunidad de W ARENA</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G45" s="1" t="n">
-        <v>46141.62370370371</v>
-      </c>
-      <c r="H45" s="1" t="n">
-        <v>46289</v>
+        <v>46213.49508101852</v>
       </c>
       <c r="I45" t="n">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="J45" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K45" t="n">
-        <v>9</v>
-      </c>
-      <c r="L45" t="n">
         <v>2026</v>
       </c>
       <c r="M45" t="inlineStr">
@@ -2417,20 +2320,25 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>exportaciones@laprovincia.com</t>
+          <t>klondono@fundacionwwbcol.org</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Ganado</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>6000000</v>
+        <v>300000</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Karla Londoño</t>
+        </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Oportunidad de PRODUCTOS LA PROVINCIA SAS</t>
+          <t>Oportunidad de Karla Londoño</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2439,37 +2347,51 @@
         </is>
       </c>
       <c r="G46" s="1" t="n">
-        <v>46141.62021990741</v>
+        <v>46212.51638888889</v>
+      </c>
+      <c r="H46" s="1" t="n">
+        <v>46217</v>
       </c>
       <c r="I46" t="n">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="J46" t="n">
         <v>2026</v>
       </c>
+      <c r="K46" t="n">
+        <v>7</v>
+      </c>
+      <c r="L46" t="n">
+        <v>2026</v>
+      </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>coordinador.mercadeo@regency.com.co</t>
+          <t>ctorres@colcobranzasnacionales.com</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Negociación</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>0</v>
+        <v>5000000</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>ctorres@colcobranzasnacionales.com</t>
+        </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Oportunidad de REGENCY TECH SAS</t>
+          <t>Oportunidad de ctorres@colcobranzasnacionales.com</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -2478,32 +2400,37 @@
         </is>
       </c>
       <c r="G47" s="1" t="n">
-        <v>46141.59664351852</v>
+        <v>46206.73804398148</v>
       </c>
       <c r="I47" t="n">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="J47" t="n">
         <v>2026</v>
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>medifar624@gmail.com</t>
+        </is>
+      </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Ganado</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>1200000</v>
+        <v>1640000</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Oportunidad de EMCALI E.I.C.E ESP</t>
+          <t>Oportunidad de MEDISFARMA SAS</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2512,46 +2439,51 @@
         </is>
       </c>
       <c r="G48" s="1" t="n">
-        <v>46141.59045138889</v>
+        <v>46203.72597222222</v>
       </c>
       <c r="H48" s="1" t="n">
-        <v>46352</v>
+        <v>46217</v>
       </c>
       <c r="I48" t="n">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="J48" t="n">
         <v>2026</v>
       </c>
       <c r="K48" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="L48" t="n">
         <v>2026</v>
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>angie_feligrana@eficacia.com.co</t>
+          <t>mercadeo@norteysur.co</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Seguimiento</t>
+          <t>Negociación</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>6000000</v>
+        <v>28190000</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Isabella Mesa</t>
+        </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Oportunidad de Eficacia sas / Angie Feligrana</t>
+          <t>Oportunidad de Isabella Mesa</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -2560,51 +2492,37 @@
         </is>
       </c>
       <c r="G49" s="1" t="n">
-        <v>46126.63210648148</v>
-      </c>
-      <c r="H49" s="1" t="n">
-        <v>46150</v>
+        <v>46191.70076388889</v>
       </c>
       <c r="I49" t="n">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="J49" t="n">
         <v>2026</v>
       </c>
-      <c r="K49" t="n">
-        <v>5</v>
-      </c>
-      <c r="L49" t="n">
-        <v>2026</v>
-      </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Estrategiadigital@zuluagaysoto.com</t>
+          <t>comercial@asertis.com.co</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C50" t="n">
         <v>0</v>
       </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>Maryuri Arguello</t>
-        </is>
-      </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Oportunidad de Maryuri Arguello</t>
+          <t>Oportunidad de IMPORTADORA CALI S.A.</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -2613,10 +2531,10 @@
         </is>
       </c>
       <c r="G50" s="1" t="n">
-        <v>46125.71925925926</v>
+        <v>46189.67539351852</v>
       </c>
       <c r="I50" t="n">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="J50" t="n">
         <v>2026</v>
@@ -2630,65 +2548,56 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>gabrielrodriguez@arrozsupremo.com</t>
+          <t>educacion@360forma.edu.co</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Ganado</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>8000000</v>
+        <v>0</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>GABRIEL RODRIGUEZ</t>
+          <t>Jorge Sanchez / jefe Comercial</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Agente de Ventas</t>
+          <t>Oportunidad de Jorge Sanchez / jefe Comercial</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Richard Castaño</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G51" s="1" t="n">
-        <v>46119.62108796297</v>
-      </c>
-      <c r="H51" s="1" t="n">
-        <v>46141</v>
+        <v>46189.65077546296</v>
       </c>
       <c r="I51" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="J51" t="n">
         <v>2026</v>
       </c>
-      <c r="K51" t="n">
-        <v>4</v>
-      </c>
-      <c r="L51" t="n">
-        <v>2026</v>
-      </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Belkis.jimenez@agrauto.com.co</t>
+          <t>directoradjunto@dclass.edu.co</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -2696,7 +2605,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Oportunidad de AGRICOLA AUTOMOTRIZ SAS</t>
+          <t>Oportunidad de DCLASS ACADEMIA SAS</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -2705,29 +2614,29 @@
         </is>
       </c>
       <c r="G52" s="1" t="n">
-        <v>46119.38914351852</v>
+        <v>46189.49674768518</v>
       </c>
       <c r="I52" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="J52" t="n">
         <v>2026</v>
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>anyela.aponza@cotel.com.co</t>
+          <t>Belkis.jimenez@agrauto.com.co</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -2735,7 +2644,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Oportunidad de COTEL SAL</t>
+          <t>Oportunidad de AGRICOLA AUTOMOTRIZ SAS / BELKYS JIMENEZ</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -2744,29 +2653,29 @@
         </is>
       </c>
       <c r="G53" s="1" t="n">
-        <v>46112.61271990741</v>
+        <v>46182.67912037037</v>
       </c>
       <c r="I53" t="n">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="J53" t="n">
         <v>2026</v>
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>liliana.patino@quironsalud.com</t>
+          <t>luisa.baena@automarcali.com</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -2774,12 +2683,12 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>CLINICA IMBANACO</t>
+          <t>luisa.baena@automarcali.com</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Oportunidad de Liliana Patiño Flórez</t>
+          <t>Oportunidad de luisa.baena@automarcali.com</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -2788,10 +2697,10 @@
         </is>
       </c>
       <c r="G54" s="1" t="n">
-        <v>46112.60853009259</v>
+        <v>46182.67809027778</v>
       </c>
       <c r="I54" t="n">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="J54" t="n">
         <v>2026</v>
@@ -2805,20 +2714,25 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>casanchez@jgb.com.co</t>
+          <t>directormercadeo@almotores.com</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C55" t="n">
         <v>0</v>
       </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Viviana Vanegas</t>
+        </is>
+      </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Oportunidad de JGB S.A.</t>
+          <t>Oportunidad de Viviana Vanegas</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -2827,29 +2741,29 @@
         </is>
       </c>
       <c r="G55" s="1" t="n">
-        <v>46112.6052662037</v>
+        <v>46182.67621527778</v>
       </c>
       <c r="I55" t="n">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="J55" t="n">
         <v>2026</v>
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>damaris.gomez@disfarma.com.co</t>
+          <t>xiomara.duran@autopacifico.com.co</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Seguimiento</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -2857,7 +2771,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Oportunidad de DISFARMA</t>
+          <t>Oportunidad de xiomara.duran@autopacifico.com.co</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -2866,10 +2780,10 @@
         </is>
       </c>
       <c r="G56" s="1" t="n">
-        <v>46112.60325231482</v>
+        <v>46182.65815972222</v>
       </c>
       <c r="I56" t="n">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="J56" t="n">
         <v>2026</v>
@@ -2883,7 +2797,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>alergologosdeoccidente@gmail.com</t>
+          <t>alejandrosaavedraconde@comfandi.com.co</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2896,12 +2810,12 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Johana Gonzalez</t>
+          <t>ALEJANDRO</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Oportunidad de Johana Gonzalez</t>
+          <t>Oportunidad de ALEJANDRO</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -2910,10 +2824,10 @@
         </is>
       </c>
       <c r="G57" s="1" t="n">
-        <v>46107.51248842593</v>
+        <v>46182.64278935185</v>
       </c>
       <c r="I57" t="n">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="J57" t="n">
         <v>2026</v>
@@ -2927,43 +2841,34 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>DavidEsteban.Porras@alfalaval.com</t>
+          <t>administracion@fiando.com.co</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Ganado</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>15000000</v>
+        <v>0</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Oportunidad de OPORTUNIDAD ENCUESTAS ALFALAVAL</t>
+          <t>Oportunidad de FIANDO LTDA</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G58" s="1" t="n">
-        <v>46101.72893518519</v>
-      </c>
-      <c r="H58" s="1" t="n">
-        <v>46141</v>
+        <v>46182.61304398148</v>
       </c>
       <c r="I58" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="J58" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K58" t="n">
-        <v>4</v>
-      </c>
-      <c r="L58" t="n">
         <v>2026</v>
       </c>
       <c r="M58" t="inlineStr">
@@ -2975,20 +2880,25 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Dr.arcarmona@gmail.com</t>
+          <t>dgamoneda@productosdrogam.com</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C59" t="n">
         <v>0</v>
       </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Diego Mauricio Gamoneda </t>
+        </is>
+      </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Oportunidad de GAMANUCLEAR LTDA - Dr Alberto Carmona</t>
+          <t xml:space="preserve">Oportunidad de Diego Mauricio Gamoneda </t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -2997,10 +2907,10 @@
         </is>
       </c>
       <c r="G59" s="1" t="n">
-        <v>46098.65114583333</v>
+        <v>46175.66417824074</v>
       </c>
       <c r="I59" t="n">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="J59" t="n">
         <v>2026</v>
@@ -3014,69 +2924,54 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>cecilia.guevara@cosmitet.net / administracion.crd@cosmitet.net</t>
+          <t>alexander.rojas@friogan.com</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
+          <t>Propuesta</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>10000000</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Oportunidad de FRIOGAN S.A</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G60" s="1" t="n">
+        <v>46175.63597222222</v>
+      </c>
+      <c r="I60" t="n">
+        <v>23</v>
+      </c>
+      <c r="J60" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>Calificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" t="inlineStr">
+        <is>
           <t>Perdido</t>
         </is>
       </c>
-      <c r="C60" t="n">
-        <v>0</v>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>Cecilia Guevara</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>Oportunidad de CLINICA REY DAVID Walter Charria</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G60" s="1" t="n">
-        <v>46094.69002314815</v>
-      </c>
-      <c r="I60" t="n">
-        <v>11</v>
-      </c>
-      <c r="J60" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M60" t="inlineStr">
-        <is>
-          <t>No calificado</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>vicerrectoriacademica@unicatolica.edu.co</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
       <c r="C61" t="n">
         <v>0</v>
       </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>Jorge Silva</t>
-        </is>
-      </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Oportunidad de Jorge Silva</t>
+          <t>Oportunidad de Agromercados la Montaña</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -3085,10 +2980,10 @@
         </is>
       </c>
       <c r="G61" s="1" t="n">
-        <v>46094.66880787037</v>
+        <v>46175.62239583334</v>
       </c>
       <c r="I61" t="n">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="J61" t="n">
         <v>2026</v>
@@ -3102,60 +2997,46 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>pedroperea02@gmail.com</t>
+          <t>juand.rios@alkosto.com.co</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Ganado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>2160000</v>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>Pedro Pablo Perea Mafla</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Oportunidad de Encuestas</t>
+          <t>Oportunidad de ALKOSTO</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G62" s="1" t="n">
-        <v>46094.65905092593</v>
-      </c>
-      <c r="H62" s="1" t="n">
-        <v>46141</v>
+        <v>46175.62055555556</v>
       </c>
       <c r="I62" t="n">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="J62" t="n">
         <v>2026</v>
       </c>
-      <c r="K62" t="n">
-        <v>4</v>
-      </c>
-      <c r="L62" t="n">
-        <v>2026</v>
-      </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>cristina.papamija@bmm.com.co</t>
+          <t>gerencia4087@grupo-exito.com</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3164,23 +3045,28 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>8071000</v>
+        <v>0</v>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Grupo exito ‒ 1007386172 - Sneider Quirama</t>
+        </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Oportunidad de BANCO MUNDO MUJER</t>
+          <t>Oportunidad de Grupo exito</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G63" s="1" t="n">
-        <v>46094.65019675926</v>
+        <v>46175.61638888889</v>
       </c>
       <c r="I63" t="n">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="J63" t="n">
         <v>2026</v>
@@ -3194,7 +3080,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>capacitacionvirtual@fundacionwwbcol.org</t>
+          <t>ldgomez@supertiendascanaveral.com</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3203,23 +3089,28 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>1600000</v>
+        <v>0</v>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Luis David Gomez</t>
+        </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Licenciamiento y ajuste WhatsApp FUNDACIÓN WWB</t>
+          <t>Oportunidad de Luis David Gomez</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G64" s="1" t="n">
-        <v>46094.64826388889</v>
+        <v>46175.60493055556</v>
       </c>
       <c r="I64" t="n">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="J64" t="n">
         <v>2026</v>
@@ -3233,73 +3124,64 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>carol.cuesta@cbolivar.com</t>
+          <t>davida_vanegas@coomeva.com.co</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Ganado</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>2900000</v>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>CAROL CUESTA</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Gestión de Subsidios CB Bogotá</t>
+          <t>Oportunidad de BANCOOMEVA</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G65" s="1" t="n">
-        <v>46094.64454861111</v>
-      </c>
-      <c r="H65" s="1" t="n">
-        <v>46135</v>
+        <v>46175.47109953704</v>
       </c>
       <c r="I65" t="n">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="J65" t="n">
         <v>2026</v>
       </c>
-      <c r="K65" t="n">
-        <v>4</v>
-      </c>
-      <c r="L65" t="n">
-        <v>2026</v>
-      </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>edwin.munoz.v@uniminuto.edu</t>
+          <t>alejandro.delgado@filedesk.com.co</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C66" t="n">
         <v>0</v>
       </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>AlejandroDelgado</t>
+        </is>
+      </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Oportunidad de UNIMINUTO</t>
+          <t>Oportunidad de AlejandroDelgado</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -3308,10 +3190,10 @@
         </is>
       </c>
       <c r="G66" s="1" t="n">
-        <v>46092.63626157407</v>
+        <v>46174.71665509259</v>
       </c>
       <c r="I66" t="n">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="J66" t="n">
         <v>2026</v>
@@ -3323,27 +3205,22 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>jaime_zuluaga@eficacia.com.co</t>
-        </is>
-      </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>0</v>
+        <v>35000000</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Jaime Alberto</t>
+          <t>Olga Lucia Hurtado</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Oportunidad de Jaime Alberto Zuluaga</t>
+          <t>Oportunidad de Olga Lucia Hurtado</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -3352,10 +3229,10 @@
         </is>
       </c>
       <c r="G67" s="1" t="n">
-        <v>46092.63153935185</v>
+        <v>46168.49854166667</v>
       </c>
       <c r="I67" t="n">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="J67" t="n">
         <v>2026</v>
@@ -3369,25 +3246,20 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>comercial@isyscol.com</t>
+          <t>comercial2@felsyn.com</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>0</v>
-      </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>Andres Nader</t>
-        </is>
+        <v>713400</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Oportunidad de Andres Nader</t>
+          <t>Oportunidad de FONDO DE EMPLEADOS FELSYN</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -3396,10 +3268,10 @@
         </is>
       </c>
       <c r="G68" s="1" t="n">
-        <v>46091.59211805555</v>
+        <v>46163.49130787037</v>
       </c>
       <c r="I68" t="n">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="J68" t="n">
         <v>2026</v>
@@ -3413,105 +3285,120 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>mercadeo@norteysur.co</t>
+          <t>mercadeo@lasevillana.com.co</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
+          <t>Contactado</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>0</v>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fabio AlbertoGallego García </t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Oportunidad de Fabio AlbertoGallego García </t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G69" s="1" t="n">
+        <v>46162.64569444444</v>
+      </c>
+      <c r="I69" t="n">
+        <v>21</v>
+      </c>
+      <c r="J69" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>No calificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>asantiago@stop.com.co</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Contactado</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>0</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Oportunidad de STOP SAS</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G70" s="1" t="n">
+        <v>46161.63508101852</v>
+      </c>
+      <c r="I70" t="n">
+        <v>21</v>
+      </c>
+      <c r="J70" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>No calificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>aestrada@teker.co</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
           <t>Perdido</t>
         </is>
       </c>
-      <c r="C69" t="n">
-        <v>0</v>
-      </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>Isabella Mesa</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>Oportunidad de Isabella Mesa</t>
-        </is>
-      </c>
-      <c r="F69" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G69" s="1" t="n">
-        <v>46091.40078703704</v>
-      </c>
-      <c r="I69" t="n">
-        <v>11</v>
-      </c>
-      <c r="J69" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M69" t="inlineStr">
-        <is>
-          <t>No calificado</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C70" t="n">
-        <v>0</v>
-      </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>Clasificación EMAIL Comfenalco Cartagena</t>
-        </is>
-      </c>
-      <c r="F70" t="inlineStr">
-        <is>
-          <t>Maria Fernanda Gaviria</t>
-        </is>
-      </c>
-      <c r="G70" s="1" t="n">
-        <v>46091.3665625</v>
-      </c>
-      <c r="I70" t="n">
-        <v>11</v>
-      </c>
-      <c r="J70" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M70" t="inlineStr">
-        <is>
-          <t>No calificado</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
       <c r="C71" t="n">
-        <v>0</v>
+        <v>16914000</v>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>TEKER SALUD SAS</t>
+        </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Oportunidad de ESE HOSPITAL LA MARIA</t>
+          <t>Oportunidad de TEKER SALUD SAS</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Laura Alejandra Castañeda</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G71" s="1" t="n">
-        <v>46083.67605324074</v>
+        <v>46161.62922453704</v>
       </c>
       <c r="I71" t="n">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="J71" t="n">
         <v>2026</v>
@@ -3525,61 +3412,71 @@
     <row r="72">
       <c r="B72" t="inlineStr">
         <is>
+          <t>Contactado</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>0</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Oportunidad de TIAN IPS SAS</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G72" s="1" t="n">
+        <v>46161.61643518518</v>
+      </c>
+      <c r="I72" t="n">
+        <v>21</v>
+      </c>
+      <c r="J72" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>No calificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>administración@fullredtotal.com</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
           <t>Perdido</t>
         </is>
       </c>
-      <c r="C72" t="n">
-        <v>0</v>
-      </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>Oportunidad de SUPER TRANSPORTE</t>
-        </is>
-      </c>
-      <c r="F72" t="inlineStr">
-        <is>
-          <t>Laura Alejandra Castañeda</t>
-        </is>
-      </c>
-      <c r="G72" s="1" t="n">
-        <v>46083.6706712963</v>
-      </c>
-      <c r="I72" t="n">
-        <v>10</v>
-      </c>
-      <c r="J72" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M72" t="inlineStr">
-        <is>
-          <t>No calificado</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
       <c r="C73" t="n">
-        <v>0</v>
+        <v>14000000</v>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Eivar Eñasco</t>
+        </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Oportunidad de ENLACES IP S.A.S</t>
+          <t>Oportunidad de Eivar Eñasco</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Laura Alejandra Castañeda</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G73" s="1" t="n">
-        <v>46083.50145833333</v>
+        <v>46154.67546296296</v>
       </c>
       <c r="I73" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="J73" t="n">
         <v>2026</v>
@@ -3593,25 +3490,25 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>accounting@diaza.com</t>
+          <t>cserna@surtifamiliar.com.co</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Ganado</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>0</v>
+        <v>975000</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>JOHANA RODRIGUEZ</t>
+          <t>Claudia Patricia Serna</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Oportunidad de JOHANA RODRIGUEZ</t>
+          <t>Oportunidad de Claudia Patricia Serna</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -3620,37 +3517,51 @@
         </is>
       </c>
       <c r="G74" s="1" t="n">
-        <v>46079.73486111111</v>
+        <v>46154.66616898148</v>
+      </c>
+      <c r="H74" s="1" t="n">
+        <v>46217</v>
       </c>
       <c r="I74" t="n">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="J74" t="n">
         <v>2026</v>
       </c>
+      <c r="K74" t="n">
+        <v>7</v>
+      </c>
+      <c r="L74" t="n">
+        <v>2026</v>
+      </c>
       <c r="M74" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>mensajeriamyr@gmail.com</t>
+          <t>coordmercadeo@pacificcenter.co</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>0</v>
+        <v>5600000</v>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Claudia Castro</t>
+        </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Oportunidad de MENSAJERIA M&amp;R SAS</t>
+          <t>Oportunidad de Claudia Castro</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -3659,24 +3570,24 @@
         </is>
       </c>
       <c r="G75" s="1" t="n">
-        <v>46079.72262731481</v>
+        <v>46154.66341435185</v>
       </c>
       <c r="I75" t="n">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="J75" t="n">
         <v>2026</v>
       </c>
       <c r="M75" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>sistemaspanaderialeal@gmail.com</t>
+          <t>isabellarengifo27@gmail.com</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -3685,16 +3596,16 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>0</v>
+        <v>28190000</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Diego Rios</t>
+          <t>Isabella Rengifo</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>JAMDAC SAS, Diego Rios</t>
+          <t>Oportunidad de Isabella Rengifo</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -3703,10 +3614,10 @@
         </is>
       </c>
       <c r="G76" s="1" t="n">
-        <v>46071.63706018519</v>
+        <v>46154.65981481481</v>
       </c>
       <c r="I76" t="n">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="J76" t="n">
         <v>2026</v>
@@ -3718,41 +3629,45 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>efernandez@unico.com.co</t>
-        </is>
-      </c>
       <c r="B77" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>0</v>
+        <v>50000000</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Erick Fernandez</t>
+          <t>Paola Gómez - Agente Inmobiliaria Independiente</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Oportunidad de Erick Fernandez</t>
+          <t>Puesto de Trabajo CC Medellin</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Richard Castaño</t>
         </is>
       </c>
       <c r="G77" s="1" t="n">
-        <v>46064.3750462963</v>
+        <v>46154.49104166667</v>
+      </c>
+      <c r="H77" s="1" t="n">
+        <v>46170</v>
       </c>
       <c r="I77" t="n">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="J77" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K77" t="n">
+        <v>5</v>
+      </c>
+      <c r="L77" t="n">
         <v>2026</v>
       </c>
       <c r="M77" t="inlineStr">
@@ -3764,69 +3679,59 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>kabenitez@icesi.edu.co</t>
+          <t>alberto.ramirez@constructorabolivar.com</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
+          <t>Ganado</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Oportunidad de NPS Relacional</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Jennifer Hoyos Gallego</t>
+        </is>
+      </c>
+      <c r="G78" s="1" t="n">
+        <v>46154.44511574074</v>
+      </c>
+      <c r="I78" t="n">
+        <v>20</v>
+      </c>
+      <c r="J78" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M78" t="inlineStr">
+        <is>
+          <t>Calificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="B79" t="inlineStr">
+        <is>
           <t>Perdido</t>
         </is>
       </c>
-      <c r="C78" t="n">
-        <v>10000000</v>
-      </c>
-      <c r="D78" t="inlineStr">
-        <is>
-          <t>KENI BENITEZ</t>
-        </is>
-      </c>
-      <c r="E78" t="inlineStr">
-        <is>
-          <t>Oportunidad de KENI BENITEZ</t>
-        </is>
-      </c>
-      <c r="F78" t="inlineStr">
-        <is>
-          <t>Jennifer Hoyos Gallego</t>
-        </is>
-      </c>
-      <c r="G78" s="1" t="n">
-        <v>46059.34918981481</v>
-      </c>
-      <c r="I78" t="n">
-        <v>6</v>
-      </c>
-      <c r="J78" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M78" t="inlineStr">
-        <is>
-          <t>No calificado</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t>patovar@uao.edu.co</t>
-        </is>
-      </c>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
       <c r="C79" t="n">
-        <v>0</v>
+        <v>3000000</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Paula Tovar</t>
+          <t>MADERKIT</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Oportunidad de UNIVERSIDAD AUTONOMA DE OCCIDENTE</t>
+          <t>Oportunidad de MADERKIT</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -3835,10 +3740,10 @@
         </is>
       </c>
       <c r="G79" s="1" t="n">
-        <v>46058.72516203704</v>
+        <v>46147.66540509259</v>
       </c>
       <c r="I79" t="n">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="J79" t="n">
         <v>2026</v>
@@ -3852,7 +3757,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>comercial@isyscol.com</t>
+          <t>omer120395@gmail.com</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -3863,9 +3768,14 @@
       <c r="C80" t="n">
         <v>0</v>
       </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Omer Peñaloza</t>
+        </is>
+      </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Oportunidad de TECNOLOGIAS ISYSCOL SAS</t>
+          <t>Oportunidad de Omer Peñaloza</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -3874,10 +3784,10 @@
         </is>
       </c>
       <c r="G80" s="1" t="n">
-        <v>46057.58993055556</v>
+        <v>46147.66090277778</v>
       </c>
       <c r="I80" t="n">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="J80" t="n">
         <v>2026</v>
@@ -3889,17 +3799,22 @@
       </c>
     </row>
     <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>directora.it@supermercadobelalcazar.com.co</t>
+        </is>
+      </c>
       <c r="B81" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>15000000</v>
+        <v>6000000</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Oportunidad de VOICE IA EFICACIA</t>
+          <t>Oportunidad de ABASTECEMOS DE OCCIDENTE</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -3908,12 +3823,21 @@
         </is>
       </c>
       <c r="G81" s="1" t="n">
-        <v>46057.3409837963</v>
+        <v>46147.64170138889</v>
+      </c>
+      <c r="H81" s="1" t="n">
+        <v>46157</v>
       </c>
       <c r="I81" t="n">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="J81" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K81" t="n">
+        <v>5</v>
+      </c>
+      <c r="L81" t="n">
         <v>2026</v>
       </c>
       <c r="M81" t="inlineStr">

</xml_diff>

<commit_message>
CRM actualizado — 14/07/2026 15:30
</commit_message>
<xml_diff>
--- a/CRM_PowerBI_BrendaLuna_actualizado.xlsx
+++ b/CRM_PowerBI_BrendaLuna_actualizado.xlsx
@@ -994,7 +994,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>coor.calidad@clinicamedical.com.co</t>
+          <t>calidad.vip@axacolpatria.co</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1007,7 +1007,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica Medical S.A.S.</t>
+          <t>Oportunidad de Clínica VIP Centro de Medicina Internacional</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1016,7 +1016,7 @@
         </is>
       </c>
       <c r="G12" s="1" t="n">
-        <v>46217.62244212963</v>
+        <v>46217.63989583333</v>
       </c>
       <c r="I12" t="n">
         <v>29</v>
@@ -1033,7 +1033,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>calidad@institutodelcorazon.com</t>
+          <t>hocen.direc@policia.gov.co</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1046,7 +1046,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Oportunidad de Instituto del Corazón de Bogotá</t>
+          <t>Oportunidad de Hospital Central Policía Nacional</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1055,7 +1055,7 @@
         </is>
       </c>
       <c r="G13" s="1" t="n">
-        <v>46217.62072916667</v>
+        <v>46217.63702546297</v>
       </c>
       <c r="I13" t="n">
         <v>29</v>
@@ -1072,7 +1072,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ana.ulloa@mederi.com.co</t>
+          <t>coor.calidad@clinicamedical.com.co</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1085,7 +1085,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Oportunidad de Hospital Universitario Mayor - Mederi</t>
+          <t>Oportunidad de Clínica Medical S.A.S.</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1094,7 +1094,7 @@
         </is>
       </c>
       <c r="G14" s="1" t="n">
-        <v>46217.61866898148</v>
+        <v>46217.62244212963</v>
       </c>
       <c r="I14" t="n">
         <v>29</v>
@@ -1111,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ayudantia@homil.gov.co</t>
+          <t>calidad@institutodelcorazon.com</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1124,7 +1124,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Oportunidad de Hospital Militar Central</t>
+          <t>Oportunidad de Instituto del Corazón de Bogotá</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1133,7 +1133,7 @@
         </is>
       </c>
       <c r="G15" s="1" t="n">
-        <v>46217.61708333333</v>
+        <v>46217.62072916667</v>
       </c>
       <c r="I15" t="n">
         <v>29</v>
@@ -1150,7 +1150,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>direccion.general@hospitalinfantildesanjose.org.co</t>
+          <t>ana.ulloa@mederi.com.co</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1163,7 +1163,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Oportunidad de Fundación Hospital Infantil Universitario de San José</t>
+          <t>Oportunidad de Hospital Universitario Mayor - Mederi</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1172,7 +1172,7 @@
         </is>
       </c>
       <c r="G16" s="1" t="n">
-        <v>46217.6153587963</v>
+        <v>46217.61866898148</v>
       </c>
       <c r="I16" t="n">
         <v>29</v>
@@ -1189,7 +1189,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>calidad@clinicadeloccidente.com</t>
+          <t>ayudantia@homil.gov.co</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1202,7 +1202,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica del Occidente S.A.</t>
+          <t>Oportunidad de Hospital Militar Central</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1211,7 +1211,7 @@
         </is>
       </c>
       <c r="G17" s="1" t="n">
-        <v>46217.61388888889</v>
+        <v>46217.61708333333</v>
       </c>
       <c r="I17" t="n">
         <v>29</v>
@@ -1228,7 +1228,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>calidad@husi.org.co</t>
+          <t>direccion.general@hospitalinfantildesanjose.org.co</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1241,7 +1241,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Oportunidad de Hospital Universitario San Ignacio</t>
+          <t>Oportunidad de Fundación Hospital Infantil Universitario de San José</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1250,7 +1250,7 @@
         </is>
       </c>
       <c r="G18" s="1" t="n">
-        <v>46217.61174768519</v>
+        <v>46217.6153587963</v>
       </c>
       <c r="I18" t="n">
         <v>29</v>
@@ -1267,7 +1267,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>cmarly@clinicademarly.com.co</t>
+          <t>calidad@clinicadeloccidente.com</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1280,7 +1280,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica de Marly</t>
+          <t>Oportunidad de Clínica del Occidente S.A.</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1289,7 +1289,7 @@
         </is>
       </c>
       <c r="G19" s="1" t="n">
-        <v>46217.60430555556</v>
+        <v>46217.61388888889</v>
       </c>
       <c r="I19" t="n">
         <v>29</v>
@@ -1306,7 +1306,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>gerencia@hus.org.co</t>
+          <t>calidad@husi.org.co</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1319,7 +1319,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Oportunidad de Hospital Universitario de la Samaritana</t>
+          <t>Oportunidad de Hospital Universitario San Ignacio</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1328,7 +1328,7 @@
         </is>
       </c>
       <c r="G20" s="1" t="n">
-        <v>46217.60261574074</v>
+        <v>46217.61174768519</v>
       </c>
       <c r="I20" t="n">
         <v>29</v>
@@ -1345,7 +1345,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>nomorales@colsanitas.com</t>
+          <t>cmarly@clinicademarly.com.co</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1358,7 +1358,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica Colsanitas Reina Sofía Pediátrica y Mujer</t>
+          <t>Oportunidad de Clínica de Marly</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1367,7 +1367,7 @@
         </is>
       </c>
       <c r="G21" s="1" t="n">
-        <v>46217.60097222222</v>
+        <v>46217.60430555556</v>
       </c>
       <c r="I21" t="n">
         <v>29</v>
@@ -1384,7 +1384,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>nomorales@colsanitas.com</t>
+          <t>gerencia@hus.org.co</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1397,7 +1397,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica Universitaria Colombia (Colsanitas)</t>
+          <t>Oportunidad de Hospital Universitario de la Samaritana</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1406,7 +1406,7 @@
         </is>
       </c>
       <c r="G22" s="1" t="n">
-        <v>46217.59863425926</v>
+        <v>46217.60261574074</v>
       </c>
       <c r="I22" t="n">
         <v>29</v>
@@ -1423,7 +1423,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>zayda.rodriguez@cpolaya.com.co</t>
+          <t>nomorales@colsanitas.com</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1436,7 +1436,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Oportunidad de Centro Policlínico del Olaya</t>
+          <t>Oportunidad de Clínica Colsanitas Reina Sofía Pediátrica y Mujer</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1445,7 +1445,7 @@
         </is>
       </c>
       <c r="G23" s="1" t="n">
-        <v>46217.59719907407</v>
+        <v>46217.60097222222</v>
       </c>
       <c r="I23" t="n">
         <v>29</v>
@@ -1462,7 +1462,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>pcasallas@lacardiol.org</t>
+          <t>nomorales@colsanitas.com</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1475,7 +1475,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Oportunidad de Fundación Cardioinfantil - Instituto de Cardiología</t>
+          <t>Oportunidad de Clínica Universitaria Colombia (Colsanitas)</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1484,7 +1484,7 @@
         </is>
       </c>
       <c r="G24" s="1" t="n">
-        <v>46217.59630787037</v>
+        <v>46217.59863425926</v>
       </c>
       <c r="I24" t="n">
         <v>29</v>
@@ -1501,7 +1501,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>dir_calidad@clinicajuanncorpas.com</t>
+          <t>zayda.rodriguez@cpolaya.com.co</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1514,7 +1514,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica Juan N Corpas Ltda</t>
+          <t>Oportunidad de Centro Policlínico del Olaya</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1523,7 +1523,7 @@
         </is>
       </c>
       <c r="G25" s="1" t="n">
-        <v>46217.52333333333</v>
+        <v>46217.59719907407</v>
       </c>
       <c r="I25" t="n">
         <v>29</v>
@@ -1540,7 +1540,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>dianaespinosanarvaez@gmail.com</t>
+          <t>pcasallas@lacardiol.org</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica Onkos</t>
+          <t>Oportunidad de Fundación Cardioinfantil - Instituto de Cardiología</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1562,7 +1562,7 @@
         </is>
       </c>
       <c r="G26" s="1" t="n">
-        <v>46217.52202546296</v>
+        <v>46217.59630787037</v>
       </c>
       <c r="I26" t="n">
         <v>29</v>
@@ -1579,7 +1579,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>gestiondecalidad@clinicapalermo.com.co</t>
+          <t>dir_calidad@clinicajuanncorpas.com</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1592,7 +1592,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica Palermo</t>
+          <t>Oportunidad de Clínica Juan N Corpas Ltda</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1601,7 +1601,7 @@
         </is>
       </c>
       <c r="G27" s="1" t="n">
-        <v>46217.51743055556</v>
+        <v>46217.52333333333</v>
       </c>
       <c r="I27" t="n">
         <v>29</v>
@@ -1618,7 +1618,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>calidad@hospitaldesanjose.org.co</t>
+          <t>dianaespinosanarvaez@gmail.com</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1631,7 +1631,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Oportunidad de Hospital San José - Sociedad de Cirugía de Bogotá</t>
+          <t>Oportunidad de Clínica Onkos</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1640,7 +1640,7 @@
         </is>
       </c>
       <c r="G28" s="1" t="n">
-        <v>46217.51425925926</v>
+        <v>46217.52202546296</v>
       </c>
       <c r="I28" t="n">
         <v>29</v>
@@ -1657,7 +1657,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>jzapata@ioir.org.co</t>
+          <t>gestiondecalidad@clinicapalermo.com.co</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1670,7 +1670,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Oportunidad de Instituto de Ortopedia Infantil Roosevelt</t>
+          <t>Oportunidad de Clínica Palermo</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1679,7 +1679,7 @@
         </is>
       </c>
       <c r="G29" s="1" t="n">
-        <v>46217.51231481481</v>
+        <v>46217.51743055556</v>
       </c>
       <c r="I29" t="n">
         <v>29</v>
@@ -1696,7 +1696,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>diana.potesno@colsubsidio.com</t>
+          <t>calidad@hospitaldesanjose.org.co</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1709,7 +1709,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica Colsubsidio Calle 100</t>
+          <t>Oportunidad de Hospital San José - Sociedad de Cirugía de Bogotá</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1718,7 +1718,7 @@
         </is>
       </c>
       <c r="G30" s="1" t="n">
-        <v>46217.51116898148</v>
+        <v>46217.51425925926</v>
       </c>
       <c r="I30" t="n">
         <v>29</v>
@@ -1735,7 +1735,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>diana.potesno@colsubsidio.com</t>
+          <t>jzapata@ioir.org.co</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1748,7 +1748,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica Colsubsidio Calle 100</t>
+          <t>Oportunidad de Instituto de Ortopedia Infantil Roosevelt</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1757,7 +1757,7 @@
         </is>
       </c>
       <c r="G31" s="1" t="n">
-        <v>46217.50983796296</v>
+        <v>46217.51231481481</v>
       </c>
       <c r="I31" t="n">
         <v>29</v>
@@ -1774,7 +1774,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>jose.chaves@colsubsidio.com</t>
+          <t>diana.potesno@colsubsidio.com</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1787,7 +1787,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica Colsubsidio Ciudad Roma</t>
+          <t>Oportunidad de Clínica Colsubsidio Calle 100</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1796,7 +1796,7 @@
         </is>
       </c>
       <c r="G32" s="1" t="n">
-        <v>46217.50767361111</v>
+        <v>46217.51116898148</v>
       </c>
       <c r="I32" t="n">
         <v>29</v>
@@ -1813,7 +1813,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>carlos.artetamo@colsubsidio.com</t>
+          <t>diana.potesno@colsubsidio.com</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1826,7 +1826,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica Infantil Colsubsidio</t>
+          <t>Oportunidad de Clínica Colsubsidio Calle 100</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1835,7 +1835,7 @@
         </is>
       </c>
       <c r="G33" s="1" t="n">
-        <v>46217.50050925926</v>
+        <v>46217.50983796296</v>
       </c>
       <c r="I33" t="n">
         <v>29</v>
@@ -1852,7 +1852,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>notificacionescdc@clinicadelcountry.com</t>
+          <t>jose.chaves@colsubsidio.com</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1865,7 +1865,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica del Country IPS</t>
+          <t>Oportunidad de Clínica Colsubsidio Ciudad Roma</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1874,7 +1874,7 @@
         </is>
       </c>
       <c r="G34" s="1" t="n">
-        <v>46217.49881944444</v>
+        <v>46217.50767361111</v>
       </c>
       <c r="I34" t="n">
         <v>29</v>
@@ -1891,7 +1891,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>direcciongeneral@shaio.org</t>
+          <t>carlos.artetamo@colsubsidio.com</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1904,7 +1904,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Oportunidad de Fundación Abood Shaio</t>
+          <t>Oportunidad de Clínica Infantil Colsubsidio</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1913,7 +1913,7 @@
         </is>
       </c>
       <c r="G35" s="1" t="n">
-        <v>46217.49715277777</v>
+        <v>46217.50050925926</v>
       </c>
       <c r="I35" t="n">
         <v>29</v>
@@ -1930,7 +1930,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>direccion@cancer.gov.co</t>
+          <t>notificacionescdc@clinicadelcountry.com</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1943,7 +1943,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Oportunidad de Instituto Nacional de Cancerología</t>
+          <t>Oportunidad de Clínica del Country IPS</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -1952,7 +1952,7 @@
         </is>
       </c>
       <c r="G36" s="1" t="n">
-        <v>46217.47924768519</v>
+        <v>46217.49881944444</v>
       </c>
       <c r="I36" t="n">
         <v>29</v>
@@ -1969,7 +1969,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>sdirmedica@clinicadelamujer.com.co</t>
+          <t>direcciongeneral@shaio.org</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1982,7 +1982,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica de la Mujer</t>
+          <t>Oportunidad de Fundación Abood Shaio</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -1991,7 +1991,7 @@
         </is>
       </c>
       <c r="G37" s="1" t="n">
-        <v>46217.47585648148</v>
+        <v>46217.49715277777</v>
       </c>
       <c r="I37" t="n">
         <v>29</v>
@@ -2008,7 +2008,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>lidercalidad@homifundacion.org.co</t>
+          <t>direccion@cancer.gov.co</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2021,7 +2021,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Oportunidad de Fundación Hospital de la Misericordia (HOMI)</t>
+          <t>Oportunidad de Instituto Nacional de Cancerología</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2030,7 +2030,7 @@
         </is>
       </c>
       <c r="G38" s="1" t="n">
-        <v>46217.47246527778</v>
+        <v>46217.47924768519</v>
       </c>
       <c r="I38" t="n">
         <v>29</v>
@@ -2047,7 +2047,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>direcciongeneral1@stewardcolombia.org</t>
+          <t>sdirmedica@clinicadelamujer.com.co</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2060,7 +2060,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Oportunidad de Hospital Universitario Clínica San Rafael</t>
+          <t>Oportunidad de Clínica de la Mujer</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2069,7 +2069,7 @@
         </is>
       </c>
       <c r="G39" s="1" t="n">
-        <v>46217.00748842592</v>
+        <v>46217.47585648148</v>
       </c>
       <c r="I39" t="n">
         <v>29</v>
@@ -2086,7 +2086,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>adriana.urrego@fsfb.org.co</t>
+          <t>lidercalidad@homifundacion.org.co</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2099,7 +2099,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Oportunidad de FUNDACION SANTA FE DE BOGOTA</t>
+          <t>Oportunidad de Fundación Hospital de la Misericordia (HOMI)</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -2108,7 +2108,7 @@
         </is>
       </c>
       <c r="G40" s="1" t="n">
-        <v>46217.00381944444</v>
+        <v>46217.47246527778</v>
       </c>
       <c r="I40" t="n">
         <v>29</v>
@@ -2125,7 +2125,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>calidadsalud@cafam.com.co</t>
+          <t>direcciongeneral1@stewardcolombia.org</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2138,7 +2138,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Oportunidad de Centro de Atención en Salud CAFAM Clínica Calle 51</t>
+          <t>Oportunidad de Hospital Universitario Clínica San Rafael</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2147,7 +2147,7 @@
         </is>
       </c>
       <c r="G41" s="1" t="n">
-        <v>46216.99954861111</v>
+        <v>46217.00748842592</v>
       </c>
       <c r="I41" t="n">
         <v>29</v>
@@ -2164,7 +2164,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>notificacionesjudiciales@fhsc.org.co</t>
+          <t>adriana.urrego@fsfb.org.co</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2177,7 +2177,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Oportunidad de Fundación Hospital San Carlos</t>
+          <t>Oportunidad de FUNDACION SANTA FE DE BOGOTA</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -2186,7 +2186,7 @@
         </is>
       </c>
       <c r="G42" s="1" t="n">
-        <v>46216.99548611111</v>
+        <v>46217.00381944444</v>
       </c>
       <c r="I42" t="n">
         <v>29</v>
@@ -2203,7 +2203,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>calidad@proseguir.org</t>
+          <t>calidadsalud@cafam.com.co</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2216,7 +2216,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Oportunidad de PROSEGUIR SEDE 3</t>
+          <t>Oportunidad de Centro de Atención en Salud CAFAM Clínica Calle 51</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2225,7 +2225,7 @@
         </is>
       </c>
       <c r="G43" s="1" t="n">
-        <v>46216.99299768519</v>
+        <v>46216.99954861111</v>
       </c>
       <c r="I43" t="n">
         <v>29</v>
@@ -2242,71 +2242,71 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>centrodecontacto@uao.edu.co</t>
+          <t>notificacionesjudiciales@fhsc.org.co</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>10000000</v>
+        <v>0</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Oportunidad de UNIVERSIDAD AUTONOMA DE OCCIDENTE</t>
+          <t>Oportunidad de Fundación Hospital San Carlos</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G44" s="1" t="n">
-        <v>46213.49821759259</v>
+        <v>46216.99548611111</v>
       </c>
       <c r="I44" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J44" t="n">
         <v>2026</v>
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>carlos.segovia@warena.co</t>
+          <t>calidad@proseguir.org</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>35000000</v>
+        <v>0</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Oportunidad de W ARENA</t>
+          <t>Oportunidad de PROSEGUIR SEDE 3</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G45" s="1" t="n">
-        <v>46213.49508101852</v>
+        <v>46216.99299768519</v>
       </c>
       <c r="I45" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J45" t="n">
         <v>2026</v>
@@ -2320,37 +2320,29 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>klondono@fundacionwwbcol.org</t>
+          <t>centrodecontacto@uao.edu.co</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Ganado</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>300000</v>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>Karla Londoño</t>
-        </is>
+        <v>10000000</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Oportunidad de Karla Londoño</t>
+          <t>Oportunidad de UNIVERSIDAD AUTONOMA DE OCCIDENTE</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G46" s="1" t="n">
-        <v>46212.51638888889</v>
-      </c>
-      <c r="H46" s="1" t="n">
-        <v>46217</v>
+        <v>46213.49821759259</v>
       </c>
       <c r="I46" t="n">
         <v>28</v>
@@ -2358,12 +2350,6 @@
       <c r="J46" t="n">
         <v>2026</v>
       </c>
-      <c r="K46" t="n">
-        <v>7</v>
-      </c>
-      <c r="L46" t="n">
-        <v>2026</v>
-      </c>
       <c r="M46" t="inlineStr">
         <is>
           <t>Calificado</t>
@@ -2373,51 +2359,46 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>ctorres@colcobranzasnacionales.com</t>
+          <t>carlos.segovia@warena.co</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Negociación</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>5000000</v>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>ctorres@colcobranzasnacionales.com</t>
-        </is>
+        <v>35000000</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Oportunidad de ctorres@colcobranzasnacionales.com</t>
+          <t>Oportunidad de W ARENA</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G47" s="1" t="n">
-        <v>46206.73804398148</v>
+        <v>46213.49508101852</v>
       </c>
       <c r="I47" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J47" t="n">
         <v>2026</v>
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>medifar624@gmail.com</t>
+          <t>klondono@fundacionwwbcol.org</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2426,11 +2407,16 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>1640000</v>
+        <v>300000</v>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Karla Londoño</t>
+        </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Oportunidad de MEDISFARMA SAS</t>
+          <t>Oportunidad de Karla Londoño</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2439,13 +2425,13 @@
         </is>
       </c>
       <c r="G48" s="1" t="n">
-        <v>46203.72597222222</v>
+        <v>46212.51638888889</v>
       </c>
       <c r="H48" s="1" t="n">
         <v>46217</v>
       </c>
       <c r="I48" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J48" t="n">
         <v>2026</v>
@@ -2465,7 +2451,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>mercadeo@norteysur.co</t>
+          <t>ctorres@colcobranzasnacionales.com</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2474,16 +2460,16 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>28190000</v>
+        <v>5000000</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Isabella Mesa</t>
+          <t>ctorres@colcobranzasnacionales.com</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Oportunidad de Isabella Mesa</t>
+          <t>Oportunidad de ctorres@colcobranzasnacionales.com</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -2492,10 +2478,10 @@
         </is>
       </c>
       <c r="G49" s="1" t="n">
-        <v>46191.70076388889</v>
+        <v>46206.73804398148</v>
       </c>
       <c r="I49" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="J49" t="n">
         <v>2026</v>
@@ -2509,20 +2495,20 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>comercial@asertis.com.co</t>
+          <t>medifar624@gmail.com</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Ganado</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>0</v>
+        <v>1640000</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Oportunidad de IMPORTADORA CALI S.A.</t>
+          <t>Oportunidad de MEDISFARMA SAS</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -2531,42 +2517,51 @@
         </is>
       </c>
       <c r="G50" s="1" t="n">
-        <v>46189.67539351852</v>
+        <v>46203.72597222222</v>
+      </c>
+      <c r="H50" s="1" t="n">
+        <v>46217</v>
       </c>
       <c r="I50" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="J50" t="n">
         <v>2026</v>
       </c>
+      <c r="K50" t="n">
+        <v>7</v>
+      </c>
+      <c r="L50" t="n">
+        <v>2026</v>
+      </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>educacion@360forma.edu.co</t>
+          <t>mercadeo@norteysur.co</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Negociación</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>0</v>
+        <v>28190000</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Jorge Sanchez / jefe Comercial</t>
+          <t>Isabella Mesa</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Oportunidad de Jorge Sanchez / jefe Comercial</t>
+          <t>Oportunidad de Isabella Mesa</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -2575,7 +2570,7 @@
         </is>
       </c>
       <c r="G51" s="1" t="n">
-        <v>46189.65077546296</v>
+        <v>46191.70076388889</v>
       </c>
       <c r="I51" t="n">
         <v>25</v>
@@ -2585,19 +2580,19 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>directoradjunto@dclass.edu.co</t>
+          <t>comercial@asertis.com.co</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -2605,7 +2600,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Oportunidad de DCLASS ACADEMIA SAS</t>
+          <t>Oportunidad de IMPORTADORA CALI S.A.</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -2614,7 +2609,7 @@
         </is>
       </c>
       <c r="G52" s="1" t="n">
-        <v>46189.49674768518</v>
+        <v>46189.67539351852</v>
       </c>
       <c r="I52" t="n">
         <v>25</v>
@@ -2624,27 +2619,32 @@
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Belkis.jimenez@agrauto.com.co</t>
+          <t>educacion@360forma.edu.co</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="C53" t="n">
         <v>0</v>
       </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Jorge Sanchez / jefe Comercial</t>
+        </is>
+      </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Oportunidad de AGRICOLA AUTOMOTRIZ SAS / BELKYS JIMENEZ</t>
+          <t>Oportunidad de Jorge Sanchez / jefe Comercial</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -2653,42 +2653,37 @@
         </is>
       </c>
       <c r="G53" s="1" t="n">
-        <v>46182.67912037037</v>
+        <v>46189.65077546296</v>
       </c>
       <c r="I53" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J53" t="n">
         <v>2026</v>
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>luisa.baena@automarcali.com</t>
+          <t>directoradjunto@dclass.edu.co</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C54" t="n">
         <v>0</v>
       </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>luisa.baena@automarcali.com</t>
-        </is>
-      </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Oportunidad de luisa.baena@automarcali.com</t>
+          <t>Oportunidad de DCLASS ACADEMIA SAS</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -2697,24 +2692,24 @@
         </is>
       </c>
       <c r="G54" s="1" t="n">
-        <v>46182.67809027778</v>
+        <v>46189.49674768518</v>
       </c>
       <c r="I54" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J54" t="n">
         <v>2026</v>
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>directormercadeo@almotores.com</t>
+          <t>Belkis.jimenez@agrauto.com.co</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2725,14 +2720,9 @@
       <c r="C55" t="n">
         <v>0</v>
       </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>Viviana Vanegas</t>
-        </is>
-      </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Oportunidad de Viviana Vanegas</t>
+          <t>Oportunidad de AGRICOLA AUTOMOTRIZ SAS / BELKYS JIMENEZ</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -2741,7 +2731,7 @@
         </is>
       </c>
       <c r="G55" s="1" t="n">
-        <v>46182.67621527778</v>
+        <v>46182.67912037037</v>
       </c>
       <c r="I55" t="n">
         <v>24</v>
@@ -2758,7 +2748,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>xiomara.duran@autopacifico.com.co</t>
+          <t>luisa.baena@automarcali.com</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2769,9 +2759,14 @@
       <c r="C56" t="n">
         <v>0</v>
       </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>luisa.baena@automarcali.com</t>
+        </is>
+      </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Oportunidad de xiomara.duran@autopacifico.com.co</t>
+          <t>Oportunidad de luisa.baena@automarcali.com</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -2780,7 +2775,7 @@
         </is>
       </c>
       <c r="G56" s="1" t="n">
-        <v>46182.65815972222</v>
+        <v>46182.67809027778</v>
       </c>
       <c r="I56" t="n">
         <v>24</v>
@@ -2797,12 +2792,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>alejandrosaavedraconde@comfandi.com.co</t>
+          <t>directormercadeo@almotores.com</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -2810,12 +2805,12 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>ALEJANDRO</t>
+          <t>Viviana Vanegas</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Oportunidad de ALEJANDRO</t>
+          <t>Oportunidad de Viviana Vanegas</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -2824,7 +2819,7 @@
         </is>
       </c>
       <c r="G57" s="1" t="n">
-        <v>46182.64278935185</v>
+        <v>46182.67621527778</v>
       </c>
       <c r="I57" t="n">
         <v>24</v>
@@ -2834,19 +2829,19 @@
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>administracion@fiando.com.co</t>
+          <t>xiomara.duran@autopacifico.com.co</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -2854,7 +2849,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Oportunidad de FIANDO LTDA</t>
+          <t>Oportunidad de xiomara.duran@autopacifico.com.co</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -2863,7 +2858,7 @@
         </is>
       </c>
       <c r="G58" s="1" t="n">
-        <v>46182.61304398148</v>
+        <v>46182.65815972222</v>
       </c>
       <c r="I58" t="n">
         <v>24</v>
@@ -2873,19 +2868,19 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>dgamoneda@productosdrogam.com</t>
+          <t>alejandrosaavedraconde@comfandi.com.co</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -2893,12 +2888,12 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t xml:space="preserve">Diego Mauricio Gamoneda </t>
+          <t>ALEJANDRO</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t xml:space="preserve">Oportunidad de Diego Mauricio Gamoneda </t>
+          <t>Oportunidad de ALEJANDRO</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -2907,10 +2902,10 @@
         </is>
       </c>
       <c r="G59" s="1" t="n">
-        <v>46175.66417824074</v>
+        <v>46182.64278935185</v>
       </c>
       <c r="I59" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J59" t="n">
         <v>2026</v>
@@ -2924,7 +2919,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>alexander.rojas@friogan.com</t>
+          <t>administracion@fiando.com.co</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2933,11 +2928,11 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>10000000</v>
+        <v>0</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Oportunidad de FRIOGAN S.A</t>
+          <t>Oportunidad de FIANDO LTDA</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -2946,10 +2941,10 @@
         </is>
       </c>
       <c r="G60" s="1" t="n">
-        <v>46175.63597222222</v>
+        <v>46182.61304398148</v>
       </c>
       <c r="I60" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J60" t="n">
         <v>2026</v>
@@ -2961,17 +2956,27 @@
       </c>
     </row>
     <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>dgamoneda@productosdrogam.com</t>
+        </is>
+      </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C61" t="n">
         <v>0</v>
       </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Diego Mauricio Gamoneda </t>
+        </is>
+      </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Oportunidad de Agromercados la Montaña</t>
+          <t xml:space="preserve">Oportunidad de Diego Mauricio Gamoneda </t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -2980,7 +2985,7 @@
         </is>
       </c>
       <c r="G61" s="1" t="n">
-        <v>46175.62239583334</v>
+        <v>46175.66417824074</v>
       </c>
       <c r="I61" t="n">
         <v>23</v>
@@ -2997,20 +3002,20 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>juand.rios@alkosto.com.co</t>
+          <t>alexander.rojas@friogan.com</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>0</v>
+        <v>10000000</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Oportunidad de ALKOSTO</t>
+          <t>Oportunidad de FRIOGAN S.A</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -3019,7 +3024,7 @@
         </is>
       </c>
       <c r="G62" s="1" t="n">
-        <v>46175.62055555556</v>
+        <v>46175.63597222222</v>
       </c>
       <c r="I62" t="n">
         <v>23</v>
@@ -3029,16 +3034,11 @@
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>gerencia4087@grupo-exito.com</t>
-        </is>
-      </c>
       <c r="B63" t="inlineStr">
         <is>
           <t>Perdido</t>
@@ -3047,14 +3047,9 @@
       <c r="C63" t="n">
         <v>0</v>
       </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>Grupo exito ‒ 1007386172 - Sneider Quirama</t>
-        </is>
-      </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Oportunidad de Grupo exito</t>
+          <t>Oportunidad de Agromercados la Montaña</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -3063,7 +3058,7 @@
         </is>
       </c>
       <c r="G63" s="1" t="n">
-        <v>46175.61638888889</v>
+        <v>46175.62239583334</v>
       </c>
       <c r="I63" t="n">
         <v>23</v>
@@ -3080,7 +3075,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>ldgomez@supertiendascanaveral.com</t>
+          <t>juand.rios@alkosto.com.co</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3091,14 +3086,9 @@
       <c r="C64" t="n">
         <v>0</v>
       </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>Luis David Gomez</t>
-        </is>
-      </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Oportunidad de Luis David Gomez</t>
+          <t>Oportunidad de ALKOSTO</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -3107,7 +3097,7 @@
         </is>
       </c>
       <c r="G64" s="1" t="n">
-        <v>46175.60493055556</v>
+        <v>46175.62055555556</v>
       </c>
       <c r="I64" t="n">
         <v>23</v>
@@ -3124,20 +3114,25 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>davida_vanegas@coomeva.com.co</t>
+          <t>gerencia4087@grupo-exito.com</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C65" t="n">
         <v>0</v>
       </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Grupo exito ‒ 1007386172 - Sneider Quirama</t>
+        </is>
+      </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Oportunidad de BANCOOMEVA</t>
+          <t>Oportunidad de Grupo exito</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -3146,7 +3141,7 @@
         </is>
       </c>
       <c r="G65" s="1" t="n">
-        <v>46175.47109953704</v>
+        <v>46175.61638888889</v>
       </c>
       <c r="I65" t="n">
         <v>23</v>
@@ -3163,12 +3158,12 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>alejandro.delgado@filedesk.com.co</t>
+          <t>ldgomez@supertiendascanaveral.com</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -3176,12 +3171,12 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>AlejandroDelgado</t>
+          <t>Luis David Gomez</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Oportunidad de AlejandroDelgado</t>
+          <t>Oportunidad de Luis David Gomez</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -3190,7 +3185,7 @@
         </is>
       </c>
       <c r="G66" s="1" t="n">
-        <v>46174.71665509259</v>
+        <v>46175.60493055556</v>
       </c>
       <c r="I66" t="n">
         <v>23</v>
@@ -3205,22 +3200,22 @@
       </c>
     </row>
     <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>davida_vanegas@coomeva.com.co</t>
+        </is>
+      </c>
       <c r="B67" t="inlineStr">
         <is>
           <t>Contactado</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>35000000</v>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>Olga Lucia Hurtado</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Oportunidad de Olga Lucia Hurtado</t>
+          <t>Oportunidad de BANCOOMEVA</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -3229,10 +3224,10 @@
         </is>
       </c>
       <c r="G67" s="1" t="n">
-        <v>46168.49854166667</v>
+        <v>46175.47109953704</v>
       </c>
       <c r="I67" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="J67" t="n">
         <v>2026</v>
@@ -3246,7 +3241,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>comercial2@felsyn.com</t>
+          <t>alejandro.delgado@filedesk.com.co</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -3255,11 +3250,16 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>713400</v>
+        <v>0</v>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>AlejandroDelgado</t>
+        </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Oportunidad de FONDO DE EMPLEADOS FELSYN</t>
+          <t>Oportunidad de AlejandroDelgado</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -3268,10 +3268,10 @@
         </is>
       </c>
       <c r="G68" s="1" t="n">
-        <v>46163.49130787037</v>
+        <v>46174.71665509259</v>
       </c>
       <c r="I68" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="J68" t="n">
         <v>2026</v>
@@ -3283,27 +3283,22 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>mercadeo@lasevillana.com.co</t>
-        </is>
-      </c>
       <c r="B69" t="inlineStr">
         <is>
           <t>Contactado</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>0</v>
+        <v>35000000</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fabio AlbertoGallego García </t>
+          <t>Olga Lucia Hurtado</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t xml:space="preserve">Oportunidad de Fabio AlbertoGallego García </t>
+          <t>Oportunidad de Olga Lucia Hurtado</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -3312,10 +3307,10 @@
         </is>
       </c>
       <c r="G69" s="1" t="n">
-        <v>46162.64569444444</v>
+        <v>46168.49854166667</v>
       </c>
       <c r="I69" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="J69" t="n">
         <v>2026</v>
@@ -3329,7 +3324,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>asantiago@stop.com.co</t>
+          <t>comercial2@felsyn.com</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -3338,11 +3333,11 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>0</v>
+        <v>713400</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Oportunidad de STOP SAS</t>
+          <t>Oportunidad de FONDO DE EMPLEADOS FELSYN</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -3351,7 +3346,7 @@
         </is>
       </c>
       <c r="G70" s="1" t="n">
-        <v>46161.63508101852</v>
+        <v>46163.49130787037</v>
       </c>
       <c r="I70" t="n">
         <v>21</v>
@@ -3368,25 +3363,25 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>aestrada@teker.co</t>
+          <t>mercadeo@lasevillana.com.co</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>16914000</v>
+        <v>0</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>TEKER SALUD SAS</t>
+          <t xml:space="preserve">Fabio AlbertoGallego García </t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Oportunidad de TEKER SALUD SAS</t>
+          <t xml:space="preserve">Oportunidad de Fabio AlbertoGallego García </t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -3395,7 +3390,7 @@
         </is>
       </c>
       <c r="G71" s="1" t="n">
-        <v>46161.62922453704</v>
+        <v>46162.64569444444</v>
       </c>
       <c r="I71" t="n">
         <v>21</v>
@@ -3410,6 +3405,11 @@
       </c>
     </row>
     <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>asantiago@stop.com.co</t>
+        </is>
+      </c>
       <c r="B72" t="inlineStr">
         <is>
           <t>Contactado</t>
@@ -3420,7 +3420,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Oportunidad de TIAN IPS SAS</t>
+          <t>Oportunidad de STOP SAS</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -3429,7 +3429,7 @@
         </is>
       </c>
       <c r="G72" s="1" t="n">
-        <v>46161.61643518518</v>
+        <v>46161.63508101852</v>
       </c>
       <c r="I72" t="n">
         <v>21</v>
@@ -3446,7 +3446,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>administración@fullredtotal.com</t>
+          <t>aestrada@teker.co</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -3455,16 +3455,16 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>14000000</v>
+        <v>16914000</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Eivar Eñasco</t>
+          <t>TEKER SALUD SAS</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Oportunidad de Eivar Eñasco</t>
+          <t>Oportunidad de TEKER SALUD SAS</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -3473,10 +3473,10 @@
         </is>
       </c>
       <c r="G73" s="1" t="n">
-        <v>46154.67546296296</v>
+        <v>46161.62922453704</v>
       </c>
       <c r="I73" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J73" t="n">
         <v>2026</v>
@@ -3488,27 +3488,17 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>cserna@surtifamiliar.com.co</t>
-        </is>
-      </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Ganado</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>975000</v>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>Claudia Patricia Serna</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Oportunidad de Claudia Patricia Serna</t>
+          <t>Oportunidad de TIAN IPS SAS</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -3517,51 +3507,42 @@
         </is>
       </c>
       <c r="G74" s="1" t="n">
-        <v>46154.66616898148</v>
-      </c>
-      <c r="H74" s="1" t="n">
-        <v>46217</v>
+        <v>46161.61643518518</v>
       </c>
       <c r="I74" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J74" t="n">
         <v>2026</v>
       </c>
-      <c r="K74" t="n">
-        <v>7</v>
-      </c>
-      <c r="L74" t="n">
-        <v>2026</v>
-      </c>
       <c r="M74" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>coordmercadeo@pacificcenter.co</t>
+          <t>administración@fullredtotal.com</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>5600000</v>
+        <v>14000000</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Claudia Castro</t>
+          <t>Eivar Eñasco</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Oportunidad de Claudia Castro</t>
+          <t>Oportunidad de Eivar Eñasco</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -3570,7 +3551,7 @@
         </is>
       </c>
       <c r="G75" s="1" t="n">
-        <v>46154.66341435185</v>
+        <v>46154.67546296296</v>
       </c>
       <c r="I75" t="n">
         <v>20</v>
@@ -3580,32 +3561,32 @@
       </c>
       <c r="M75" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>isabellarengifo27@gmail.com</t>
+          <t>cserna@surtifamiliar.com.co</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Ganado</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>28190000</v>
+        <v>975000</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Isabella Rengifo</t>
+          <t>Claudia Patricia Serna</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Oportunidad de Isabella Rengifo</t>
+          <t>Oportunidad de Claudia Patricia Serna</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -3614,7 +3595,10 @@
         </is>
       </c>
       <c r="G76" s="1" t="n">
-        <v>46154.65981481481</v>
+        <v>46154.66616898148</v>
+      </c>
+      <c r="H76" s="1" t="n">
+        <v>46217</v>
       </c>
       <c r="I76" t="n">
         <v>20</v>
@@ -3622,41 +3606,49 @@
       <c r="J76" t="n">
         <v>2026</v>
       </c>
+      <c r="K76" t="n">
+        <v>7</v>
+      </c>
+      <c r="L76" t="n">
+        <v>2026</v>
+      </c>
       <c r="M76" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>coordmercadeo@pacificcenter.co</t>
+        </is>
+      </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>50000000</v>
+        <v>5600000</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Paola Gómez - Agente Inmobiliaria Independiente</t>
+          <t>Claudia Castro</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Puesto de Trabajo CC Medellin</t>
+          <t>Oportunidad de Claudia Castro</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Richard Castaño</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G77" s="1" t="n">
-        <v>46154.49104166667</v>
-      </c>
-      <c r="H77" s="1" t="n">
-        <v>46170</v>
+        <v>46154.66341435185</v>
       </c>
       <c r="I77" t="n">
         <v>20</v>
@@ -3664,44 +3656,43 @@
       <c r="J77" t="n">
         <v>2026</v>
       </c>
-      <c r="K77" t="n">
-        <v>5</v>
-      </c>
-      <c r="L77" t="n">
-        <v>2026</v>
-      </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>alberto.ramirez@constructorabolivar.com</t>
+          <t>isabellarengifo27@gmail.com</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Ganado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>3000000</v>
+        <v>28190000</v>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Isabella Rengifo</t>
+        </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Oportunidad de NPS Relacional</t>
+          <t>Oportunidad de Isabella Rengifo</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G78" s="1" t="n">
-        <v>46154.44511574074</v>
+        <v>46154.65981481481</v>
       </c>
       <c r="I78" t="n">
         <v>20</v>
@@ -3711,7 +3702,7 @@
       </c>
       <c r="M78" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
@@ -3722,30 +3713,39 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>3000000</v>
+        <v>50000000</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>MADERKIT</t>
+          <t>Paola Gómez - Agente Inmobiliaria Independiente</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Oportunidad de MADERKIT</t>
+          <t>Puesto de Trabajo CC Medellin</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Richard Castaño</t>
         </is>
       </c>
       <c r="G79" s="1" t="n">
-        <v>46147.66540509259</v>
+        <v>46154.49104166667</v>
+      </c>
+      <c r="H79" s="1" t="n">
+        <v>46170</v>
       </c>
       <c r="I79" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J79" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K79" t="n">
+        <v>5</v>
+      </c>
+      <c r="L79" t="n">
         <v>2026</v>
       </c>
       <c r="M79" t="inlineStr">
@@ -3757,64 +3757,59 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>omer120395@gmail.com</t>
+          <t>alberto.ramirez@constructorabolivar.com</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
+          <t>Ganado</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Oportunidad de NPS Relacional</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Jennifer Hoyos Gallego</t>
+        </is>
+      </c>
+      <c r="G80" s="1" t="n">
+        <v>46154.44511574074</v>
+      </c>
+      <c r="I80" t="n">
+        <v>20</v>
+      </c>
+      <c r="J80" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M80" t="inlineStr">
+        <is>
+          <t>Calificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="B81" t="inlineStr">
+        <is>
           <t>Perdido</t>
         </is>
       </c>
-      <c r="C80" t="n">
-        <v>0</v>
-      </c>
-      <c r="D80" t="inlineStr">
-        <is>
-          <t>Omer Peñaloza</t>
-        </is>
-      </c>
-      <c r="E80" t="inlineStr">
-        <is>
-          <t>Oportunidad de Omer Peñaloza</t>
-        </is>
-      </c>
-      <c r="F80" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G80" s="1" t="n">
-        <v>46147.66090277778</v>
-      </c>
-      <c r="I80" t="n">
-        <v>19</v>
-      </c>
-      <c r="J80" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M80" t="inlineStr">
-        <is>
-          <t>No calificado</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t>directora.it@supermercadobelalcazar.com.co</t>
-        </is>
-      </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
       <c r="C81" t="n">
-        <v>6000000</v>
+        <v>3000000</v>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>MADERKIT</t>
+        </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Oportunidad de ABASTECEMOS DE OCCIDENTE</t>
+          <t>Oportunidad de MADERKIT</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -3823,21 +3818,12 @@
         </is>
       </c>
       <c r="G81" s="1" t="n">
-        <v>46147.64170138889</v>
-      </c>
-      <c r="H81" s="1" t="n">
-        <v>46157</v>
+        <v>46147.66540509259</v>
       </c>
       <c r="I81" t="n">
         <v>19</v>
       </c>
       <c r="J81" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K81" t="n">
-        <v>5</v>
-      </c>
-      <c r="L81" t="n">
         <v>2026</v>
       </c>
       <c r="M81" t="inlineStr">

</xml_diff>

<commit_message>
CRM actualizado — 14/07/2026 16:56
</commit_message>
<xml_diff>
--- a/CRM_PowerBI_BrendaLuna_actualizado.xlsx
+++ b/CRM_PowerBI_BrendaLuna_actualizado.xlsx
@@ -992,14 +992,9 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>calidad.vip@axacolpatria.co</t>
-        </is>
-      </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1007,7 +1002,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica VIP Centro de Medicina Internacional</t>
+          <t>Oportunidad de Fajas Gama Alta</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1016,7 +1011,7 @@
         </is>
       </c>
       <c r="G12" s="1" t="n">
-        <v>46217.63989583333</v>
+        <v>46217.64614583334</v>
       </c>
       <c r="I12" t="n">
         <v>29</v>
@@ -1033,12 +1028,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>hocen.direc@policia.gov.co</t>
+          <t>calidad.vip@axacolpatria.co</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -1046,7 +1041,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Oportunidad de Hospital Central Policía Nacional</t>
+          <t>Oportunidad de Clínica VIP Centro de Medicina Internacional</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1055,7 +1050,7 @@
         </is>
       </c>
       <c r="G13" s="1" t="n">
-        <v>46217.63702546297</v>
+        <v>46217.63989583333</v>
       </c>
       <c r="I13" t="n">
         <v>29</v>
@@ -1072,12 +1067,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>coor.calidad@clinicamedical.com.co</t>
+          <t>hocen.direc@policia.gov.co</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -1085,7 +1080,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica Medical S.A.S.</t>
+          <t>Oportunidad de Hospital Central Policía Nacional</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1094,7 +1089,7 @@
         </is>
       </c>
       <c r="G14" s="1" t="n">
-        <v>46217.62244212963</v>
+        <v>46217.63702546297</v>
       </c>
       <c r="I14" t="n">
         <v>29</v>
@@ -1111,12 +1106,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>calidad@institutodelcorazon.com</t>
+          <t>coor.calidad@clinicamedical.com.co</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -1124,7 +1119,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Oportunidad de Instituto del Corazón de Bogotá</t>
+          <t>Oportunidad de Clínica Medical S.A.S.</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1133,7 +1128,7 @@
         </is>
       </c>
       <c r="G15" s="1" t="n">
-        <v>46217.62072916667</v>
+        <v>46217.62244212963</v>
       </c>
       <c r="I15" t="n">
         <v>29</v>
@@ -1150,12 +1145,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ana.ulloa@mederi.com.co</t>
+          <t>calidad@institutodelcorazon.com</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -1163,7 +1158,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Oportunidad de Hospital Universitario Mayor - Mederi</t>
+          <t>Oportunidad de Instituto del Corazón de Bogotá</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1172,7 +1167,7 @@
         </is>
       </c>
       <c r="G16" s="1" t="n">
-        <v>46217.61866898148</v>
+        <v>46217.62072916667</v>
       </c>
       <c r="I16" t="n">
         <v>29</v>
@@ -1189,12 +1184,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ayudantia@homil.gov.co</t>
+          <t>ana.ulloa@mederi.com.co</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -1202,7 +1197,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Oportunidad de Hospital Militar Central</t>
+          <t>Oportunidad de Hospital Universitario Mayor - Mederi</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1211,7 +1206,7 @@
         </is>
       </c>
       <c r="G17" s="1" t="n">
-        <v>46217.61708333333</v>
+        <v>46217.61866898148</v>
       </c>
       <c r="I17" t="n">
         <v>29</v>
@@ -1228,12 +1223,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>direccion.general@hospitalinfantildesanjose.org.co</t>
+          <t>ayudantia@homil.gov.co</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -1241,7 +1236,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Oportunidad de Fundación Hospital Infantil Universitario de San José</t>
+          <t>Oportunidad de Hospital Militar Central</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1250,7 +1245,7 @@
         </is>
       </c>
       <c r="G18" s="1" t="n">
-        <v>46217.6153587963</v>
+        <v>46217.61708333333</v>
       </c>
       <c r="I18" t="n">
         <v>29</v>
@@ -1267,12 +1262,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>calidad@clinicadeloccidente.com</t>
+          <t>direccion.general@hospitalinfantildesanjose.org.co</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -1280,7 +1275,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica del Occidente S.A.</t>
+          <t>Oportunidad de Fundación Hospital Infantil Universitario de San José</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1289,7 +1284,7 @@
         </is>
       </c>
       <c r="G19" s="1" t="n">
-        <v>46217.61388888889</v>
+        <v>46217.6153587963</v>
       </c>
       <c r="I19" t="n">
         <v>29</v>
@@ -1306,12 +1301,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>calidad@husi.org.co</t>
+          <t>calidad@clinicadeloccidente.com</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -1319,7 +1314,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Oportunidad de Hospital Universitario San Ignacio</t>
+          <t>Oportunidad de Clínica del Occidente S.A.</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1328,7 +1323,7 @@
         </is>
       </c>
       <c r="G20" s="1" t="n">
-        <v>46217.61174768519</v>
+        <v>46217.61388888889</v>
       </c>
       <c r="I20" t="n">
         <v>29</v>
@@ -1345,12 +1340,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>cmarly@clinicademarly.com.co</t>
+          <t>calidad@husi.org.co</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -1358,7 +1353,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica de Marly</t>
+          <t>Oportunidad de Hospital Universitario San Ignacio</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1367,7 +1362,7 @@
         </is>
       </c>
       <c r="G21" s="1" t="n">
-        <v>46217.60430555556</v>
+        <v>46217.61174768519</v>
       </c>
       <c r="I21" t="n">
         <v>29</v>
@@ -1384,12 +1379,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>gerencia@hus.org.co</t>
+          <t>cmarly@clinicademarly.com.co</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -1397,7 +1392,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Oportunidad de Hospital Universitario de la Samaritana</t>
+          <t>Oportunidad de Clínica de Marly</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1406,7 +1401,7 @@
         </is>
       </c>
       <c r="G22" s="1" t="n">
-        <v>46217.60261574074</v>
+        <v>46217.60430555556</v>
       </c>
       <c r="I22" t="n">
         <v>29</v>
@@ -1423,12 +1418,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>nomorales@colsanitas.com</t>
+          <t>gerencia@hus.org.co</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -1436,7 +1431,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica Colsanitas Reina Sofía Pediátrica y Mujer</t>
+          <t>Oportunidad de Hospital Universitario de la Samaritana</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1445,7 +1440,7 @@
         </is>
       </c>
       <c r="G23" s="1" t="n">
-        <v>46217.60097222222</v>
+        <v>46217.60261574074</v>
       </c>
       <c r="I23" t="n">
         <v>29</v>
@@ -1467,7 +1462,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -1475,7 +1470,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica Universitaria Colombia (Colsanitas)</t>
+          <t>Oportunidad de Clínica Colsanitas Reina Sofía Pediátrica y Mujer</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1484,7 +1479,7 @@
         </is>
       </c>
       <c r="G24" s="1" t="n">
-        <v>46217.59863425926</v>
+        <v>46217.60097222222</v>
       </c>
       <c r="I24" t="n">
         <v>29</v>
@@ -1501,12 +1496,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>zayda.rodriguez@cpolaya.com.co</t>
+          <t>nomorales@colsanitas.com</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -1514,7 +1509,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Oportunidad de Centro Policlínico del Olaya</t>
+          <t>Oportunidad de Clínica Universitaria Colombia (Colsanitas)</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1523,7 +1518,7 @@
         </is>
       </c>
       <c r="G25" s="1" t="n">
-        <v>46217.59719907407</v>
+        <v>46217.59863425926</v>
       </c>
       <c r="I25" t="n">
         <v>29</v>
@@ -1540,12 +1535,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>pcasallas@lacardiol.org</t>
+          <t>zayda.rodriguez@cpolaya.com.co</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -1553,7 +1548,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Oportunidad de Fundación Cardioinfantil - Instituto de Cardiología</t>
+          <t>Oportunidad de Centro Policlínico del Olaya</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1562,7 +1557,7 @@
         </is>
       </c>
       <c r="G26" s="1" t="n">
-        <v>46217.59630787037</v>
+        <v>46217.59719907407</v>
       </c>
       <c r="I26" t="n">
         <v>29</v>
@@ -1579,12 +1574,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>dir_calidad@clinicajuanncorpas.com</t>
+          <t>pcasallas@lacardiol.org</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -1592,7 +1587,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica Juan N Corpas Ltda</t>
+          <t>Oportunidad de Fundación Cardioinfantil - Instituto de Cardiología</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1601,7 +1596,7 @@
         </is>
       </c>
       <c r="G27" s="1" t="n">
-        <v>46217.52333333333</v>
+        <v>46217.59630787037</v>
       </c>
       <c r="I27" t="n">
         <v>29</v>
@@ -1618,12 +1613,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>dianaespinosanarvaez@gmail.com</t>
+          <t>dir_calidad@clinicajuanncorpas.com</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -1631,7 +1626,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica Onkos</t>
+          <t>Oportunidad de Clínica Juan N Corpas Ltda</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1640,7 +1635,7 @@
         </is>
       </c>
       <c r="G28" s="1" t="n">
-        <v>46217.52202546296</v>
+        <v>46217.52333333333</v>
       </c>
       <c r="I28" t="n">
         <v>29</v>
@@ -1657,12 +1652,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>gestiondecalidad@clinicapalermo.com.co</t>
+          <t>dianaespinosanarvaez@gmail.com</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -1670,7 +1665,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica Palermo</t>
+          <t>Oportunidad de Clínica Onkos</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1679,7 +1674,7 @@
         </is>
       </c>
       <c r="G29" s="1" t="n">
-        <v>46217.51743055556</v>
+        <v>46217.52202546296</v>
       </c>
       <c r="I29" t="n">
         <v>29</v>
@@ -1696,12 +1691,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>calidad@hospitaldesanjose.org.co</t>
+          <t>gestiondecalidad@clinicapalermo.com.co</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -1709,7 +1704,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Oportunidad de Hospital San José - Sociedad de Cirugía de Bogotá</t>
+          <t>Oportunidad de Clínica Palermo</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1718,7 +1713,7 @@
         </is>
       </c>
       <c r="G30" s="1" t="n">
-        <v>46217.51425925926</v>
+        <v>46217.51743055556</v>
       </c>
       <c r="I30" t="n">
         <v>29</v>
@@ -1735,12 +1730,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>jzapata@ioir.org.co</t>
+          <t>calidad@hospitaldesanjose.org.co</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -1748,7 +1743,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Oportunidad de Instituto de Ortopedia Infantil Roosevelt</t>
+          <t>Oportunidad de Hospital San José - Sociedad de Cirugía de Bogotá</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1757,7 +1752,7 @@
         </is>
       </c>
       <c r="G31" s="1" t="n">
-        <v>46217.51231481481</v>
+        <v>46217.51425925926</v>
       </c>
       <c r="I31" t="n">
         <v>29</v>
@@ -1774,12 +1769,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>diana.potesno@colsubsidio.com</t>
+          <t>jzapata@ioir.org.co</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -1787,7 +1782,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica Colsubsidio Calle 100</t>
+          <t>Oportunidad de Instituto de Ortopedia Infantil Roosevelt</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1796,7 +1791,7 @@
         </is>
       </c>
       <c r="G32" s="1" t="n">
-        <v>46217.51116898148</v>
+        <v>46217.51231481481</v>
       </c>
       <c r="I32" t="n">
         <v>29</v>
@@ -1818,7 +1813,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -1835,7 +1830,7 @@
         </is>
       </c>
       <c r="G33" s="1" t="n">
-        <v>46217.50983796296</v>
+        <v>46217.51116898148</v>
       </c>
       <c r="I33" t="n">
         <v>29</v>
@@ -1852,12 +1847,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>jose.chaves@colsubsidio.com</t>
+          <t>diana.potesno@colsubsidio.com</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -1865,7 +1860,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica Colsubsidio Ciudad Roma</t>
+          <t>Oportunidad de Clínica Colsubsidio Calle 100</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1874,7 +1869,7 @@
         </is>
       </c>
       <c r="G34" s="1" t="n">
-        <v>46217.50767361111</v>
+        <v>46217.50983796296</v>
       </c>
       <c r="I34" t="n">
         <v>29</v>
@@ -1891,12 +1886,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>carlos.artetamo@colsubsidio.com</t>
+          <t>jose.chaves@colsubsidio.com</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -1904,7 +1899,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica Infantil Colsubsidio</t>
+          <t>Oportunidad de Clínica Colsubsidio Ciudad Roma</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1913,7 +1908,7 @@
         </is>
       </c>
       <c r="G35" s="1" t="n">
-        <v>46217.50050925926</v>
+        <v>46217.50767361111</v>
       </c>
       <c r="I35" t="n">
         <v>29</v>
@@ -1930,12 +1925,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>notificacionescdc@clinicadelcountry.com</t>
+          <t>carlos.artetamo@colsubsidio.com</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -1943,7 +1938,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica del Country IPS</t>
+          <t>Oportunidad de Clínica Infantil Colsubsidio</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -1952,7 +1947,7 @@
         </is>
       </c>
       <c r="G36" s="1" t="n">
-        <v>46217.49881944444</v>
+        <v>46217.50050925926</v>
       </c>
       <c r="I36" t="n">
         <v>29</v>
@@ -1969,12 +1964,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>direcciongeneral@shaio.org</t>
+          <t>notificacionescdc@clinicadelcountry.com</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -1982,7 +1977,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Oportunidad de Fundación Abood Shaio</t>
+          <t>Oportunidad de Clínica del Country IPS</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -1991,7 +1986,7 @@
         </is>
       </c>
       <c r="G37" s="1" t="n">
-        <v>46217.49715277777</v>
+        <v>46217.49881944444</v>
       </c>
       <c r="I37" t="n">
         <v>29</v>
@@ -2008,12 +2003,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>direccion@cancer.gov.co</t>
+          <t>direcciongeneral@shaio.org</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -2021,7 +2016,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Oportunidad de Instituto Nacional de Cancerología</t>
+          <t>Oportunidad de Fundación Abood Shaio</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2030,7 +2025,7 @@
         </is>
       </c>
       <c r="G38" s="1" t="n">
-        <v>46217.47924768519</v>
+        <v>46217.49715277777</v>
       </c>
       <c r="I38" t="n">
         <v>29</v>
@@ -2047,12 +2042,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>sdirmedica@clinicadelamujer.com.co</t>
+          <t>direccion@cancer.gov.co</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -2060,7 +2055,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica de la Mujer</t>
+          <t>Oportunidad de Instituto Nacional de Cancerología</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2069,7 +2064,7 @@
         </is>
       </c>
       <c r="G39" s="1" t="n">
-        <v>46217.47585648148</v>
+        <v>46217.47924768519</v>
       </c>
       <c r="I39" t="n">
         <v>29</v>
@@ -2086,12 +2081,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>lidercalidad@homifundacion.org.co</t>
+          <t>sdirmedica@clinicadelamujer.com.co</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -2099,7 +2094,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Oportunidad de Fundación Hospital de la Misericordia (HOMI)</t>
+          <t>Oportunidad de Clínica de la Mujer</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -2108,7 +2103,7 @@
         </is>
       </c>
       <c r="G40" s="1" t="n">
-        <v>46217.47246527778</v>
+        <v>46217.47585648148</v>
       </c>
       <c r="I40" t="n">
         <v>29</v>
@@ -2125,12 +2120,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>direcciongeneral1@stewardcolombia.org</t>
+          <t>lidercalidad@homifundacion.org.co</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -2138,7 +2133,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Oportunidad de Hospital Universitario Clínica San Rafael</t>
+          <t>Oportunidad de Fundación Hospital de la Misericordia (HOMI)</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2147,7 +2142,7 @@
         </is>
       </c>
       <c r="G41" s="1" t="n">
-        <v>46217.00748842592</v>
+        <v>46217.47246527778</v>
       </c>
       <c r="I41" t="n">
         <v>29</v>
@@ -2164,12 +2159,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>adriana.urrego@fsfb.org.co</t>
+          <t>direcciongeneral1@stewardcolombia.org</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -2177,7 +2172,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Oportunidad de FUNDACION SANTA FE DE BOGOTA</t>
+          <t>Oportunidad de Hospital Universitario Clínica San Rafael</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -2186,7 +2181,7 @@
         </is>
       </c>
       <c r="G42" s="1" t="n">
-        <v>46217.00381944444</v>
+        <v>46217.00748842592</v>
       </c>
       <c r="I42" t="n">
         <v>29</v>
@@ -2203,12 +2198,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>calidadsalud@cafam.com.co</t>
+          <t>adriana.urrego@fsfb.org.co</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -2216,7 +2211,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Oportunidad de Centro de Atención en Salud CAFAM Clínica Calle 51</t>
+          <t>Oportunidad de FUNDACION SANTA FE DE BOGOTA</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2225,7 +2220,7 @@
         </is>
       </c>
       <c r="G43" s="1" t="n">
-        <v>46216.99954861111</v>
+        <v>46217.00381944444</v>
       </c>
       <c r="I43" t="n">
         <v>29</v>
@@ -2242,12 +2237,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>notificacionesjudiciales@fhsc.org.co</t>
+          <t>calidadsalud@cafam.com.co</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -2255,7 +2250,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Oportunidad de Fundación Hospital San Carlos</t>
+          <t>Oportunidad de Centro de Atención en Salud CAFAM Clínica Calle 51</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -2264,7 +2259,7 @@
         </is>
       </c>
       <c r="G44" s="1" t="n">
-        <v>46216.99548611111</v>
+        <v>46216.99954861111</v>
       </c>
       <c r="I44" t="n">
         <v>29</v>
@@ -2281,12 +2276,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>calidad@proseguir.org</t>
+          <t>notificacionesjudiciales@fhsc.org.co</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -2294,7 +2289,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Oportunidad de PROSEGUIR SEDE 3</t>
+          <t>Oportunidad de Fundación Hospital San Carlos</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -2303,7 +2298,7 @@
         </is>
       </c>
       <c r="G45" s="1" t="n">
-        <v>46216.99299768519</v>
+        <v>46216.99548611111</v>
       </c>
       <c r="I45" t="n">
         <v>29</v>
@@ -2320,59 +2315,59 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>centrodecontacto@uao.edu.co</t>
+          <t>calidad@proseguir.org</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>10000000</v>
+        <v>0</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Oportunidad de UNIVERSIDAD AUTONOMA DE OCCIDENTE</t>
+          <t>Oportunidad de PROSEGUIR SEDE 3</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G46" s="1" t="n">
-        <v>46213.49821759259</v>
+        <v>46216.99299768519</v>
       </c>
       <c r="I46" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J46" t="n">
         <v>2026</v>
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>carlos.segovia@warena.co</t>
+          <t>centrodecontacto@uao.edu.co</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>35000000</v>
+        <v>10000000</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Oportunidad de W ARENA</t>
+          <t>Oportunidad de UNIVERSIDAD AUTONOMA DE OCCIDENTE</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -2381,7 +2376,7 @@
         </is>
       </c>
       <c r="G47" s="1" t="n">
-        <v>46213.49508101852</v>
+        <v>46213.49821759259</v>
       </c>
       <c r="I47" t="n">
         <v>28</v>
@@ -2391,44 +2386,36 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>klondono@fundacionwwbcol.org</t>
+          <t>carlos.segovia@warena.co</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Ganado</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>300000</v>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>Karla Londoño</t>
-        </is>
+        <v>35000000</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Oportunidad de Karla Londoño</t>
+          <t>Oportunidad de W ARENA</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G48" s="1" t="n">
-        <v>46212.51638888889</v>
-      </c>
-      <c r="H48" s="1" t="n">
-        <v>46217</v>
+        <v>46213.49508101852</v>
       </c>
       <c r="I48" t="n">
         <v>28</v>
@@ -2436,40 +2423,34 @@
       <c r="J48" t="n">
         <v>2026</v>
       </c>
-      <c r="K48" t="n">
-        <v>7</v>
-      </c>
-      <c r="L48" t="n">
-        <v>2026</v>
-      </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>ctorres@colcobranzasnacionales.com</t>
+          <t>klondono@fundacionwwbcol.org</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Negociación</t>
+          <t>Ganado</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>5000000</v>
+        <v>300000</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>ctorres@colcobranzasnacionales.com</t>
+          <t>Karla Londoño</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Oportunidad de ctorres@colcobranzasnacionales.com</t>
+          <t>Oportunidad de Karla Londoño</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -2478,12 +2459,21 @@
         </is>
       </c>
       <c r="G49" s="1" t="n">
-        <v>46206.73804398148</v>
+        <v>46212.51638888889</v>
+      </c>
+      <c r="H49" s="1" t="n">
+        <v>46217</v>
       </c>
       <c r="I49" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J49" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K49" t="n">
+        <v>7</v>
+      </c>
+      <c r="L49" t="n">
         <v>2026</v>
       </c>
       <c r="M49" t="inlineStr">
@@ -2495,20 +2485,25 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>medifar624@gmail.com</t>
+          <t>ctorres@colcobranzasnacionales.com</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Ganado</t>
+          <t>Negociación</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>1640000</v>
+        <v>5000000</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>ctorres@colcobranzasnacionales.com</t>
+        </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Oportunidad de MEDISFARMA SAS</t>
+          <t>Oportunidad de ctorres@colcobranzasnacionales.com</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -2517,10 +2512,7 @@
         </is>
       </c>
       <c r="G50" s="1" t="n">
-        <v>46203.72597222222</v>
-      </c>
-      <c r="H50" s="1" t="n">
-        <v>46217</v>
+        <v>46206.73804398148</v>
       </c>
       <c r="I50" t="n">
         <v>27</v>
@@ -2528,12 +2520,6 @@
       <c r="J50" t="n">
         <v>2026</v>
       </c>
-      <c r="K50" t="n">
-        <v>7</v>
-      </c>
-      <c r="L50" t="n">
-        <v>2026</v>
-      </c>
       <c r="M50" t="inlineStr">
         <is>
           <t>Calificado</t>
@@ -2543,25 +2529,20 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>mercadeo@norteysur.co</t>
+          <t>medifar624@gmail.com</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Negociación</t>
+          <t>Ganado</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>28190000</v>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>Isabella Mesa</t>
-        </is>
+        <v>1640000</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Oportunidad de Isabella Mesa</t>
+          <t>Oportunidad de MEDISFARMA SAS</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -2570,12 +2551,21 @@
         </is>
       </c>
       <c r="G51" s="1" t="n">
-        <v>46191.70076388889</v>
+        <v>46203.72597222222</v>
+      </c>
+      <c r="H51" s="1" t="n">
+        <v>46199</v>
       </c>
       <c r="I51" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="J51" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K51" t="n">
+        <v>6</v>
+      </c>
+      <c r="L51" t="n">
         <v>2026</v>
       </c>
       <c r="M51" t="inlineStr">
@@ -2587,20 +2577,25 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>comercial@asertis.com.co</t>
+          <t>mercadeo@norteysur.co</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Negociación</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>0</v>
+        <v>28190000</v>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Isabella Mesa</t>
+        </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Oportunidad de IMPORTADORA CALI S.A.</t>
+          <t>Oportunidad de Isabella Mesa</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -2609,7 +2604,7 @@
         </is>
       </c>
       <c r="G52" s="1" t="n">
-        <v>46189.67539351852</v>
+        <v>46191.70076388889</v>
       </c>
       <c r="I52" t="n">
         <v>25</v>
@@ -2619,32 +2614,27 @@
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>educacion@360forma.edu.co</t>
+          <t>comercial@asertis.com.co</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C53" t="n">
         <v>0</v>
       </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>Jorge Sanchez / jefe Comercial</t>
-        </is>
-      </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Oportunidad de Jorge Sanchez / jefe Comercial</t>
+          <t>Oportunidad de IMPORTADORA CALI S.A.</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -2653,7 +2643,7 @@
         </is>
       </c>
       <c r="G53" s="1" t="n">
-        <v>46189.65077546296</v>
+        <v>46189.67539351852</v>
       </c>
       <c r="I53" t="n">
         <v>25</v>
@@ -2670,20 +2660,25 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>directoradjunto@dclass.edu.co</t>
+          <t>educacion@360forma.edu.co</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C54" t="n">
         <v>0</v>
       </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Jorge Sanchez / jefe Comercial</t>
+        </is>
+      </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Oportunidad de DCLASS ACADEMIA SAS</t>
+          <t>Oportunidad de Jorge Sanchez / jefe Comercial</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -2692,7 +2687,7 @@
         </is>
       </c>
       <c r="G54" s="1" t="n">
-        <v>46189.49674768518</v>
+        <v>46189.65077546296</v>
       </c>
       <c r="I54" t="n">
         <v>25</v>
@@ -2702,19 +2697,19 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Belkis.jimenez@agrauto.com.co</t>
+          <t>directoradjunto@dclass.edu.co</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -2722,7 +2717,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Oportunidad de AGRICOLA AUTOMOTRIZ SAS / BELKYS JIMENEZ</t>
+          <t>Oportunidad de DCLASS ACADEMIA SAS</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -2731,24 +2726,24 @@
         </is>
       </c>
       <c r="G55" s="1" t="n">
-        <v>46182.67912037037</v>
+        <v>46189.49674768518</v>
       </c>
       <c r="I55" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J55" t="n">
         <v>2026</v>
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>luisa.baena@automarcali.com</t>
+          <t>Belkis.jimenez@agrauto.com.co</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2759,14 +2754,9 @@
       <c r="C56" t="n">
         <v>0</v>
       </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>luisa.baena@automarcali.com</t>
-        </is>
-      </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Oportunidad de luisa.baena@automarcali.com</t>
+          <t>Oportunidad de AGRICOLA AUTOMOTRIZ SAS / BELKYS JIMENEZ</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -2775,7 +2765,7 @@
         </is>
       </c>
       <c r="G56" s="1" t="n">
-        <v>46182.67809027778</v>
+        <v>46182.67912037037</v>
       </c>
       <c r="I56" t="n">
         <v>24</v>
@@ -2792,12 +2782,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>directormercadeo@almotores.com</t>
+          <t>luisa.baena@automarcali.com</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -2805,12 +2795,12 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Viviana Vanegas</t>
+          <t>luisa.baena@automarcali.com</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Oportunidad de Viviana Vanegas</t>
+          <t>Oportunidad de luisa.baena@automarcali.com</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -2819,7 +2809,7 @@
         </is>
       </c>
       <c r="G57" s="1" t="n">
-        <v>46182.67621527778</v>
+        <v>46182.67809027778</v>
       </c>
       <c r="I57" t="n">
         <v>24</v>
@@ -2829,14 +2819,14 @@
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>xiomara.duran@autopacifico.com.co</t>
+          <t>directormercadeo@almotores.com</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2847,9 +2837,14 @@
       <c r="C58" t="n">
         <v>0</v>
       </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Viviana Vanegas</t>
+        </is>
+      </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Oportunidad de xiomara.duran@autopacifico.com.co</t>
+          <t>Oportunidad de Viviana Vanegas</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -2858,7 +2853,7 @@
         </is>
       </c>
       <c r="G58" s="1" t="n">
-        <v>46182.65815972222</v>
+        <v>46182.67621527778</v>
       </c>
       <c r="I58" t="n">
         <v>24</v>
@@ -2875,25 +2870,20 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>alejandrosaavedraconde@comfandi.com.co</t>
+          <t>xiomara.duran@autopacifico.com.co</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C59" t="n">
         <v>0</v>
       </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>ALEJANDRO</t>
-        </is>
-      </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Oportunidad de ALEJANDRO</t>
+          <t>Oportunidad de xiomara.duran@autopacifico.com.co</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -2902,7 +2892,7 @@
         </is>
       </c>
       <c r="G59" s="1" t="n">
-        <v>46182.64278935185</v>
+        <v>46182.65815972222</v>
       </c>
       <c r="I59" t="n">
         <v>24</v>
@@ -2919,20 +2909,25 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>administracion@fiando.com.co</t>
+          <t>alejandrosaavedraconde@comfandi.com.co</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C60" t="n">
         <v>0</v>
       </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>ALEJANDRO</t>
+        </is>
+      </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Oportunidad de FIANDO LTDA</t>
+          <t>Oportunidad de ALEJANDRO</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -2941,7 +2936,7 @@
         </is>
       </c>
       <c r="G60" s="1" t="n">
-        <v>46182.61304398148</v>
+        <v>46182.64278935185</v>
       </c>
       <c r="I60" t="n">
         <v>24</v>
@@ -2951,32 +2946,27 @@
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>dgamoneda@productosdrogam.com</t>
+          <t>administracion@fiando.com.co</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C61" t="n">
         <v>0</v>
       </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Diego Mauricio Gamoneda </t>
-        </is>
-      </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t xml:space="preserve">Oportunidad de Diego Mauricio Gamoneda </t>
+          <t>Oportunidad de FIANDO LTDA</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -2985,37 +2975,42 @@
         </is>
       </c>
       <c r="G61" s="1" t="n">
-        <v>46175.66417824074</v>
+        <v>46182.61304398148</v>
       </c>
       <c r="I61" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J61" t="n">
         <v>2026</v>
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>alexander.rojas@friogan.com</t>
+          <t>dgamoneda@productosdrogam.com</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>10000000</v>
+        <v>0</v>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Diego Mauricio Gamoneda </t>
+        </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Oportunidad de FRIOGAN S.A</t>
+          <t xml:space="preserve">Oportunidad de Diego Mauricio Gamoneda </t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -3024,7 +3019,7 @@
         </is>
       </c>
       <c r="G62" s="1" t="n">
-        <v>46175.63597222222</v>
+        <v>46175.66417824074</v>
       </c>
       <c r="I62" t="n">
         <v>23</v>
@@ -3034,22 +3029,27 @@
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>alexander.rojas@friogan.com</t>
+        </is>
+      </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>0</v>
+        <v>10000000</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Oportunidad de Agromercados la Montaña</t>
+          <t>Oportunidad de FRIOGAN S.A</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -3058,7 +3058,7 @@
         </is>
       </c>
       <c r="G63" s="1" t="n">
-        <v>46175.62239583334</v>
+        <v>46175.63597222222</v>
       </c>
       <c r="I63" t="n">
         <v>23</v>
@@ -3068,16 +3068,11 @@
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>juand.rios@alkosto.com.co</t>
-        </is>
-      </c>
       <c r="B64" t="inlineStr">
         <is>
           <t>Perdido</t>
@@ -3088,7 +3083,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Oportunidad de ALKOSTO</t>
+          <t>Oportunidad de Agromercados la Montaña</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -3097,7 +3092,7 @@
         </is>
       </c>
       <c r="G64" s="1" t="n">
-        <v>46175.62055555556</v>
+        <v>46175.62239583334</v>
       </c>
       <c r="I64" t="n">
         <v>23</v>
@@ -3114,7 +3109,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>gerencia4087@grupo-exito.com</t>
+          <t>juand.rios@alkosto.com.co</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -3125,14 +3120,9 @@
       <c r="C65" t="n">
         <v>0</v>
       </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>Grupo exito ‒ 1007386172 - Sneider Quirama</t>
-        </is>
-      </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Oportunidad de Grupo exito</t>
+          <t>Oportunidad de ALKOSTO</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -3141,7 +3131,7 @@
         </is>
       </c>
       <c r="G65" s="1" t="n">
-        <v>46175.61638888889</v>
+        <v>46175.62055555556</v>
       </c>
       <c r="I65" t="n">
         <v>23</v>
@@ -3158,7 +3148,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>ldgomez@supertiendascanaveral.com</t>
+          <t>gerencia4087@grupo-exito.com</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -3171,12 +3161,12 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Luis David Gomez</t>
+          <t>Grupo exito ‒ 1007386172 - Sneider Quirama</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Oportunidad de Luis David Gomez</t>
+          <t>Oportunidad de Grupo exito</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -3185,7 +3175,7 @@
         </is>
       </c>
       <c r="G66" s="1" t="n">
-        <v>46175.60493055556</v>
+        <v>46175.61638888889</v>
       </c>
       <c r="I66" t="n">
         <v>23</v>
@@ -3202,20 +3192,25 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>davida_vanegas@coomeva.com.co</t>
+          <t>ldgomez@supertiendascanaveral.com</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C67" t="n">
         <v>0</v>
       </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Luis David Gomez</t>
+        </is>
+      </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Oportunidad de BANCOOMEVA</t>
+          <t>Oportunidad de Luis David Gomez</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -3224,7 +3219,7 @@
         </is>
       </c>
       <c r="G67" s="1" t="n">
-        <v>46175.47109953704</v>
+        <v>46175.60493055556</v>
       </c>
       <c r="I67" t="n">
         <v>23</v>
@@ -3241,7 +3236,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>alejandro.delgado@filedesk.com.co</t>
+          <t>davida_vanegas@coomeva.com.co</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -3252,14 +3247,9 @@
       <c r="C68" t="n">
         <v>0</v>
       </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>AlejandroDelgado</t>
-        </is>
-      </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Oportunidad de AlejandroDelgado</t>
+          <t>Oportunidad de BANCOOMEVA</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -3268,7 +3258,7 @@
         </is>
       </c>
       <c r="G68" s="1" t="n">
-        <v>46174.71665509259</v>
+        <v>46175.47109953704</v>
       </c>
       <c r="I68" t="n">
         <v>23</v>
@@ -3283,105 +3273,105 @@
       </c>
     </row>
     <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>alejandro.delgado@filedesk.com.co</t>
+        </is>
+      </c>
       <c r="B69" t="inlineStr">
         <is>
           <t>Contactado</t>
         </is>
       </c>
       <c r="C69" t="n">
+        <v>0</v>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>AlejandroDelgado</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Oportunidad de AlejandroDelgado</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G69" s="1" t="n">
+        <v>46174.71665509259</v>
+      </c>
+      <c r="I69" t="n">
+        <v>23</v>
+      </c>
+      <c r="J69" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>No calificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Propuesta</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
         <v>35000000</v>
       </c>
-      <c r="D69" t="inlineStr">
+      <c r="D70" t="inlineStr">
         <is>
           <t>Olga Lucia Hurtado</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr">
+      <c r="E70" t="inlineStr">
         <is>
           <t>Oportunidad de Olga Lucia Hurtado</t>
         </is>
       </c>
-      <c r="F69" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G69" s="1" t="n">
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G70" s="1" t="n">
         <v>46168.49854166667</v>
       </c>
-      <c r="I69" t="n">
+      <c r="I70" t="n">
         <v>22</v>
       </c>
-      <c r="J69" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M69" t="inlineStr">
-        <is>
-          <t>No calificado</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>comercial2@felsyn.com</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>Contactado</t>
-        </is>
-      </c>
-      <c r="C70" t="n">
-        <v>713400</v>
-      </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>Oportunidad de FONDO DE EMPLEADOS FELSYN</t>
-        </is>
-      </c>
-      <c r="F70" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G70" s="1" t="n">
-        <v>46163.49130787037</v>
-      </c>
-      <c r="I70" t="n">
-        <v>21</v>
-      </c>
       <c r="J70" t="n">
         <v>2026</v>
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>mercadeo@lasevillana.com.co</t>
+          <t>comercial2@felsyn.com</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>0</v>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fabio AlbertoGallego García </t>
-        </is>
+        <v>713400</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t xml:space="preserve">Oportunidad de Fabio AlbertoGallego García </t>
+          <t>Oportunidad de FONDO DE EMPLEADOS FELSYN</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -3390,7 +3380,7 @@
         </is>
       </c>
       <c r="G71" s="1" t="n">
-        <v>46162.64569444444</v>
+        <v>46163.49130787037</v>
       </c>
       <c r="I71" t="n">
         <v>21</v>
@@ -3400,14 +3390,14 @@
       </c>
       <c r="M71" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>asantiago@stop.com.co</t>
+          <t>mercadeo@lasevillana.com.co</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -3418,9 +3408,14 @@
       <c r="C72" t="n">
         <v>0</v>
       </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fabio AlbertoGallego García </t>
+        </is>
+      </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Oportunidad de STOP SAS</t>
+          <t xml:space="preserve">Oportunidad de Fabio AlbertoGallego García </t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -3429,7 +3424,7 @@
         </is>
       </c>
       <c r="G72" s="1" t="n">
-        <v>46161.63508101852</v>
+        <v>46162.64569444444</v>
       </c>
       <c r="I72" t="n">
         <v>21</v>
@@ -3446,25 +3441,20 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>aestrada@teker.co</t>
+          <t>asantiago@stop.com.co</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>16914000</v>
-      </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>TEKER SALUD SAS</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Oportunidad de TEKER SALUD SAS</t>
+          <t>Oportunidad de STOP SAS</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -3473,7 +3463,7 @@
         </is>
       </c>
       <c r="G73" s="1" t="n">
-        <v>46161.62922453704</v>
+        <v>46161.63508101852</v>
       </c>
       <c r="I73" t="n">
         <v>21</v>
@@ -3488,17 +3478,27 @@
       </c>
     </row>
     <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>aestrada@teker.co</t>
+        </is>
+      </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>0</v>
+        <v>16914000</v>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>TEKER SALUD SAS</t>
+        </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Oportunidad de TIAN IPS SAS</t>
+          <t>Oportunidad de TEKER SALUD SAS</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -3507,7 +3507,7 @@
         </is>
       </c>
       <c r="G74" s="1" t="n">
-        <v>46161.61643518518</v>
+        <v>46161.62922453704</v>
       </c>
       <c r="I74" t="n">
         <v>21</v>
@@ -3522,27 +3522,17 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>administración@fullredtotal.com</t>
-        </is>
-      </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>14000000</v>
-      </c>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>Eivar Eñasco</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Oportunidad de Eivar Eñasco</t>
+          <t>Oportunidad de TIAN IPS SAS</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -3551,10 +3541,10 @@
         </is>
       </c>
       <c r="G75" s="1" t="n">
-        <v>46154.67546296296</v>
+        <v>46161.61643518518</v>
       </c>
       <c r="I75" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J75" t="n">
         <v>2026</v>
@@ -3568,25 +3558,25 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>cserna@surtifamiliar.com.co</t>
+          <t>administración@fullredtotal.com</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Ganado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>975000</v>
+        <v>14000000</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Claudia Patricia Serna</t>
+          <t>Eivar Eñasco</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Oportunidad de Claudia Patricia Serna</t>
+          <t>Oportunidad de Eivar Eñasco</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -3595,10 +3585,7 @@
         </is>
       </c>
       <c r="G76" s="1" t="n">
-        <v>46154.66616898148</v>
-      </c>
-      <c r="H76" s="1" t="n">
-        <v>46217</v>
+        <v>46154.67546296296</v>
       </c>
       <c r="I76" t="n">
         <v>20</v>
@@ -3606,40 +3593,34 @@
       <c r="J76" t="n">
         <v>2026</v>
       </c>
-      <c r="K76" t="n">
-        <v>7</v>
-      </c>
-      <c r="L76" t="n">
-        <v>2026</v>
-      </c>
       <c r="M76" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>coordmercadeo@pacificcenter.co</t>
+          <t>cserna@surtifamiliar.com.co</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Ganado</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>5600000</v>
+        <v>975000</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Claudia Castro</t>
+          <t>Claudia Patricia Serna</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Oportunidad de Claudia Castro</t>
+          <t>Oportunidad de Claudia Patricia Serna</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -3648,7 +3629,10 @@
         </is>
       </c>
       <c r="G77" s="1" t="n">
-        <v>46154.66341435185</v>
+        <v>46154.66616898148</v>
+      </c>
+      <c r="H77" s="1" t="n">
+        <v>46217</v>
       </c>
       <c r="I77" t="n">
         <v>20</v>
@@ -3656,6 +3640,12 @@
       <c r="J77" t="n">
         <v>2026</v>
       </c>
+      <c r="K77" t="n">
+        <v>7</v>
+      </c>
+      <c r="L77" t="n">
+        <v>2026</v>
+      </c>
       <c r="M77" t="inlineStr">
         <is>
           <t>Calificado</t>
@@ -3665,25 +3655,25 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>isabellarengifo27@gmail.com</t>
+          <t>coordmercadeo@pacificcenter.co</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>28190000</v>
+        <v>5600000</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Isabella Rengifo</t>
+          <t>Claudia Castro</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Oportunidad de Isabella Rengifo</t>
+          <t>Oportunidad de Claudia Castro</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -3692,7 +3682,7 @@
         </is>
       </c>
       <c r="G78" s="1" t="n">
-        <v>46154.65981481481</v>
+        <v>46154.66341435185</v>
       </c>
       <c r="I78" t="n">
         <v>20</v>
@@ -3702,39 +3692,41 @@
       </c>
       <c r="M78" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>isabellarengifo27@gmail.com</t>
+        </is>
+      </c>
       <c r="B79" t="inlineStr">
         <is>
           <t>Perdido</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>50000000</v>
+        <v>28190000</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Paola Gómez - Agente Inmobiliaria Independiente</t>
+          <t>Isabella Rengifo</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Puesto de Trabajo CC Medellin</t>
+          <t>Oportunidad de Isabella Rengifo</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Richard Castaño</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G79" s="1" t="n">
-        <v>46154.49104166667</v>
-      </c>
-      <c r="H79" s="1" t="n">
-        <v>46170</v>
+        <v>46154.65981481481</v>
       </c>
       <c r="I79" t="n">
         <v>20</v>
@@ -3742,12 +3734,6 @@
       <c r="J79" t="n">
         <v>2026</v>
       </c>
-      <c r="K79" t="n">
-        <v>5</v>
-      </c>
-      <c r="L79" t="n">
-        <v>2026</v>
-      </c>
       <c r="M79" t="inlineStr">
         <is>
           <t>No calificado</t>
@@ -3755,31 +3741,34 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t>alberto.ramirez@constructorabolivar.com</t>
-        </is>
-      </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Ganado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>3000000</v>
+        <v>50000000</v>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Paola Gómez - Agente Inmobiliaria Independiente</t>
+        </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Oportunidad de NPS Relacional</t>
+          <t>Puesto de Trabajo CC Medellin</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Richard Castaño</t>
         </is>
       </c>
       <c r="G80" s="1" t="n">
-        <v>46154.44511574074</v>
+        <v>46154.49104166667</v>
+      </c>
+      <c r="H80" s="1" t="n">
+        <v>46170</v>
       </c>
       <c r="I80" t="n">
         <v>20</v>
@@ -3787,48 +3776,54 @@
       <c r="J80" t="n">
         <v>2026</v>
       </c>
+      <c r="K80" t="n">
+        <v>5</v>
+      </c>
+      <c r="L80" t="n">
+        <v>2026</v>
+      </c>
       <c r="M80" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>alberto.ramirez@constructorabolivar.com</t>
+        </is>
+      </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Ganado</t>
         </is>
       </c>
       <c r="C81" t="n">
         <v>3000000</v>
       </c>
-      <c r="D81" t="inlineStr">
-        <is>
-          <t>MADERKIT</t>
-        </is>
-      </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Oportunidad de MADERKIT</t>
+          <t>Oportunidad de NPS Relacional</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G81" s="1" t="n">
-        <v>46147.66540509259</v>
+        <v>46154.44511574074</v>
       </c>
       <c r="I81" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J81" t="n">
         <v>2026</v>
       </c>
       <c r="M81" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
CRM actualizado — 17/07/2026 16:14
</commit_message>
<xml_diff>
--- a/CRM_PowerBI_BrendaLuna_actualizado.xlsx
+++ b/CRM_PowerBI_BrendaLuna_actualizado.xlsx
@@ -992,9 +992,14 @@
       </c>
     </row>
     <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Vidanteips@gmail.com</t>
+        </is>
+      </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1002,7 +1007,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Oportunidad de Fajas Gama Alta</t>
+          <t>Oportunidad de VIDANTE IPS SAS</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1011,7 +1016,7 @@
         </is>
       </c>
       <c r="G12" s="1" t="n">
-        <v>46217.64614583334</v>
+        <v>46219.71274305556</v>
       </c>
       <c r="I12" t="n">
         <v>29</v>
@@ -1021,14 +1026,14 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>calidad.vip@axacolpatria.co</t>
+          <t>francisco.alzate@aficenter.com.co</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1037,11 +1042,16 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0</v>
+        <v>30000000</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>francisco.alzate@aficenter.com.co</t>
+        </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica VIP Centro de Medicina Internacional</t>
+          <t>Oportunidad de francisco.alzate@aficenter.com.co</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1050,7 +1060,7 @@
         </is>
       </c>
       <c r="G13" s="1" t="n">
-        <v>46217.63989583333</v>
+        <v>46217.71496527778</v>
       </c>
       <c r="I13" t="n">
         <v>29</v>
@@ -1065,11 +1075,6 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>hocen.direc@policia.gov.co</t>
-        </is>
-      </c>
       <c r="B14" t="inlineStr">
         <is>
           <t>Contactado</t>
@@ -1080,7 +1085,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Oportunidad de Hospital Central Policía Nacional</t>
+          <t>Oportunidad de Fajas Gama Alta</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1089,7 +1094,7 @@
         </is>
       </c>
       <c r="G14" s="1" t="n">
-        <v>46217.63702546297</v>
+        <v>46217.64614583334</v>
       </c>
       <c r="I14" t="n">
         <v>29</v>
@@ -1106,7 +1111,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>coor.calidad@clinicamedical.com.co</t>
+          <t>calidad.vip@axacolpatria.co</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1119,7 +1124,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica Medical S.A.S.</t>
+          <t>Oportunidad de Clínica VIP Centro de Medicina Internacional</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1128,7 +1133,7 @@
         </is>
       </c>
       <c r="G15" s="1" t="n">
-        <v>46217.62244212963</v>
+        <v>46217.63989583333</v>
       </c>
       <c r="I15" t="n">
         <v>29</v>
@@ -1145,7 +1150,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>calidad@institutodelcorazon.com</t>
+          <t>hocen.direc@policia.gov.co</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1158,7 +1163,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Oportunidad de Instituto del Corazón de Bogotá</t>
+          <t>Oportunidad de Hospital Central Policía Nacional</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1167,7 +1172,7 @@
         </is>
       </c>
       <c r="G16" s="1" t="n">
-        <v>46217.62072916667</v>
+        <v>46217.63702546297</v>
       </c>
       <c r="I16" t="n">
         <v>29</v>
@@ -1184,7 +1189,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ana.ulloa@mederi.com.co</t>
+          <t>coor.calidad@clinicamedical.com.co</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1197,7 +1202,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Oportunidad de Hospital Universitario Mayor - Mederi</t>
+          <t>Oportunidad de Clínica Medical S.A.S.</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1206,7 +1211,7 @@
         </is>
       </c>
       <c r="G17" s="1" t="n">
-        <v>46217.61866898148</v>
+        <v>46217.62244212963</v>
       </c>
       <c r="I17" t="n">
         <v>29</v>
@@ -1223,7 +1228,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ayudantia@homil.gov.co</t>
+          <t>calidad@institutodelcorazon.com</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1236,7 +1241,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Oportunidad de Hospital Militar Central</t>
+          <t>Oportunidad de Instituto del Corazón de Bogotá</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1245,7 +1250,7 @@
         </is>
       </c>
       <c r="G18" s="1" t="n">
-        <v>46217.61708333333</v>
+        <v>46217.62072916667</v>
       </c>
       <c r="I18" t="n">
         <v>29</v>
@@ -1262,7 +1267,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>direccion.general@hospitalinfantildesanjose.org.co</t>
+          <t>ana.ulloa@mederi.com.co</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1275,7 +1280,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Oportunidad de Fundación Hospital Infantil Universitario de San José</t>
+          <t>Oportunidad de Hospital Universitario Mayor - Mederi</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1284,7 +1289,7 @@
         </is>
       </c>
       <c r="G19" s="1" t="n">
-        <v>46217.6153587963</v>
+        <v>46217.61866898148</v>
       </c>
       <c r="I19" t="n">
         <v>29</v>
@@ -1301,7 +1306,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>calidad@clinicadeloccidente.com</t>
+          <t>ayudantia@homil.gov.co</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1314,7 +1319,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica del Occidente S.A.</t>
+          <t>Oportunidad de Hospital Militar Central</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1323,7 +1328,7 @@
         </is>
       </c>
       <c r="G20" s="1" t="n">
-        <v>46217.61388888889</v>
+        <v>46217.61708333333</v>
       </c>
       <c r="I20" t="n">
         <v>29</v>
@@ -1340,7 +1345,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>calidad@husi.org.co</t>
+          <t>direccion.general@hospitalinfantildesanjose.org.co</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1353,7 +1358,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Oportunidad de Hospital Universitario San Ignacio</t>
+          <t>Oportunidad de Fundación Hospital Infantil Universitario de San José</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1362,7 +1367,7 @@
         </is>
       </c>
       <c r="G21" s="1" t="n">
-        <v>46217.61174768519</v>
+        <v>46217.6153587963</v>
       </c>
       <c r="I21" t="n">
         <v>29</v>
@@ -1379,7 +1384,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>cmarly@clinicademarly.com.co</t>
+          <t>calidad@clinicadeloccidente.com</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1392,7 +1397,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica de Marly</t>
+          <t>Oportunidad de Clínica del Occidente S.A.</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1401,7 +1406,7 @@
         </is>
       </c>
       <c r="G22" s="1" t="n">
-        <v>46217.60430555556</v>
+        <v>46217.61388888889</v>
       </c>
       <c r="I22" t="n">
         <v>29</v>
@@ -1418,7 +1423,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>gerencia@hus.org.co</t>
+          <t>calidad@husi.org.co</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1431,7 +1436,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Oportunidad de Hospital Universitario de la Samaritana</t>
+          <t>Oportunidad de Hospital Universitario San Ignacio</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1440,7 +1445,7 @@
         </is>
       </c>
       <c r="G23" s="1" t="n">
-        <v>46217.60261574074</v>
+        <v>46217.61174768519</v>
       </c>
       <c r="I23" t="n">
         <v>29</v>
@@ -1457,7 +1462,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>nomorales@colsanitas.com</t>
+          <t>cmarly@clinicademarly.com.co</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1470,7 +1475,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica Colsanitas Reina Sofía Pediátrica y Mujer</t>
+          <t>Oportunidad de Clínica de Marly</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1479,7 +1484,7 @@
         </is>
       </c>
       <c r="G24" s="1" t="n">
-        <v>46217.60097222222</v>
+        <v>46217.60430555556</v>
       </c>
       <c r="I24" t="n">
         <v>29</v>
@@ -1496,7 +1501,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>nomorales@colsanitas.com</t>
+          <t>gerencia@hus.org.co</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1509,7 +1514,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica Universitaria Colombia (Colsanitas)</t>
+          <t>Oportunidad de Hospital Universitario de la Samaritana</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1518,7 +1523,7 @@
         </is>
       </c>
       <c r="G25" s="1" t="n">
-        <v>46217.59863425926</v>
+        <v>46217.60261574074</v>
       </c>
       <c r="I25" t="n">
         <v>29</v>
@@ -1535,7 +1540,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>zayda.rodriguez@cpolaya.com.co</t>
+          <t>nomorales@colsanitas.com</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1548,7 +1553,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Oportunidad de Centro Policlínico del Olaya</t>
+          <t>Oportunidad de Clínica Colsanitas Reina Sofía Pediátrica y Mujer</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1557,7 +1562,7 @@
         </is>
       </c>
       <c r="G26" s="1" t="n">
-        <v>46217.59719907407</v>
+        <v>46217.60097222222</v>
       </c>
       <c r="I26" t="n">
         <v>29</v>
@@ -1574,7 +1579,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>pcasallas@lacardiol.org</t>
+          <t>nomorales@colsanitas.com</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1587,7 +1592,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Oportunidad de Fundación Cardioinfantil - Instituto de Cardiología</t>
+          <t>Oportunidad de Clínica Universitaria Colombia (Colsanitas)</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1596,7 +1601,7 @@
         </is>
       </c>
       <c r="G27" s="1" t="n">
-        <v>46217.59630787037</v>
+        <v>46217.59863425926</v>
       </c>
       <c r="I27" t="n">
         <v>29</v>
@@ -1613,7 +1618,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>dir_calidad@clinicajuanncorpas.com</t>
+          <t>zayda.rodriguez@cpolaya.com.co</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1626,7 +1631,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica Juan N Corpas Ltda</t>
+          <t>Oportunidad de Centro Policlínico del Olaya</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1635,7 +1640,7 @@
         </is>
       </c>
       <c r="G28" s="1" t="n">
-        <v>46217.52333333333</v>
+        <v>46217.59719907407</v>
       </c>
       <c r="I28" t="n">
         <v>29</v>
@@ -1652,7 +1657,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>dianaespinosanarvaez@gmail.com</t>
+          <t>pcasallas@lacardiol.org</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1665,7 +1670,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica Onkos</t>
+          <t>Oportunidad de Fundación Cardioinfantil - Instituto de Cardiología</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1674,7 +1679,7 @@
         </is>
       </c>
       <c r="G29" s="1" t="n">
-        <v>46217.52202546296</v>
+        <v>46217.59630787037</v>
       </c>
       <c r="I29" t="n">
         <v>29</v>
@@ -1691,7 +1696,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>gestiondecalidad@clinicapalermo.com.co</t>
+          <t>dir_calidad@clinicajuanncorpas.com</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1704,7 +1709,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica Palermo</t>
+          <t>Oportunidad de Clínica Juan N Corpas Ltda</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1713,7 +1718,7 @@
         </is>
       </c>
       <c r="G30" s="1" t="n">
-        <v>46217.51743055556</v>
+        <v>46217.52333333333</v>
       </c>
       <c r="I30" t="n">
         <v>29</v>
@@ -1730,7 +1735,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>calidad@hospitaldesanjose.org.co</t>
+          <t>dianaespinosanarvaez@gmail.com</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1743,7 +1748,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Oportunidad de Hospital San José - Sociedad de Cirugía de Bogotá</t>
+          <t>Oportunidad de Clínica Onkos</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1752,7 +1757,7 @@
         </is>
       </c>
       <c r="G31" s="1" t="n">
-        <v>46217.51425925926</v>
+        <v>46217.52202546296</v>
       </c>
       <c r="I31" t="n">
         <v>29</v>
@@ -1769,7 +1774,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>jzapata@ioir.org.co</t>
+          <t>gestiondecalidad@clinicapalermo.com.co</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1782,7 +1787,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Oportunidad de Instituto de Ortopedia Infantil Roosevelt</t>
+          <t>Oportunidad de Clínica Palermo</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1791,7 +1796,7 @@
         </is>
       </c>
       <c r="G32" s="1" t="n">
-        <v>46217.51231481481</v>
+        <v>46217.51743055556</v>
       </c>
       <c r="I32" t="n">
         <v>29</v>
@@ -1808,7 +1813,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>diana.potesno@colsubsidio.com</t>
+          <t>calidad@hospitaldesanjose.org.co</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1821,7 +1826,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica Colsubsidio Calle 100</t>
+          <t>Oportunidad de Hospital San José - Sociedad de Cirugía de Bogotá</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1830,7 +1835,7 @@
         </is>
       </c>
       <c r="G33" s="1" t="n">
-        <v>46217.51116898148</v>
+        <v>46217.51425925926</v>
       </c>
       <c r="I33" t="n">
         <v>29</v>
@@ -1847,7 +1852,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>diana.potesno@colsubsidio.com</t>
+          <t>jzapata@ioir.org.co</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1860,7 +1865,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica Colsubsidio Calle 100</t>
+          <t>Oportunidad de Instituto de Ortopedia Infantil Roosevelt</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1869,7 +1874,7 @@
         </is>
       </c>
       <c r="G34" s="1" t="n">
-        <v>46217.50983796296</v>
+        <v>46217.51231481481</v>
       </c>
       <c r="I34" t="n">
         <v>29</v>
@@ -1886,7 +1891,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>jose.chaves@colsubsidio.com</t>
+          <t>diana.potesno@colsubsidio.com</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1899,7 +1904,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica Colsubsidio Ciudad Roma</t>
+          <t>Oportunidad de Clínica Colsubsidio Calle 100</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1908,7 +1913,7 @@
         </is>
       </c>
       <c r="G35" s="1" t="n">
-        <v>46217.50767361111</v>
+        <v>46217.51116898148</v>
       </c>
       <c r="I35" t="n">
         <v>29</v>
@@ -1925,7 +1930,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>carlos.artetamo@colsubsidio.com</t>
+          <t>diana.potesno@colsubsidio.com</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1938,7 +1943,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica Infantil Colsubsidio</t>
+          <t>Oportunidad de Clínica Colsubsidio Calle 100</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -1947,7 +1952,7 @@
         </is>
       </c>
       <c r="G36" s="1" t="n">
-        <v>46217.50050925926</v>
+        <v>46217.50983796296</v>
       </c>
       <c r="I36" t="n">
         <v>29</v>
@@ -1964,7 +1969,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>notificacionescdc@clinicadelcountry.com</t>
+          <t>jose.chaves@colsubsidio.com</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1977,7 +1982,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica del Country IPS</t>
+          <t>Oportunidad de Clínica Colsubsidio Ciudad Roma</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -1986,7 +1991,7 @@
         </is>
       </c>
       <c r="G37" s="1" t="n">
-        <v>46217.49881944444</v>
+        <v>46217.50767361111</v>
       </c>
       <c r="I37" t="n">
         <v>29</v>
@@ -2003,7 +2008,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>direcciongeneral@shaio.org</t>
+          <t>carlos.artetamo@colsubsidio.com</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2016,7 +2021,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Oportunidad de Fundación Abood Shaio</t>
+          <t>Oportunidad de Clínica Infantil Colsubsidio</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2025,7 +2030,7 @@
         </is>
       </c>
       <c r="G38" s="1" t="n">
-        <v>46217.49715277777</v>
+        <v>46217.50050925926</v>
       </c>
       <c r="I38" t="n">
         <v>29</v>
@@ -2042,7 +2047,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>direccion@cancer.gov.co</t>
+          <t>notificacionescdc@clinicadelcountry.com</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2055,7 +2060,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Oportunidad de Instituto Nacional de Cancerología</t>
+          <t>Oportunidad de Clínica del Country IPS</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2064,7 +2069,7 @@
         </is>
       </c>
       <c r="G39" s="1" t="n">
-        <v>46217.47924768519</v>
+        <v>46217.49881944444</v>
       </c>
       <c r="I39" t="n">
         <v>29</v>
@@ -2081,7 +2086,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>sdirmedica@clinicadelamujer.com.co</t>
+          <t>direcciongeneral@shaio.org</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2094,7 +2099,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica de la Mujer</t>
+          <t>Oportunidad de Fundación Abood Shaio</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -2103,7 +2108,7 @@
         </is>
       </c>
       <c r="G40" s="1" t="n">
-        <v>46217.47585648148</v>
+        <v>46217.49715277777</v>
       </c>
       <c r="I40" t="n">
         <v>29</v>
@@ -2120,7 +2125,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>lidercalidad@homifundacion.org.co</t>
+          <t>direccion@cancer.gov.co</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2133,7 +2138,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Oportunidad de Fundación Hospital de la Misericordia (HOMI)</t>
+          <t>Oportunidad de Instituto Nacional de Cancerología</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2142,7 +2147,7 @@
         </is>
       </c>
       <c r="G41" s="1" t="n">
-        <v>46217.47246527778</v>
+        <v>46217.47924768519</v>
       </c>
       <c r="I41" t="n">
         <v>29</v>
@@ -2159,7 +2164,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>direcciongeneral1@stewardcolombia.org</t>
+          <t>sdirmedica@clinicadelamujer.com.co</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2172,7 +2177,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Oportunidad de Hospital Universitario Clínica San Rafael</t>
+          <t>Oportunidad de Clínica de la Mujer</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -2181,7 +2186,7 @@
         </is>
       </c>
       <c r="G42" s="1" t="n">
-        <v>46217.00748842592</v>
+        <v>46217.47585648148</v>
       </c>
       <c r="I42" t="n">
         <v>29</v>
@@ -2198,7 +2203,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>adriana.urrego@fsfb.org.co</t>
+          <t>lidercalidad@homifundacion.org.co</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2211,7 +2216,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Oportunidad de FUNDACION SANTA FE DE BOGOTA</t>
+          <t>Oportunidad de Fundación Hospital de la Misericordia (HOMI)</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2220,7 +2225,7 @@
         </is>
       </c>
       <c r="G43" s="1" t="n">
-        <v>46217.00381944444</v>
+        <v>46217.47246527778</v>
       </c>
       <c r="I43" t="n">
         <v>29</v>
@@ -2237,7 +2242,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>calidadsalud@cafam.com.co</t>
+          <t>direcciongeneral1@stewardcolombia.org</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2250,7 +2255,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Oportunidad de Centro de Atención en Salud CAFAM Clínica Calle 51</t>
+          <t>Oportunidad de Hospital Universitario Clínica San Rafael</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -2259,7 +2264,7 @@
         </is>
       </c>
       <c r="G44" s="1" t="n">
-        <v>46216.99954861111</v>
+        <v>46217.00748842592</v>
       </c>
       <c r="I44" t="n">
         <v>29</v>
@@ -2276,7 +2281,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>notificacionesjudiciales@fhsc.org.co</t>
+          <t>adriana.urrego@fsfb.org.co</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2289,7 +2294,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Oportunidad de Fundación Hospital San Carlos</t>
+          <t>Oportunidad de FUNDACION SANTA FE DE BOGOTA</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -2298,7 +2303,7 @@
         </is>
       </c>
       <c r="G45" s="1" t="n">
-        <v>46216.99548611111</v>
+        <v>46217.00381944444</v>
       </c>
       <c r="I45" t="n">
         <v>29</v>
@@ -2315,7 +2320,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>calidad@proseguir.org</t>
+          <t>calidadsalud@cafam.com.co</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2328,7 +2333,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Oportunidad de PROSEGUIR SEDE 3</t>
+          <t>Oportunidad de Centro de Atención en Salud CAFAM Clínica Calle 51</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2337,7 +2342,7 @@
         </is>
       </c>
       <c r="G46" s="1" t="n">
-        <v>46216.99299768519</v>
+        <v>46216.99954861111</v>
       </c>
       <c r="I46" t="n">
         <v>29</v>
@@ -2354,46 +2359,46 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>centrodecontacto@uao.edu.co</t>
+          <t>notificacionesjudiciales@fhsc.org.co</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>10000000</v>
+        <v>0</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Oportunidad de UNIVERSIDAD AUTONOMA DE OCCIDENTE</t>
+          <t>Oportunidad de Fundación Hospital San Carlos</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G47" s="1" t="n">
-        <v>46213.49821759259</v>
+        <v>46216.99548611111</v>
       </c>
       <c r="I47" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J47" t="n">
         <v>2026</v>
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>carlos.segovia@warena.co</t>
+          <t>calidad@proseguir.org</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2402,23 +2407,23 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>35000000</v>
+        <v>0</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Oportunidad de W ARENA</t>
+          <t>Oportunidad de PROSEGUIR SEDE 3</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G48" s="1" t="n">
-        <v>46213.49508101852</v>
+        <v>46216.99299768519</v>
       </c>
       <c r="I48" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J48" t="n">
         <v>2026</v>
@@ -2432,37 +2437,29 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>klondono@fundacionwwbcol.org</t>
+          <t>centrodecontacto@uao.edu.co</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Ganado</t>
+          <t>Negociación</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>300000</v>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>Karla Londoño</t>
-        </is>
+        <v>10000000</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Oportunidad de Karla Londoño</t>
+          <t>Oportunidad de UNIVERSIDAD AUTONOMA DE OCCIDENTE</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G49" s="1" t="n">
-        <v>46212.51638888889</v>
-      </c>
-      <c r="H49" s="1" t="n">
-        <v>46217</v>
+        <v>46213.49821759259</v>
       </c>
       <c r="I49" t="n">
         <v>28</v>
@@ -2470,12 +2467,6 @@
       <c r="J49" t="n">
         <v>2026</v>
       </c>
-      <c r="K49" t="n">
-        <v>7</v>
-      </c>
-      <c r="L49" t="n">
-        <v>2026</v>
-      </c>
       <c r="M49" t="inlineStr">
         <is>
           <t>Calificado</t>
@@ -2485,7 +2476,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>ctorres@colcobranzasnacionales.com</t>
+          <t>carlos.segovia@warena.co</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2494,28 +2485,23 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>5000000</v>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>ctorres@colcobranzasnacionales.com</t>
-        </is>
+        <v>35000000</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Oportunidad de ctorres@colcobranzasnacionales.com</t>
+          <t>Oportunidad de W ARENA</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G50" s="1" t="n">
-        <v>46206.73804398148</v>
+        <v>46213.49508101852</v>
       </c>
       <c r="I50" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J50" t="n">
         <v>2026</v>
@@ -2529,7 +2515,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>medifar624@gmail.com</t>
+          <t>klondono@fundacionwwbcol.org</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2538,11 +2524,16 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>1640000</v>
+        <v>300000</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Karla Londoño</t>
+        </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Oportunidad de MEDISFARMA SAS</t>
+          <t>Oportunidad de Karla Londoño</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -2551,19 +2542,19 @@
         </is>
       </c>
       <c r="G51" s="1" t="n">
-        <v>46203.72597222222</v>
+        <v>46212.51638888889</v>
       </c>
       <c r="H51" s="1" t="n">
-        <v>46199</v>
+        <v>46217</v>
       </c>
       <c r="I51" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J51" t="n">
         <v>2026</v>
       </c>
       <c r="K51" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L51" t="n">
         <v>2026</v>
@@ -2577,7 +2568,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>mercadeo@norteysur.co</t>
+          <t>ctorres@colcobranzasnacionales.com</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2586,16 +2577,16 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>28190000</v>
+        <v>5000000</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Isabella Mesa</t>
+          <t>ctorres@colcobranzasnacionales.com</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Oportunidad de Isabella Mesa</t>
+          <t>Oportunidad de ctorres@colcobranzasnacionales.com</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -2604,10 +2595,10 @@
         </is>
       </c>
       <c r="G52" s="1" t="n">
-        <v>46191.70076388889</v>
+        <v>46206.73804398148</v>
       </c>
       <c r="I52" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="J52" t="n">
         <v>2026</v>
@@ -2621,20 +2612,20 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>comercial@asertis.com.co</t>
+          <t>medifar624@gmail.com</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Ganado</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>0</v>
+        <v>1640000</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Oportunidad de IMPORTADORA CALI S.A.</t>
+          <t>Oportunidad de MEDISFARMA SAS</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -2643,42 +2634,51 @@
         </is>
       </c>
       <c r="G53" s="1" t="n">
-        <v>46189.67539351852</v>
+        <v>46203.72597222222</v>
+      </c>
+      <c r="H53" s="1" t="n">
+        <v>46199</v>
       </c>
       <c r="I53" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="J53" t="n">
         <v>2026</v>
       </c>
+      <c r="K53" t="n">
+        <v>6</v>
+      </c>
+      <c r="L53" t="n">
+        <v>2026</v>
+      </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>educacion@360forma.edu.co</t>
+          <t>mercadeo@norteysur.co</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Negociación</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>0</v>
+        <v>28190000</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Jorge Sanchez / jefe Comercial</t>
+          <t>Isabella Mesa</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Oportunidad de Jorge Sanchez / jefe Comercial</t>
+          <t>Oportunidad de Isabella Mesa</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -2687,7 +2687,7 @@
         </is>
       </c>
       <c r="G54" s="1" t="n">
-        <v>46189.65077546296</v>
+        <v>46191.70076388889</v>
       </c>
       <c r="I54" t="n">
         <v>25</v>
@@ -2697,19 +2697,19 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>directoradjunto@dclass.edu.co</t>
+          <t>comercial@asertis.com.co</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -2717,7 +2717,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Oportunidad de DCLASS ACADEMIA SAS</t>
+          <t>Oportunidad de IMPORTADORA CALI S.A.</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -2726,7 +2726,7 @@
         </is>
       </c>
       <c r="G55" s="1" t="n">
-        <v>46189.49674768518</v>
+        <v>46189.67539351852</v>
       </c>
       <c r="I55" t="n">
         <v>25</v>
@@ -2743,7 +2743,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Belkis.jimenez@agrauto.com.co</t>
+          <t>educacion@360forma.edu.co</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2754,9 +2754,14 @@
       <c r="C56" t="n">
         <v>0</v>
       </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Jorge Sanchez / jefe Comercial</t>
+        </is>
+      </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Oportunidad de AGRICOLA AUTOMOTRIZ SAS / BELKYS JIMENEZ</t>
+          <t>Oportunidad de Jorge Sanchez / jefe Comercial</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -2765,10 +2770,10 @@
         </is>
       </c>
       <c r="G56" s="1" t="n">
-        <v>46182.67912037037</v>
+        <v>46189.65077546296</v>
       </c>
       <c r="I56" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J56" t="n">
         <v>2026</v>
@@ -2782,25 +2787,20 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>luisa.baena@automarcali.com</t>
+          <t>directoradjunto@dclass.edu.co</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C57" t="n">
         <v>0</v>
       </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>luisa.baena@automarcali.com</t>
-        </is>
-      </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Oportunidad de luisa.baena@automarcali.com</t>
+          <t>Oportunidad de DCLASS ACADEMIA SAS</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -2809,10 +2809,10 @@
         </is>
       </c>
       <c r="G57" s="1" t="n">
-        <v>46182.67809027778</v>
+        <v>46189.49674768518</v>
       </c>
       <c r="I57" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J57" t="n">
         <v>2026</v>
@@ -2826,7 +2826,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>directormercadeo@almotores.com</t>
+          <t>Belkis.jimenez@agrauto.com.co</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2837,14 +2837,9 @@
       <c r="C58" t="n">
         <v>0</v>
       </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>Viviana Vanegas</t>
-        </is>
-      </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Oportunidad de Viviana Vanegas</t>
+          <t>Oportunidad de AGRICOLA AUTOMOTRIZ SAS / BELKYS JIMENEZ</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -2853,7 +2848,7 @@
         </is>
       </c>
       <c r="G58" s="1" t="n">
-        <v>46182.67621527778</v>
+        <v>46182.67912037037</v>
       </c>
       <c r="I58" t="n">
         <v>24</v>
@@ -2870,7 +2865,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>xiomara.duran@autopacifico.com.co</t>
+          <t>luisa.baena@automarcali.com</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2881,9 +2876,14 @@
       <c r="C59" t="n">
         <v>0</v>
       </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>luisa.baena@automarcali.com</t>
+        </is>
+      </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Oportunidad de xiomara.duran@autopacifico.com.co</t>
+          <t>Oportunidad de luisa.baena@automarcali.com</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -2892,7 +2892,7 @@
         </is>
       </c>
       <c r="G59" s="1" t="n">
-        <v>46182.65815972222</v>
+        <v>46182.67809027778</v>
       </c>
       <c r="I59" t="n">
         <v>24</v>
@@ -2909,12 +2909,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>alejandrosaavedraconde@comfandi.com.co</t>
+          <t>directormercadeo@almotores.com</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -2922,12 +2922,12 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>ALEJANDRO</t>
+          <t>Viviana Vanegas</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Oportunidad de ALEJANDRO</t>
+          <t>Oportunidad de Viviana Vanegas</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -2936,7 +2936,7 @@
         </is>
       </c>
       <c r="G60" s="1" t="n">
-        <v>46182.64278935185</v>
+        <v>46182.67621527778</v>
       </c>
       <c r="I60" t="n">
         <v>24</v>
@@ -2953,12 +2953,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>administracion@fiando.com.co</t>
+          <t>xiomara.duran@autopacifico.com.co</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -2966,7 +2966,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Oportunidad de FIANDO LTDA</t>
+          <t>Oportunidad de xiomara.duran@autopacifico.com.co</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -2975,7 +2975,7 @@
         </is>
       </c>
       <c r="G61" s="1" t="n">
-        <v>46182.61304398148</v>
+        <v>46182.65815972222</v>
       </c>
       <c r="I61" t="n">
         <v>24</v>
@@ -2985,19 +2985,19 @@
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>dgamoneda@productosdrogam.com</t>
+          <t>alejandrosaavedraconde@comfandi.com.co</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -3005,12 +3005,12 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t xml:space="preserve">Diego Mauricio Gamoneda </t>
+          <t>ALEJANDRO</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t xml:space="preserve">Oportunidad de Diego Mauricio Gamoneda </t>
+          <t>Oportunidad de ALEJANDRO</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -3019,10 +3019,10 @@
         </is>
       </c>
       <c r="G62" s="1" t="n">
-        <v>46175.66417824074</v>
+        <v>46182.64278935185</v>
       </c>
       <c r="I62" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J62" t="n">
         <v>2026</v>
@@ -3036,7 +3036,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>alexander.rojas@friogan.com</t>
+          <t>administracion@fiando.com.co</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3045,11 +3045,11 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>10000000</v>
+        <v>0</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Oportunidad de FRIOGAN S.A</t>
+          <t>Oportunidad de FIANDO LTDA</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -3058,10 +3058,10 @@
         </is>
       </c>
       <c r="G63" s="1" t="n">
-        <v>46175.63597222222</v>
+        <v>46182.61304398148</v>
       </c>
       <c r="I63" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J63" t="n">
         <v>2026</v>
@@ -3073,17 +3073,27 @@
       </c>
     </row>
     <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>dgamoneda@productosdrogam.com</t>
+        </is>
+      </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C64" t="n">
         <v>0</v>
       </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Diego Mauricio Gamoneda </t>
+        </is>
+      </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Oportunidad de Agromercados la Montaña</t>
+          <t xml:space="preserve">Oportunidad de Diego Mauricio Gamoneda </t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -3092,7 +3102,7 @@
         </is>
       </c>
       <c r="G64" s="1" t="n">
-        <v>46175.62239583334</v>
+        <v>46175.66417824074</v>
       </c>
       <c r="I64" t="n">
         <v>23</v>
@@ -3109,20 +3119,20 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>juand.rios@alkosto.com.co</t>
+          <t>alexander.rojas@friogan.com</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>0</v>
+        <v>10000000</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Oportunidad de ALKOSTO</t>
+          <t>Oportunidad de FRIOGAN S.A</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -3131,7 +3141,7 @@
         </is>
       </c>
       <c r="G65" s="1" t="n">
-        <v>46175.62055555556</v>
+        <v>46175.63597222222</v>
       </c>
       <c r="I65" t="n">
         <v>23</v>
@@ -3141,16 +3151,11 @@
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>gerencia4087@grupo-exito.com</t>
-        </is>
-      </c>
       <c r="B66" t="inlineStr">
         <is>
           <t>Perdido</t>
@@ -3159,14 +3164,9 @@
       <c r="C66" t="n">
         <v>0</v>
       </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>Grupo exito ‒ 1007386172 - Sneider Quirama</t>
-        </is>
-      </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Oportunidad de Grupo exito</t>
+          <t>Oportunidad de Agromercados la Montaña</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -3175,7 +3175,7 @@
         </is>
       </c>
       <c r="G66" s="1" t="n">
-        <v>46175.61638888889</v>
+        <v>46175.62239583334</v>
       </c>
       <c r="I66" t="n">
         <v>23</v>
@@ -3192,7 +3192,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>ldgomez@supertiendascanaveral.com</t>
+          <t>juand.rios@alkosto.com.co</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3203,14 +3203,9 @@
       <c r="C67" t="n">
         <v>0</v>
       </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>Luis David Gomez</t>
-        </is>
-      </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Oportunidad de Luis David Gomez</t>
+          <t>Oportunidad de ALKOSTO</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -3219,7 +3214,7 @@
         </is>
       </c>
       <c r="G67" s="1" t="n">
-        <v>46175.60493055556</v>
+        <v>46175.62055555556</v>
       </c>
       <c r="I67" t="n">
         <v>23</v>
@@ -3236,20 +3231,25 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>davida_vanegas@coomeva.com.co</t>
+          <t>gerencia4087@grupo-exito.com</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C68" t="n">
         <v>0</v>
       </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Grupo exito ‒ 1007386172 - Sneider Quirama</t>
+        </is>
+      </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Oportunidad de BANCOOMEVA</t>
+          <t>Oportunidad de Grupo exito</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -3258,7 +3258,7 @@
         </is>
       </c>
       <c r="G68" s="1" t="n">
-        <v>46175.47109953704</v>
+        <v>46175.61638888889</v>
       </c>
       <c r="I68" t="n">
         <v>23</v>
@@ -3275,12 +3275,12 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>alejandro.delgado@filedesk.com.co</t>
+          <t>ldgomez@supertiendascanaveral.com</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -3288,12 +3288,12 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>AlejandroDelgado</t>
+          <t>Luis David Gomez</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Oportunidad de AlejandroDelgado</t>
+          <t>Oportunidad de Luis David Gomez</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -3302,7 +3302,7 @@
         </is>
       </c>
       <c r="G69" s="1" t="n">
-        <v>46174.71665509259</v>
+        <v>46175.60493055556</v>
       </c>
       <c r="I69" t="n">
         <v>23</v>
@@ -3317,22 +3317,22 @@
       </c>
     </row>
     <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>davida_vanegas@coomeva.com.co</t>
+        </is>
+      </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>35000000</v>
-      </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>Olga Lucia Hurtado</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Oportunidad de Olga Lucia Hurtado</t>
+          <t>Oportunidad de BANCOOMEVA</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -3341,120 +3341,120 @@
         </is>
       </c>
       <c r="G70" s="1" t="n">
-        <v>46168.49854166667</v>
+        <v>46175.47109953704</v>
       </c>
       <c r="I70" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="J70" t="n">
         <v>2026</v>
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>comercial2@felsyn.com</t>
+          <t>alejandro.delgado@filedesk.com.co</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
+          <t>Contactado</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>0</v>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>AlejandroDelgado</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Oportunidad de AlejandroDelgado</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G71" s="1" t="n">
+        <v>46174.71665509259</v>
+      </c>
+      <c r="I71" t="n">
+        <v>23</v>
+      </c>
+      <c r="J71" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>No calificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="B72" t="inlineStr">
+        <is>
           <t>Propuesta</t>
         </is>
       </c>
-      <c r="C71" t="n">
-        <v>713400</v>
-      </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>Oportunidad de FONDO DE EMPLEADOS FELSYN</t>
-        </is>
-      </c>
-      <c r="F71" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G71" s="1" t="n">
-        <v>46163.49130787037</v>
-      </c>
-      <c r="I71" t="n">
-        <v>21</v>
-      </c>
-      <c r="J71" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M71" t="inlineStr">
+      <c r="C72" t="n">
+        <v>35000000</v>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Olga Lucia Hurtado</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Oportunidad de Olga Lucia Hurtado</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G72" s="1" t="n">
+        <v>46168.49854166667</v>
+      </c>
+      <c r="I72" t="n">
+        <v>22</v>
+      </c>
+      <c r="J72" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M72" t="inlineStr">
         <is>
           <t>Calificado</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>mercadeo@lasevillana.com.co</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>Contactado</t>
-        </is>
-      </c>
-      <c r="C72" t="n">
-        <v>0</v>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fabio AlbertoGallego García </t>
-        </is>
-      </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Oportunidad de Fabio AlbertoGallego García </t>
-        </is>
-      </c>
-      <c r="F72" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G72" s="1" t="n">
-        <v>46162.64569444444</v>
-      </c>
-      <c r="I72" t="n">
-        <v>21</v>
-      </c>
-      <c r="J72" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M72" t="inlineStr">
-        <is>
-          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>asantiago@stop.com.co</t>
+          <t>comercial2@felsyn.com</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>0</v>
+        <v>713400</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Oportunidad de STOP SAS</t>
+          <t>Oportunidad de FONDO DE EMPLEADOS FELSYN</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -3463,7 +3463,7 @@
         </is>
       </c>
       <c r="G73" s="1" t="n">
-        <v>46161.63508101852</v>
+        <v>46163.49130787037</v>
       </c>
       <c r="I73" t="n">
         <v>21</v>
@@ -3473,32 +3473,32 @@
       </c>
       <c r="M73" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>aestrada@teker.co</t>
+          <t>mercadeo@lasevillana.com.co</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>16914000</v>
+        <v>0</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>TEKER SALUD SAS</t>
+          <t xml:space="preserve">Fabio AlbertoGallego García </t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Oportunidad de TEKER SALUD SAS</t>
+          <t xml:space="preserve">Oportunidad de Fabio AlbertoGallego García </t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -3507,7 +3507,7 @@
         </is>
       </c>
       <c r="G74" s="1" t="n">
-        <v>46161.62922453704</v>
+        <v>46162.64569444444</v>
       </c>
       <c r="I74" t="n">
         <v>21</v>
@@ -3522,6 +3522,11 @@
       </c>
     </row>
     <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>asantiago@stop.com.co</t>
+        </is>
+      </c>
       <c r="B75" t="inlineStr">
         <is>
           <t>Contactado</t>
@@ -3532,7 +3537,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Oportunidad de TIAN IPS SAS</t>
+          <t>Oportunidad de STOP SAS</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -3541,7 +3546,7 @@
         </is>
       </c>
       <c r="G75" s="1" t="n">
-        <v>46161.61643518518</v>
+        <v>46161.63508101852</v>
       </c>
       <c r="I75" t="n">
         <v>21</v>
@@ -3558,7 +3563,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>administración@fullredtotal.com</t>
+          <t>aestrada@teker.co</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -3567,16 +3572,16 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>14000000</v>
+        <v>16914000</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Eivar Eñasco</t>
+          <t>TEKER SALUD SAS</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Oportunidad de Eivar Eñasco</t>
+          <t>Oportunidad de TEKER SALUD SAS</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -3585,10 +3590,10 @@
         </is>
       </c>
       <c r="G76" s="1" t="n">
-        <v>46154.67546296296</v>
+        <v>46161.62922453704</v>
       </c>
       <c r="I76" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J76" t="n">
         <v>2026</v>
@@ -3600,27 +3605,17 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>cserna@surtifamiliar.com.co</t>
-        </is>
-      </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Ganado</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>975000</v>
-      </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>Claudia Patricia Serna</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Oportunidad de Claudia Patricia Serna</t>
+          <t>Oportunidad de TIAN IPS SAS</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -3629,51 +3624,42 @@
         </is>
       </c>
       <c r="G77" s="1" t="n">
-        <v>46154.66616898148</v>
-      </c>
-      <c r="H77" s="1" t="n">
-        <v>46217</v>
+        <v>46161.61643518518</v>
       </c>
       <c r="I77" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J77" t="n">
         <v>2026</v>
       </c>
-      <c r="K77" t="n">
-        <v>7</v>
-      </c>
-      <c r="L77" t="n">
-        <v>2026</v>
-      </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>coordmercadeo@pacificcenter.co</t>
+          <t>administración@fullredtotal.com</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>5600000</v>
+        <v>14000000</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Claudia Castro</t>
+          <t>Eivar Eñasco</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Oportunidad de Claudia Castro</t>
+          <t>Oportunidad de Eivar Eñasco</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -3682,7 +3668,7 @@
         </is>
       </c>
       <c r="G78" s="1" t="n">
-        <v>46154.66341435185</v>
+        <v>46154.67546296296</v>
       </c>
       <c r="I78" t="n">
         <v>20</v>
@@ -3692,32 +3678,32 @@
       </c>
       <c r="M78" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>isabellarengifo27@gmail.com</t>
+          <t>cserna@surtifamiliar.com.co</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Ganado</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>28190000</v>
+        <v>975000</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Isabella Rengifo</t>
+          <t>Claudia Patricia Serna</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Oportunidad de Isabella Rengifo</t>
+          <t>Oportunidad de Claudia Patricia Serna</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -3726,7 +3712,10 @@
         </is>
       </c>
       <c r="G79" s="1" t="n">
-        <v>46154.65981481481</v>
+        <v>46154.66616898148</v>
+      </c>
+      <c r="H79" s="1" t="n">
+        <v>46217</v>
       </c>
       <c r="I79" t="n">
         <v>20</v>
@@ -3734,41 +3723,49 @@
       <c r="J79" t="n">
         <v>2026</v>
       </c>
+      <c r="K79" t="n">
+        <v>7</v>
+      </c>
+      <c r="L79" t="n">
+        <v>2026</v>
+      </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>coordmercadeo@pacificcenter.co</t>
+        </is>
+      </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>50000000</v>
+        <v>5600000</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Paola Gómez - Agente Inmobiliaria Independiente</t>
+          <t>Claudia Castro</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Puesto de Trabajo CC Medellin</t>
+          <t>Oportunidad de Claudia Castro</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Richard Castaño</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G80" s="1" t="n">
-        <v>46154.49104166667</v>
-      </c>
-      <c r="H80" s="1" t="n">
-        <v>46170</v>
+        <v>46154.66341435185</v>
       </c>
       <c r="I80" t="n">
         <v>20</v>
@@ -3776,44 +3773,43 @@
       <c r="J80" t="n">
         <v>2026</v>
       </c>
-      <c r="K80" t="n">
-        <v>5</v>
-      </c>
-      <c r="L80" t="n">
-        <v>2026</v>
-      </c>
       <c r="M80" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>alberto.ramirez@constructorabolivar.com</t>
+          <t>isabellarengifo27@gmail.com</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Ganado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>3000000</v>
+        <v>28190000</v>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Isabella Rengifo</t>
+        </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Oportunidad de NPS Relacional</t>
+          <t>Oportunidad de Isabella Rengifo</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G81" s="1" t="n">
-        <v>46154.44511574074</v>
+        <v>46154.65981481481</v>
       </c>
       <c r="I81" t="n">
         <v>20</v>
@@ -3823,7 +3819,7 @@
       </c>
       <c r="M81" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
CRM actualizado — 21/07/2026 14:54
</commit_message>
<xml_diff>
--- a/CRM_PowerBI_BrendaLuna_actualizado.xlsx
+++ b/CRM_PowerBI_BrendaLuna_actualizado.xlsx
@@ -992,14 +992,9 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Vidanteips@gmail.com</t>
-        </is>
-      </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1007,77 +1002,91 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Oportunidad de VIDANTE IPS SAS</t>
+          <t>Oportunidad de CLINICA DE OFTALMOLOGIA DE CALI S A</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G12" s="1" t="n">
-        <v>46219.71274305556</v>
+        <v>46224.46891203704</v>
       </c>
       <c r="I12" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="J12" t="n">
         <v>2026</v>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>francisco.alzate@aficenter.com.co</t>
+          <t>hrodriguez@jaramillomora.com</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>30000000</v>
+        <v>48600000</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>francisco.alzate@aficenter.com.co</t>
+          <t>HANNA RODRIGUEZ</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Oportunidad de francisco.alzate@aficenter.com.co</t>
+          <t>Oportunidad de HANNA RODRIGUEZ</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G13" s="1" t="n">
-        <v>46217.71496527778</v>
+        <v>46224.45887731481</v>
+      </c>
+      <c r="H13" s="1" t="n">
+        <v>46265</v>
       </c>
       <c r="I13" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="J13" t="n">
         <v>2026</v>
       </c>
+      <c r="K13" t="n">
+        <v>8</v>
+      </c>
+      <c r="L13" t="n">
+        <v>2026</v>
+      </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Vidanteips@gmail.com</t>
+        </is>
+      </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -1085,7 +1094,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Oportunidad de Fajas Gama Alta</t>
+          <t>Oportunidad de VIDANTE IPS SAS</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1094,7 +1103,7 @@
         </is>
       </c>
       <c r="G14" s="1" t="n">
-        <v>46217.64614583334</v>
+        <v>46219.71274305556</v>
       </c>
       <c r="I14" t="n">
         <v>29</v>
@@ -1104,14 +1113,14 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>calidad.vip@axacolpatria.co</t>
+          <t>francisco.alzate@aficenter.com.co</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1120,11 +1129,16 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0</v>
+        <v>30000000</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>francisco.alzate@aficenter.com.co</t>
+        </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica VIP Centro de Medicina Internacional</t>
+          <t>Oportunidad de francisco.alzate@aficenter.com.co</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1133,7 +1147,7 @@
         </is>
       </c>
       <c r="G15" s="1" t="n">
-        <v>46217.63989583333</v>
+        <v>46217.71496527778</v>
       </c>
       <c r="I15" t="n">
         <v>29</v>
@@ -1148,11 +1162,6 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>hocen.direc@policia.gov.co</t>
-        </is>
-      </c>
       <c r="B16" t="inlineStr">
         <is>
           <t>Contactado</t>
@@ -1163,7 +1172,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Oportunidad de Hospital Central Policía Nacional</t>
+          <t>Oportunidad de Fajas Gama Alta</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1172,7 +1181,7 @@
         </is>
       </c>
       <c r="G16" s="1" t="n">
-        <v>46217.63702546297</v>
+        <v>46217.64614583334</v>
       </c>
       <c r="I16" t="n">
         <v>29</v>
@@ -1189,7 +1198,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>coor.calidad@clinicamedical.com.co</t>
+          <t>calidad.vip@axacolpatria.co</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1202,7 +1211,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica Medical S.A.S.</t>
+          <t>Oportunidad de Clínica VIP Centro de Medicina Internacional</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1211,7 +1220,7 @@
         </is>
       </c>
       <c r="G17" s="1" t="n">
-        <v>46217.62244212963</v>
+        <v>46217.63989583333</v>
       </c>
       <c r="I17" t="n">
         <v>29</v>
@@ -1228,7 +1237,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>calidad@institutodelcorazon.com</t>
+          <t>hocen.direc@policia.gov.co</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1241,7 +1250,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Oportunidad de Instituto del Corazón de Bogotá</t>
+          <t>Oportunidad de Hospital Central Policía Nacional</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1250,7 +1259,7 @@
         </is>
       </c>
       <c r="G18" s="1" t="n">
-        <v>46217.62072916667</v>
+        <v>46217.63702546297</v>
       </c>
       <c r="I18" t="n">
         <v>29</v>
@@ -1267,7 +1276,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ana.ulloa@mederi.com.co</t>
+          <t>coor.calidad@clinicamedical.com.co</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1280,7 +1289,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Oportunidad de Hospital Universitario Mayor - Mederi</t>
+          <t>Oportunidad de Clínica Medical S.A.S.</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1289,7 +1298,7 @@
         </is>
       </c>
       <c r="G19" s="1" t="n">
-        <v>46217.61866898148</v>
+        <v>46217.62244212963</v>
       </c>
       <c r="I19" t="n">
         <v>29</v>
@@ -1306,7 +1315,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ayudantia@homil.gov.co</t>
+          <t>calidad@institutodelcorazon.com</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1319,7 +1328,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Oportunidad de Hospital Militar Central</t>
+          <t>Oportunidad de Instituto del Corazón de Bogotá</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1328,7 +1337,7 @@
         </is>
       </c>
       <c r="G20" s="1" t="n">
-        <v>46217.61708333333</v>
+        <v>46217.62072916667</v>
       </c>
       <c r="I20" t="n">
         <v>29</v>
@@ -1345,7 +1354,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>direccion.general@hospitalinfantildesanjose.org.co</t>
+          <t>ana.ulloa@mederi.com.co</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1358,7 +1367,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Oportunidad de Fundación Hospital Infantil Universitario de San José</t>
+          <t>Oportunidad de Hospital Universitario Mayor - Mederi</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1367,7 +1376,7 @@
         </is>
       </c>
       <c r="G21" s="1" t="n">
-        <v>46217.6153587963</v>
+        <v>46217.61866898148</v>
       </c>
       <c r="I21" t="n">
         <v>29</v>
@@ -1384,7 +1393,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>calidad@clinicadeloccidente.com</t>
+          <t>ayudantia@homil.gov.co</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1397,7 +1406,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica del Occidente S.A.</t>
+          <t>Oportunidad de Hospital Militar Central</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1406,7 +1415,7 @@
         </is>
       </c>
       <c r="G22" s="1" t="n">
-        <v>46217.61388888889</v>
+        <v>46217.61708333333</v>
       </c>
       <c r="I22" t="n">
         <v>29</v>
@@ -1423,7 +1432,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>calidad@husi.org.co</t>
+          <t>direccion.general@hospitalinfantildesanjose.org.co</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1436,7 +1445,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Oportunidad de Hospital Universitario San Ignacio</t>
+          <t>Oportunidad de Fundación Hospital Infantil Universitario de San José</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1445,7 +1454,7 @@
         </is>
       </c>
       <c r="G23" s="1" t="n">
-        <v>46217.61174768519</v>
+        <v>46217.6153587963</v>
       </c>
       <c r="I23" t="n">
         <v>29</v>
@@ -1462,7 +1471,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>cmarly@clinicademarly.com.co</t>
+          <t>calidad@clinicadeloccidente.com</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1475,7 +1484,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica de Marly</t>
+          <t>Oportunidad de Clínica del Occidente S.A.</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1484,7 +1493,7 @@
         </is>
       </c>
       <c r="G24" s="1" t="n">
-        <v>46217.60430555556</v>
+        <v>46217.61388888889</v>
       </c>
       <c r="I24" t="n">
         <v>29</v>
@@ -1501,7 +1510,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>gerencia@hus.org.co</t>
+          <t>calidad@husi.org.co</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1514,7 +1523,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Oportunidad de Hospital Universitario de la Samaritana</t>
+          <t>Oportunidad de Hospital Universitario San Ignacio</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1523,7 +1532,7 @@
         </is>
       </c>
       <c r="G25" s="1" t="n">
-        <v>46217.60261574074</v>
+        <v>46217.61174768519</v>
       </c>
       <c r="I25" t="n">
         <v>29</v>
@@ -1540,7 +1549,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>nomorales@colsanitas.com</t>
+          <t>cmarly@clinicademarly.com.co</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1553,7 +1562,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica Colsanitas Reina Sofía Pediátrica y Mujer</t>
+          <t>Oportunidad de Clínica de Marly</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1562,7 +1571,7 @@
         </is>
       </c>
       <c r="G26" s="1" t="n">
-        <v>46217.60097222222</v>
+        <v>46217.60430555556</v>
       </c>
       <c r="I26" t="n">
         <v>29</v>
@@ -1579,7 +1588,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>nomorales@colsanitas.com</t>
+          <t>gerencia@hus.org.co</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1592,7 +1601,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica Universitaria Colombia (Colsanitas)</t>
+          <t>Oportunidad de Hospital Universitario de la Samaritana</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1601,7 +1610,7 @@
         </is>
       </c>
       <c r="G27" s="1" t="n">
-        <v>46217.59863425926</v>
+        <v>46217.60261574074</v>
       </c>
       <c r="I27" t="n">
         <v>29</v>
@@ -1618,7 +1627,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>zayda.rodriguez@cpolaya.com.co</t>
+          <t>nomorales@colsanitas.com</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1631,7 +1640,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Oportunidad de Centro Policlínico del Olaya</t>
+          <t>Oportunidad de Clínica Colsanitas Reina Sofía Pediátrica y Mujer</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1640,7 +1649,7 @@
         </is>
       </c>
       <c r="G28" s="1" t="n">
-        <v>46217.59719907407</v>
+        <v>46217.60097222222</v>
       </c>
       <c r="I28" t="n">
         <v>29</v>
@@ -1657,7 +1666,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>pcasallas@lacardiol.org</t>
+          <t>nomorales@colsanitas.com</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1670,7 +1679,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Oportunidad de Fundación Cardioinfantil - Instituto de Cardiología</t>
+          <t>Oportunidad de Clínica Universitaria Colombia (Colsanitas)</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1679,7 +1688,7 @@
         </is>
       </c>
       <c r="G29" s="1" t="n">
-        <v>46217.59630787037</v>
+        <v>46217.59863425926</v>
       </c>
       <c r="I29" t="n">
         <v>29</v>
@@ -1696,7 +1705,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>dir_calidad@clinicajuanncorpas.com</t>
+          <t>zayda.rodriguez@cpolaya.com.co</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1709,7 +1718,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica Juan N Corpas Ltda</t>
+          <t>Oportunidad de Centro Policlínico del Olaya</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1718,7 +1727,7 @@
         </is>
       </c>
       <c r="G30" s="1" t="n">
-        <v>46217.52333333333</v>
+        <v>46217.59719907407</v>
       </c>
       <c r="I30" t="n">
         <v>29</v>
@@ -1735,7 +1744,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>dianaespinosanarvaez@gmail.com</t>
+          <t>pcasallas@lacardiol.org</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1748,7 +1757,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica Onkos</t>
+          <t>Oportunidad de Fundación Cardioinfantil - Instituto de Cardiología</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1757,7 +1766,7 @@
         </is>
       </c>
       <c r="G31" s="1" t="n">
-        <v>46217.52202546296</v>
+        <v>46217.59630787037</v>
       </c>
       <c r="I31" t="n">
         <v>29</v>
@@ -1774,7 +1783,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>gestiondecalidad@clinicapalermo.com.co</t>
+          <t>dir_calidad@clinicajuanncorpas.com</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1787,7 +1796,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica Palermo</t>
+          <t>Oportunidad de Clínica Juan N Corpas Ltda</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1796,7 +1805,7 @@
         </is>
       </c>
       <c r="G32" s="1" t="n">
-        <v>46217.51743055556</v>
+        <v>46217.52333333333</v>
       </c>
       <c r="I32" t="n">
         <v>29</v>
@@ -1813,7 +1822,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>calidad@hospitaldesanjose.org.co</t>
+          <t>dianaespinosanarvaez@gmail.com</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1826,7 +1835,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Oportunidad de Hospital San José - Sociedad de Cirugía de Bogotá</t>
+          <t>Oportunidad de Clínica Onkos</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1835,7 +1844,7 @@
         </is>
       </c>
       <c r="G33" s="1" t="n">
-        <v>46217.51425925926</v>
+        <v>46217.52202546296</v>
       </c>
       <c r="I33" t="n">
         <v>29</v>
@@ -1852,7 +1861,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>jzapata@ioir.org.co</t>
+          <t>gestiondecalidad@clinicapalermo.com.co</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1865,7 +1874,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Oportunidad de Instituto de Ortopedia Infantil Roosevelt</t>
+          <t>Oportunidad de Clínica Palermo</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1874,7 +1883,7 @@
         </is>
       </c>
       <c r="G34" s="1" t="n">
-        <v>46217.51231481481</v>
+        <v>46217.51743055556</v>
       </c>
       <c r="I34" t="n">
         <v>29</v>
@@ -1891,7 +1900,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>diana.potesno@colsubsidio.com</t>
+          <t>calidad@hospitaldesanjose.org.co</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1904,7 +1913,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica Colsubsidio Calle 100</t>
+          <t>Oportunidad de Hospital San José - Sociedad de Cirugía de Bogotá</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1913,7 +1922,7 @@
         </is>
       </c>
       <c r="G35" s="1" t="n">
-        <v>46217.51116898148</v>
+        <v>46217.51425925926</v>
       </c>
       <c r="I35" t="n">
         <v>29</v>
@@ -1930,7 +1939,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>diana.potesno@colsubsidio.com</t>
+          <t>jzapata@ioir.org.co</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1943,7 +1952,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica Colsubsidio Calle 100</t>
+          <t>Oportunidad de Instituto de Ortopedia Infantil Roosevelt</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -1952,7 +1961,7 @@
         </is>
       </c>
       <c r="G36" s="1" t="n">
-        <v>46217.50983796296</v>
+        <v>46217.51231481481</v>
       </c>
       <c r="I36" t="n">
         <v>29</v>
@@ -1969,7 +1978,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>jose.chaves@colsubsidio.com</t>
+          <t>diana.potesno@colsubsidio.com</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1982,7 +1991,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica Colsubsidio Ciudad Roma</t>
+          <t>Oportunidad de Clínica Colsubsidio Calle 100</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -1991,7 +2000,7 @@
         </is>
       </c>
       <c r="G37" s="1" t="n">
-        <v>46217.50767361111</v>
+        <v>46217.51116898148</v>
       </c>
       <c r="I37" t="n">
         <v>29</v>
@@ -2008,7 +2017,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>carlos.artetamo@colsubsidio.com</t>
+          <t>diana.potesno@colsubsidio.com</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2021,7 +2030,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica Infantil Colsubsidio</t>
+          <t>Oportunidad de Clínica Colsubsidio Calle 100</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2030,7 +2039,7 @@
         </is>
       </c>
       <c r="G38" s="1" t="n">
-        <v>46217.50050925926</v>
+        <v>46217.50983796296</v>
       </c>
       <c r="I38" t="n">
         <v>29</v>
@@ -2047,7 +2056,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>notificacionescdc@clinicadelcountry.com</t>
+          <t>jose.chaves@colsubsidio.com</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2060,7 +2069,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica del Country IPS</t>
+          <t>Oportunidad de Clínica Colsubsidio Ciudad Roma</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2069,7 +2078,7 @@
         </is>
       </c>
       <c r="G39" s="1" t="n">
-        <v>46217.49881944444</v>
+        <v>46217.50767361111</v>
       </c>
       <c r="I39" t="n">
         <v>29</v>
@@ -2086,7 +2095,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>direcciongeneral@shaio.org</t>
+          <t>carlos.artetamo@colsubsidio.com</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2099,7 +2108,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Oportunidad de Fundación Abood Shaio</t>
+          <t>Oportunidad de Clínica Infantil Colsubsidio</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -2108,7 +2117,7 @@
         </is>
       </c>
       <c r="G40" s="1" t="n">
-        <v>46217.49715277777</v>
+        <v>46217.50050925926</v>
       </c>
       <c r="I40" t="n">
         <v>29</v>
@@ -2125,7 +2134,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>direccion@cancer.gov.co</t>
+          <t>notificacionescdc@clinicadelcountry.com</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2138,7 +2147,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Oportunidad de Instituto Nacional de Cancerología</t>
+          <t>Oportunidad de Clínica del Country IPS</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2147,7 +2156,7 @@
         </is>
       </c>
       <c r="G41" s="1" t="n">
-        <v>46217.47924768519</v>
+        <v>46217.49881944444</v>
       </c>
       <c r="I41" t="n">
         <v>29</v>
@@ -2164,7 +2173,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>sdirmedica@clinicadelamujer.com.co</t>
+          <t>direcciongeneral@shaio.org</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2177,7 +2186,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica de la Mujer</t>
+          <t>Oportunidad de Fundación Abood Shaio</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -2186,7 +2195,7 @@
         </is>
       </c>
       <c r="G42" s="1" t="n">
-        <v>46217.47585648148</v>
+        <v>46217.49715277777</v>
       </c>
       <c r="I42" t="n">
         <v>29</v>
@@ -2203,7 +2212,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>lidercalidad@homifundacion.org.co</t>
+          <t>direccion@cancer.gov.co</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2216,7 +2225,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Oportunidad de Fundación Hospital de la Misericordia (HOMI)</t>
+          <t>Oportunidad de Instituto Nacional de Cancerología</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2225,7 +2234,7 @@
         </is>
       </c>
       <c r="G43" s="1" t="n">
-        <v>46217.47246527778</v>
+        <v>46217.47924768519</v>
       </c>
       <c r="I43" t="n">
         <v>29</v>
@@ -2242,7 +2251,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>direcciongeneral1@stewardcolombia.org</t>
+          <t>sdirmedica@clinicadelamujer.com.co</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2255,7 +2264,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Oportunidad de Hospital Universitario Clínica San Rafael</t>
+          <t>Oportunidad de Clínica de la Mujer</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -2264,7 +2273,7 @@
         </is>
       </c>
       <c r="G44" s="1" t="n">
-        <v>46217.00748842592</v>
+        <v>46217.47585648148</v>
       </c>
       <c r="I44" t="n">
         <v>29</v>
@@ -2281,7 +2290,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>adriana.urrego@fsfb.org.co</t>
+          <t>lidercalidad@homifundacion.org.co</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2294,7 +2303,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Oportunidad de FUNDACION SANTA FE DE BOGOTA</t>
+          <t>Oportunidad de Fundación Hospital de la Misericordia (HOMI)</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -2303,7 +2312,7 @@
         </is>
       </c>
       <c r="G45" s="1" t="n">
-        <v>46217.00381944444</v>
+        <v>46217.47246527778</v>
       </c>
       <c r="I45" t="n">
         <v>29</v>
@@ -2320,7 +2329,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>calidadsalud@cafam.com.co</t>
+          <t>direcciongeneral1@stewardcolombia.org</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2333,7 +2342,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Oportunidad de Centro de Atención en Salud CAFAM Clínica Calle 51</t>
+          <t>Oportunidad de Hospital Universitario Clínica San Rafael</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2342,7 +2351,7 @@
         </is>
       </c>
       <c r="G46" s="1" t="n">
-        <v>46216.99954861111</v>
+        <v>46217.00748842592</v>
       </c>
       <c r="I46" t="n">
         <v>29</v>
@@ -2359,7 +2368,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>notificacionesjudiciales@fhsc.org.co</t>
+          <t>adriana.urrego@fsfb.org.co</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2372,7 +2381,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Oportunidad de Fundación Hospital San Carlos</t>
+          <t>Oportunidad de FUNDACION SANTA FE DE BOGOTA</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -2381,7 +2390,7 @@
         </is>
       </c>
       <c r="G47" s="1" t="n">
-        <v>46216.99548611111</v>
+        <v>46217.00381944444</v>
       </c>
       <c r="I47" t="n">
         <v>29</v>
@@ -2398,7 +2407,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>calidad@proseguir.org</t>
+          <t>calidadsalud@cafam.com.co</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2411,7 +2420,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Oportunidad de PROSEGUIR SEDE 3</t>
+          <t>Oportunidad de Centro de Atención en Salud CAFAM Clínica Calle 51</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2420,7 +2429,7 @@
         </is>
       </c>
       <c r="G48" s="1" t="n">
-        <v>46216.99299768519</v>
+        <v>46216.99954861111</v>
       </c>
       <c r="I48" t="n">
         <v>29</v>
@@ -2437,115 +2446,107 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>centrodecontacto@uao.edu.co</t>
+          <t>notificacionesjudiciales@fhsc.org.co</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Negociación</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>10000000</v>
+        <v>0</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Oportunidad de UNIVERSIDAD AUTONOMA DE OCCIDENTE</t>
+          <t>Oportunidad de Fundación Hospital San Carlos</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G49" s="1" t="n">
-        <v>46213.49821759259</v>
+        <v>46216.99548611111</v>
       </c>
       <c r="I49" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J49" t="n">
         <v>2026</v>
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>carlos.segovia@warena.co</t>
+          <t>calidad@proseguir.org</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Negociación</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>35000000</v>
+        <v>0</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Oportunidad de W ARENA</t>
+          <t>Oportunidad de PROSEGUIR SEDE 3</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G50" s="1" t="n">
-        <v>46213.49508101852</v>
+        <v>46216.99299768519</v>
       </c>
       <c r="I50" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J50" t="n">
         <v>2026</v>
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>klondono@fundacionwwbcol.org</t>
+          <t>centrodecontacto@uao.edu.co</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Ganado</t>
+          <t>Negociación</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>300000</v>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>Karla Londoño</t>
-        </is>
+        <v>10000000</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Oportunidad de Karla Londoño</t>
+          <t>Oportunidad de UNIVERSIDAD AUTONOMA DE OCCIDENTE</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G51" s="1" t="n">
-        <v>46212.51638888889</v>
-      </c>
-      <c r="H51" s="1" t="n">
-        <v>46217</v>
+        <v>46213.49821759259</v>
       </c>
       <c r="I51" t="n">
         <v>28</v>
@@ -2553,12 +2554,6 @@
       <c r="J51" t="n">
         <v>2026</v>
       </c>
-      <c r="K51" t="n">
-        <v>7</v>
-      </c>
-      <c r="L51" t="n">
-        <v>2026</v>
-      </c>
       <c r="M51" t="inlineStr">
         <is>
           <t>Calificado</t>
@@ -2568,7 +2563,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>ctorres@colcobranzasnacionales.com</t>
+          <t>carlos.segovia@warena.co</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2577,28 +2572,23 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>5000000</v>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>ctorres@colcobranzasnacionales.com</t>
-        </is>
+        <v>35000000</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Oportunidad de ctorres@colcobranzasnacionales.com</t>
+          <t>Oportunidad de W ARENA</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G52" s="1" t="n">
-        <v>46206.73804398148</v>
+        <v>46213.49508101852</v>
       </c>
       <c r="I52" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J52" t="n">
         <v>2026</v>
@@ -2612,7 +2602,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>medifar624@gmail.com</t>
+          <t>klondono@fundacionwwbcol.org</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2621,11 +2611,16 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>1640000</v>
+        <v>300000</v>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Karla Londoño</t>
+        </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Oportunidad de MEDISFARMA SAS</t>
+          <t>Oportunidad de Karla Londoño</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -2634,19 +2629,19 @@
         </is>
       </c>
       <c r="G53" s="1" t="n">
-        <v>46203.72597222222</v>
+        <v>46212.51638888889</v>
       </c>
       <c r="H53" s="1" t="n">
-        <v>46199</v>
+        <v>46217</v>
       </c>
       <c r="I53" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J53" t="n">
         <v>2026</v>
       </c>
       <c r="K53" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L53" t="n">
         <v>2026</v>
@@ -2660,7 +2655,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>mercadeo@norteysur.co</t>
+          <t>ctorres@colcobranzasnacionales.com</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2669,16 +2664,16 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>28190000</v>
+        <v>5000000</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Isabella Mesa</t>
+          <t>ctorres@colcobranzasnacionales.com</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Oportunidad de Isabella Mesa</t>
+          <t>Oportunidad de ctorres@colcobranzasnacionales.com</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -2687,10 +2682,10 @@
         </is>
       </c>
       <c r="G54" s="1" t="n">
-        <v>46191.70076388889</v>
+        <v>46206.73804398148</v>
       </c>
       <c r="I54" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="J54" t="n">
         <v>2026</v>
@@ -2704,20 +2699,20 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>comercial@asertis.com.co</t>
+          <t>medifar624@gmail.com</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Ganado</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>0</v>
+        <v>1640000</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Oportunidad de IMPORTADORA CALI S.A.</t>
+          <t>Oportunidad de MEDISFARMA SAS</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -2726,42 +2721,51 @@
         </is>
       </c>
       <c r="G55" s="1" t="n">
-        <v>46189.67539351852</v>
+        <v>46203.72597222222</v>
+      </c>
+      <c r="H55" s="1" t="n">
+        <v>46199</v>
       </c>
       <c r="I55" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="J55" t="n">
         <v>2026</v>
       </c>
+      <c r="K55" t="n">
+        <v>6</v>
+      </c>
+      <c r="L55" t="n">
+        <v>2026</v>
+      </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>educacion@360forma.edu.co</t>
+          <t>mercadeo@norteysur.co</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Negociación</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>0</v>
+        <v>28190000</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Jorge Sanchez / jefe Comercial</t>
+          <t>Isabella Mesa</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Oportunidad de Jorge Sanchez / jefe Comercial</t>
+          <t>Oportunidad de Isabella Mesa</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -2770,7 +2774,7 @@
         </is>
       </c>
       <c r="G56" s="1" t="n">
-        <v>46189.65077546296</v>
+        <v>46191.70076388889</v>
       </c>
       <c r="I56" t="n">
         <v>25</v>
@@ -2780,19 +2784,19 @@
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>directoradjunto@dclass.edu.co</t>
+          <t>comercial@asertis.com.co</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -2800,7 +2804,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Oportunidad de DCLASS ACADEMIA SAS</t>
+          <t>Oportunidad de IMPORTADORA CALI S.A.</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -2809,7 +2813,7 @@
         </is>
       </c>
       <c r="G57" s="1" t="n">
-        <v>46189.49674768518</v>
+        <v>46189.67539351852</v>
       </c>
       <c r="I57" t="n">
         <v>25</v>
@@ -2826,7 +2830,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Belkis.jimenez@agrauto.com.co</t>
+          <t>educacion@360forma.edu.co</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2837,9 +2841,14 @@
       <c r="C58" t="n">
         <v>0</v>
       </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Jorge Sanchez / jefe Comercial</t>
+        </is>
+      </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Oportunidad de AGRICOLA AUTOMOTRIZ SAS / BELKYS JIMENEZ</t>
+          <t>Oportunidad de Jorge Sanchez / jefe Comercial</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -2848,10 +2857,10 @@
         </is>
       </c>
       <c r="G58" s="1" t="n">
-        <v>46182.67912037037</v>
+        <v>46189.65077546296</v>
       </c>
       <c r="I58" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J58" t="n">
         <v>2026</v>
@@ -2865,25 +2874,20 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>luisa.baena@automarcali.com</t>
+          <t>directoradjunto@dclass.edu.co</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C59" t="n">
         <v>0</v>
       </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>luisa.baena@automarcali.com</t>
-        </is>
-      </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Oportunidad de luisa.baena@automarcali.com</t>
+          <t>Oportunidad de DCLASS ACADEMIA SAS</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -2892,10 +2896,10 @@
         </is>
       </c>
       <c r="G59" s="1" t="n">
-        <v>46182.67809027778</v>
+        <v>46189.49674768518</v>
       </c>
       <c r="I59" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J59" t="n">
         <v>2026</v>
@@ -2909,7 +2913,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>directormercadeo@almotores.com</t>
+          <t>Belkis.jimenez@agrauto.com.co</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2920,14 +2924,9 @@
       <c r="C60" t="n">
         <v>0</v>
       </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>Viviana Vanegas</t>
-        </is>
-      </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Oportunidad de Viviana Vanegas</t>
+          <t>Oportunidad de AGRICOLA AUTOMOTRIZ SAS / BELKYS JIMENEZ</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -2936,7 +2935,7 @@
         </is>
       </c>
       <c r="G60" s="1" t="n">
-        <v>46182.67621527778</v>
+        <v>46182.67912037037</v>
       </c>
       <c r="I60" t="n">
         <v>24</v>
@@ -2953,7 +2952,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>xiomara.duran@autopacifico.com.co</t>
+          <t>luisa.baena@automarcali.com</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2964,9 +2963,14 @@
       <c r="C61" t="n">
         <v>0</v>
       </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>luisa.baena@automarcali.com</t>
+        </is>
+      </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Oportunidad de xiomara.duran@autopacifico.com.co</t>
+          <t>Oportunidad de luisa.baena@automarcali.com</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -2975,7 +2979,7 @@
         </is>
       </c>
       <c r="G61" s="1" t="n">
-        <v>46182.65815972222</v>
+        <v>46182.67809027778</v>
       </c>
       <c r="I61" t="n">
         <v>24</v>
@@ -2992,12 +2996,12 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>alejandrosaavedraconde@comfandi.com.co</t>
+          <t>directormercadeo@almotores.com</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -3005,12 +3009,12 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>ALEJANDRO</t>
+          <t>Viviana Vanegas</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Oportunidad de ALEJANDRO</t>
+          <t>Oportunidad de Viviana Vanegas</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -3019,7 +3023,7 @@
         </is>
       </c>
       <c r="G62" s="1" t="n">
-        <v>46182.64278935185</v>
+        <v>46182.67621527778</v>
       </c>
       <c r="I62" t="n">
         <v>24</v>
@@ -3036,12 +3040,12 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>administracion@fiando.com.co</t>
+          <t>xiomara.duran@autopacifico.com.co</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -3049,7 +3053,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Oportunidad de FIANDO LTDA</t>
+          <t>Oportunidad de xiomara.duran@autopacifico.com.co</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -3058,7 +3062,7 @@
         </is>
       </c>
       <c r="G63" s="1" t="n">
-        <v>46182.61304398148</v>
+        <v>46182.65815972222</v>
       </c>
       <c r="I63" t="n">
         <v>24</v>
@@ -3068,19 +3072,19 @@
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>dgamoneda@productosdrogam.com</t>
+          <t>alejandrosaavedraconde@comfandi.com.co</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -3088,12 +3092,12 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t xml:space="preserve">Diego Mauricio Gamoneda </t>
+          <t>ALEJANDRO</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t xml:space="preserve">Oportunidad de Diego Mauricio Gamoneda </t>
+          <t>Oportunidad de ALEJANDRO</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -3102,10 +3106,10 @@
         </is>
       </c>
       <c r="G64" s="1" t="n">
-        <v>46175.66417824074</v>
+        <v>46182.64278935185</v>
       </c>
       <c r="I64" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J64" t="n">
         <v>2026</v>
@@ -3119,7 +3123,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>alexander.rojas@friogan.com</t>
+          <t>administracion@fiando.com.co</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -3128,11 +3132,11 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>10000000</v>
+        <v>0</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Oportunidad de FRIOGAN S.A</t>
+          <t>Oportunidad de FIANDO LTDA</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -3141,10 +3145,10 @@
         </is>
       </c>
       <c r="G65" s="1" t="n">
-        <v>46175.63597222222</v>
+        <v>46182.61304398148</v>
       </c>
       <c r="I65" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J65" t="n">
         <v>2026</v>
@@ -3156,17 +3160,27 @@
       </c>
     </row>
     <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>dgamoneda@productosdrogam.com</t>
+        </is>
+      </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C66" t="n">
         <v>0</v>
       </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Diego Mauricio Gamoneda </t>
+        </is>
+      </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Oportunidad de Agromercados la Montaña</t>
+          <t xml:space="preserve">Oportunidad de Diego Mauricio Gamoneda </t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -3175,7 +3189,7 @@
         </is>
       </c>
       <c r="G66" s="1" t="n">
-        <v>46175.62239583334</v>
+        <v>46175.66417824074</v>
       </c>
       <c r="I66" t="n">
         <v>23</v>
@@ -3192,20 +3206,20 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>juand.rios@alkosto.com.co</t>
+          <t>alexander.rojas@friogan.com</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>0</v>
+        <v>10000000</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Oportunidad de ALKOSTO</t>
+          <t>Oportunidad de FRIOGAN S.A</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -3214,7 +3228,7 @@
         </is>
       </c>
       <c r="G67" s="1" t="n">
-        <v>46175.62055555556</v>
+        <v>46175.63597222222</v>
       </c>
       <c r="I67" t="n">
         <v>23</v>
@@ -3224,16 +3238,11 @@
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>gerencia4087@grupo-exito.com</t>
-        </is>
-      </c>
       <c r="B68" t="inlineStr">
         <is>
           <t>Perdido</t>
@@ -3242,14 +3251,9 @@
       <c r="C68" t="n">
         <v>0</v>
       </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>Grupo exito ‒ 1007386172 - Sneider Quirama</t>
-        </is>
-      </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Oportunidad de Grupo exito</t>
+          <t>Oportunidad de Agromercados la Montaña</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -3258,7 +3262,7 @@
         </is>
       </c>
       <c r="G68" s="1" t="n">
-        <v>46175.61638888889</v>
+        <v>46175.62239583334</v>
       </c>
       <c r="I68" t="n">
         <v>23</v>
@@ -3275,7 +3279,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>ldgomez@supertiendascanaveral.com</t>
+          <t>juand.rios@alkosto.com.co</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -3286,14 +3290,9 @@
       <c r="C69" t="n">
         <v>0</v>
       </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>Luis David Gomez</t>
-        </is>
-      </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Oportunidad de Luis David Gomez</t>
+          <t>Oportunidad de ALKOSTO</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -3302,7 +3301,7 @@
         </is>
       </c>
       <c r="G69" s="1" t="n">
-        <v>46175.60493055556</v>
+        <v>46175.62055555556</v>
       </c>
       <c r="I69" t="n">
         <v>23</v>
@@ -3319,20 +3318,25 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>davida_vanegas@coomeva.com.co</t>
+          <t>gerencia4087@grupo-exito.com</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C70" t="n">
         <v>0</v>
       </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Grupo exito ‒ 1007386172 - Sneider Quirama</t>
+        </is>
+      </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Oportunidad de BANCOOMEVA</t>
+          <t>Oportunidad de Grupo exito</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -3341,7 +3345,7 @@
         </is>
       </c>
       <c r="G70" s="1" t="n">
-        <v>46175.47109953704</v>
+        <v>46175.61638888889</v>
       </c>
       <c r="I70" t="n">
         <v>23</v>
@@ -3358,12 +3362,12 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>alejandro.delgado@filedesk.com.co</t>
+          <t>ldgomez@supertiendascanaveral.com</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -3371,12 +3375,12 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>AlejandroDelgado</t>
+          <t>Luis David Gomez</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Oportunidad de AlejandroDelgado</t>
+          <t>Oportunidad de Luis David Gomez</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -3385,7 +3389,7 @@
         </is>
       </c>
       <c r="G71" s="1" t="n">
-        <v>46174.71665509259</v>
+        <v>46175.60493055556</v>
       </c>
       <c r="I71" t="n">
         <v>23</v>
@@ -3400,22 +3404,22 @@
       </c>
     </row>
     <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>davida_vanegas@coomeva.com.co</t>
+        </is>
+      </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>35000000</v>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>Olga Lucia Hurtado</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Oportunidad de Olga Lucia Hurtado</t>
+          <t>Oportunidad de BANCOOMEVA</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -3424,120 +3428,120 @@
         </is>
       </c>
       <c r="G72" s="1" t="n">
-        <v>46168.49854166667</v>
+        <v>46175.47109953704</v>
       </c>
       <c r="I72" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="J72" t="n">
         <v>2026</v>
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>comercial2@felsyn.com</t>
+          <t>alejandro.delgado@filedesk.com.co</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
+          <t>Contactado</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>0</v>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>AlejandroDelgado</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Oportunidad de AlejandroDelgado</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G73" s="1" t="n">
+        <v>46174.71665509259</v>
+      </c>
+      <c r="I73" t="n">
+        <v>23</v>
+      </c>
+      <c r="J73" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>No calificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="B74" t="inlineStr">
+        <is>
           <t>Propuesta</t>
         </is>
       </c>
-      <c r="C73" t="n">
-        <v>713400</v>
-      </c>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>Oportunidad de FONDO DE EMPLEADOS FELSYN</t>
-        </is>
-      </c>
-      <c r="F73" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G73" s="1" t="n">
-        <v>46163.49130787037</v>
-      </c>
-      <c r="I73" t="n">
-        <v>21</v>
-      </c>
-      <c r="J73" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M73" t="inlineStr">
+      <c r="C74" t="n">
+        <v>35000000</v>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Olga Lucia Hurtado</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Oportunidad de Olga Lucia Hurtado</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G74" s="1" t="n">
+        <v>46168.49854166667</v>
+      </c>
+      <c r="I74" t="n">
+        <v>22</v>
+      </c>
+      <c r="J74" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M74" t="inlineStr">
         <is>
           <t>Calificado</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>mercadeo@lasevillana.com.co</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>Contactado</t>
-        </is>
-      </c>
-      <c r="C74" t="n">
-        <v>0</v>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fabio AlbertoGallego García </t>
-        </is>
-      </c>
-      <c r="E74" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Oportunidad de Fabio AlbertoGallego García </t>
-        </is>
-      </c>
-      <c r="F74" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G74" s="1" t="n">
-        <v>46162.64569444444</v>
-      </c>
-      <c r="I74" t="n">
-        <v>21</v>
-      </c>
-      <c r="J74" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M74" t="inlineStr">
-        <is>
-          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>asantiago@stop.com.co</t>
+          <t>comercial2@felsyn.com</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>0</v>
+        <v>713400</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Oportunidad de STOP SAS</t>
+          <t>Oportunidad de FONDO DE EMPLEADOS FELSYN</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -3546,7 +3550,7 @@
         </is>
       </c>
       <c r="G75" s="1" t="n">
-        <v>46161.63508101852</v>
+        <v>46163.49130787037</v>
       </c>
       <c r="I75" t="n">
         <v>21</v>
@@ -3556,32 +3560,32 @@
       </c>
       <c r="M75" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>aestrada@teker.co</t>
+          <t>mercadeo@lasevillana.com.co</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>16914000</v>
+        <v>0</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>TEKER SALUD SAS</t>
+          <t xml:space="preserve">Fabio AlbertoGallego García </t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Oportunidad de TEKER SALUD SAS</t>
+          <t xml:space="preserve">Oportunidad de Fabio AlbertoGallego García </t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -3590,7 +3594,7 @@
         </is>
       </c>
       <c r="G76" s="1" t="n">
-        <v>46161.62922453704</v>
+        <v>46162.64569444444</v>
       </c>
       <c r="I76" t="n">
         <v>21</v>
@@ -3605,6 +3609,11 @@
       </c>
     </row>
     <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>asantiago@stop.com.co</t>
+        </is>
+      </c>
       <c r="B77" t="inlineStr">
         <is>
           <t>Contactado</t>
@@ -3615,7 +3624,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Oportunidad de TIAN IPS SAS</t>
+          <t>Oportunidad de STOP SAS</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -3624,7 +3633,7 @@
         </is>
       </c>
       <c r="G77" s="1" t="n">
-        <v>46161.61643518518</v>
+        <v>46161.63508101852</v>
       </c>
       <c r="I77" t="n">
         <v>21</v>
@@ -3641,7 +3650,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>administración@fullredtotal.com</t>
+          <t>aestrada@teker.co</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -3650,16 +3659,16 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>14000000</v>
+        <v>16914000</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Eivar Eñasco</t>
+          <t>TEKER SALUD SAS</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Oportunidad de Eivar Eñasco</t>
+          <t>Oportunidad de TEKER SALUD SAS</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -3668,10 +3677,10 @@
         </is>
       </c>
       <c r="G78" s="1" t="n">
-        <v>46154.67546296296</v>
+        <v>46161.62922453704</v>
       </c>
       <c r="I78" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J78" t="n">
         <v>2026</v>
@@ -3683,27 +3692,17 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t>cserna@surtifamiliar.com.co</t>
-        </is>
-      </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Ganado</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>975000</v>
-      </c>
-      <c r="D79" t="inlineStr">
-        <is>
-          <t>Claudia Patricia Serna</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Oportunidad de Claudia Patricia Serna</t>
+          <t>Oportunidad de TIAN IPS SAS</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -3712,51 +3711,42 @@
         </is>
       </c>
       <c r="G79" s="1" t="n">
-        <v>46154.66616898148</v>
-      </c>
-      <c r="H79" s="1" t="n">
-        <v>46217</v>
+        <v>46161.61643518518</v>
       </c>
       <c r="I79" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J79" t="n">
         <v>2026</v>
       </c>
-      <c r="K79" t="n">
-        <v>7</v>
-      </c>
-      <c r="L79" t="n">
-        <v>2026</v>
-      </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>coordmercadeo@pacificcenter.co</t>
+          <t>administración@fullredtotal.com</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>5600000</v>
+        <v>14000000</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Claudia Castro</t>
+          <t>Eivar Eñasco</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Oportunidad de Claudia Castro</t>
+          <t>Oportunidad de Eivar Eñasco</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -3765,7 +3755,7 @@
         </is>
       </c>
       <c r="G80" s="1" t="n">
-        <v>46154.66341435185</v>
+        <v>46154.67546296296</v>
       </c>
       <c r="I80" t="n">
         <v>20</v>
@@ -3775,32 +3765,32 @@
       </c>
       <c r="M80" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>isabellarengifo27@gmail.com</t>
+          <t>cserna@surtifamiliar.com.co</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Ganado</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>28190000</v>
+        <v>975000</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Isabella Rengifo</t>
+          <t>Claudia Patricia Serna</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Oportunidad de Isabella Rengifo</t>
+          <t>Oportunidad de Claudia Patricia Serna</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -3809,7 +3799,10 @@
         </is>
       </c>
       <c r="G81" s="1" t="n">
-        <v>46154.65981481481</v>
+        <v>46154.66616898148</v>
+      </c>
+      <c r="H81" s="1" t="n">
+        <v>46217</v>
       </c>
       <c r="I81" t="n">
         <v>20</v>
@@ -3817,9 +3810,15 @@
       <c r="J81" t="n">
         <v>2026</v>
       </c>
+      <c r="K81" t="n">
+        <v>7</v>
+      </c>
+      <c r="L81" t="n">
+        <v>2026</v>
+      </c>
       <c r="M81" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
CRM actualizado — 22/07/2026 07:39
</commit_message>
<xml_diff>
--- a/CRM_PowerBI_BrendaLuna_actualizado.xlsx
+++ b/CRM_PowerBI_BrendaLuna_actualizado.xlsx
@@ -992,26 +992,36 @@
       </c>
     </row>
     <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Kelly.rodriguez@claro.com.co</t>
+        </is>
+      </c>
       <c r="B12" t="inlineStr">
         <is>
           <t>Contactado</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0</v>
+        <v>169000000</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Hermes Alfonso Duarte Mendoza</t>
+        </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Oportunidad de CLINICA DE OFTALMOLOGIA DE CALI S A</t>
+          <t>Oportunidad de Kelly Rodriguez</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G12" s="1" t="n">
-        <v>46224.46891203704</v>
+        <v>46224.67548611111</v>
       </c>
       <c r="I12" t="n">
         <v>30</v>
@@ -1028,37 +1038,34 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>hrodriguez@jaramillomora.com</t>
+          <t>maryuri.urbano@impocali.com</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>48600000</v>
+        <v>0</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>HANNA RODRIGUEZ</t>
+          <t>IMPOCALI</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Oportunidad de HANNA RODRIGUEZ</t>
+          <t>Oportunidad de maryuri.urbano@impocali.com</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G13" s="1" t="n">
-        <v>46224.45887731481</v>
-      </c>
-      <c r="H13" s="1" t="n">
-        <v>46265</v>
+        <v>46224.66466435185</v>
       </c>
       <c r="I13" t="n">
         <v>30</v>
@@ -1066,144 +1073,152 @@
       <c r="J13" t="n">
         <v>2026</v>
       </c>
-      <c r="K13" t="n">
-        <v>8</v>
-      </c>
-      <c r="L13" t="n">
-        <v>2026</v>
-      </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Vidanteips@gmail.com</t>
+          <t>calidad@sumivalle.com</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
+          <t>Contactado</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>calidad@sumivalle.com</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Oportunidad de calidad@sumivalle.com</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G14" s="1" t="n">
+        <v>46224.63564814815</v>
+      </c>
+      <c r="I14" t="n">
+        <v>30</v>
+      </c>
+      <c r="J14" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>No calificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Contactado</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Oportunidad de CLINICA DE OFTALMOLOGIA DE CALI S A</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Jennifer Hoyos Gallego</t>
+        </is>
+      </c>
+      <c r="G15" s="1" t="n">
+        <v>46224.46891203704</v>
+      </c>
+      <c r="I15" t="n">
+        <v>30</v>
+      </c>
+      <c r="J15" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>No calificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>hrodriguez@jaramillomora.com</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
           <t>Propuesta</t>
         </is>
       </c>
-      <c r="C14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Oportunidad de VIDANTE IPS SAS</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G14" s="1" t="n">
-        <v>46219.71274305556</v>
-      </c>
-      <c r="I14" t="n">
-        <v>29</v>
-      </c>
-      <c r="J14" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M14" t="inlineStr">
+      <c r="C16" t="n">
+        <v>48600000</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>HANNA RODRIGUEZ</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Oportunidad de HANNA RODRIGUEZ</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Jennifer Hoyos Gallego</t>
+        </is>
+      </c>
+      <c r="G16" s="1" t="n">
+        <v>46224.45887731481</v>
+      </c>
+      <c r="H16" s="1" t="n">
+        <v>46265</v>
+      </c>
+      <c r="I16" t="n">
+        <v>30</v>
+      </c>
+      <c r="J16" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K16" t="n">
+        <v>8</v>
+      </c>
+      <c r="L16" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M16" t="inlineStr">
         <is>
           <t>Calificado</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>francisco.alzate@aficenter.com.co</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Contactado</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>30000000</v>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>francisco.alzate@aficenter.com.co</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Oportunidad de francisco.alzate@aficenter.com.co</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G15" s="1" t="n">
-        <v>46217.71496527778</v>
-      </c>
-      <c r="I15" t="n">
-        <v>29</v>
-      </c>
-      <c r="J15" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>No calificado</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Contactado</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Oportunidad de Fajas Gama Alta</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G16" s="1" t="n">
-        <v>46217.64614583334</v>
-      </c>
-      <c r="I16" t="n">
-        <v>29</v>
-      </c>
-      <c r="J16" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>calidad.vip@axacolpatria.co</t>
+          <t>Vidanteips@gmail.com</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -1211,7 +1226,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica VIP Centro de Medicina Internacional</t>
+          <t>Oportunidad de VIDANTE IPS SAS</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1220,7 +1235,7 @@
         </is>
       </c>
       <c r="G17" s="1" t="n">
-        <v>46217.63989583333</v>
+        <v>46219.71274305556</v>
       </c>
       <c r="I17" t="n">
         <v>29</v>
@@ -1230,14 +1245,14 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>hocen.direc@policia.gov.co</t>
+          <t>francisco.alzate@aficenter.com.co</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1246,11 +1261,16 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>0</v>
+        <v>30000000</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>francisco.alzate@aficenter.com.co</t>
+        </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Oportunidad de Hospital Central Policía Nacional</t>
+          <t>Oportunidad de francisco.alzate@aficenter.com.co</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1259,7 +1279,7 @@
         </is>
       </c>
       <c r="G18" s="1" t="n">
-        <v>46217.63702546297</v>
+        <v>46217.71496527778</v>
       </c>
       <c r="I18" t="n">
         <v>29</v>
@@ -1274,11 +1294,6 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>coor.calidad@clinicamedical.com.co</t>
-        </is>
-      </c>
       <c r="B19" t="inlineStr">
         <is>
           <t>Contactado</t>
@@ -1289,7 +1304,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica Medical S.A.S.</t>
+          <t>Oportunidad de Fajas Gama Alta</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1298,7 +1313,7 @@
         </is>
       </c>
       <c r="G19" s="1" t="n">
-        <v>46217.62244212963</v>
+        <v>46217.64614583334</v>
       </c>
       <c r="I19" t="n">
         <v>29</v>
@@ -1315,7 +1330,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>calidad@institutodelcorazon.com</t>
+          <t>calidad.vip@axacolpatria.co</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1328,7 +1343,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Oportunidad de Instituto del Corazón de Bogotá</t>
+          <t>Oportunidad de Clínica VIP Centro de Medicina Internacional</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1337,7 +1352,7 @@
         </is>
       </c>
       <c r="G20" s="1" t="n">
-        <v>46217.62072916667</v>
+        <v>46217.63989583333</v>
       </c>
       <c r="I20" t="n">
         <v>29</v>
@@ -1354,7 +1369,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ana.ulloa@mederi.com.co</t>
+          <t>hocen.direc@policia.gov.co</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1367,7 +1382,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Oportunidad de Hospital Universitario Mayor - Mederi</t>
+          <t>Oportunidad de Hospital Central Policía Nacional</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1376,7 +1391,7 @@
         </is>
       </c>
       <c r="G21" s="1" t="n">
-        <v>46217.61866898148</v>
+        <v>46217.63702546297</v>
       </c>
       <c r="I21" t="n">
         <v>29</v>
@@ -1393,7 +1408,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ayudantia@homil.gov.co</t>
+          <t>coor.calidad@clinicamedical.com.co</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1406,7 +1421,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Oportunidad de Hospital Militar Central</t>
+          <t>Oportunidad de Clínica Medical S.A.S.</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1415,7 +1430,7 @@
         </is>
       </c>
       <c r="G22" s="1" t="n">
-        <v>46217.61708333333</v>
+        <v>46217.62244212963</v>
       </c>
       <c r="I22" t="n">
         <v>29</v>
@@ -1432,7 +1447,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>direccion.general@hospitalinfantildesanjose.org.co</t>
+          <t>calidad@institutodelcorazon.com</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1445,7 +1460,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Oportunidad de Fundación Hospital Infantil Universitario de San José</t>
+          <t>Oportunidad de Instituto del Corazón de Bogotá</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1454,7 +1469,7 @@
         </is>
       </c>
       <c r="G23" s="1" t="n">
-        <v>46217.6153587963</v>
+        <v>46217.62072916667</v>
       </c>
       <c r="I23" t="n">
         <v>29</v>
@@ -1471,7 +1486,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>calidad@clinicadeloccidente.com</t>
+          <t>ana.ulloa@mederi.com.co</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1484,7 +1499,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica del Occidente S.A.</t>
+          <t>Oportunidad de Hospital Universitario Mayor - Mederi</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1493,7 +1508,7 @@
         </is>
       </c>
       <c r="G24" s="1" t="n">
-        <v>46217.61388888889</v>
+        <v>46217.61866898148</v>
       </c>
       <c r="I24" t="n">
         <v>29</v>
@@ -1510,7 +1525,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>calidad@husi.org.co</t>
+          <t>ayudantia@homil.gov.co</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1523,7 +1538,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Oportunidad de Hospital Universitario San Ignacio</t>
+          <t>Oportunidad de Hospital Militar Central</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1532,7 +1547,7 @@
         </is>
       </c>
       <c r="G25" s="1" t="n">
-        <v>46217.61174768519</v>
+        <v>46217.61708333333</v>
       </c>
       <c r="I25" t="n">
         <v>29</v>
@@ -1549,7 +1564,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>cmarly@clinicademarly.com.co</t>
+          <t>direccion.general@hospitalinfantildesanjose.org.co</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1562,7 +1577,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica de Marly</t>
+          <t>Oportunidad de Fundación Hospital Infantil Universitario de San José</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1571,7 +1586,7 @@
         </is>
       </c>
       <c r="G26" s="1" t="n">
-        <v>46217.60430555556</v>
+        <v>46217.6153587963</v>
       </c>
       <c r="I26" t="n">
         <v>29</v>
@@ -1588,7 +1603,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>gerencia@hus.org.co</t>
+          <t>calidad@clinicadeloccidente.com</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1601,7 +1616,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Oportunidad de Hospital Universitario de la Samaritana</t>
+          <t>Oportunidad de Clínica del Occidente S.A.</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1610,7 +1625,7 @@
         </is>
       </c>
       <c r="G27" s="1" t="n">
-        <v>46217.60261574074</v>
+        <v>46217.61388888889</v>
       </c>
       <c r="I27" t="n">
         <v>29</v>
@@ -1627,7 +1642,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>nomorales@colsanitas.com</t>
+          <t>calidad@husi.org.co</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1640,7 +1655,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica Colsanitas Reina Sofía Pediátrica y Mujer</t>
+          <t>Oportunidad de Hospital Universitario San Ignacio</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1649,7 +1664,7 @@
         </is>
       </c>
       <c r="G28" s="1" t="n">
-        <v>46217.60097222222</v>
+        <v>46217.61174768519</v>
       </c>
       <c r="I28" t="n">
         <v>29</v>
@@ -1666,7 +1681,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>nomorales@colsanitas.com</t>
+          <t>cmarly@clinicademarly.com.co</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1679,7 +1694,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica Universitaria Colombia (Colsanitas)</t>
+          <t>Oportunidad de Clínica de Marly</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1688,7 +1703,7 @@
         </is>
       </c>
       <c r="G29" s="1" t="n">
-        <v>46217.59863425926</v>
+        <v>46217.60430555556</v>
       </c>
       <c r="I29" t="n">
         <v>29</v>
@@ -1705,7 +1720,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>zayda.rodriguez@cpolaya.com.co</t>
+          <t>gerencia@hus.org.co</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1718,7 +1733,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Oportunidad de Centro Policlínico del Olaya</t>
+          <t>Oportunidad de Hospital Universitario de la Samaritana</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1727,7 +1742,7 @@
         </is>
       </c>
       <c r="G30" s="1" t="n">
-        <v>46217.59719907407</v>
+        <v>46217.60261574074</v>
       </c>
       <c r="I30" t="n">
         <v>29</v>
@@ -1744,7 +1759,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>pcasallas@lacardiol.org</t>
+          <t>nomorales@colsanitas.com</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1757,7 +1772,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Oportunidad de Fundación Cardioinfantil - Instituto de Cardiología</t>
+          <t>Oportunidad de Clínica Colsanitas Reina Sofía Pediátrica y Mujer</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1766,7 +1781,7 @@
         </is>
       </c>
       <c r="G31" s="1" t="n">
-        <v>46217.59630787037</v>
+        <v>46217.60097222222</v>
       </c>
       <c r="I31" t="n">
         <v>29</v>
@@ -1783,7 +1798,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>dir_calidad@clinicajuanncorpas.com</t>
+          <t>nomorales@colsanitas.com</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1796,7 +1811,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica Juan N Corpas Ltda</t>
+          <t>Oportunidad de Clínica Universitaria Colombia (Colsanitas)</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1805,7 +1820,7 @@
         </is>
       </c>
       <c r="G32" s="1" t="n">
-        <v>46217.52333333333</v>
+        <v>46217.59863425926</v>
       </c>
       <c r="I32" t="n">
         <v>29</v>
@@ -1822,7 +1837,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>dianaespinosanarvaez@gmail.com</t>
+          <t>zayda.rodriguez@cpolaya.com.co</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1835,7 +1850,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica Onkos</t>
+          <t>Oportunidad de Centro Policlínico del Olaya</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1844,7 +1859,7 @@
         </is>
       </c>
       <c r="G33" s="1" t="n">
-        <v>46217.52202546296</v>
+        <v>46217.59719907407</v>
       </c>
       <c r="I33" t="n">
         <v>29</v>
@@ -1861,7 +1876,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>gestiondecalidad@clinicapalermo.com.co</t>
+          <t>pcasallas@lacardiol.org</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1874,7 +1889,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica Palermo</t>
+          <t>Oportunidad de Fundación Cardioinfantil - Instituto de Cardiología</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1883,7 +1898,7 @@
         </is>
       </c>
       <c r="G34" s="1" t="n">
-        <v>46217.51743055556</v>
+        <v>46217.59630787037</v>
       </c>
       <c r="I34" t="n">
         <v>29</v>
@@ -1900,7 +1915,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>calidad@hospitaldesanjose.org.co</t>
+          <t>dir_calidad@clinicajuanncorpas.com</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1913,7 +1928,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Oportunidad de Hospital San José - Sociedad de Cirugía de Bogotá</t>
+          <t>Oportunidad de Clínica Juan N Corpas Ltda</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1922,7 +1937,7 @@
         </is>
       </c>
       <c r="G35" s="1" t="n">
-        <v>46217.51425925926</v>
+        <v>46217.52333333333</v>
       </c>
       <c r="I35" t="n">
         <v>29</v>
@@ -1939,7 +1954,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>jzapata@ioir.org.co</t>
+          <t>dianaespinosanarvaez@gmail.com</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1952,7 +1967,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Oportunidad de Instituto de Ortopedia Infantil Roosevelt</t>
+          <t>Oportunidad de Clínica Onkos</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -1961,7 +1976,7 @@
         </is>
       </c>
       <c r="G36" s="1" t="n">
-        <v>46217.51231481481</v>
+        <v>46217.52202546296</v>
       </c>
       <c r="I36" t="n">
         <v>29</v>
@@ -1978,7 +1993,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>diana.potesno@colsubsidio.com</t>
+          <t>gestiondecalidad@clinicapalermo.com.co</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1991,7 +2006,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica Colsubsidio Calle 100</t>
+          <t>Oportunidad de Clínica Palermo</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -2000,7 +2015,7 @@
         </is>
       </c>
       <c r="G37" s="1" t="n">
-        <v>46217.51116898148</v>
+        <v>46217.51743055556</v>
       </c>
       <c r="I37" t="n">
         <v>29</v>
@@ -2017,7 +2032,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>diana.potesno@colsubsidio.com</t>
+          <t>calidad@hospitaldesanjose.org.co</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2030,7 +2045,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica Colsubsidio Calle 100</t>
+          <t>Oportunidad de Hospital San José - Sociedad de Cirugía de Bogotá</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2039,7 +2054,7 @@
         </is>
       </c>
       <c r="G38" s="1" t="n">
-        <v>46217.50983796296</v>
+        <v>46217.51425925926</v>
       </c>
       <c r="I38" t="n">
         <v>29</v>
@@ -2056,7 +2071,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>jose.chaves@colsubsidio.com</t>
+          <t>jzapata@ioir.org.co</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2069,7 +2084,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica Colsubsidio Ciudad Roma</t>
+          <t>Oportunidad de Instituto de Ortopedia Infantil Roosevelt</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2078,7 +2093,7 @@
         </is>
       </c>
       <c r="G39" s="1" t="n">
-        <v>46217.50767361111</v>
+        <v>46217.51231481481</v>
       </c>
       <c r="I39" t="n">
         <v>29</v>
@@ -2095,7 +2110,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>carlos.artetamo@colsubsidio.com</t>
+          <t>diana.potesno@colsubsidio.com</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2108,7 +2123,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica Infantil Colsubsidio</t>
+          <t>Oportunidad de Clínica Colsubsidio Calle 100</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -2117,7 +2132,7 @@
         </is>
       </c>
       <c r="G40" s="1" t="n">
-        <v>46217.50050925926</v>
+        <v>46217.51116898148</v>
       </c>
       <c r="I40" t="n">
         <v>29</v>
@@ -2134,7 +2149,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>notificacionescdc@clinicadelcountry.com</t>
+          <t>diana.potesno@colsubsidio.com</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2147,7 +2162,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica del Country IPS</t>
+          <t>Oportunidad de Clínica Colsubsidio Calle 100</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2156,7 +2171,7 @@
         </is>
       </c>
       <c r="G41" s="1" t="n">
-        <v>46217.49881944444</v>
+        <v>46217.50983796296</v>
       </c>
       <c r="I41" t="n">
         <v>29</v>
@@ -2173,7 +2188,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>direcciongeneral@shaio.org</t>
+          <t>jose.chaves@colsubsidio.com</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2186,7 +2201,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Oportunidad de Fundación Abood Shaio</t>
+          <t>Oportunidad de Clínica Colsubsidio Ciudad Roma</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -2195,7 +2210,7 @@
         </is>
       </c>
       <c r="G42" s="1" t="n">
-        <v>46217.49715277777</v>
+        <v>46217.50767361111</v>
       </c>
       <c r="I42" t="n">
         <v>29</v>
@@ -2212,7 +2227,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>direccion@cancer.gov.co</t>
+          <t>carlos.artetamo@colsubsidio.com</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2225,7 +2240,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Oportunidad de Instituto Nacional de Cancerología</t>
+          <t>Oportunidad de Clínica Infantil Colsubsidio</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2234,7 +2249,7 @@
         </is>
       </c>
       <c r="G43" s="1" t="n">
-        <v>46217.47924768519</v>
+        <v>46217.50050925926</v>
       </c>
       <c r="I43" t="n">
         <v>29</v>
@@ -2251,7 +2266,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>sdirmedica@clinicadelamujer.com.co</t>
+          <t>notificacionescdc@clinicadelcountry.com</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2264,7 +2279,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Oportunidad de Clínica de la Mujer</t>
+          <t>Oportunidad de Clínica del Country IPS</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -2273,7 +2288,7 @@
         </is>
       </c>
       <c r="G44" s="1" t="n">
-        <v>46217.47585648148</v>
+        <v>46217.49881944444</v>
       </c>
       <c r="I44" t="n">
         <v>29</v>
@@ -2290,7 +2305,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>lidercalidad@homifundacion.org.co</t>
+          <t>direcciongeneral@shaio.org</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2303,7 +2318,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Oportunidad de Fundación Hospital de la Misericordia (HOMI)</t>
+          <t>Oportunidad de Fundación Abood Shaio</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -2312,7 +2327,7 @@
         </is>
       </c>
       <c r="G45" s="1" t="n">
-        <v>46217.47246527778</v>
+        <v>46217.49715277777</v>
       </c>
       <c r="I45" t="n">
         <v>29</v>
@@ -2329,7 +2344,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>direcciongeneral1@stewardcolombia.org</t>
+          <t>direccion@cancer.gov.co</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2342,7 +2357,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Oportunidad de Hospital Universitario Clínica San Rafael</t>
+          <t>Oportunidad de Instituto Nacional de Cancerología</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2351,7 +2366,7 @@
         </is>
       </c>
       <c r="G46" s="1" t="n">
-        <v>46217.00748842592</v>
+        <v>46217.47924768519</v>
       </c>
       <c r="I46" t="n">
         <v>29</v>
@@ -2368,7 +2383,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>adriana.urrego@fsfb.org.co</t>
+          <t>sdirmedica@clinicadelamujer.com.co</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2381,7 +2396,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Oportunidad de FUNDACION SANTA FE DE BOGOTA</t>
+          <t>Oportunidad de Clínica de la Mujer</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -2390,7 +2405,7 @@
         </is>
       </c>
       <c r="G47" s="1" t="n">
-        <v>46217.00381944444</v>
+        <v>46217.47585648148</v>
       </c>
       <c r="I47" t="n">
         <v>29</v>
@@ -2407,7 +2422,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>calidadsalud@cafam.com.co</t>
+          <t>lidercalidad@homifundacion.org.co</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2420,7 +2435,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Oportunidad de Centro de Atención en Salud CAFAM Clínica Calle 51</t>
+          <t>Oportunidad de Fundación Hospital de la Misericordia (HOMI)</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2429,7 +2444,7 @@
         </is>
       </c>
       <c r="G48" s="1" t="n">
-        <v>46216.99954861111</v>
+        <v>46217.47246527778</v>
       </c>
       <c r="I48" t="n">
         <v>29</v>
@@ -2446,7 +2461,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>notificacionesjudiciales@fhsc.org.co</t>
+          <t>direcciongeneral1@stewardcolombia.org</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2459,7 +2474,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Oportunidad de Fundación Hospital San Carlos</t>
+          <t>Oportunidad de Hospital Universitario Clínica San Rafael</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -2468,7 +2483,7 @@
         </is>
       </c>
       <c r="G49" s="1" t="n">
-        <v>46216.99548611111</v>
+        <v>46217.00748842592</v>
       </c>
       <c r="I49" t="n">
         <v>29</v>
@@ -2485,7 +2500,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>calidad@proseguir.org</t>
+          <t>adriana.urrego@fsfb.org.co</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2498,7 +2513,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Oportunidad de PROSEGUIR SEDE 3</t>
+          <t>Oportunidad de FUNDACION SANTA FE DE BOGOTA</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -2507,7 +2522,7 @@
         </is>
       </c>
       <c r="G50" s="1" t="n">
-        <v>46216.99299768519</v>
+        <v>46217.00381944444</v>
       </c>
       <c r="I50" t="n">
         <v>29</v>
@@ -2524,103 +2539,98 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>centrodecontacto@uao.edu.co</t>
+          <t>calidadsalud@cafam.com.co</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Negociación</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>10000000</v>
+        <v>0</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Oportunidad de UNIVERSIDAD AUTONOMA DE OCCIDENTE</t>
+          <t>Oportunidad de Centro de Atención en Salud CAFAM Clínica Calle 51</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G51" s="1" t="n">
-        <v>46213.49821759259</v>
+        <v>46216.99954861111</v>
       </c>
       <c r="I51" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J51" t="n">
         <v>2026</v>
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>carlos.segovia@warena.co</t>
+          <t>notificacionesjudiciales@fhsc.org.co</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Negociación</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>35000000</v>
+        <v>0</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Oportunidad de W ARENA</t>
+          <t>Oportunidad de Fundación Hospital San Carlos</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Jennifer Hoyos Gallego</t>
+          <t>Brenda Maria Luna Fontalvo</t>
         </is>
       </c>
       <c r="G52" s="1" t="n">
-        <v>46213.49508101852</v>
+        <v>46216.99548611111</v>
       </c>
       <c r="I52" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J52" t="n">
         <v>2026</v>
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>klondono@fundacionwwbcol.org</t>
+          <t>calidad@proseguir.org</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Ganado</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>300000</v>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>Karla Londoño</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Oportunidad de Karla Londoño</t>
+          <t>Oportunidad de PROSEGUIR SEDE 3</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -2629,33 +2639,24 @@
         </is>
       </c>
       <c r="G53" s="1" t="n">
-        <v>46212.51638888889</v>
-      </c>
-      <c r="H53" s="1" t="n">
-        <v>46217</v>
+        <v>46216.99299768519</v>
       </c>
       <c r="I53" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J53" t="n">
         <v>2026</v>
       </c>
-      <c r="K53" t="n">
-        <v>7</v>
-      </c>
-      <c r="L53" t="n">
-        <v>2026</v>
-      </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>ctorres@colcobranzasnacionales.com</t>
+          <t>centrodecontacto@uao.edu.co</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2664,28 +2665,23 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>5000000</v>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>ctorres@colcobranzasnacionales.com</t>
-        </is>
+        <v>10000000</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Oportunidad de ctorres@colcobranzasnacionales.com</t>
+          <t>Oportunidad de UNIVERSIDAD AUTONOMA DE OCCIDENTE</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G54" s="1" t="n">
-        <v>46206.73804398148</v>
+        <v>46213.49821759259</v>
       </c>
       <c r="I54" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J54" t="n">
         <v>2026</v>
@@ -2699,43 +2695,34 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>medifar624@gmail.com</t>
+          <t>carlos.segovia@warena.co</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Ganado</t>
+          <t>Negociación</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>1640000</v>
+        <v>35000000</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Oportunidad de MEDISFARMA SAS</t>
+          <t>Oportunidad de W ARENA</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Brenda Maria Luna Fontalvo</t>
+          <t>Jennifer Hoyos Gallego</t>
         </is>
       </c>
       <c r="G55" s="1" t="n">
-        <v>46203.72597222222</v>
-      </c>
-      <c r="H55" s="1" t="n">
-        <v>46199</v>
+        <v>46213.49508101852</v>
       </c>
       <c r="I55" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J55" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K55" t="n">
-        <v>6</v>
-      </c>
-      <c r="L55" t="n">
         <v>2026</v>
       </c>
       <c r="M55" t="inlineStr">
@@ -2747,25 +2734,25 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>mercadeo@norteysur.co</t>
+          <t>klondono@fundacionwwbcol.org</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Negociación</t>
+          <t>Ganado</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>28190000</v>
+        <v>300000</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Isabella Mesa</t>
+          <t>Karla Londoño</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Oportunidad de Isabella Mesa</t>
+          <t>Oportunidad de Karla Londoño</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -2774,12 +2761,21 @@
         </is>
       </c>
       <c r="G56" s="1" t="n">
-        <v>46191.70076388889</v>
+        <v>46212.51638888889</v>
+      </c>
+      <c r="H56" s="1" t="n">
+        <v>46217</v>
       </c>
       <c r="I56" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="J56" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K56" t="n">
+        <v>7</v>
+      </c>
+      <c r="L56" t="n">
         <v>2026</v>
       </c>
       <c r="M56" t="inlineStr">
@@ -2791,20 +2787,25 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>comercial@asertis.com.co</t>
+          <t>ctorres@colcobranzasnacionales.com</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Negociación</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>0</v>
+        <v>5000000</v>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>ctorres@colcobranzasnacionales.com</t>
+        </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Oportunidad de IMPORTADORA CALI S.A.</t>
+          <t>Oportunidad de ctorres@colcobranzasnacionales.com</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -2813,42 +2814,37 @@
         </is>
       </c>
       <c r="G57" s="1" t="n">
-        <v>46189.67539351852</v>
+        <v>46206.73804398148</v>
       </c>
       <c r="I57" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="J57" t="n">
         <v>2026</v>
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>educacion@360forma.edu.co</t>
+          <t>medifar624@gmail.com</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Ganado</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>0</v>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>Jorge Sanchez / jefe Comercial</t>
-        </is>
+        <v>1640000</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Oportunidad de Jorge Sanchez / jefe Comercial</t>
+          <t>Oportunidad de MEDISFARMA SAS</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -2857,37 +2853,51 @@
         </is>
       </c>
       <c r="G58" s="1" t="n">
-        <v>46189.65077546296</v>
+        <v>46203.72597222222</v>
+      </c>
+      <c r="H58" s="1" t="n">
+        <v>46199</v>
       </c>
       <c r="I58" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="J58" t="n">
         <v>2026</v>
       </c>
+      <c r="K58" t="n">
+        <v>6</v>
+      </c>
+      <c r="L58" t="n">
+        <v>2026</v>
+      </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>directoradjunto@dclass.edu.co</t>
+          <t>mercadeo@norteysur.co</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Negociación</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>0</v>
+        <v>28190000</v>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Isabella Mesa</t>
+        </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Oportunidad de DCLASS ACADEMIA SAS</t>
+          <t>Oportunidad de Isabella Mesa</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -2896,7 +2906,7 @@
         </is>
       </c>
       <c r="G59" s="1" t="n">
-        <v>46189.49674768518</v>
+        <v>46191.70076388889</v>
       </c>
       <c r="I59" t="n">
         <v>25</v>
@@ -2906,14 +2916,14 @@
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Belkis.jimenez@agrauto.com.co</t>
+          <t>comercial@asertis.com.co</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2926,7 +2936,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Oportunidad de AGRICOLA AUTOMOTRIZ SAS / BELKYS JIMENEZ</t>
+          <t>Oportunidad de IMPORTADORA CALI S.A.</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -2935,10 +2945,10 @@
         </is>
       </c>
       <c r="G60" s="1" t="n">
-        <v>46182.67912037037</v>
+        <v>46189.67539351852</v>
       </c>
       <c r="I60" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J60" t="n">
         <v>2026</v>
@@ -2952,7 +2962,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>luisa.baena@automarcali.com</t>
+          <t>educacion@360forma.edu.co</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2965,12 +2975,12 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>luisa.baena@automarcali.com</t>
+          <t>Jorge Sanchez / jefe Comercial</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Oportunidad de luisa.baena@automarcali.com</t>
+          <t>Oportunidad de Jorge Sanchez / jefe Comercial</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -2979,10 +2989,10 @@
         </is>
       </c>
       <c r="G61" s="1" t="n">
-        <v>46182.67809027778</v>
+        <v>46189.65077546296</v>
       </c>
       <c r="I61" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J61" t="n">
         <v>2026</v>
@@ -2996,25 +3006,20 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>directormercadeo@almotores.com</t>
+          <t>directoradjunto@dclass.edu.co</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C62" t="n">
         <v>0</v>
       </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>Viviana Vanegas</t>
-        </is>
-      </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Oportunidad de Viviana Vanegas</t>
+          <t>Oportunidad de DCLASS ACADEMIA SAS</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -3023,10 +3028,10 @@
         </is>
       </c>
       <c r="G62" s="1" t="n">
-        <v>46182.67621527778</v>
+        <v>46189.49674768518</v>
       </c>
       <c r="I62" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J62" t="n">
         <v>2026</v>
@@ -3040,7 +3045,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>xiomara.duran@autopacifico.com.co</t>
+          <t>Belkis.jimenez@agrauto.com.co</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3053,7 +3058,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Oportunidad de xiomara.duran@autopacifico.com.co</t>
+          <t>Oportunidad de AGRICOLA AUTOMOTRIZ SAS / BELKYS JIMENEZ</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -3062,7 +3067,7 @@
         </is>
       </c>
       <c r="G63" s="1" t="n">
-        <v>46182.65815972222</v>
+        <v>46182.67912037037</v>
       </c>
       <c r="I63" t="n">
         <v>24</v>
@@ -3079,12 +3084,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>alejandrosaavedraconde@comfandi.com.co</t>
+          <t>luisa.baena@automarcali.com</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -3092,12 +3097,12 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>ALEJANDRO</t>
+          <t>luisa.baena@automarcali.com</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Oportunidad de ALEJANDRO</t>
+          <t>Oportunidad de luisa.baena@automarcali.com</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -3106,7 +3111,7 @@
         </is>
       </c>
       <c r="G64" s="1" t="n">
-        <v>46182.64278935185</v>
+        <v>46182.67809027778</v>
       </c>
       <c r="I64" t="n">
         <v>24</v>
@@ -3123,20 +3128,25 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>administracion@fiando.com.co</t>
+          <t>directormercadeo@almotores.com</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C65" t="n">
         <v>0</v>
       </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Viviana Vanegas</t>
+        </is>
+      </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Oportunidad de FIANDO LTDA</t>
+          <t>Oportunidad de Viviana Vanegas</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -3145,7 +3155,7 @@
         </is>
       </c>
       <c r="G65" s="1" t="n">
-        <v>46182.61304398148</v>
+        <v>46182.67621527778</v>
       </c>
       <c r="I65" t="n">
         <v>24</v>
@@ -3155,14 +3165,14 @@
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>dgamoneda@productosdrogam.com</t>
+          <t>xiomara.duran@autopacifico.com.co</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -3173,14 +3183,9 @@
       <c r="C66" t="n">
         <v>0</v>
       </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Diego Mauricio Gamoneda </t>
-        </is>
-      </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t xml:space="preserve">Oportunidad de Diego Mauricio Gamoneda </t>
+          <t>Oportunidad de xiomara.duran@autopacifico.com.co</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -3189,10 +3194,10 @@
         </is>
       </c>
       <c r="G66" s="1" t="n">
-        <v>46175.66417824074</v>
+        <v>46182.65815972222</v>
       </c>
       <c r="I66" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J66" t="n">
         <v>2026</v>
@@ -3206,93 +3211,108 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>alexander.rojas@friogan.com</t>
+          <t>alejandrosaavedraconde@comfandi.com.co</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>0</v>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>ALEJANDRO</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Oportunidad de ALEJANDRO</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G67" s="1" t="n">
+        <v>46182.64278935185</v>
+      </c>
+      <c r="I67" t="n">
+        <v>24</v>
+      </c>
+      <c r="J67" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>No calificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>administracion@fiando.com.co</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
           <t>Propuesta</t>
         </is>
       </c>
-      <c r="C67" t="n">
-        <v>10000000</v>
-      </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>Oportunidad de FRIOGAN S.A</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G67" s="1" t="n">
-        <v>46175.63597222222</v>
-      </c>
-      <c r="I67" t="n">
-        <v>23</v>
-      </c>
-      <c r="J67" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M67" t="inlineStr">
+      <c r="C68" t="n">
+        <v>0</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Oportunidad de FIANDO LTDA</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Brenda Maria Luna Fontalvo</t>
+        </is>
+      </c>
+      <c r="G68" s="1" t="n">
+        <v>46182.61304398148</v>
+      </c>
+      <c r="I68" t="n">
+        <v>24</v>
+      </c>
+      <c r="J68" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M68" t="inlineStr">
         <is>
           <t>Calificado</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>Perdido</t>
-        </is>
-      </c>
-      <c r="C68" t="n">
-        <v>0</v>
-      </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>Oportunidad de Agromercados la Montaña</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t>Brenda Maria Luna Fontalvo</t>
-        </is>
-      </c>
-      <c r="G68" s="1" t="n">
-        <v>46175.62239583334</v>
-      </c>
-      <c r="I68" t="n">
-        <v>23</v>
-      </c>
-      <c r="J68" t="n">
-        <v>2026</v>
-      </c>
-      <c r="M68" t="inlineStr">
-        <is>
-          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>juand.rios@alkosto.com.co</t>
+          <t>dgamoneda@productosdrogam.com</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C69" t="n">
         <v>0</v>
       </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Diego Mauricio Gamoneda </t>
+        </is>
+      </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Oportunidad de ALKOSTO</t>
+          <t xml:space="preserve">Oportunidad de Diego Mauricio Gamoneda </t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -3301,7 +3321,7 @@
         </is>
       </c>
       <c r="G69" s="1" t="n">
-        <v>46175.62055555556</v>
+        <v>46175.66417824074</v>
       </c>
       <c r="I69" t="n">
         <v>23</v>
@@ -3318,25 +3338,20 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>gerencia4087@grupo-exito.com</t>
+          <t>alexander.rojas@friogan.com</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>0</v>
-      </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>Grupo exito ‒ 1007386172 - Sneider Quirama</t>
-        </is>
+        <v>10000000</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Oportunidad de Grupo exito</t>
+          <t>Oportunidad de FRIOGAN S.A</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -3345,7 +3360,7 @@
         </is>
       </c>
       <c r="G70" s="1" t="n">
-        <v>46175.61638888889</v>
+        <v>46175.63597222222</v>
       </c>
       <c r="I70" t="n">
         <v>23</v>
@@ -3355,16 +3370,11 @@
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>ldgomez@supertiendascanaveral.com</t>
-        </is>
-      </c>
       <c r="B71" t="inlineStr">
         <is>
           <t>Perdido</t>
@@ -3373,14 +3383,9 @@
       <c r="C71" t="n">
         <v>0</v>
       </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>Luis David Gomez</t>
-        </is>
-      </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Oportunidad de Luis David Gomez</t>
+          <t>Oportunidad de Agromercados la Montaña</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -3389,7 +3394,7 @@
         </is>
       </c>
       <c r="G71" s="1" t="n">
-        <v>46175.60493055556</v>
+        <v>46175.62239583334</v>
       </c>
       <c r="I71" t="n">
         <v>23</v>
@@ -3406,12 +3411,12 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>davida_vanegas@coomeva.com.co</t>
+          <t>juand.rios@alkosto.com.co</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -3419,7 +3424,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Oportunidad de BANCOOMEVA</t>
+          <t>Oportunidad de ALKOSTO</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -3428,7 +3433,7 @@
         </is>
       </c>
       <c r="G72" s="1" t="n">
-        <v>46175.47109953704</v>
+        <v>46175.62055555556</v>
       </c>
       <c r="I72" t="n">
         <v>23</v>
@@ -3445,12 +3450,12 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>alejandro.delgado@filedesk.com.co</t>
+          <t>gerencia4087@grupo-exito.com</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -3458,12 +3463,12 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>AlejandroDelgado</t>
+          <t>Grupo exito ‒ 1007386172 - Sneider Quirama</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Oportunidad de AlejandroDelgado</t>
+          <t>Oportunidad de Grupo exito</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -3472,7 +3477,7 @@
         </is>
       </c>
       <c r="G73" s="1" t="n">
-        <v>46174.71665509259</v>
+        <v>46175.61638888889</v>
       </c>
       <c r="I73" t="n">
         <v>23</v>
@@ -3487,22 +3492,27 @@
       </c>
     </row>
     <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>ldgomez@supertiendascanaveral.com</t>
+        </is>
+      </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>35000000</v>
+        <v>0</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Olga Lucia Hurtado</t>
+          <t>Luis David Gomez</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Oportunidad de Olga Lucia Hurtado</t>
+          <t>Oportunidad de Luis David Gomez</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -3511,37 +3521,37 @@
         </is>
       </c>
       <c r="G74" s="1" t="n">
-        <v>46168.49854166667</v>
+        <v>46175.60493055556</v>
       </c>
       <c r="I74" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="J74" t="n">
         <v>2026</v>
       </c>
       <c r="M74" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>comercial2@felsyn.com</t>
+          <t>davida_vanegas@coomeva.com.co</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Propuesta</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>713400</v>
+        <v>0</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Oportunidad de FONDO DE EMPLEADOS FELSYN</t>
+          <t>Oportunidad de BANCOOMEVA</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -3550,24 +3560,24 @@
         </is>
       </c>
       <c r="G75" s="1" t="n">
-        <v>46163.49130787037</v>
+        <v>46175.47109953704</v>
       </c>
       <c r="I75" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="J75" t="n">
         <v>2026</v>
       </c>
       <c r="M75" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>mercadeo@lasevillana.com.co</t>
+          <t>alejandro.delgado@filedesk.com.co</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -3580,12 +3590,12 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fabio AlbertoGallego García </t>
+          <t>AlejandroDelgado</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t xml:space="preserve">Oportunidad de Fabio AlbertoGallego García </t>
+          <t>Oportunidad de AlejandroDelgado</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -3594,10 +3604,10 @@
         </is>
       </c>
       <c r="G76" s="1" t="n">
-        <v>46162.64569444444</v>
+        <v>46174.71665509259</v>
       </c>
       <c r="I76" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="J76" t="n">
         <v>2026</v>
@@ -3609,22 +3619,22 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>asantiago@stop.com.co</t>
-        </is>
-      </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Contactado</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>0</v>
+        <v>35000000</v>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Olga Lucia Hurtado</t>
+        </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Oportunidad de STOP SAS</t>
+          <t>Oportunidad de Olga Lucia Hurtado</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -3633,42 +3643,37 @@
         </is>
       </c>
       <c r="G77" s="1" t="n">
-        <v>46161.63508101852</v>
+        <v>46168.49854166667</v>
       </c>
       <c r="I77" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="J77" t="n">
         <v>2026</v>
       </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>aestrada@teker.co</t>
+          <t>comercial2@felsyn.com</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Propuesta</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>16914000</v>
-      </c>
-      <c r="D78" t="inlineStr">
-        <is>
-          <t>TEKER SALUD SAS</t>
-        </is>
+        <v>713400</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Oportunidad de TEKER SALUD SAS</t>
+          <t>Oportunidad de FONDO DE EMPLEADOS FELSYN</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -3677,7 +3682,7 @@
         </is>
       </c>
       <c r="G78" s="1" t="n">
-        <v>46161.62922453704</v>
+        <v>46163.49130787037</v>
       </c>
       <c r="I78" t="n">
         <v>21</v>
@@ -3687,11 +3692,16 @@
       </c>
       <c r="M78" t="inlineStr">
         <is>
-          <t>No calificado</t>
+          <t>Calificado</t>
         </is>
       </c>
     </row>
     <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>mercadeo@lasevillana.com.co</t>
+        </is>
+      </c>
       <c r="B79" t="inlineStr">
         <is>
           <t>Contactado</t>
@@ -3700,9 +3710,14 @@
       <c r="C79" t="n">
         <v>0</v>
       </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fabio AlbertoGallego García </t>
+        </is>
+      </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Oportunidad de TIAN IPS SAS</t>
+          <t xml:space="preserve">Oportunidad de Fabio AlbertoGallego García </t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -3711,7 +3726,7 @@
         </is>
       </c>
       <c r="G79" s="1" t="n">
-        <v>46161.61643518518</v>
+        <v>46162.64569444444</v>
       </c>
       <c r="I79" t="n">
         <v>21</v>
@@ -3728,25 +3743,20 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>administración@fullredtotal.com</t>
+          <t>asantiago@stop.com.co</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Perdido</t>
+          <t>Contactado</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>14000000</v>
-      </c>
-      <c r="D80" t="inlineStr">
-        <is>
-          <t>Eivar Eñasco</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Oportunidad de Eivar Eñasco</t>
+          <t>Oportunidad de STOP SAS</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -3755,10 +3765,10 @@
         </is>
       </c>
       <c r="G80" s="1" t="n">
-        <v>46154.67546296296</v>
+        <v>46161.63508101852</v>
       </c>
       <c r="I80" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J80" t="n">
         <v>2026</v>
@@ -3772,25 +3782,25 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>cserna@surtifamiliar.com.co</t>
+          <t>aestrada@teker.co</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Ganado</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>975000</v>
+        <v>16914000</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Claudia Patricia Serna</t>
+          <t>TEKER SALUD SAS</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Oportunidad de Claudia Patricia Serna</t>
+          <t>Oportunidad de TEKER SALUD SAS</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -3799,26 +3809,17 @@
         </is>
       </c>
       <c r="G81" s="1" t="n">
-        <v>46154.66616898148</v>
-      </c>
-      <c r="H81" s="1" t="n">
-        <v>46217</v>
+        <v>46161.62922453704</v>
       </c>
       <c r="I81" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J81" t="n">
         <v>2026</v>
       </c>
-      <c r="K81" t="n">
-        <v>7</v>
-      </c>
-      <c r="L81" t="n">
-        <v>2026</v>
-      </c>
       <c r="M81" t="inlineStr">
         <is>
-          <t>Calificado</t>
+          <t>No calificado</t>
         </is>
       </c>
     </row>

</xml_diff>